<commit_message>
Arquiva dados, recalibra e atualiza docs (2026-07-16)
</commit_message>
<xml_diff>
--- a/backtest_results/resultados_backtest.xlsx
+++ b/backtest_results/resultados_backtest.xlsx
@@ -1,17 +1,17 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Resumo" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Por cidade" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Confiança ≥90%" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Calibração" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Meta" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="Resumo" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Por cidade" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Confiança ≥90%" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Calibração" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Meta" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -516,28 +516,28 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>43</v>
+        <v>50</v>
       </c>
       <c r="C2" s="2" t="n">
-        <v>0.9302325581395349</v>
+        <v>0.9399999999999999</v>
       </c>
       <c r="D2" s="3" t="n">
-        <v>0.9452393026621347</v>
+        <v>1.167035015843559</v>
       </c>
       <c r="E2" s="4" t="n">
-        <v>2.298278417306298</v>
+        <v>2.790558363237093</v>
       </c>
       <c r="F2" s="2" t="n">
-        <v>0.3237961514479204</v>
+        <v>0.3974428553235143</v>
       </c>
       <c r="G2" s="2" t="n">
         <v>0.01500000000000012</v>
       </c>
       <c r="H2" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="I2" s="3" t="n">
-        <v>0.8224302325581395</v>
+        <v>0.81289</v>
       </c>
     </row>
     <row r="3">
@@ -547,28 +547,28 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>605</v>
+        <v>799</v>
       </c>
       <c r="C3" s="2" t="n">
-        <v>0.9933884297520661</v>
+        <v>0.9949937421777222</v>
       </c>
       <c r="D3" s="3" t="n">
-        <v>0.610291547347061</v>
+        <v>0.9108378539494695</v>
       </c>
       <c r="E3" s="4" t="n">
-        <v>1.532243549788371</v>
+        <v>1.824304190053051</v>
       </c>
       <c r="F3" s="2" t="n">
-        <v>0.1547023390404267</v>
+        <v>0.2165792628473568</v>
       </c>
       <c r="G3" s="2" t="n">
-        <v>0.06205548829455021</v>
+        <v>0.05833537351557738</v>
       </c>
       <c r="H3" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="I3" s="3" t="n">
-        <v>0.9857570247933884</v>
+        <v>0.985328535669587</v>
       </c>
     </row>
     <row r="4">
@@ -578,28 +578,28 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>386</v>
+        <v>584</v>
       </c>
       <c r="C4" s="2" t="n">
-        <v>0.9922279792746114</v>
+        <v>0.9948630136986302</v>
       </c>
       <c r="D4" s="3" t="n">
-        <v>0.3344072484430783</v>
+        <v>0.6337816300886023</v>
       </c>
       <c r="E4" s="4" t="n">
-        <v>1.303270782690179</v>
+        <v>1.604346618374838</v>
       </c>
       <c r="F4" s="2" t="n">
-        <v>0.09339158668902825</v>
+        <v>0.1666620371164005</v>
       </c>
       <c r="G4" s="2" t="n">
-        <v>0.05867506981975656</v>
+        <v>0.05450205413924314</v>
       </c>
       <c r="H4" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="I4" s="3" t="n">
-        <v>0.9872279792746114</v>
+        <v>0.9862585616438356</v>
       </c>
     </row>
     <row r="5">
@@ -609,28 +609,28 @@
         </is>
       </c>
       <c r="B5" s="5" t="n">
-        <v>152</v>
+        <v>316</v>
       </c>
       <c r="C5" s="6" t="n">
         <v>1</v>
       </c>
       <c r="D5" s="7" t="n">
-        <v>0.1419116277595212</v>
+        <v>0.375727490456135</v>
       </c>
       <c r="E5" s="8" t="n">
-        <v>1.136926707180735</v>
+        <v>1.386549407279066</v>
       </c>
       <c r="F5" s="6" t="n">
-        <v>0.04420609856527014</v>
+        <v>0.1124570846138906</v>
       </c>
       <c r="G5" s="6" t="n">
-        <v>0.01500000000000001</v>
+        <v>0.01386579723875592</v>
       </c>
       <c r="H5" s="5" t="n">
         <v>2</v>
       </c>
       <c r="I5" s="7" t="n">
-        <v>0.9886250000000001</v>
+        <v>0.9872626582278482</v>
       </c>
     </row>
     <row r="6">
@@ -640,34 +640,34 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>195</v>
+        <v>366</v>
       </c>
       <c r="C6" s="2" t="n">
-        <v>0.9846153846153847</v>
+        <v>0.9918032786885246</v>
       </c>
       <c r="D6" s="3" t="n">
-        <v>1.087150930421656</v>
+        <v>1.542762506299694</v>
       </c>
       <c r="E6" s="4" t="n">
-        <v>2.533519618922796</v>
+        <v>3.526947895152975</v>
       </c>
       <c r="F6" s="2" t="n">
-        <v>0.3680023176452523</v>
+        <v>0.5083415275368819</v>
       </c>
       <c r="G6" s="2" t="n">
-        <v>0.02842499999999992</v>
+        <v>0.02127438923763536</v>
       </c>
       <c r="H6" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="I6" s="3" t="n">
-        <v>0.9519769230769232</v>
+        <v>0.9634412568306011</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Atualizado em 2026-07-13T20:48:50+00:00 · arquivo de 1610 dias-cidade (~89 dias corridos) · 18 cidades</t>
+          <t>Atualizado em 2026-07-16T09:05:53+00:00 · arquivo de 1664 dias-cidade (~92 dias corridos) · 18 cidades</t>
         </is>
       </c>
     </row>
@@ -801,13 +801,13 @@
         </is>
       </c>
       <c r="C5" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="D5" s="2" t="n">
-        <v>0.5</v>
+        <v>0.75</v>
       </c>
       <c r="E5" s="3" t="n">
-        <v>0.04003875968992247</v>
+        <v>0.1297630704668648</v>
       </c>
     </row>
     <row r="6">
@@ -948,13 +948,13 @@
         </is>
       </c>
       <c r="C12" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="D12" s="2" t="n">
         <v>1</v>
       </c>
       <c r="E12" s="3" t="n">
-        <v>0.013021778584392</v>
+        <v>0.1246779442009537</v>
       </c>
     </row>
     <row r="13">
@@ -969,13 +969,13 @@
         </is>
       </c>
       <c r="C13" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="D13" s="2" t="n">
         <v>1</v>
       </c>
       <c r="E13" s="3" t="n">
-        <v>0.3453851615193468</v>
+        <v>0.359417419583863</v>
       </c>
     </row>
     <row r="14">
@@ -1032,13 +1032,13 @@
         </is>
       </c>
       <c r="C16" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D16" s="2" t="n">
         <v>1</v>
       </c>
       <c r="E16" s="3" t="n">
-        <v>0.05236838018325828</v>
+        <v>0.05875135890666253</v>
       </c>
     </row>
     <row r="17">
@@ -1053,13 +1053,13 @@
         </is>
       </c>
       <c r="C17" t="n">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="D17" s="2" t="n">
-        <v>0.9166666666666666</v>
+        <v>0.9285714285714286</v>
       </c>
       <c r="E17" s="3" t="n">
-        <v>0.001126628647129417</v>
+        <v>0.00526332678942815</v>
       </c>
     </row>
     <row r="18">
@@ -1074,13 +1074,13 @@
         </is>
       </c>
       <c r="C18" t="n">
-        <v>19</v>
+        <v>28</v>
       </c>
       <c r="D18" s="2" t="n">
         <v>1</v>
       </c>
       <c r="E18" s="3" t="n">
-        <v>0.0479095129217771</v>
+        <v>0.06388759741877117</v>
       </c>
     </row>
     <row r="19">
@@ -1095,13 +1095,13 @@
         </is>
       </c>
       <c r="C19" t="n">
-        <v>23</v>
+        <v>42</v>
       </c>
       <c r="D19" s="2" t="n">
         <v>1</v>
       </c>
       <c r="E19" s="3" t="n">
-        <v>0.0222035787522157</v>
+        <v>0.0470542006317368</v>
       </c>
     </row>
     <row r="20">
@@ -1116,13 +1116,13 @@
         </is>
       </c>
       <c r="C20" t="n">
-        <v>9</v>
+        <v>14</v>
       </c>
       <c r="D20" s="2" t="n">
-        <v>0.8888888888888888</v>
+        <v>0.9285714285714286</v>
       </c>
       <c r="E20" s="3" t="n">
-        <v>0.04735313115653037</v>
+        <v>0.1439081708138227</v>
       </c>
     </row>
     <row r="21">
@@ -1137,13 +1137,13 @@
         </is>
       </c>
       <c r="C21" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D21" s="2" t="n">
         <v>1</v>
       </c>
       <c r="E21" s="3" t="n">
-        <v>0.00442641974059972</v>
+        <v>0.005385531300417991</v>
       </c>
     </row>
     <row r="22">
@@ -1158,13 +1158,13 @@
         </is>
       </c>
       <c r="C22" t="n">
-        <v>3</v>
+        <v>7</v>
       </c>
       <c r="D22" s="2" t="n">
         <v>1</v>
       </c>
       <c r="E22" s="3" t="n">
-        <v>0.003244057280757295</v>
+        <v>0.009569509080958683</v>
       </c>
     </row>
     <row r="23">
@@ -1179,13 +1179,13 @@
         </is>
       </c>
       <c r="C23" t="n">
-        <v>29</v>
+        <v>48</v>
       </c>
       <c r="D23" s="2" t="n">
         <v>1</v>
       </c>
       <c r="E23" s="3" t="n">
-        <v>0.1010788596880604</v>
+        <v>0.1324955366147939</v>
       </c>
     </row>
     <row r="24">
@@ -1200,13 +1200,13 @@
         </is>
       </c>
       <c r="C24" t="n">
-        <v>7</v>
+        <v>15</v>
       </c>
       <c r="D24" s="2" t="n">
-        <v>0.8571428571428571</v>
+        <v>0.9333333333333333</v>
       </c>
       <c r="E24" s="3" t="n">
-        <v>0.0001540608447643408</v>
+        <v>0.008152139544279196</v>
       </c>
     </row>
     <row r="25">
@@ -1221,13 +1221,13 @@
         </is>
       </c>
       <c r="C25" t="n">
-        <v>9</v>
+        <v>31</v>
       </c>
       <c r="D25" s="2" t="n">
         <v>1</v>
       </c>
       <c r="E25" s="3" t="n">
-        <v>0.03612824745940195</v>
+        <v>0.06882017260898085</v>
       </c>
     </row>
     <row r="26">
@@ -1242,13 +1242,13 @@
         </is>
       </c>
       <c r="C26" t="n">
-        <v>14</v>
+        <v>29</v>
       </c>
       <c r="D26" s="2" t="n">
         <v>1</v>
       </c>
       <c r="E26" s="3" t="n">
-        <v>0.1294413161520027</v>
+        <v>0.149150473154086</v>
       </c>
     </row>
     <row r="27">
@@ -1284,13 +1284,13 @@
         </is>
       </c>
       <c r="C28" t="n">
-        <v>8</v>
+        <v>21</v>
       </c>
       <c r="D28" s="2" t="n">
         <v>1</v>
       </c>
       <c r="E28" s="3" t="n">
-        <v>0.09834929017629578</v>
+        <v>0.12045292685178</v>
       </c>
     </row>
     <row r="29">
@@ -1305,13 +1305,13 @@
         </is>
       </c>
       <c r="C29" t="n">
-        <v>12</v>
+        <v>34</v>
       </c>
       <c r="D29" s="2" t="n">
         <v>1</v>
       </c>
       <c r="E29" s="3" t="n">
-        <v>0.02375437679063087</v>
+        <v>0.1643362114715348</v>
       </c>
     </row>
     <row r="30">
@@ -1326,13 +1326,13 @@
         </is>
       </c>
       <c r="C30" t="n">
-        <v>19</v>
+        <v>26</v>
       </c>
       <c r="D30" s="2" t="n">
         <v>1</v>
       </c>
       <c r="E30" s="3" t="n">
-        <v>0.3611268961512431</v>
+        <v>0.3824485469655075</v>
       </c>
     </row>
     <row r="31">
@@ -1347,13 +1347,13 @@
         </is>
       </c>
       <c r="C31" t="n">
-        <v>4</v>
+        <v>15</v>
       </c>
       <c r="D31" s="2" t="n">
         <v>1</v>
       </c>
       <c r="E31" s="3" t="n">
-        <v>0.07741719247522236</v>
+        <v>0.08584108705952805</v>
       </c>
     </row>
     <row r="32">
@@ -1389,13 +1389,13 @@
         </is>
       </c>
       <c r="C33" t="n">
-        <v>8</v>
+        <v>22</v>
       </c>
       <c r="D33" s="2" t="n">
         <v>1</v>
       </c>
       <c r="E33" s="3" t="n">
-        <v>0.05808558576517504</v>
+        <v>0.08064529957421883</v>
       </c>
     </row>
   </sheetData>
@@ -1447,13 +1447,13 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>902</v>
+        <v>923</v>
       </c>
       <c r="C2" s="2" t="n">
-        <v>0.8681</v>
+        <v>0.8711</v>
       </c>
       <c r="D2" s="2" t="n">
-        <v>0.9926</v>
+        <v>0.9923</v>
       </c>
     </row>
     <row r="3">
@@ -1463,13 +1463,13 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>908</v>
+        <v>930</v>
       </c>
       <c r="C3" s="2" t="n">
-        <v>0.8601</v>
+        <v>0.8633999999999999</v>
       </c>
       <c r="D3" s="2" t="n">
-        <v>0.9955000000000001</v>
+        <v>0.9952</v>
       </c>
     </row>
     <row r="4">
@@ -1479,13 +1479,13 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>929</v>
+        <v>957</v>
       </c>
       <c r="C4" s="2" t="n">
-        <v>0.8665</v>
+        <v>0.8704</v>
       </c>
       <c r="D4" s="2" t="n">
-        <v>0.9961</v>
+        <v>0.9957</v>
       </c>
     </row>
     <row r="5">
@@ -1495,13 +1495,13 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>924</v>
+        <v>951</v>
       </c>
       <c r="C5" s="2" t="n">
-        <v>0.8582</v>
+        <v>0.8623</v>
       </c>
       <c r="D5" s="2" t="n">
-        <v>0.9974</v>
+        <v>0.9969</v>
       </c>
     </row>
     <row r="6">
@@ -1511,13 +1511,13 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>948</v>
+        <v>972</v>
       </c>
       <c r="C6" s="2" t="n">
-        <v>0.8386</v>
+        <v>0.8426</v>
       </c>
       <c r="D6" s="2" t="n">
-        <v>0.9976</v>
+        <v>0.9975000000000001</v>
       </c>
     </row>
     <row r="7">
@@ -1527,13 +1527,13 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>927</v>
+        <v>948</v>
       </c>
       <c r="C7" s="2" t="n">
-        <v>0.8511</v>
+        <v>0.8544</v>
       </c>
       <c r="D7" s="2" t="n">
-        <v>0.9976</v>
+        <v>0.9972</v>
       </c>
     </row>
     <row r="8">
@@ -1543,13 +1543,13 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>949</v>
+        <v>972</v>
       </c>
       <c r="C8" s="2" t="n">
-        <v>0.8367</v>
+        <v>0.8405</v>
       </c>
       <c r="D8" s="2" t="n">
-        <v>0.9976</v>
+        <v>0.9971</v>
       </c>
     </row>
     <row r="9">
@@ -1559,13 +1559,13 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>887</v>
+        <v>906</v>
       </c>
       <c r="C9" s="2" t="n">
-        <v>0.8963</v>
+        <v>0.8985</v>
       </c>
       <c r="D9" s="2" t="n">
-        <v>0.992</v>
+        <v>0.9917</v>
       </c>
     </row>
     <row r="10">
@@ -1575,13 +1575,13 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>863</v>
+        <v>883</v>
       </c>
       <c r="C10" s="2" t="n">
-        <v>0.8667</v>
+        <v>0.8698</v>
       </c>
       <c r="D10" s="2" t="n">
-        <v>0.9931</v>
+        <v>0.9923</v>
       </c>
     </row>
     <row r="11">
@@ -1591,13 +1591,13 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>878</v>
+        <v>908</v>
       </c>
       <c r="C11" s="2" t="n">
-        <v>0.9237</v>
+        <v>0.9262</v>
       </c>
       <c r="D11" s="2" t="n">
-        <v>0.9939</v>
+        <v>0.9937</v>
       </c>
     </row>
     <row r="12">
@@ -1607,13 +1607,13 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>879</v>
+        <v>902</v>
       </c>
       <c r="C12" s="2" t="n">
-        <v>0.909</v>
+        <v>0.9113</v>
       </c>
       <c r="D12" s="2" t="n">
-        <v>0.9885</v>
+        <v>0.9881</v>
       </c>
     </row>
     <row r="13">
@@ -1623,13 +1623,13 @@
         </is>
       </c>
       <c r="B13" t="n">
-        <v>874</v>
+        <v>895</v>
       </c>
       <c r="C13" s="2" t="n">
-        <v>0.897</v>
+        <v>0.8994</v>
       </c>
       <c r="D13" s="2" t="n">
-        <v>0.9877</v>
+        <v>0.9873</v>
       </c>
     </row>
     <row r="14">
@@ -1639,13 +1639,13 @@
         </is>
       </c>
       <c r="B14" t="n">
-        <v>861</v>
+        <v>887</v>
       </c>
       <c r="C14" s="2" t="n">
-        <v>0.8663999999999999</v>
+        <v>0.8692</v>
       </c>
       <c r="D14" s="2" t="n">
-        <v>0.9939</v>
+        <v>0.9933</v>
       </c>
     </row>
     <row r="15">
@@ -1655,13 +1655,13 @@
         </is>
       </c>
       <c r="B15" t="n">
-        <v>903</v>
+        <v>929</v>
       </c>
       <c r="C15" s="2" t="n">
-        <v>0.8616</v>
+        <v>0.8653999999999999</v>
       </c>
       <c r="D15" s="2" t="n">
-        <v>0.9946</v>
+        <v>0.9941</v>
       </c>
     </row>
     <row r="16">
@@ -1671,13 +1671,13 @@
         </is>
       </c>
       <c r="B16" t="n">
-        <v>884</v>
+        <v>911</v>
       </c>
       <c r="C16" s="2" t="n">
-        <v>0.8676</v>
+        <v>0.8716</v>
       </c>
       <c r="D16" s="2" t="n">
-        <v>0.9908</v>
+        <v>0.9905</v>
       </c>
     </row>
     <row r="17">
@@ -1687,13 +1687,13 @@
         </is>
       </c>
       <c r="B17" t="n">
-        <v>849</v>
+        <v>875</v>
       </c>
       <c r="C17" s="2" t="n">
-        <v>0.9117</v>
+        <v>0.9143</v>
       </c>
       <c r="D17" s="2" t="n">
-        <v>0.9922</v>
+        <v>0.9919</v>
       </c>
     </row>
     <row r="18">
@@ -1703,13 +1703,13 @@
         </is>
       </c>
       <c r="B18" t="n">
-        <v>931</v>
+        <v>952</v>
       </c>
       <c r="C18" s="2" t="n">
-        <v>0.8539</v>
+        <v>0.8571</v>
       </c>
       <c r="D18" s="2" t="n">
-        <v>0.9975000000000001</v>
+        <v>0.9969</v>
       </c>
     </row>
     <row r="19">
@@ -1719,13 +1719,13 @@
         </is>
       </c>
       <c r="B19" t="n">
-        <v>922</v>
+        <v>947</v>
       </c>
       <c r="C19" s="2" t="n">
-        <v>0.8807</v>
+        <v>0.8828</v>
       </c>
       <c r="D19" s="2" t="n">
-        <v>0.9923</v>
+        <v>0.9917</v>
       </c>
     </row>
   </sheetData>
@@ -1789,19 +1789,19 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>0.142</v>
+        <v>0.1393</v>
       </c>
       <c r="C2" t="n">
-        <v>0.142</v>
+        <v>0.1393</v>
       </c>
       <c r="D2" t="n">
-        <v>1.4745</v>
+        <v>0.0094</v>
       </c>
       <c r="E2" t="n">
-        <v>-0.1847</v>
+        <v>1.0582</v>
       </c>
       <c r="F2" t="n">
-        <v>0.1825</v>
+        <v>0.0721</v>
       </c>
     </row>
     <row r="3">
@@ -1811,19 +1811,19 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>0.135</v>
+        <v>0.132</v>
       </c>
       <c r="C3" t="n">
-        <v>0.1243</v>
+        <v>0.1223</v>
       </c>
       <c r="D3" t="n">
-        <v>0.001</v>
+        <v>0.0026</v>
       </c>
       <c r="E3" t="n">
-        <v>1.0602</v>
+        <v>1.0596</v>
       </c>
       <c r="F3" t="n">
-        <v>0.0799</v>
+        <v>0.0798</v>
       </c>
     </row>
     <row r="4">
@@ -1833,19 +1833,19 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>0.0456</v>
+        <v>0.0449</v>
       </c>
       <c r="C4" t="n">
-        <v>0.0396</v>
+        <v>0.0387</v>
       </c>
       <c r="D4" t="n">
-        <v>0.111</v>
+        <v>0.1206</v>
       </c>
       <c r="E4" t="n">
-        <v>0.9853</v>
+        <v>0.9749</v>
       </c>
       <c r="F4" t="n">
-        <v>0.0604</v>
+        <v>0.0608</v>
       </c>
     </row>
   </sheetData>
@@ -1874,7 +1874,7 @@
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>2026-07-13T20:48:50+00:00</t>
+          <t>2026-07-16T09:05:53+00:00</t>
         </is>
       </c>
     </row>
@@ -1885,7 +1885,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>1610</v>
+        <v>1664</v>
       </c>
     </row>
     <row r="3">
@@ -1895,7 +1895,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>89</v>
+        <v>92</v>
       </c>
     </row>
     <row r="4">

</xml_diff>

<commit_message>
Arquiva dados, recalibra e atualiza docs (2026-07-19)
</commit_message>
<xml_diff>
--- a/backtest_results/resultados_backtest.xlsx
+++ b/backtest_results/resultados_backtest.xlsx
@@ -516,19 +516,19 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>50</v>
+        <v>54</v>
       </c>
       <c r="C2" s="2" t="n">
-        <v>0.9399999999999999</v>
+        <v>0.9444444444444444</v>
       </c>
       <c r="D2" s="3" t="n">
-        <v>1.167035015843559</v>
+        <v>1.211494616704504</v>
       </c>
       <c r="E2" s="4" t="n">
-        <v>2.790558363237093</v>
+        <v>2.909810215614418</v>
       </c>
       <c r="F2" s="2" t="n">
-        <v>0.3974428553235143</v>
+        <v>0.4011466028965043</v>
       </c>
       <c r="G2" s="2" t="n">
         <v>0.01500000000000012</v>
@@ -537,7 +537,7 @@
         <v>5</v>
       </c>
       <c r="I2" s="3" t="n">
-        <v>0.81289</v>
+        <v>0.8193981481481482</v>
       </c>
     </row>
     <row r="3">
@@ -547,19 +547,19 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>799</v>
+        <v>810</v>
       </c>
       <c r="C3" s="2" t="n">
-        <v>0.9949937421777222</v>
+        <v>0.9950617283950617</v>
       </c>
       <c r="D3" s="3" t="n">
-        <v>0.9108378539494695</v>
+        <v>0.9244216055834175</v>
       </c>
       <c r="E3" s="4" t="n">
-        <v>1.824304190053051</v>
+        <v>1.845107080764028</v>
       </c>
       <c r="F3" s="2" t="n">
-        <v>0.2165792628473568</v>
+        <v>0.2134078865496956</v>
       </c>
       <c r="G3" s="2" t="n">
         <v>0.05833537351557738</v>
@@ -568,7 +568,7 @@
         <v>17</v>
       </c>
       <c r="I3" s="3" t="n">
-        <v>0.985328535669587</v>
+        <v>0.9853623456790124</v>
       </c>
     </row>
     <row r="4">
@@ -578,19 +578,19 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>584</v>
+        <v>592</v>
       </c>
       <c r="C4" s="2" t="n">
-        <v>0.9948630136986302</v>
+        <v>0.9949324324324325</v>
       </c>
       <c r="D4" s="3" t="n">
-        <v>0.6337816300886023</v>
+        <v>0.6432573461737613</v>
       </c>
       <c r="E4" s="4" t="n">
-        <v>1.604346618374838</v>
+        <v>1.618144640085836</v>
       </c>
       <c r="F4" s="2" t="n">
-        <v>0.1666620371164005</v>
+        <v>0.164140706524158</v>
       </c>
       <c r="G4" s="2" t="n">
         <v>0.05450205413924314</v>
@@ -599,7 +599,7 @@
         <v>11</v>
       </c>
       <c r="I4" s="3" t="n">
-        <v>0.9862585616438356</v>
+        <v>0.9862863175675675</v>
       </c>
     </row>
     <row r="5">
@@ -609,28 +609,28 @@
         </is>
       </c>
       <c r="B5" s="5" t="n">
-        <v>316</v>
+        <v>320</v>
       </c>
       <c r="C5" s="6" t="n">
         <v>1</v>
       </c>
       <c r="D5" s="7" t="n">
-        <v>0.375727490456135</v>
+        <v>0.3809635051512486</v>
       </c>
       <c r="E5" s="8" t="n">
-        <v>1.386549407279066</v>
+        <v>1.392274030837791</v>
       </c>
       <c r="F5" s="6" t="n">
-        <v>0.1124570846138906</v>
+        <v>0.1101630143863725</v>
       </c>
       <c r="G5" s="6" t="n">
-        <v>0.01386579723875592</v>
+        <v>0.01386579723875603</v>
       </c>
       <c r="H5" s="5" t="n">
         <v>2</v>
       </c>
       <c r="I5" s="7" t="n">
-        <v>0.9872626582278482</v>
+        <v>0.9872609375</v>
       </c>
     </row>
     <row r="6">
@@ -640,34 +640,34 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>366</v>
+        <v>374</v>
       </c>
       <c r="C6" s="2" t="n">
-        <v>0.9918032786885246</v>
+        <v>0.9919786096256684</v>
       </c>
       <c r="D6" s="3" t="n">
-        <v>1.542762506299694</v>
+        <v>1.592458121855753</v>
       </c>
       <c r="E6" s="4" t="n">
-        <v>3.526947895152975</v>
+        <v>3.688480226999131</v>
       </c>
       <c r="F6" s="2" t="n">
-        <v>0.5083415275368819</v>
+        <v>0.5100956653419606</v>
       </c>
       <c r="G6" s="2" t="n">
-        <v>0.02127438923763536</v>
+        <v>0.02127438923763525</v>
       </c>
       <c r="H6" t="n">
         <v>7</v>
       </c>
       <c r="I6" s="3" t="n">
-        <v>0.9634412568306011</v>
+        <v>0.963024064171123</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Atualizado em 2026-07-16T09:05:53+00:00 · arquivo de 1664 dias-cidade (~92 dias corridos) · 18 cidades</t>
+          <t>Atualizado em 2026-07-19T09:06:05+00:00 · arquivo de 1718 dias-cidade (~95 dias corridos) · 18 cidades</t>
         </is>
       </c>
     </row>
@@ -780,13 +780,13 @@
         </is>
       </c>
       <c r="C4" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="D4" s="2" t="n">
         <v>1</v>
       </c>
       <c r="E4" s="3" t="n">
-        <v>0.01745987540471589</v>
+        <v>0.02881845001496088</v>
       </c>
     </row>
     <row r="5">
@@ -885,13 +885,13 @@
         </is>
       </c>
       <c r="C9" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="D9" s="2" t="n">
         <v>1</v>
       </c>
       <c r="E9" s="3" t="n">
-        <v>0.116414868833568</v>
+        <v>0.1339089586680833</v>
       </c>
     </row>
     <row r="10">
@@ -927,13 +927,13 @@
         </is>
       </c>
       <c r="C11" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="D11" s="2" t="n">
         <v>1</v>
       </c>
       <c r="E11" s="3" t="n">
-        <v>0.09552888816451663</v>
+        <v>0.1111358245807016</v>
       </c>
     </row>
     <row r="12">
@@ -1053,13 +1053,13 @@
         </is>
       </c>
       <c r="C17" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="D17" s="2" t="n">
-        <v>0.9285714285714286</v>
+        <v>0.9333333333333333</v>
       </c>
       <c r="E17" s="3" t="n">
-        <v>0.00526332678942815</v>
+        <v>0.007722343182870766</v>
       </c>
     </row>
     <row r="18">
@@ -1095,13 +1095,13 @@
         </is>
       </c>
       <c r="C19" t="n">
-        <v>42</v>
+        <v>44</v>
       </c>
       <c r="D19" s="2" t="n">
         <v>1</v>
       </c>
       <c r="E19" s="3" t="n">
-        <v>0.0470542006317368</v>
+        <v>0.05952500982236602</v>
       </c>
     </row>
     <row r="20">
@@ -1242,13 +1242,13 @@
         </is>
       </c>
       <c r="C26" t="n">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="D26" s="2" t="n">
         <v>1</v>
       </c>
       <c r="E26" s="3" t="n">
-        <v>0.149150473154086</v>
+        <v>0.1666445629886013</v>
       </c>
     </row>
     <row r="27">
@@ -1284,13 +1284,13 @@
         </is>
       </c>
       <c r="C28" t="n">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="D28" s="2" t="n">
         <v>1</v>
       </c>
       <c r="E28" s="3" t="n">
-        <v>0.12045292685178</v>
+        <v>0.1366634849983473</v>
       </c>
     </row>
     <row r="29">
@@ -1326,13 +1326,13 @@
         </is>
       </c>
       <c r="C30" t="n">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="D30" s="2" t="n">
         <v>1</v>
       </c>
       <c r="E30" s="3" t="n">
-        <v>0.3824485469655075</v>
+        <v>0.383509688956412</v>
       </c>
     </row>
     <row r="31">
@@ -1447,13 +1447,13 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>923</v>
+        <v>943</v>
       </c>
       <c r="C2" s="2" t="n">
-        <v>0.8711</v>
+        <v>0.8727</v>
       </c>
       <c r="D2" s="2" t="n">
-        <v>0.9923</v>
+        <v>0.992</v>
       </c>
     </row>
     <row r="3">
@@ -1463,13 +1463,13 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>930</v>
+        <v>952</v>
       </c>
       <c r="C3" s="2" t="n">
-        <v>0.8633999999999999</v>
+        <v>0.8666</v>
       </c>
       <c r="D3" s="2" t="n">
-        <v>0.9952</v>
+        <v>0.9949</v>
       </c>
     </row>
     <row r="4">
@@ -1479,13 +1479,13 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>957</v>
+        <v>982</v>
       </c>
       <c r="C4" s="2" t="n">
-        <v>0.8704</v>
+        <v>0.8737</v>
       </c>
       <c r="D4" s="2" t="n">
-        <v>0.9957</v>
+        <v>0.9953</v>
       </c>
     </row>
     <row r="5">
@@ -1495,13 +1495,13 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>951</v>
+        <v>976</v>
       </c>
       <c r="C5" s="2" t="n">
-        <v>0.8623</v>
+        <v>0.8658</v>
       </c>
       <c r="D5" s="2" t="n">
-        <v>0.9969</v>
+        <v>0.9964</v>
       </c>
     </row>
     <row r="6">
@@ -1511,13 +1511,13 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>972</v>
+        <v>996</v>
       </c>
       <c r="C6" s="2" t="n">
-        <v>0.8426</v>
+        <v>0.8464</v>
       </c>
       <c r="D6" s="2" t="n">
-        <v>0.9975000000000001</v>
+        <v>0.9974</v>
       </c>
     </row>
     <row r="7">
@@ -1527,13 +1527,13 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>948</v>
+        <v>969</v>
       </c>
       <c r="C7" s="2" t="n">
-        <v>0.8544</v>
+        <v>0.8576</v>
       </c>
       <c r="D7" s="2" t="n">
-        <v>0.9972</v>
+        <v>0.997</v>
       </c>
     </row>
     <row r="8">
@@ -1543,13 +1543,13 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>972</v>
+        <v>993</v>
       </c>
       <c r="C8" s="2" t="n">
-        <v>0.8405</v>
+        <v>0.8439</v>
       </c>
       <c r="D8" s="2" t="n">
-        <v>0.9971</v>
+        <v>0.9968</v>
       </c>
     </row>
     <row r="9">
@@ -1559,13 +1559,13 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>906</v>
+        <v>926</v>
       </c>
       <c r="C9" s="2" t="n">
         <v>0.8985</v>
       </c>
       <c r="D9" s="2" t="n">
-        <v>0.9917</v>
+        <v>0.9912</v>
       </c>
     </row>
     <row r="10">
@@ -1575,13 +1575,13 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>883</v>
+        <v>902</v>
       </c>
       <c r="C10" s="2" t="n">
-        <v>0.8698</v>
+        <v>0.8725000000000001</v>
       </c>
       <c r="D10" s="2" t="n">
-        <v>0.9923</v>
+        <v>0.9913999999999999</v>
       </c>
     </row>
     <row r="11">
@@ -1591,13 +1591,13 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>908</v>
+        <v>937</v>
       </c>
       <c r="C11" s="2" t="n">
-        <v>0.9262</v>
+        <v>0.9274</v>
       </c>
       <c r="D11" s="2" t="n">
-        <v>0.9937</v>
+        <v>0.9935</v>
       </c>
     </row>
     <row r="12">
@@ -1607,13 +1607,13 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>902</v>
+        <v>925</v>
       </c>
       <c r="C12" s="2" t="n">
-        <v>0.9113</v>
+        <v>0.9124</v>
       </c>
       <c r="D12" s="2" t="n">
-        <v>0.9881</v>
+        <v>0.9878</v>
       </c>
     </row>
     <row r="13">
@@ -1623,10 +1623,10 @@
         </is>
       </c>
       <c r="B13" t="n">
-        <v>895</v>
+        <v>916</v>
       </c>
       <c r="C13" s="2" t="n">
-        <v>0.8994</v>
+        <v>0.9016999999999999</v>
       </c>
       <c r="D13" s="2" t="n">
         <v>0.9873</v>
@@ -1639,13 +1639,13 @@
         </is>
       </c>
       <c r="B14" t="n">
-        <v>887</v>
+        <v>914</v>
       </c>
       <c r="C14" s="2" t="n">
-        <v>0.8692</v>
+        <v>0.8731</v>
       </c>
       <c r="D14" s="2" t="n">
-        <v>0.9933</v>
+        <v>0.9928</v>
       </c>
     </row>
     <row r="15">
@@ -1655,13 +1655,13 @@
         </is>
       </c>
       <c r="B15" t="n">
-        <v>929</v>
+        <v>951</v>
       </c>
       <c r="C15" s="2" t="n">
-        <v>0.8653999999999999</v>
+        <v>0.8686</v>
       </c>
       <c r="D15" s="2" t="n">
-        <v>0.9941</v>
+        <v>0.9938</v>
       </c>
     </row>
     <row r="16">
@@ -1671,13 +1671,13 @@
         </is>
       </c>
       <c r="B16" t="n">
-        <v>911</v>
+        <v>935</v>
       </c>
       <c r="C16" s="2" t="n">
-        <v>0.8716</v>
+        <v>0.8738</v>
       </c>
       <c r="D16" s="2" t="n">
-        <v>0.9905</v>
+        <v>0.9902</v>
       </c>
     </row>
     <row r="17">
@@ -1687,13 +1687,13 @@
         </is>
       </c>
       <c r="B17" t="n">
-        <v>875</v>
+        <v>900</v>
       </c>
       <c r="C17" s="2" t="n">
-        <v>0.9143</v>
+        <v>0.9167</v>
       </c>
       <c r="D17" s="2" t="n">
-        <v>0.9919</v>
+        <v>0.9916</v>
       </c>
     </row>
     <row r="18">
@@ -1703,13 +1703,13 @@
         </is>
       </c>
       <c r="B18" t="n">
-        <v>952</v>
+        <v>971</v>
       </c>
       <c r="C18" s="2" t="n">
-        <v>0.8571</v>
+        <v>0.8599</v>
       </c>
       <c r="D18" s="2" t="n">
-        <v>0.9969</v>
+        <v>0.9966</v>
       </c>
     </row>
     <row r="19">
@@ -1719,13 +1719,13 @@
         </is>
       </c>
       <c r="B19" t="n">
-        <v>947</v>
+        <v>971</v>
       </c>
       <c r="C19" s="2" t="n">
-        <v>0.8828</v>
+        <v>0.8847</v>
       </c>
       <c r="D19" s="2" t="n">
-        <v>0.9917</v>
+        <v>0.9913</v>
       </c>
     </row>
   </sheetData>
@@ -1789,19 +1789,19 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>0.1393</v>
+        <v>0.1372</v>
       </c>
       <c r="C2" t="n">
-        <v>0.1393</v>
+        <v>0.1372</v>
       </c>
       <c r="D2" t="n">
-        <v>0.0094</v>
+        <v>1.2781</v>
       </c>
       <c r="E2" t="n">
-        <v>1.0582</v>
+        <v>-0.6977</v>
       </c>
       <c r="F2" t="n">
-        <v>0.0721</v>
+        <v>0.2158</v>
       </c>
     </row>
     <row r="3">
@@ -1811,19 +1811,19 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>0.132</v>
+        <v>0.1305</v>
       </c>
       <c r="C3" t="n">
-        <v>0.1223</v>
+        <v>0.1207</v>
       </c>
       <c r="D3" t="n">
-        <v>0.0026</v>
+        <v>0.0036</v>
       </c>
       <c r="E3" t="n">
-        <v>1.0596</v>
+        <v>1.0469</v>
       </c>
       <c r="F3" t="n">
-        <v>0.0798</v>
+        <v>0.08069999999999999</v>
       </c>
     </row>
     <row r="4">
@@ -1833,19 +1833,19 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>0.0449</v>
+        <v>0.0445</v>
       </c>
       <c r="C4" t="n">
-        <v>0.0387</v>
+        <v>0.0386</v>
       </c>
       <c r="D4" t="n">
-        <v>0.1206</v>
+        <v>0.1218</v>
       </c>
       <c r="E4" t="n">
-        <v>0.9749</v>
+        <v>0.9756</v>
       </c>
       <c r="F4" t="n">
-        <v>0.0608</v>
+        <v>0.0609</v>
       </c>
     </row>
   </sheetData>
@@ -1874,7 +1874,7 @@
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>2026-07-16T09:05:53+00:00</t>
+          <t>2026-07-19T09:06:05+00:00</t>
         </is>
       </c>
     </row>
@@ -1885,7 +1885,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>1664</v>
+        <v>1718</v>
       </c>
     </row>
     <row r="3">
@@ -1895,7 +1895,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>92</v>
+        <v>95</v>
       </c>
     </row>
     <row r="4">
@@ -1925,7 +1925,7 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>42</v>
+        <v>44</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Arquiva dados, recalibra e atualiza docs (2026-07-25)
</commit_message>
<xml_diff>
--- a/backtest_results/resultados_backtest.xlsx
+++ b/backtest_results/resultados_backtest.xlsx
@@ -516,28 +516,28 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>57</v>
+        <v>94</v>
       </c>
       <c r="C2" s="2" t="n">
-        <v>0.9298245614035088</v>
+        <v>0.925531914893617</v>
       </c>
       <c r="D2" s="3" t="n">
-        <v>1.230936658375462</v>
+        <v>2.023534694440274</v>
       </c>
       <c r="E2" s="4" t="n">
-        <v>2.965699092143766</v>
+        <v>5.812032957769755</v>
       </c>
       <c r="F2" s="2" t="n">
-        <v>0.3948538299914004</v>
+        <v>0.6866623052571255</v>
       </c>
       <c r="G2" s="2" t="n">
-        <v>0.01500000000000012</v>
+        <v>0.03601705784261244</v>
       </c>
       <c r="H2" t="n">
-        <v>6</v>
+        <v>13</v>
       </c>
       <c r="I2" s="3" t="n">
-        <v>0.8214035087719298</v>
+        <v>0.8057021276595745</v>
       </c>
     </row>
     <row r="3">
@@ -547,28 +547,28 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>823</v>
+        <v>849</v>
       </c>
       <c r="C3" s="2" t="n">
-        <v>0.9951397326852977</v>
+        <v>0.9952885747938751</v>
       </c>
       <c r="D3" s="3" t="n">
-        <v>0.942253938858188</v>
+        <v>0.9546705330339486</v>
       </c>
       <c r="E3" s="4" t="n">
-        <v>1.872624840485766</v>
+        <v>1.89194217630363</v>
       </c>
       <c r="F3" s="2" t="n">
-        <v>0.2117228565766469</v>
+        <v>0.2085089166253642</v>
       </c>
       <c r="G3" s="2" t="n">
         <v>0.05833537351557738</v>
       </c>
       <c r="H3" t="n">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="I3" s="3" t="n">
-        <v>0.9853809234507899</v>
+        <v>0.9854746760895171</v>
       </c>
     </row>
     <row r="4">
@@ -578,28 +578,28 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>603</v>
+        <v>624</v>
       </c>
       <c r="C4" s="2" t="n">
-        <v>0.9950248756218906</v>
+        <v>0.9951923076923077</v>
       </c>
       <c r="D4" s="3" t="n">
-        <v>0.6554387811951277</v>
+        <v>0.6620819621075029</v>
       </c>
       <c r="E4" s="4" t="n">
-        <v>1.634704427506083</v>
+        <v>1.644046841016263</v>
       </c>
       <c r="F4" s="2" t="n">
-        <v>0.1623543426650389</v>
+        <v>0.1591320836060908</v>
       </c>
       <c r="G4" s="2" t="n">
         <v>0.05450205413924314</v>
       </c>
       <c r="H4" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="I4" s="3" t="n">
-        <v>0.986337479270315</v>
+        <v>0.9864070512820513</v>
       </c>
     </row>
     <row r="5">
@@ -609,19 +609,19 @@
         </is>
       </c>
       <c r="B5" s="5" t="n">
-        <v>324</v>
+        <v>339</v>
       </c>
       <c r="C5" s="6" t="n">
         <v>1</v>
       </c>
       <c r="D5" s="7" t="n">
-        <v>0.3857104020819992</v>
+        <v>0.4040889134516599</v>
       </c>
       <c r="E5" s="8" t="n">
-        <v>1.398234154216364</v>
+        <v>1.420067351952305</v>
       </c>
       <c r="F5" s="6" t="n">
-        <v>0.1080651026370896</v>
+        <v>0.1097886529941046</v>
       </c>
       <c r="G5" s="6" t="n">
         <v>0.01386579723875603</v>
@@ -630,7 +630,7 @@
         <v>2</v>
       </c>
       <c r="I5" s="7" t="n">
-        <v>0.9872746913580247</v>
+        <v>0.9873038348082597</v>
       </c>
     </row>
     <row r="6">
@@ -640,34 +640,34 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>381</v>
+        <v>433</v>
       </c>
       <c r="C6" s="2" t="n">
-        <v>0.9895013123359579</v>
+        <v>0.9838337182448037</v>
       </c>
       <c r="D6" s="3" t="n">
-        <v>1.616647060457461</v>
+        <v>2.427623607891934</v>
       </c>
       <c r="E6" s="4" t="n">
-        <v>3.773057879979477</v>
+        <v>7.267363409300844</v>
       </c>
       <c r="F6" s="2" t="n">
-        <v>0.5015466056877711</v>
+        <v>0.8024138594850778</v>
       </c>
       <c r="G6" s="2" t="n">
-        <v>0.02127438923763525</v>
+        <v>0.0238814380190151</v>
       </c>
       <c r="H6" t="n">
-        <v>8</v>
+        <v>15</v>
       </c>
       <c r="I6" s="3" t="n">
-        <v>0.9624593175853019</v>
+        <v>0.9478799076212472</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Atualizado em 2026-07-22T09:07:15+00:00 · arquivo de 1772 dias-cidade (~98 dias corridos) · 18 cidades</t>
+          <t>Atualizado em 2026-07-25T09:07:30+00:00 · arquivo de 1826 dias-cidade (~101 dias corridos) · 18 cidades</t>
         </is>
       </c>
     </row>
@@ -738,13 +738,13 @@
         </is>
       </c>
       <c r="C2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D2" s="2" t="n">
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="E2" s="3" t="n">
-        <v>-0.015</v>
+        <v>-0.03</v>
       </c>
     </row>
     <row r="3">
@@ -780,13 +780,13 @@
         </is>
       </c>
       <c r="C4" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="D4" s="2" t="n">
         <v>1</v>
       </c>
       <c r="E4" s="3" t="n">
-        <v>0.02881845001496088</v>
+        <v>0.04310416430067517</v>
       </c>
     </row>
     <row r="5">
@@ -822,13 +822,13 @@
         </is>
       </c>
       <c r="C6" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D6" s="2" t="n">
-        <v>1</v>
+        <v>0.6666666666666666</v>
       </c>
       <c r="E6" s="3" t="n">
-        <v>0.06998597475455821</v>
+        <v>0.05498597475455821</v>
       </c>
     </row>
     <row r="7">
@@ -864,13 +864,13 @@
         </is>
       </c>
       <c r="C8" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="D8" s="2" t="n">
         <v>1</v>
       </c>
       <c r="E8" s="3" t="n">
-        <v>0.0478553995303817</v>
+        <v>0.06465915981240283</v>
       </c>
     </row>
     <row r="9">
@@ -885,13 +885,13 @@
         </is>
       </c>
       <c r="C9" t="n">
-        <v>7</v>
+        <v>11</v>
       </c>
       <c r="D9" s="2" t="n">
         <v>1</v>
       </c>
       <c r="E9" s="3" t="n">
-        <v>0.1339089586680833</v>
+        <v>0.2520383017006383</v>
       </c>
     </row>
     <row r="10">
@@ -906,13 +906,13 @@
         </is>
       </c>
       <c r="C10" t="n">
-        <v>3</v>
+        <v>9</v>
       </c>
       <c r="D10" s="2" t="n">
-        <v>0.6666666666666666</v>
+        <v>0.7777777777777778</v>
       </c>
       <c r="E10" s="3" t="n">
-        <v>0.02618168176312127</v>
+        <v>0.1028257775440028</v>
       </c>
     </row>
     <row r="11">
@@ -927,13 +927,13 @@
         </is>
       </c>
       <c r="C11" t="n">
-        <v>6</v>
+        <v>16</v>
       </c>
       <c r="D11" s="2" t="n">
-        <v>1</v>
+        <v>0.9375</v>
       </c>
       <c r="E11" s="3" t="n">
-        <v>0.131617752291545</v>
+        <v>0.4816544603275433</v>
       </c>
     </row>
     <row r="12">
@@ -948,13 +948,13 @@
         </is>
       </c>
       <c r="C12" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="D12" s="2" t="n">
         <v>1</v>
       </c>
       <c r="E12" s="3" t="n">
-        <v>0.1246779442009537</v>
+        <v>0.1096779442009537</v>
       </c>
     </row>
     <row r="13">
@@ -969,13 +969,13 @@
         </is>
       </c>
       <c r="C13" t="n">
-        <v>7</v>
+        <v>12</v>
       </c>
       <c r="D13" s="2" t="n">
         <v>1</v>
       </c>
       <c r="E13" s="3" t="n">
-        <v>0.359417419583863</v>
+        <v>0.499460054103122</v>
       </c>
     </row>
     <row r="14">
@@ -990,13 +990,13 @@
         </is>
       </c>
       <c r="C14" t="n">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="D14" s="2" t="n">
         <v>1</v>
       </c>
       <c r="E14" s="3" t="n">
-        <v>0.07498384322006901</v>
+        <v>0.1458534598264396</v>
       </c>
     </row>
     <row r="15">
@@ -1011,13 +1011,13 @@
         </is>
       </c>
       <c r="C15" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D15" s="2" t="n">
         <v>1</v>
       </c>
       <c r="E15" s="3" t="n">
-        <v>0.03533294402859619</v>
+        <v>0.06111910755060877</v>
       </c>
     </row>
     <row r="16">
@@ -1032,13 +1032,13 @@
         </is>
       </c>
       <c r="C16" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D16" s="2" t="n">
         <v>1</v>
       </c>
       <c r="E16" s="3" t="n">
-        <v>0.05875135890666253</v>
+        <v>0.08375135890666252</v>
       </c>
     </row>
     <row r="17">
@@ -1053,13 +1053,13 @@
         </is>
       </c>
       <c r="C17" t="n">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="D17" s="2" t="n">
-        <v>0.9333333333333333</v>
+        <v>0.9375</v>
       </c>
       <c r="E17" s="3" t="n">
-        <v>0.007722343182870766</v>
+        <v>-0.007277656817129237</v>
       </c>
     </row>
     <row r="18">
@@ -1095,13 +1095,13 @@
         </is>
       </c>
       <c r="C19" t="n">
-        <v>45</v>
+        <v>48</v>
       </c>
       <c r="D19" s="2" t="n">
         <v>1</v>
       </c>
       <c r="E19" s="3" t="n">
-        <v>0.06251162156283976</v>
+        <v>0.08026961197471519</v>
       </c>
     </row>
     <row r="20">
@@ -1179,13 +1179,13 @@
         </is>
       </c>
       <c r="C23" t="n">
-        <v>48</v>
+        <v>53</v>
       </c>
       <c r="D23" s="2" t="n">
-        <v>1</v>
+        <v>0.9811320754716981</v>
       </c>
       <c r="E23" s="3" t="n">
-        <v>0.1324955366147939</v>
+        <v>0.1204182766073854</v>
       </c>
     </row>
     <row r="24">
@@ -1221,13 +1221,13 @@
         </is>
       </c>
       <c r="C25" t="n">
-        <v>31</v>
+        <v>34</v>
       </c>
       <c r="D25" s="2" t="n">
         <v>1</v>
       </c>
       <c r="E25" s="3" t="n">
-        <v>0.06882017260898085</v>
+        <v>0.08714677553059588</v>
       </c>
     </row>
     <row r="26">
@@ -1242,13 +1242,13 @@
         </is>
       </c>
       <c r="C26" t="n">
-        <v>32</v>
+        <v>38</v>
       </c>
       <c r="D26" s="2" t="n">
         <v>1</v>
       </c>
       <c r="E26" s="3" t="n">
-        <v>0.1672481847189836</v>
+        <v>0.2866355040228434</v>
       </c>
     </row>
     <row r="27">
@@ -1263,13 +1263,13 @@
         </is>
       </c>
       <c r="C27" t="n">
-        <v>9</v>
+        <v>17</v>
       </c>
       <c r="D27" s="2" t="n">
-        <v>0.8888888888888888</v>
+        <v>0.8823529411764706</v>
       </c>
       <c r="E27" s="3" t="n">
-        <v>0.03139044076973562</v>
+        <v>0.1114445636874697</v>
       </c>
     </row>
     <row r="28">
@@ -1284,13 +1284,13 @@
         </is>
       </c>
       <c r="C28" t="n">
-        <v>24</v>
+        <v>36</v>
       </c>
       <c r="D28" s="2" t="n">
-        <v>1</v>
+        <v>0.9722222222222222</v>
       </c>
       <c r="E28" s="3" t="n">
-        <v>0.1571454127091907</v>
+        <v>0.5101247894412824</v>
       </c>
     </row>
     <row r="29">
@@ -1305,13 +1305,13 @@
         </is>
       </c>
       <c r="C29" t="n">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="D29" s="2" t="n">
         <v>1</v>
       </c>
       <c r="E29" s="3" t="n">
-        <v>0.1643362114715348</v>
+        <v>0.1493362114715348</v>
       </c>
     </row>
     <row r="30">
@@ -1326,13 +1326,13 @@
         </is>
       </c>
       <c r="C30" t="n">
-        <v>27</v>
+        <v>33</v>
       </c>
       <c r="D30" s="2" t="n">
         <v>1</v>
       </c>
       <c r="E30" s="3" t="n">
-        <v>0.383509688956412</v>
+        <v>0.5256973694409416</v>
       </c>
     </row>
     <row r="31">
@@ -1347,13 +1347,13 @@
         </is>
       </c>
       <c r="C31" t="n">
-        <v>16</v>
+        <v>20</v>
       </c>
       <c r="D31" s="2" t="n">
         <v>1</v>
       </c>
       <c r="E31" s="3" t="n">
-        <v>0.08639412878904036</v>
+        <v>0.157263745395411</v>
       </c>
     </row>
     <row r="32">
@@ -1368,13 +1368,13 @@
         </is>
       </c>
       <c r="C32" t="n">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="D32" s="2" t="n">
         <v>1</v>
       </c>
       <c r="E32" s="3" t="n">
-        <v>0.0435250713406103</v>
+        <v>0.07001616940441541</v>
       </c>
     </row>
     <row r="33">
@@ -1389,13 +1389,13 @@
         </is>
       </c>
       <c r="C33" t="n">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="D33" s="2" t="n">
         <v>1</v>
       </c>
       <c r="E33" s="3" t="n">
-        <v>0.08064529957421883</v>
+        <v>0.1056452995742188</v>
       </c>
     </row>
   </sheetData>
@@ -1447,13 +1447,13 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>964</v>
+        <v>821</v>
       </c>
       <c r="C2" s="2" t="n">
-        <v>0.8754999999999999</v>
+        <v>0.8733</v>
       </c>
       <c r="D2" s="2" t="n">
-        <v>0.9916</v>
+        <v>0.995</v>
       </c>
     </row>
     <row r="3">
@@ -1463,13 +1463,13 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>973</v>
+        <v>904</v>
       </c>
       <c r="C3" s="2" t="n">
         <v>0.8695000000000001</v>
       </c>
       <c r="D3" s="2" t="n">
-        <v>0.9946</v>
+        <v>0.9961</v>
       </c>
     </row>
     <row r="4">
@@ -1479,13 +1479,13 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>1008</v>
+        <v>967</v>
       </c>
       <c r="C4" s="2" t="n">
-        <v>0.877</v>
+        <v>0.88</v>
       </c>
       <c r="D4" s="2" t="n">
-        <v>0.9949</v>
+        <v>0.995</v>
       </c>
     </row>
     <row r="5">
@@ -1495,13 +1495,13 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>998</v>
+        <v>951</v>
       </c>
       <c r="C5" s="2" t="n">
-        <v>0.8687</v>
+        <v>0.8665</v>
       </c>
       <c r="D5" s="2" t="n">
-        <v>0.9962</v>
+        <v>0.9969</v>
       </c>
     </row>
     <row r="6">
@@ -1511,13 +1511,13 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>1021</v>
+        <v>996</v>
       </c>
       <c r="C6" s="2" t="n">
-        <v>0.8501</v>
+        <v>0.8534</v>
       </c>
       <c r="D6" s="2" t="n">
-        <v>0.9972</v>
+        <v>0.9975000000000001</v>
       </c>
     </row>
     <row r="7">
@@ -1527,13 +1527,13 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>990</v>
+        <v>933</v>
       </c>
       <c r="C7" s="2" t="n">
-        <v>0.8606</v>
+        <v>0.8564000000000001</v>
       </c>
       <c r="D7" s="2" t="n">
-        <v>0.9967</v>
+        <v>0.9968</v>
       </c>
     </row>
     <row r="8">
@@ -1543,13 +1543,13 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>1015</v>
+        <v>973</v>
       </c>
       <c r="C8" s="2" t="n">
-        <v>0.8473000000000001</v>
+        <v>0.8438</v>
       </c>
       <c r="D8" s="2" t="n">
-        <v>0.9965000000000001</v>
+        <v>0.9972</v>
       </c>
     </row>
     <row r="9">
@@ -1559,13 +1559,13 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>948</v>
+        <v>878</v>
       </c>
       <c r="C9" s="2" t="n">
-        <v>0.8987000000000001</v>
+        <v>0.9055</v>
       </c>
       <c r="D9" s="2" t="n">
-        <v>0.9906</v>
+        <v>0.9919</v>
       </c>
     </row>
     <row r="10">
@@ -1575,13 +1575,13 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>920</v>
+        <v>800</v>
       </c>
       <c r="C10" s="2" t="n">
-        <v>0.875</v>
+        <v>0.8625</v>
       </c>
       <c r="D10" s="2" t="n">
-        <v>0.9908</v>
+        <v>0.9933999999999999</v>
       </c>
     </row>
     <row r="11">
@@ -1591,13 +1591,13 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>962</v>
+        <v>921</v>
       </c>
       <c r="C11" s="2" t="n">
-        <v>0.9293</v>
+        <v>0.9446</v>
       </c>
       <c r="D11" s="2" t="n">
-        <v>0.9935</v>
+        <v>0.9941</v>
       </c>
     </row>
     <row r="12">
@@ -1607,13 +1607,13 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>945</v>
+        <v>848</v>
       </c>
       <c r="C12" s="2" t="n">
-        <v>0.9132</v>
+        <v>0.9281</v>
       </c>
       <c r="D12" s="2" t="n">
-        <v>0.9873</v>
+        <v>0.993</v>
       </c>
     </row>
     <row r="13">
@@ -1623,13 +1623,13 @@
         </is>
       </c>
       <c r="B13" t="n">
-        <v>938</v>
+        <v>807</v>
       </c>
       <c r="C13" s="2" t="n">
-        <v>0.903</v>
+        <v>0.8996</v>
       </c>
       <c r="D13" s="2" t="n">
-        <v>0.987</v>
+        <v>0.9903</v>
       </c>
     </row>
     <row r="14">
@@ -1639,13 +1639,13 @@
         </is>
       </c>
       <c r="B14" t="n">
-        <v>938</v>
+        <v>854</v>
       </c>
       <c r="C14" s="2" t="n">
-        <v>0.8763</v>
+        <v>0.8782</v>
       </c>
       <c r="D14" s="2" t="n">
-        <v>0.9925</v>
+        <v>0.9944</v>
       </c>
     </row>
     <row r="15">
@@ -1655,13 +1655,13 @@
         </is>
       </c>
       <c r="B15" t="n">
-        <v>974</v>
+        <v>917</v>
       </c>
       <c r="C15" s="2" t="n">
-        <v>0.8717</v>
+        <v>0.8691</v>
       </c>
       <c r="D15" s="2" t="n">
-        <v>0.9936</v>
+        <v>0.9955000000000001</v>
       </c>
     </row>
     <row r="16">
@@ -1671,13 +1671,13 @@
         </is>
       </c>
       <c r="B16" t="n">
-        <v>956</v>
+        <v>830</v>
       </c>
       <c r="C16" s="2" t="n">
-        <v>0.8766</v>
+        <v>0.888</v>
       </c>
       <c r="D16" s="2" t="n">
-        <v>0.9902</v>
+        <v>0.9901</v>
       </c>
     </row>
     <row r="17">
@@ -1687,13 +1687,13 @@
         </is>
       </c>
       <c r="B17" t="n">
-        <v>920</v>
+        <v>852</v>
       </c>
       <c r="C17" s="2" t="n">
-        <v>0.9185</v>
+        <v>0.919</v>
       </c>
       <c r="D17" s="2" t="n">
-        <v>0.9915</v>
+        <v>0.9921</v>
       </c>
     </row>
     <row r="18">
@@ -1703,10 +1703,10 @@
         </is>
       </c>
       <c r="B18" t="n">
-        <v>993</v>
+        <v>949</v>
       </c>
       <c r="C18" s="2" t="n">
-        <v>0.863</v>
+        <v>0.8662</v>
       </c>
       <c r="D18" s="2" t="n">
         <v>0.9963</v>
@@ -1719,13 +1719,13 @@
         </is>
       </c>
       <c r="B19" t="n">
-        <v>998</v>
+        <v>946</v>
       </c>
       <c r="C19" s="2" t="n">
-        <v>0.8868</v>
+        <v>0.9112</v>
       </c>
       <c r="D19" s="2" t="n">
-        <v>0.9912</v>
+        <v>0.9923999999999999</v>
       </c>
     </row>
   </sheetData>
@@ -1789,19 +1789,19 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>0.1351</v>
+        <v>0.133</v>
       </c>
       <c r="C2" t="n">
-        <v>0.1351</v>
+        <v>0.1224</v>
       </c>
       <c r="D2" t="n">
-        <v>1.4556</v>
+        <v>0.0051</v>
       </c>
       <c r="E2" t="n">
-        <v>-0.393</v>
+        <v>1.0466</v>
       </c>
       <c r="F2" t="n">
-        <v>0.1874</v>
+        <v>0.073</v>
       </c>
     </row>
     <row r="3">
@@ -1811,19 +1811,19 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>0.1291</v>
+        <v>0.1271</v>
       </c>
       <c r="C3" t="n">
-        <v>0.1197</v>
+        <v>0.1092</v>
       </c>
       <c r="D3" t="n">
-        <v>0.0034</v>
+        <v>0.0017</v>
       </c>
       <c r="E3" t="n">
-        <v>1.051</v>
+        <v>1.0421</v>
       </c>
       <c r="F3" t="n">
-        <v>0.08069999999999999</v>
+        <v>0.08110000000000001</v>
       </c>
     </row>
     <row r="4">
@@ -1833,19 +1833,19 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>0.0442</v>
+        <v>0.0436</v>
       </c>
       <c r="C4" t="n">
-        <v>0.0385</v>
+        <v>0.0383</v>
       </c>
       <c r="D4" t="n">
-        <v>0.1216</v>
+        <v>0.1211</v>
       </c>
       <c r="E4" t="n">
-        <v>0.9785</v>
+        <v>0.995</v>
       </c>
       <c r="F4" t="n">
-        <v>0.0608</v>
+        <v>0.0602</v>
       </c>
     </row>
   </sheetData>
@@ -1874,7 +1874,7 @@
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>2026-07-22T09:07:15+00:00</t>
+          <t>2026-07-25T09:07:30+00:00</t>
         </is>
       </c>
     </row>
@@ -1885,7 +1885,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>1772</v>
+        <v>1826</v>
       </c>
     </row>
     <row r="3">
@@ -1895,7 +1895,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>98</v>
+        <v>101</v>
       </c>
     </row>
     <row r="4">

</xml_diff>

<commit_message>
Arquiva dados, recalibra e atualiza docs (2026-07-28)
</commit_message>
<xml_diff>
--- a/backtest_results/resultados_backtest.xlsx
+++ b/backtest_results/resultados_backtest.xlsx
@@ -516,28 +516,28 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>94</v>
+        <v>322</v>
       </c>
       <c r="C2" s="2" t="n">
-        <v>0.925531914893617</v>
+        <v>0.8975155279503105</v>
       </c>
       <c r="D2" s="3" t="n">
-        <v>2.023534694440274</v>
+        <v>4.037473155639022</v>
       </c>
       <c r="E2" s="4" t="n">
-        <v>5.812032957769755</v>
+        <v>20.19841346343609</v>
       </c>
       <c r="F2" s="2" t="n">
-        <v>0.6866623052571255</v>
+        <v>1.46374171808818</v>
       </c>
       <c r="G2" s="2" t="n">
-        <v>0.03601705784261244</v>
+        <v>0.2170352923628444</v>
       </c>
       <c r="H2" t="n">
-        <v>13</v>
+        <v>62</v>
       </c>
       <c r="I2" s="3" t="n">
-        <v>0.8057021276595745</v>
+        <v>0.8386086956521739</v>
       </c>
     </row>
     <row r="3">
@@ -547,28 +547,28 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>849</v>
+        <v>1679</v>
       </c>
       <c r="C3" s="2" t="n">
-        <v>0.9952885747938751</v>
+        <v>0.9940440738534843</v>
       </c>
       <c r="D3" s="3" t="n">
-        <v>0.9546705330339486</v>
+        <v>1.890835831197596</v>
       </c>
       <c r="E3" s="4" t="n">
-        <v>1.89194217630363</v>
+        <v>2.748689574300068</v>
       </c>
       <c r="F3" s="2" t="n">
-        <v>0.2085089166253642</v>
+        <v>0.3543711950145478</v>
       </c>
       <c r="G3" s="2" t="n">
-        <v>0.05833537351557738</v>
+        <v>0.08704657533117888</v>
       </c>
       <c r="H3" t="n">
-        <v>18</v>
+        <v>33</v>
       </c>
       <c r="I3" s="3" t="n">
-        <v>0.9854746760895171</v>
+        <v>0.9857066706372841</v>
       </c>
     </row>
     <row r="4">
@@ -578,28 +578,28 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>624</v>
+        <v>1214</v>
       </c>
       <c r="C4" s="2" t="n">
-        <v>0.9951923076923077</v>
+        <v>0.9950576606260296</v>
       </c>
       <c r="D4" s="3" t="n">
-        <v>0.6620819621075029</v>
+        <v>1.325577596940686</v>
       </c>
       <c r="E4" s="4" t="n">
-        <v>1.644046841016263</v>
+        <v>2.313242463695541</v>
       </c>
       <c r="F4" s="2" t="n">
-        <v>0.1591320836060908</v>
+        <v>0.2860751501989593</v>
       </c>
       <c r="G4" s="2" t="n">
-        <v>0.05450205413924314</v>
+        <v>0.08016721391959125</v>
       </c>
       <c r="H4" t="n">
-        <v>12</v>
+        <v>19</v>
       </c>
       <c r="I4" s="3" t="n">
-        <v>0.9864070512820513</v>
+        <v>0.9866803953871499</v>
       </c>
     </row>
     <row r="5">
@@ -609,28 +609,28 @@
         </is>
       </c>
       <c r="B5" s="5" t="n">
-        <v>339</v>
+        <v>636</v>
       </c>
       <c r="C5" s="6" t="n">
-        <v>1</v>
+        <v>0.9984276729559748</v>
       </c>
       <c r="D5" s="7" t="n">
-        <v>0.4040889134516599</v>
+        <v>0.7252985342410232</v>
       </c>
       <c r="E5" s="8" t="n">
-        <v>1.420067351952305</v>
+        <v>1.759873310506253</v>
       </c>
       <c r="F5" s="6" t="n">
-        <v>0.1097886529941046</v>
+        <v>0.1847982976405755</v>
       </c>
       <c r="G5" s="6" t="n">
-        <v>0.01386579723875603</v>
+        <v>0.02619857308701179</v>
       </c>
       <c r="H5" s="5" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="I5" s="7" t="n">
-        <v>0.9873038348082597</v>
+        <v>0.987495283018868</v>
       </c>
     </row>
     <row r="6">
@@ -640,34 +640,34 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>433</v>
+        <v>958</v>
       </c>
       <c r="C6" s="2" t="n">
-        <v>0.9838337182448037</v>
+        <v>0.964509394572025</v>
       </c>
       <c r="D6" s="3" t="n">
-        <v>2.427623607891934</v>
+        <v>4.762771689880045</v>
       </c>
       <c r="E6" s="4" t="n">
-        <v>7.267363409300844</v>
+        <v>24.84427521783187</v>
       </c>
       <c r="F6" s="2" t="n">
-        <v>0.8024138594850778</v>
+        <v>1.621608880265423</v>
       </c>
       <c r="G6" s="2" t="n">
-        <v>0.0238814380190151</v>
+        <v>0.1983925675638193</v>
       </c>
       <c r="H6" t="n">
-        <v>15</v>
+        <v>67</v>
       </c>
       <c r="I6" s="3" t="n">
-        <v>0.9478799076212472</v>
+        <v>0.9374519832985387</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Atualizado em 2026-07-25T09:07:30+00:00 · arquivo de 1826 dias-cidade (~101 dias corridos) · 18 cidades</t>
+          <t>Atualizado em 2026-07-28T09:48:16+00:00 · arquivo de 3881 dias-cidade (~100 dias corridos) · 39 cidades</t>
         </is>
       </c>
     </row>
@@ -689,7 +689,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E33"/>
+  <dimension ref="A1:E73"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -738,13 +738,13 @@
         </is>
       </c>
       <c r="C2" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D2" s="2" t="n">
-        <v>0.5</v>
+        <v>0.6666666666666666</v>
       </c>
       <c r="E2" s="3" t="n">
-        <v>-0.03</v>
+        <v>0.00623474540887469</v>
       </c>
     </row>
     <row r="3">
@@ -755,17 +755,17 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Londres (EGLC)</t>
+          <t>Munique (EDDM)</t>
         </is>
       </c>
       <c r="C3" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D3" s="2" t="n">
         <v>1</v>
       </c>
       <c r="E3" s="3" t="n">
-        <v>0.03205713797646388</v>
+        <v>0.02250133372388761</v>
       </c>
     </row>
     <row r="4">
@@ -776,17 +776,17 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Amsterdã (EHAM)</t>
+          <t>Helsinque (EFHK)</t>
         </is>
       </c>
       <c r="C4" t="n">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="D4" s="2" t="n">
         <v>1</v>
       </c>
       <c r="E4" s="3" t="n">
-        <v>0.04310416430067517</v>
+        <v>-0.01807874151893931</v>
       </c>
     </row>
     <row r="5">
@@ -797,17 +797,17 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Varsóvia (EPWA)</t>
+          <t>Londres (EGLC)</t>
         </is>
       </c>
       <c r="C5" t="n">
-        <v>4</v>
+        <v>8</v>
       </c>
       <c r="D5" s="2" t="n">
-        <v>0.75</v>
+        <v>0.875</v>
       </c>
       <c r="E5" s="3" t="n">
-        <v>0.1297630704668648</v>
+        <v>0.03322151580128275</v>
       </c>
     </row>
     <row r="6">
@@ -818,17 +818,17 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Istambul (LTFM)</t>
+          <t>Amsterdã (EHAM)</t>
         </is>
       </c>
       <c r="C6" t="n">
-        <v>3</v>
+        <v>14</v>
       </c>
       <c r="D6" s="2" t="n">
-        <v>0.6666666666666666</v>
+        <v>0.9285714285714286</v>
       </c>
       <c r="E6" s="3" t="n">
-        <v>0.05498597475455821</v>
+        <v>0.01843717445760852</v>
       </c>
     </row>
     <row r="7">
@@ -839,17 +839,17 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Cidade do México (MMMX)</t>
+          <t>Varsóvia (EPWA)</t>
         </is>
       </c>
       <c r="C7" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="D7" s="2" t="n">
-        <v>0.5</v>
+        <v>0.8</v>
       </c>
       <c r="E7" s="3" t="n">
-        <v>-0.007415277030661634</v>
+        <v>0.1431748022405707</v>
       </c>
     </row>
     <row r="8">
@@ -860,17 +860,17 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Wellington (NZWN)</t>
+          <t>Cidade do Cabo (FACT)</t>
         </is>
       </c>
       <c r="C8" t="n">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="D8" s="2" t="n">
         <v>1</v>
       </c>
       <c r="E8" s="3" t="n">
-        <v>0.06465915981240283</v>
+        <v>0.007052021389959679</v>
       </c>
     </row>
     <row r="9">
@@ -881,17 +881,17 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Tóquio (RJTT)</t>
+          <t>Atlanta (KATL)</t>
         </is>
       </c>
       <c r="C9" t="n">
-        <v>11</v>
+        <v>2</v>
       </c>
       <c r="D9" s="2" t="n">
-        <v>1</v>
+        <v>0.5</v>
       </c>
       <c r="E9" s="3" t="n">
-        <v>0.2520383017006383</v>
+        <v>-0.008617021276595745</v>
       </c>
     </row>
     <row r="10">
@@ -902,17 +902,17 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Seul (RKSI)</t>
+          <t>Denver (KBKF)</t>
         </is>
       </c>
       <c r="C10" t="n">
-        <v>9</v>
+        <v>4</v>
       </c>
       <c r="D10" s="2" t="n">
-        <v>0.7777777777777778</v>
+        <v>1</v>
       </c>
       <c r="E10" s="3" t="n">
-        <v>0.1028257775440028</v>
+        <v>0.08075556783620651</v>
       </c>
     </row>
     <row r="11">
@@ -923,17 +923,17 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Buenos Aires (SAEZ)</t>
+          <t>Dallas (KDAL)</t>
         </is>
       </c>
       <c r="C11" t="n">
-        <v>16</v>
+        <v>2</v>
       </c>
       <c r="D11" s="2" t="n">
-        <v>0.9375</v>
+        <v>1</v>
       </c>
       <c r="E11" s="3" t="n">
-        <v>0.4816544603275433</v>
+        <v>0.01248377447937243</v>
       </c>
     </row>
     <row r="12">
@@ -944,17 +944,17 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Guarulhos (SBGR)</t>
+          <t>Houston (KHOU)</t>
         </is>
       </c>
       <c r="C12" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="D12" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E12" s="3" t="n">
-        <v>0.1096779442009537</v>
+        <v>-0.06</v>
       </c>
     </row>
     <row r="13">
@@ -965,17 +965,17 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Moscou (UUWW)</t>
+          <t>Los Angeles (KLAX)</t>
         </is>
       </c>
       <c r="C13" t="n">
-        <v>12</v>
+        <v>5</v>
       </c>
       <c r="D13" s="2" t="n">
-        <v>1</v>
+        <v>0.6</v>
       </c>
       <c r="E13" s="3" t="n">
-        <v>0.499460054103122</v>
+        <v>0.006890414114194828</v>
       </c>
     </row>
     <row r="14">
@@ -986,17 +986,17 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Singapura (WSSS)</t>
+          <t>Nova York (KLGA)</t>
         </is>
       </c>
       <c r="C14" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="D14" s="2" t="n">
-        <v>1</v>
+        <v>0.75</v>
       </c>
       <c r="E14" s="3" t="n">
-        <v>0.1458534598264396</v>
+        <v>0.0767850392492342</v>
       </c>
     </row>
     <row r="15">
@@ -1007,17 +1007,17 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Pequim (ZBAA)</t>
+          <t>Miami (KMIA)</t>
         </is>
       </c>
       <c r="C15" t="n">
-        <v>4</v>
+        <v>9</v>
       </c>
       <c r="D15" s="2" t="n">
-        <v>1</v>
+        <v>0.8888888888888888</v>
       </c>
       <c r="E15" s="3" t="n">
-        <v>0.06111910755060877</v>
+        <v>0.1206121803170523</v>
       </c>
     </row>
     <row r="16">
@@ -1028,317 +1028,317 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Xangai (ZSPD)</t>
+          <t>Chicago (KORD)</t>
         </is>
       </c>
       <c r="C16" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="D16" s="2" t="n">
         <v>1</v>
       </c>
       <c r="E16" s="3" t="n">
-        <v>0.08375135890666252</v>
+        <v>0.02063570816437714</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Combinado</t>
+          <t>Edge</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Toronto (CYYZ)</t>
+          <t>Seattle (KSEA)</t>
         </is>
       </c>
       <c r="C17" t="n">
-        <v>16</v>
+        <v>6</v>
       </c>
       <c r="D17" s="2" t="n">
-        <v>0.9375</v>
+        <v>0.8333333333333334</v>
       </c>
       <c r="E17" s="3" t="n">
-        <v>-0.007277656817129237</v>
+        <v>-0.04666569575854426</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>Combinado</t>
+          <t>Edge</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Londres (EGLC)</t>
+          <t>Milão (LIMC)</t>
         </is>
       </c>
       <c r="C18" t="n">
-        <v>28</v>
+        <v>2</v>
       </c>
       <c r="D18" s="2" t="n">
         <v>1</v>
       </c>
       <c r="E18" s="3" t="n">
-        <v>0.06388759741877117</v>
+        <v>0.01419268854547966</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>Combinado</t>
+          <t>Edge</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>Amsterdã (EHAM)</t>
+          <t>Ancara (LTAC)</t>
         </is>
       </c>
       <c r="C19" t="n">
-        <v>48</v>
+        <v>1</v>
       </c>
       <c r="D19" s="2" t="n">
         <v>1</v>
       </c>
       <c r="E19" s="3" t="n">
-        <v>0.08026961197471519</v>
+        <v>0.007584722969338365</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>Combinado</t>
+          <t>Edge</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>Varsóvia (EPWA)</t>
+          <t>Istambul (LTFM)</t>
         </is>
       </c>
       <c r="C20" t="n">
-        <v>14</v>
+        <v>7</v>
       </c>
       <c r="D20" s="2" t="n">
-        <v>0.9285714285714286</v>
+        <v>1</v>
       </c>
       <c r="E20" s="3" t="n">
-        <v>0.1439081708138227</v>
+        <v>0.2123882871456879</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>Combinado</t>
+          <t>Edge</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>Madri (LEMD)</t>
+          <t>Cidade do México (MMMX)</t>
         </is>
       </c>
       <c r="C21" t="n">
         <v>4</v>
       </c>
       <c r="D21" s="2" t="n">
-        <v>1</v>
+        <v>0.75</v>
       </c>
       <c r="E21" s="3" t="n">
-        <v>0.005385531300417991</v>
+        <v>0.006895137313328397</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>Combinado</t>
+          <t>Edge</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>Ancara (LTAC)</t>
+          <t>Wellington (NZWN)</t>
         </is>
       </c>
       <c r="C22" t="n">
-        <v>7</v>
+        <v>15</v>
       </c>
       <c r="D22" s="2" t="n">
-        <v>1</v>
+        <v>0.8666666666666667</v>
       </c>
       <c r="E22" s="3" t="n">
-        <v>0.009569509080958683</v>
+        <v>0.395586087922119</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>Combinado</t>
+          <t>Edge</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>Istambul (LTFM)</t>
+          <t>Taipé (RCSS)</t>
         </is>
       </c>
       <c r="C23" t="n">
-        <v>53</v>
+        <v>22</v>
       </c>
       <c r="D23" s="2" t="n">
-        <v>0.9811320754716981</v>
+        <v>0.9090909090909091</v>
       </c>
       <c r="E23" s="3" t="n">
-        <v>0.1204182766073854</v>
+        <v>0.2295774625433846</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>Combinado</t>
+          <t>Edge</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>Cidade do México (MMMX)</t>
+          <t>Tóquio (RJTT)</t>
         </is>
       </c>
       <c r="C24" t="n">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="D24" s="2" t="n">
-        <v>0.9333333333333333</v>
+        <v>1</v>
       </c>
       <c r="E24" s="3" t="n">
-        <v>0.008152139544279196</v>
+        <v>0.1844042105660792</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>Combinado</t>
+          <t>Edge</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>Wellington (NZWN)</t>
+          <t>Seul (RKSI)</t>
         </is>
       </c>
       <c r="C25" t="n">
-        <v>34</v>
+        <v>13</v>
       </c>
       <c r="D25" s="2" t="n">
-        <v>1</v>
+        <v>0.9230769230769231</v>
       </c>
       <c r="E25" s="3" t="n">
-        <v>0.08714677553059588</v>
+        <v>0.2566434903166885</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>Combinado</t>
+          <t>Edge</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>Tóquio (RJTT)</t>
+          <t>Manila (RPLL)</t>
         </is>
       </c>
       <c r="C26" t="n">
-        <v>38</v>
+        <v>17</v>
       </c>
       <c r="D26" s="2" t="n">
         <v>1</v>
       </c>
       <c r="E26" s="3" t="n">
-        <v>0.2866355040228434</v>
+        <v>0.2056511408541294</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>Combinado</t>
+          <t>Edge</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>Seul (RKSI)</t>
+          <t>Buenos Aires (SAEZ)</t>
         </is>
       </c>
       <c r="C27" t="n">
         <v>17</v>
       </c>
       <c r="D27" s="2" t="n">
-        <v>0.8823529411764706</v>
+        <v>1</v>
       </c>
       <c r="E27" s="3" t="n">
-        <v>0.1114445636874697</v>
+        <v>0.5673435632805013</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>Combinado</t>
+          <t>Edge</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>Buenos Aires (SAEZ)</t>
+          <t>Guarulhos (SBGR)</t>
         </is>
       </c>
       <c r="C28" t="n">
-        <v>36</v>
+        <v>6</v>
       </c>
       <c r="D28" s="2" t="n">
-        <v>0.9722222222222222</v>
+        <v>0.8333333333333334</v>
       </c>
       <c r="E28" s="3" t="n">
-        <v>0.5101247894412824</v>
+        <v>0.1298913520808539</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>Combinado</t>
+          <t>Edge</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>Guarulhos (SBGR)</t>
+          <t>Moscou (UUWW)</t>
         </is>
       </c>
       <c r="C29" t="n">
-        <v>35</v>
+        <v>14</v>
       </c>
       <c r="D29" s="2" t="n">
-        <v>1</v>
+        <v>0.8571428571428571</v>
       </c>
       <c r="E29" s="3" t="n">
-        <v>0.1493362114715348</v>
+        <v>0.4721726782662505</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>Combinado</t>
+          <t>Edge</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>Moscou (UUWW)</t>
+          <t>Kuala Lumpur (WMKK)</t>
         </is>
       </c>
       <c r="C30" t="n">
-        <v>33</v>
+        <v>3</v>
       </c>
       <c r="D30" s="2" t="n">
         <v>1</v>
       </c>
       <c r="E30" s="3" t="n">
-        <v>0.5256973694409416</v>
+        <v>0.01972871211600642</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>Combinado</t>
+          <t>Edge</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
@@ -1347,19 +1347,19 @@
         </is>
       </c>
       <c r="C31" t="n">
-        <v>20</v>
+        <v>10</v>
       </c>
       <c r="D31" s="2" t="n">
-        <v>1</v>
+        <v>0.9</v>
       </c>
       <c r="E31" s="3" t="n">
-        <v>0.157263745395411</v>
+        <v>0.06741812387731545</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>Combinado</t>
+          <t>Edge</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
@@ -1368,34 +1368,874 @@
         </is>
       </c>
       <c r="C32" t="n">
-        <v>12</v>
+        <v>7</v>
       </c>
       <c r="D32" s="2" t="n">
         <v>1</v>
       </c>
       <c r="E32" s="3" t="n">
-        <v>0.07001616940441541</v>
+        <v>0.09010581559877134</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>Combinado</t>
+          <t>Edge</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
+          <t>Guangzhou (ZGGG)</t>
+        </is>
+      </c>
+      <c r="C33" t="n">
+        <v>21</v>
+      </c>
+      <c r="D33" s="2" t="n">
+        <v>0.8095238095238095</v>
+      </c>
+      <c r="E33" s="3" t="n">
+        <v>0.1065260645220891</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>Edge</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>Shenzhen (ZGSZ)</t>
+        </is>
+      </c>
+      <c r="C34" t="n">
+        <v>43</v>
+      </c>
+      <c r="D34" s="2" t="n">
+        <v>0.9069767441860465</v>
+      </c>
+      <c r="E34" s="3" t="n">
+        <v>0.4367327818601304</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>Edge</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>Wuhan (ZHHH)</t>
+        </is>
+      </c>
+      <c r="C35" t="n">
+        <v>8</v>
+      </c>
+      <c r="D35" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="E35" s="3" t="n">
+        <v>0.05065203240622935</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>Edge</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
           <t>Xangai (ZSPD)</t>
         </is>
       </c>
-      <c r="C33" t="n">
+      <c r="C36" t="n">
+        <v>12</v>
+      </c>
+      <c r="D36" s="2" t="n">
+        <v>0.9166666666666666</v>
+      </c>
+      <c r="E36" s="3" t="n">
+        <v>0.1685559848260972</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>Combinado</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>Toronto (CYYZ)</t>
+        </is>
+      </c>
+      <c r="C37" t="n">
+        <v>16</v>
+      </c>
+      <c r="D37" s="2" t="n">
+        <v>0.9375</v>
+      </c>
+      <c r="E37" s="3" t="n">
+        <v>0.02649807219830284</v>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>Combinado</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>Munique (EDDM)</t>
+        </is>
+      </c>
+      <c r="C38" t="n">
+        <v>21</v>
+      </c>
+      <c r="D38" s="2" t="n">
+        <v>0.9523809523809523</v>
+      </c>
+      <c r="E38" s="3" t="n">
+        <v>0.02897737559373625</v>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>Combinado</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>Helsinque (EFHK)</t>
+        </is>
+      </c>
+      <c r="C39" t="n">
+        <v>29</v>
+      </c>
+      <c r="D39" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="E39" s="3" t="n">
+        <v>0.01943847144601079</v>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>Combinado</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>Londres (EGLC)</t>
+        </is>
+      </c>
+      <c r="C40" t="n">
+        <v>32</v>
+      </c>
+      <c r="D40" s="2" t="n">
+        <v>0.96875</v>
+      </c>
+      <c r="E40" s="3" t="n">
+        <v>0.06505197524359005</v>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>Combinado</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>Amsterdã (EHAM)</t>
+        </is>
+      </c>
+      <c r="C41" t="n">
+        <v>54</v>
+      </c>
+      <c r="D41" s="2" t="n">
+        <v>0.9814814814814815</v>
+      </c>
+      <c r="E41" s="3" t="n">
+        <v>0.05499900040126621</v>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>Combinado</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>Varsóvia (EPWA)</t>
+        </is>
+      </c>
+      <c r="C42" t="n">
+        <v>15</v>
+      </c>
+      <c r="D42" s="2" t="n">
+        <v>0.9333333333333333</v>
+      </c>
+      <c r="E42" s="3" t="n">
+        <v>0.1573199025875285</v>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>Combinado</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>Cidade do Cabo (FACT)</t>
+        </is>
+      </c>
+      <c r="C43" t="n">
         <v>23</v>
       </c>
-      <c r="D33" s="2" t="n">
+      <c r="D43" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="E33" s="3" t="n">
-        <v>0.1056452995742188</v>
+      <c r="E43" s="3" t="n">
+        <v>0.02646317118320567</v>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>Combinado</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>Atlanta (KATL)</t>
+        </is>
+      </c>
+      <c r="C44" t="n">
+        <v>16</v>
+      </c>
+      <c r="D44" s="2" t="n">
+        <v>0.9375</v>
+      </c>
+      <c r="E44" s="3" t="n">
+        <v>0.003500706411286052</v>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>Combinado</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>Denver (KBKF)</t>
+        </is>
+      </c>
+      <c r="C45" t="n">
+        <v>5</v>
+      </c>
+      <c r="D45" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="E45" s="3" t="n">
+        <v>0.08135918956658879</v>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>Combinado</t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>Dallas (KDAL)</t>
+        </is>
+      </c>
+      <c r="C46" t="n">
+        <v>6</v>
+      </c>
+      <c r="D46" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="E46" s="3" t="n">
+        <v>0.01731065767370086</v>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>Combinado</t>
+        </is>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>Houston (KHOU)</t>
+        </is>
+      </c>
+      <c r="C47" t="n">
+        <v>10</v>
+      </c>
+      <c r="D47" s="2" t="n">
+        <v>0.6</v>
+      </c>
+      <c r="E47" s="3" t="n">
+        <v>-0.05112262463304137</v>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>Combinado</t>
+        </is>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>Los Angeles (KLAX)</t>
+        </is>
+      </c>
+      <c r="C48" t="n">
+        <v>14</v>
+      </c>
+      <c r="D48" s="2" t="n">
+        <v>0.8571428571428571</v>
+      </c>
+      <c r="E48" s="3" t="n">
+        <v>0.01528237604625361</v>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>Combinado</t>
+        </is>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>Nova York (KLGA)</t>
+        </is>
+      </c>
+      <c r="C49" t="n">
+        <v>16</v>
+      </c>
+      <c r="D49" s="2" t="n">
+        <v>0.9375</v>
+      </c>
+      <c r="E49" s="3" t="n">
+        <v>0.09285061569441484</v>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>Combinado</t>
+        </is>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>Miami (KMIA)</t>
+        </is>
+      </c>
+      <c r="C50" t="n">
+        <v>29</v>
+      </c>
+      <c r="D50" s="2" t="n">
+        <v>0.9655172413793104</v>
+      </c>
+      <c r="E50" s="3" t="n">
+        <v>0.1437867028586853</v>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>Combinado</t>
+        </is>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>Chicago (KORD)</t>
+        </is>
+      </c>
+      <c r="C51" t="n">
+        <v>21</v>
+      </c>
+      <c r="D51" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="E51" s="3" t="n">
+        <v>0.04168440738044763</v>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>Combinado</t>
+        </is>
+      </c>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>Seattle (KSEA)</t>
+        </is>
+      </c>
+      <c r="C52" t="n">
+        <v>22</v>
+      </c>
+      <c r="D52" s="2" t="n">
+        <v>0.9545454545454546</v>
+      </c>
+      <c r="E52" s="3" t="n">
+        <v>-0.02457179188325269</v>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>Combinado</t>
+        </is>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>Madri (LEMD)</t>
+        </is>
+      </c>
+      <c r="C53" t="n">
+        <v>4</v>
+      </c>
+      <c r="D53" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="E53" s="3" t="n">
+        <v>0.005385531300417991</v>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>Combinado</t>
+        </is>
+      </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>Milão (LIMC)</t>
+        </is>
+      </c>
+      <c r="C54" t="n">
+        <v>19</v>
+      </c>
+      <c r="D54" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="E54" s="3" t="n">
+        <v>0.03465308375945613</v>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>Combinado</t>
+        </is>
+      </c>
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>Tel Aviv (LLBG)</t>
+        </is>
+      </c>
+      <c r="C55" t="n">
+        <v>4</v>
+      </c>
+      <c r="D55" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="E55" s="3" t="n">
+        <v>0.005115058255058735</v>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
+          <t>Combinado</t>
+        </is>
+      </c>
+      <c r="B56" t="inlineStr">
+        <is>
+          <t>Ancara (LTAC)</t>
+        </is>
+      </c>
+      <c r="C56" t="n">
+        <v>9</v>
+      </c>
+      <c r="D56" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="E56" s="3" t="n">
+        <v>0.01770727377980937</v>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="inlineStr">
+        <is>
+          <t>Combinado</t>
+        </is>
+      </c>
+      <c r="B57" t="inlineStr">
+        <is>
+          <t>Istambul (LTFM)</t>
+        </is>
+      </c>
+      <c r="C57" t="n">
+        <v>61</v>
+      </c>
+      <c r="D57" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="E57" s="3" t="n">
+        <v>0.2820296780107753</v>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="inlineStr">
+        <is>
+          <t>Combinado</t>
+        </is>
+      </c>
+      <c r="B58" t="inlineStr">
+        <is>
+          <t>Cidade do México (MMMX)</t>
+        </is>
+      </c>
+      <c r="C58" t="n">
+        <v>17</v>
+      </c>
+      <c r="D58" s="2" t="n">
+        <v>0.9411764705882353</v>
+      </c>
+      <c r="E58" s="3" t="n">
+        <v>0.02246255388826923</v>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="inlineStr">
+        <is>
+          <t>Combinado</t>
+        </is>
+      </c>
+      <c r="B59" t="inlineStr">
+        <is>
+          <t>Wellington (NZWN)</t>
+        </is>
+      </c>
+      <c r="C59" t="n">
+        <v>43</v>
+      </c>
+      <c r="D59" s="2" t="n">
+        <v>0.9534883720930233</v>
+      </c>
+      <c r="E59" s="3" t="n">
+        <v>0.4156127746967782</v>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="inlineStr">
+        <is>
+          <t>Combinado</t>
+        </is>
+      </c>
+      <c r="B60" t="inlineStr">
+        <is>
+          <t>Taipé (RCSS)</t>
+        </is>
+      </c>
+      <c r="C60" t="n">
+        <v>24</v>
+      </c>
+      <c r="D60" s="2" t="n">
+        <v>0.9166666666666666</v>
+      </c>
+      <c r="E60" s="3" t="n">
+        <v>0.2310896158327151</v>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="inlineStr">
+        <is>
+          <t>Combinado</t>
+        </is>
+      </c>
+      <c r="B61" t="inlineStr">
+        <is>
+          <t>Tóquio (RJTT)</t>
+        </is>
+      </c>
+      <c r="C61" t="n">
+        <v>40</v>
+      </c>
+      <c r="D61" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="E61" s="3" t="n">
+        <v>0.218397791157902</v>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="inlineStr">
+        <is>
+          <t>Combinado</t>
+        </is>
+      </c>
+      <c r="B62" t="inlineStr">
+        <is>
+          <t>Seul (RKSI)</t>
+        </is>
+      </c>
+      <c r="C62" t="n">
+        <v>20</v>
+      </c>
+      <c r="D62" s="2" t="n">
+        <v>0.95</v>
+      </c>
+      <c r="E62" s="3" t="n">
+        <v>0.2631693719170212</v>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="inlineStr">
+        <is>
+          <t>Combinado</t>
+        </is>
+      </c>
+      <c r="B63" t="inlineStr">
+        <is>
+          <t>Manila (RPLL)</t>
+        </is>
+      </c>
+      <c r="C63" t="n">
+        <v>43</v>
+      </c>
+      <c r="D63" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="E63" s="3" t="n">
+        <v>0.2052968984655665</v>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="inlineStr">
+        <is>
+          <t>Combinado</t>
+        </is>
+      </c>
+      <c r="B64" t="inlineStr">
+        <is>
+          <t>Buenos Aires (SAEZ)</t>
+        </is>
+      </c>
+      <c r="C64" t="n">
+        <v>36</v>
+      </c>
+      <c r="D64" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="E64" s="3" t="n">
+        <v>0.5943425580461936</v>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" t="inlineStr">
+        <is>
+          <t>Combinado</t>
+        </is>
+      </c>
+      <c r="B65" t="inlineStr">
+        <is>
+          <t>Guarulhos (SBGR)</t>
+        </is>
+      </c>
+      <c r="C65" t="n">
+        <v>38</v>
+      </c>
+      <c r="D65" s="2" t="n">
+        <v>0.9736842105263158</v>
+      </c>
+      <c r="E65" s="3" t="n">
+        <v>0.1716760837214112</v>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" t="inlineStr">
+        <is>
+          <t>Combinado</t>
+        </is>
+      </c>
+      <c r="B66" t="inlineStr">
+        <is>
+          <t>Moscou (UUWW)</t>
+        </is>
+      </c>
+      <c r="C66" t="n">
+        <v>34</v>
+      </c>
+      <c r="D66" s="2" t="n">
+        <v>0.9411764705882353</v>
+      </c>
+      <c r="E66" s="3" t="n">
+        <v>0.4957568473774073</v>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" t="inlineStr">
+        <is>
+          <t>Combinado</t>
+        </is>
+      </c>
+      <c r="B67" t="inlineStr">
+        <is>
+          <t>Kuala Lumpur (WMKK)</t>
+        </is>
+      </c>
+      <c r="C67" t="n">
+        <v>6</v>
+      </c>
+      <c r="D67" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="E67" s="3" t="n">
+        <v>0.02281118910147331</v>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" t="inlineStr">
+        <is>
+          <t>Combinado</t>
+        </is>
+      </c>
+      <c r="B68" t="inlineStr">
+        <is>
+          <t>Singapura (WSSS)</t>
+        </is>
+      </c>
+      <c r="C68" t="n">
+        <v>23</v>
+      </c>
+      <c r="D68" s="2" t="n">
+        <v>0.9565217391304348</v>
+      </c>
+      <c r="E68" s="3" t="n">
+        <v>0.07827536771677449</v>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" t="inlineStr">
+        <is>
+          <t>Combinado</t>
+        </is>
+      </c>
+      <c r="B69" t="inlineStr">
+        <is>
+          <t>Pequim (ZBAA)</t>
+        </is>
+      </c>
+      <c r="C69" t="n">
+        <v>15</v>
+      </c>
+      <c r="D69" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="E69" s="3" t="n">
+        <v>0.09900287745257799</v>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" t="inlineStr">
+        <is>
+          <t>Combinado</t>
+        </is>
+      </c>
+      <c r="B70" t="inlineStr">
+        <is>
+          <t>Guangzhou (ZGGG)</t>
+        </is>
+      </c>
+      <c r="C70" t="n">
+        <v>35</v>
+      </c>
+      <c r="D70" s="2" t="n">
+        <v>0.8857142857142857</v>
+      </c>
+      <c r="E70" s="3" t="n">
+        <v>0.1242287830957168</v>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" t="inlineStr">
+        <is>
+          <t>Combinado</t>
+        </is>
+      </c>
+      <c r="B71" t="inlineStr">
+        <is>
+          <t>Shenzhen (ZGSZ)</t>
+        </is>
+      </c>
+      <c r="C71" t="n">
+        <v>92</v>
+      </c>
+      <c r="D71" s="2" t="n">
+        <v>0.9565217391304348</v>
+      </c>
+      <c r="E71" s="3" t="n">
+        <v>0.499676072759845</v>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" t="inlineStr">
+        <is>
+          <t>Combinado</t>
+        </is>
+      </c>
+      <c r="B72" t="inlineStr">
+        <is>
+          <t>Wuhan (ZHHH)</t>
+        </is>
+      </c>
+      <c r="C72" t="n">
+        <v>35</v>
+      </c>
+      <c r="D72" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="E72" s="3" t="n">
+        <v>0.08680414628249902</v>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" t="inlineStr">
+        <is>
+          <t>Combinado</t>
+        </is>
+      </c>
+      <c r="B73" t="inlineStr">
+        <is>
+          <t>Xangai (ZSPD)</t>
+        </is>
+      </c>
+      <c r="C73" t="n">
+        <v>31</v>
+      </c>
+      <c r="D73" s="2" t="n">
+        <v>0.967741935483871</v>
+      </c>
+      <c r="E73" s="3" t="n">
+        <v>0.1904499254936535</v>
       </c>
     </row>
   </sheetData>
@@ -1409,7 +2249,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D19"/>
+  <dimension ref="A1:D40"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
@@ -1447,285 +2287,621 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>821</v>
+        <v>1004</v>
       </c>
       <c r="C2" s="2" t="n">
-        <v>0.8733</v>
+        <v>0.8794999999999999</v>
       </c>
       <c r="D2" s="2" t="n">
-        <v>0.995</v>
+        <v>0.9907</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Londres (EGLC)</t>
+          <t>Munique (EDDM)</t>
         </is>
       </c>
       <c r="B3" t="n">
-        <v>904</v>
+        <v>931</v>
       </c>
       <c r="C3" s="2" t="n">
-        <v>0.8695000000000001</v>
+        <v>0.8464</v>
       </c>
       <c r="D3" s="2" t="n">
-        <v>0.9961</v>
+        <v>0.9974</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Amsterdã (EHAM)</t>
+          <t>Helsinque (EFHK)</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>967</v>
+        <v>895</v>
       </c>
       <c r="C4" s="2" t="n">
-        <v>0.88</v>
+        <v>0.8715000000000001</v>
       </c>
       <c r="D4" s="2" t="n">
-        <v>0.995</v>
+        <v>0.9933999999999999</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Varsóvia (EPWA)</t>
+          <t>Londres (EGLC)</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>951</v>
+        <v>1017</v>
       </c>
       <c r="C5" s="2" t="n">
-        <v>0.8665</v>
+        <v>0.8751</v>
       </c>
       <c r="D5" s="2" t="n">
-        <v>0.9969</v>
+        <v>0.9939</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Madri (LEMD)</t>
+          <t>Amsterdã (EHAM)</t>
         </is>
       </c>
       <c r="B6" t="n">
-        <v>996</v>
+        <v>1050</v>
       </c>
       <c r="C6" s="2" t="n">
-        <v>0.8534</v>
+        <v>0.881</v>
       </c>
       <c r="D6" s="2" t="n">
-        <v>0.9975000000000001</v>
+        <v>0.9943</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Paris (LFPB)</t>
+          <t>Varsóvia (EPWA)</t>
         </is>
       </c>
       <c r="B7" t="n">
-        <v>933</v>
+        <v>1041</v>
       </c>
       <c r="C7" s="2" t="n">
-        <v>0.8564000000000001</v>
+        <v>0.8742</v>
       </c>
       <c r="D7" s="2" t="n">
-        <v>0.9968</v>
+        <v>0.996</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Ancara (LTAC)</t>
+          <t>Cidade do Cabo (FACT)</t>
         </is>
       </c>
       <c r="B8" t="n">
-        <v>973</v>
+        <v>875</v>
       </c>
       <c r="C8" s="2" t="n">
-        <v>0.8438</v>
+        <v>0.8823</v>
       </c>
       <c r="D8" s="2" t="n">
-        <v>0.9972</v>
+        <v>0.9913999999999999</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Istambul (LTFM)</t>
+          <t>Atlanta (KATL)</t>
         </is>
       </c>
       <c r="B9" t="n">
-        <v>878</v>
+        <v>1047</v>
       </c>
       <c r="C9" s="2" t="n">
-        <v>0.9055</v>
+        <v>0.852</v>
       </c>
       <c r="D9" s="2" t="n">
-        <v>0.9919</v>
+        <v>0.9965000000000001</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Cidade do México (MMMX)</t>
+          <t>Denver (KBKF)</t>
         </is>
       </c>
       <c r="B10" t="n">
-        <v>800</v>
+        <v>1040</v>
       </c>
       <c r="C10" s="2" t="n">
-        <v>0.8625</v>
+        <v>0.8683</v>
       </c>
       <c r="D10" s="2" t="n">
-        <v>0.9933999999999999</v>
+        <v>0.9971</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Wellington (NZWN)</t>
+          <t>Dallas (KDAL)</t>
         </is>
       </c>
       <c r="B11" t="n">
-        <v>921</v>
+        <v>1004</v>
       </c>
       <c r="C11" s="2" t="n">
-        <v>0.9446</v>
+        <v>0.8825</v>
       </c>
       <c r="D11" s="2" t="n">
-        <v>0.9941</v>
+        <v>0.9947</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Tóquio (RJTT)</t>
+          <t>Houston (KHOU)</t>
         </is>
       </c>
       <c r="B12" t="n">
-        <v>848</v>
+        <v>993</v>
       </c>
       <c r="C12" s="2" t="n">
-        <v>0.9281</v>
+        <v>0.8802</v>
       </c>
       <c r="D12" s="2" t="n">
-        <v>0.993</v>
+        <v>0.9944</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Seul (RKSI)</t>
+          <t>Los Angeles (KLAX)</t>
         </is>
       </c>
       <c r="B13" t="n">
-        <v>807</v>
+        <v>1015</v>
       </c>
       <c r="C13" s="2" t="n">
-        <v>0.8996</v>
+        <v>0.8966</v>
       </c>
       <c r="D13" s="2" t="n">
-        <v>0.9903</v>
+        <v>0.9847</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Buenos Aires (SAEZ)</t>
+          <t>Nova York (KLGA)</t>
         </is>
       </c>
       <c r="B14" t="n">
-        <v>854</v>
+        <v>1009</v>
       </c>
       <c r="C14" s="2" t="n">
-        <v>0.8782</v>
+        <v>0.8811</v>
       </c>
       <c r="D14" s="2" t="n">
-        <v>0.9944</v>
+        <v>0.9942</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Guarulhos (SBGR)</t>
+          <t>Miami (KMIA)</t>
         </is>
       </c>
       <c r="B15" t="n">
-        <v>917</v>
+        <v>1017</v>
       </c>
       <c r="C15" s="2" t="n">
-        <v>0.8691</v>
+        <v>0.8653</v>
       </c>
       <c r="D15" s="2" t="n">
-        <v>0.9955000000000001</v>
+        <v>0.9933</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Moscou (UUWW)</t>
+          <t>Chicago (KORD)</t>
         </is>
       </c>
       <c r="B16" t="n">
-        <v>830</v>
+        <v>1046</v>
       </c>
       <c r="C16" s="2" t="n">
-        <v>0.888</v>
+        <v>0.8901</v>
       </c>
       <c r="D16" s="2" t="n">
-        <v>0.9901</v>
+        <v>0.9958</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Singapura (WSSS)</t>
+          <t>Seattle (KSEA)</t>
         </is>
       </c>
       <c r="B17" t="n">
-        <v>852</v>
+        <v>1016</v>
       </c>
       <c r="C17" s="2" t="n">
-        <v>0.919</v>
+        <v>0.875</v>
       </c>
       <c r="D17" s="2" t="n">
-        <v>0.9921</v>
+        <v>0.9956</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>Pequim (ZBAA)</t>
+          <t>Madri (LEMD)</t>
         </is>
       </c>
       <c r="B18" t="n">
-        <v>949</v>
+        <v>1071</v>
       </c>
       <c r="C18" s="2" t="n">
-        <v>0.8662</v>
+        <v>0.8571</v>
       </c>
       <c r="D18" s="2" t="n">
-        <v>0.9963</v>
+        <v>0.9968</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
+          <t>Paris (LFPB)</t>
+        </is>
+      </c>
+      <c r="B19" t="n">
+        <v>1031</v>
+      </c>
+      <c r="C19" s="2" t="n">
+        <v>0.8661</v>
+      </c>
+      <c r="D19" s="2" t="n">
+        <v>0.996</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>Milão (LIMC)</t>
+        </is>
+      </c>
+      <c r="B20" t="n">
+        <v>928</v>
+      </c>
+      <c r="C20" s="2" t="n">
+        <v>0.8481</v>
+      </c>
+      <c r="D20" s="2" t="n">
+        <v>0.9975000000000001</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>Tel Aviv (LLBG)</t>
+        </is>
+      </c>
+      <c r="B21" t="n">
+        <v>917</v>
+      </c>
+      <c r="C21" s="2" t="n">
+        <v>0.8484</v>
+      </c>
+      <c r="D21" s="2" t="n">
+        <v>0.9944</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>Ancara (LTAC)</t>
+        </is>
+      </c>
+      <c r="B22" t="n">
+        <v>1059</v>
+      </c>
+      <c r="C22" s="2" t="n">
+        <v>0.8527</v>
+      </c>
+      <c r="D22" s="2" t="n">
+        <v>0.996</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>Istambul (LTFM)</t>
+        </is>
+      </c>
+      <c r="B23" t="n">
+        <v>997</v>
+      </c>
+      <c r="C23" s="2" t="n">
+        <v>0.9056999999999999</v>
+      </c>
+      <c r="D23" s="2" t="n">
+        <v>0.9899</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>Cidade do México (MMMX)</t>
+        </is>
+      </c>
+      <c r="B24" t="n">
+        <v>951</v>
+      </c>
+      <c r="C24" s="2" t="n">
+        <v>0.8791</v>
+      </c>
+      <c r="D24" s="2" t="n">
+        <v>0.99</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>Wellington (NZWN)</t>
+        </is>
+      </c>
+      <c r="B25" t="n">
+        <v>1009</v>
+      </c>
+      <c r="C25" s="2" t="n">
+        <v>0.9326</v>
+      </c>
+      <c r="D25" s="2" t="n">
+        <v>0.9932</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>Taipé (RCSS)</t>
+        </is>
+      </c>
+      <c r="B26" t="n">
+        <v>860</v>
+      </c>
+      <c r="C26" s="2" t="n">
+        <v>0.8907</v>
+      </c>
+      <c r="D26" s="2" t="n">
+        <v>0.9921</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>Tóquio (RJTT)</t>
+        </is>
+      </c>
+      <c r="B27" t="n">
+        <v>986</v>
+      </c>
+      <c r="C27" s="2" t="n">
+        <v>0.9147999999999999</v>
+      </c>
+      <c r="D27" s="2" t="n">
+        <v>0.9859</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>Seul (RKSI)</t>
+        </is>
+      </c>
+      <c r="B28" t="n">
+        <v>987</v>
+      </c>
+      <c r="C28" s="2" t="n">
+        <v>0.9078000000000001</v>
+      </c>
+      <c r="D28" s="2" t="n">
+        <v>0.9866</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>Manila (RPLL)</t>
+        </is>
+      </c>
+      <c r="B29" t="n">
+        <v>859</v>
+      </c>
+      <c r="C29" s="2" t="n">
+        <v>0.8964</v>
+      </c>
+      <c r="D29" s="2" t="n">
+        <v>0.9935</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>Buenos Aires (SAEZ)</t>
+        </is>
+      </c>
+      <c r="B30" t="n">
+        <v>982</v>
+      </c>
+      <c r="C30" s="2" t="n">
+        <v>0.8829</v>
+      </c>
+      <c r="D30" s="2" t="n">
+        <v>0.9917</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>Guarulhos (SBGR)</t>
+        </is>
+      </c>
+      <c r="B31" t="n">
+        <v>1024</v>
+      </c>
+      <c r="C31" s="2" t="n">
+        <v>0.877</v>
+      </c>
+      <c r="D31" s="2" t="n">
+        <v>0.9928</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>Moscou (UUWW)</t>
+        </is>
+      </c>
+      <c r="B32" t="n">
+        <v>1006</v>
+      </c>
+      <c r="C32" s="2" t="n">
+        <v>0.8817</v>
+      </c>
+      <c r="D32" s="2" t="n">
+        <v>0.9898</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>Kuala Lumpur (WMKK)</t>
+        </is>
+      </c>
+      <c r="B33" t="n">
+        <v>814</v>
+      </c>
+      <c r="C33" s="2" t="n">
+        <v>0.8968</v>
+      </c>
+      <c r="D33" s="2" t="n">
+        <v>0.9889</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>Singapura (WSSS)</t>
+        </is>
+      </c>
+      <c r="B34" t="n">
+        <v>964</v>
+      </c>
+      <c r="C34" s="2" t="n">
+        <v>0.9222</v>
+      </c>
+      <c r="D34" s="2" t="n">
+        <v>0.9909</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>Pequim (ZBAA)</t>
+        </is>
+      </c>
+      <c r="B35" t="n">
+        <v>1038</v>
+      </c>
+      <c r="C35" s="2" t="n">
+        <v>0.8671</v>
+      </c>
+      <c r="D35" s="2" t="n">
+        <v>0.995</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>Guangzhou (ZGGG)</t>
+        </is>
+      </c>
+      <c r="B36" t="n">
+        <v>820</v>
+      </c>
+      <c r="C36" s="2" t="n">
+        <v>0.8976</v>
+      </c>
+      <c r="D36" s="2" t="n">
+        <v>0.9909</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>Shenzhen (ZGSZ)</t>
+        </is>
+      </c>
+      <c r="B37" t="n">
+        <v>894</v>
+      </c>
+      <c r="C37" s="2" t="n">
+        <v>0.9116</v>
+      </c>
+      <c r="D37" s="2" t="n">
+        <v>0.9926</v>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>Wuhan (ZHHH)</t>
+        </is>
+      </c>
+      <c r="B38" t="n">
+        <v>868</v>
+      </c>
+      <c r="C38" s="2" t="n">
+        <v>0.8871</v>
+      </c>
+      <c r="D38" s="2" t="n">
+        <v>0.9913</v>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
           <t>Xangai (ZSPD)</t>
         </is>
       </c>
-      <c r="B19" t="n">
-        <v>946</v>
-      </c>
-      <c r="C19" s="2" t="n">
-        <v>0.9112</v>
-      </c>
-      <c r="D19" s="2" t="n">
-        <v>0.9923999999999999</v>
+      <c r="B39" t="n">
+        <v>1047</v>
+      </c>
+      <c r="C39" s="2" t="n">
+        <v>0.8911</v>
+      </c>
+      <c r="D39" s="2" t="n">
+        <v>0.9896</v>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>Chengdu (ZUUU)</t>
+        </is>
+      </c>
+      <c r="B40" t="n">
+        <v>854</v>
+      </c>
+      <c r="C40" s="2" t="n">
+        <v>0.8712</v>
+      </c>
+      <c r="D40" s="2" t="n">
+        <v>0.9926</v>
       </c>
     </row>
   </sheetData>
@@ -1789,19 +2965,19 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>0.133</v>
+        <v>0.135</v>
       </c>
       <c r="C2" t="n">
-        <v>0.1224</v>
+        <v>0.135</v>
       </c>
       <c r="D2" t="n">
-        <v>0.0051</v>
+        <v>0.0049</v>
       </c>
       <c r="E2" t="n">
-        <v>1.0466</v>
+        <v>1.0403</v>
       </c>
       <c r="F2" t="n">
-        <v>0.073</v>
+        <v>0.0742</v>
       </c>
     </row>
     <row r="3">
@@ -1811,19 +2987,19 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>0.1271</v>
+        <v>0.13</v>
       </c>
       <c r="C3" t="n">
-        <v>0.1092</v>
+        <v>0.13</v>
       </c>
       <c r="D3" t="n">
-        <v>0.0017</v>
+        <v>-0.008500000000000001</v>
       </c>
       <c r="E3" t="n">
-        <v>1.0421</v>
+        <v>1.0613</v>
       </c>
       <c r="F3" t="n">
-        <v>0.08110000000000001</v>
+        <v>0.0815</v>
       </c>
     </row>
     <row r="4">
@@ -1833,19 +3009,19 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>0.0436</v>
+        <v>0.0509</v>
       </c>
       <c r="C4" t="n">
-        <v>0.0383</v>
+        <v>0.0447</v>
       </c>
       <c r="D4" t="n">
-        <v>0.1211</v>
+        <v>0.0858</v>
       </c>
       <c r="E4" t="n">
-        <v>0.995</v>
+        <v>1.0179</v>
       </c>
       <c r="F4" t="n">
-        <v>0.0602</v>
+        <v>0.0629</v>
       </c>
     </row>
   </sheetData>
@@ -1874,7 +3050,7 @@
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>2026-07-25T09:07:30+00:00</t>
+          <t>2026-07-28T09:48:16+00:00</t>
         </is>
       </c>
     </row>
@@ -1885,7 +3061,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>1826</v>
+        <v>3881</v>
       </c>
     </row>
     <row r="3">
@@ -1895,7 +3071,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>101</v>
+        <v>100</v>
       </c>
     </row>
     <row r="4">
@@ -1905,7 +3081,7 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>18</v>
+        <v>39</v>
       </c>
     </row>
     <row r="5">
@@ -1925,7 +3101,7 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>46</v>
+        <v>186</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Arquiva dados, recalibra e atualiza docs (2026-07-31)
</commit_message>
<xml_diff>
--- a/backtest_results/resultados_backtest.xlsx
+++ b/backtest_results/resultados_backtest.xlsx
@@ -516,28 +516,28 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>322</v>
+        <v>343</v>
       </c>
       <c r="C2" s="2" t="n">
-        <v>0.8975155279503105</v>
+        <v>0.8950437317784257</v>
       </c>
       <c r="D2" s="3" t="n">
-        <v>4.037473155639022</v>
+        <v>4.560707689951263</v>
       </c>
       <c r="E2" s="4" t="n">
-        <v>20.19841346343609</v>
+        <v>28.02788094283614</v>
       </c>
       <c r="F2" s="2" t="n">
-        <v>1.46374171808818</v>
+        <v>1.640147752218049</v>
       </c>
       <c r="G2" s="2" t="n">
         <v>0.2170352923628444</v>
       </c>
       <c r="H2" t="n">
-        <v>62</v>
+        <v>68</v>
       </c>
       <c r="I2" s="3" t="n">
-        <v>0.8386086956521739</v>
+        <v>0.8323381924198251</v>
       </c>
     </row>
     <row r="3">
@@ -547,28 +547,28 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>1679</v>
+        <v>1736</v>
       </c>
       <c r="C3" s="2" t="n">
-        <v>0.9940440738534843</v>
+        <v>0.993663594470046</v>
       </c>
       <c r="D3" s="3" t="n">
-        <v>1.890835831197596</v>
+        <v>1.948048719175096</v>
       </c>
       <c r="E3" s="4" t="n">
-        <v>2.748689574300068</v>
+        <v>2.837148066055549</v>
       </c>
       <c r="F3" s="2" t="n">
-        <v>0.3543711950145478</v>
+        <v>0.3549004252321757</v>
       </c>
       <c r="G3" s="2" t="n">
-        <v>0.08704657533117888</v>
+        <v>0.08704657533117932</v>
       </c>
       <c r="H3" t="n">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="I3" s="3" t="n">
-        <v>0.9857066706372841</v>
+        <v>0.9857531682027649</v>
       </c>
     </row>
     <row r="4">
@@ -578,28 +578,28 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>1214</v>
+        <v>1259</v>
       </c>
       <c r="C4" s="2" t="n">
-        <v>0.9950576606260296</v>
+        <v>0.9944400317712471</v>
       </c>
       <c r="D4" s="3" t="n">
-        <v>1.325577596940686</v>
+        <v>1.367908183446105</v>
       </c>
       <c r="E4" s="4" t="n">
-        <v>2.313242463695541</v>
+        <v>2.365867722085081</v>
       </c>
       <c r="F4" s="2" t="n">
-        <v>0.2860751501989593</v>
+        <v>0.2850773230877728</v>
       </c>
       <c r="G4" s="2" t="n">
-        <v>0.08016721391959125</v>
+        <v>0.08016721391959114</v>
       </c>
       <c r="H4" t="n">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="I4" s="3" t="n">
-        <v>0.9866803953871499</v>
+        <v>0.9866898332009532</v>
       </c>
     </row>
     <row r="5">
@@ -609,19 +609,19 @@
         </is>
       </c>
       <c r="B5" s="5" t="n">
-        <v>636</v>
+        <v>664</v>
       </c>
       <c r="C5" s="6" t="n">
-        <v>0.9984276729559748</v>
+        <v>0.9984939759036144</v>
       </c>
       <c r="D5" s="7" t="n">
-        <v>0.7252985342410232</v>
+        <v>0.765749080790208</v>
       </c>
       <c r="E5" s="8" t="n">
-        <v>1.759873310506253</v>
+        <v>1.81177862053934</v>
       </c>
       <c r="F5" s="6" t="n">
-        <v>0.1847982976405755</v>
+        <v>0.1889846603581167</v>
       </c>
       <c r="G5" s="6" t="n">
         <v>0.02619857308701179</v>
@@ -630,7 +630,7 @@
         <v>5</v>
       </c>
       <c r="I5" s="7" t="n">
-        <v>0.987495283018868</v>
+        <v>0.9874239457831325</v>
       </c>
     </row>
     <row r="6">
@@ -640,34 +640,34 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>958</v>
+        <v>1007</v>
       </c>
       <c r="C6" s="2" t="n">
-        <v>0.964509394572025</v>
+        <v>0.9632571996027806</v>
       </c>
       <c r="D6" s="3" t="n">
-        <v>4.762771689880045</v>
+        <v>5.326456770741472</v>
       </c>
       <c r="E6" s="4" t="n">
-        <v>24.84427521783187</v>
+        <v>34.11269547699197</v>
       </c>
       <c r="F6" s="2" t="n">
-        <v>1.621608880265423</v>
+        <v>1.795634550883839</v>
       </c>
       <c r="G6" s="2" t="n">
         <v>0.1983925675638193</v>
       </c>
       <c r="H6" t="n">
-        <v>67</v>
+        <v>73</v>
       </c>
       <c r="I6" s="3" t="n">
-        <v>0.9374519832985387</v>
+        <v>0.9345993048659385</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Atualizado em 2026-07-28T09:48:16+00:00 · arquivo de 3881 dias-cidade (~100 dias corridos) · 39 cidades</t>
+          <t>Atualizado em 2026-07-31T09:10:36+00:00 · arquivo de 3998 dias-cidade (~103 dias corridos) · 39 cidades</t>
         </is>
       </c>
     </row>
@@ -689,7 +689,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E73"/>
+  <dimension ref="A1:E75"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -822,13 +822,13 @@
         </is>
       </c>
       <c r="C6" t="n">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="D6" s="2" t="n">
-        <v>0.9285714285714286</v>
+        <v>0.9375</v>
       </c>
       <c r="E6" s="3" t="n">
-        <v>0.01843717445760852</v>
+        <v>0.0708055546408668</v>
       </c>
     </row>
     <row r="7">
@@ -969,13 +969,13 @@
         </is>
       </c>
       <c r="C13" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="D13" s="2" t="n">
-        <v>0.6</v>
+        <v>0.7142857142857143</v>
       </c>
       <c r="E13" s="3" t="n">
-        <v>0.006890414114194828</v>
+        <v>0.1799384187411469</v>
       </c>
     </row>
     <row r="14">
@@ -1074,13 +1074,13 @@
         </is>
       </c>
       <c r="C18" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D18" s="2" t="n">
         <v>1</v>
       </c>
       <c r="E18" s="3" t="n">
-        <v>0.01419268854547966</v>
+        <v>0.02847840283119394</v>
       </c>
     </row>
     <row r="19">
@@ -1137,13 +1137,13 @@
         </is>
       </c>
       <c r="C21" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="D21" s="2" t="n">
-        <v>0.75</v>
+        <v>0.8333333333333334</v>
       </c>
       <c r="E21" s="3" t="n">
-        <v>0.006895137313328397</v>
+        <v>0.02092739537784452</v>
       </c>
     </row>
     <row r="22">
@@ -1179,13 +1179,13 @@
         </is>
       </c>
       <c r="C23" t="n">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="D23" s="2" t="n">
-        <v>0.9090909090909091</v>
+        <v>0.9130434782608695</v>
       </c>
       <c r="E23" s="3" t="n">
-        <v>0.2295774625433846</v>
+        <v>0.2694376024035244</v>
       </c>
     </row>
     <row r="24">
@@ -1200,13 +1200,13 @@
         </is>
       </c>
       <c r="C24" t="n">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="D24" s="2" t="n">
         <v>1</v>
       </c>
       <c r="E24" s="3" t="n">
-        <v>0.1844042105660792</v>
+        <v>0.2986899248517935</v>
       </c>
     </row>
     <row r="25">
@@ -1221,13 +1221,13 @@
         </is>
       </c>
       <c r="C25" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="D25" s="2" t="n">
-        <v>0.9230769230769231</v>
+        <v>0.9285714285714286</v>
       </c>
       <c r="E25" s="3" t="n">
-        <v>0.2566434903166885</v>
+        <v>0.2659331078030273</v>
       </c>
     </row>
     <row r="26">
@@ -1263,13 +1263,13 @@
         </is>
       </c>
       <c r="C27" t="n">
-        <v>17</v>
+        <v>20</v>
       </c>
       <c r="D27" s="2" t="n">
-        <v>1</v>
+        <v>0.95</v>
       </c>
       <c r="E27" s="3" t="n">
-        <v>0.5673435632805013</v>
+        <v>0.7046621818573011</v>
       </c>
     </row>
     <row r="28">
@@ -1326,13 +1326,13 @@
         </is>
       </c>
       <c r="C30" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D30" s="2" t="n">
         <v>1</v>
       </c>
       <c r="E30" s="3" t="n">
-        <v>0.01972871211600642</v>
+        <v>0.02901832960234521</v>
       </c>
     </row>
     <row r="31">
@@ -1389,13 +1389,13 @@
         </is>
       </c>
       <c r="C33" t="n">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="D33" s="2" t="n">
-        <v>0.8095238095238095</v>
+        <v>0.8181818181818182</v>
       </c>
       <c r="E33" s="3" t="n">
-        <v>0.1065260645220891</v>
+        <v>0.1201624281584527</v>
       </c>
     </row>
     <row r="34">
@@ -1410,13 +1410,13 @@
         </is>
       </c>
       <c r="C34" t="n">
-        <v>43</v>
+        <v>45</v>
       </c>
       <c r="D34" s="2" t="n">
-        <v>0.9069767441860465</v>
+        <v>0.8888888888888888</v>
       </c>
       <c r="E34" s="3" t="n">
-        <v>0.4367327818601304</v>
+        <v>0.4067327818601304</v>
       </c>
     </row>
     <row r="35">
@@ -1464,22 +1464,22 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>Combinado</t>
+          <t>Edge</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>Toronto (CYYZ)</t>
+          <t>Chengdu (ZUUU)</t>
         </is>
       </c>
       <c r="C37" t="n">
-        <v>16</v>
+        <v>3</v>
       </c>
       <c r="D37" s="2" t="n">
-        <v>0.9375</v>
+        <v>0.6666666666666666</v>
       </c>
       <c r="E37" s="3" t="n">
-        <v>0.02649807219830284</v>
+        <v>-0.02417989417989416</v>
       </c>
     </row>
     <row r="38">
@@ -1490,17 +1490,17 @@
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>Munique (EDDM)</t>
+          <t>Toronto (CYYZ)</t>
         </is>
       </c>
       <c r="C38" t="n">
-        <v>21</v>
+        <v>17</v>
       </c>
       <c r="D38" s="2" t="n">
-        <v>0.9523809523809523</v>
+        <v>0.9411764705882353</v>
       </c>
       <c r="E38" s="3" t="n">
-        <v>0.02897737559373625</v>
+        <v>0.02895708859174546</v>
       </c>
     </row>
     <row r="39">
@@ -1511,17 +1511,17 @@
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>Helsinque (EFHK)</t>
+          <t>Munique (EDDM)</t>
         </is>
       </c>
       <c r="C39" t="n">
-        <v>29</v>
+        <v>21</v>
       </c>
       <c r="D39" s="2" t="n">
-        <v>1</v>
+        <v>0.9523809523809523</v>
       </c>
       <c r="E39" s="3" t="n">
-        <v>0.01943847144601079</v>
+        <v>0.02897737559373625</v>
       </c>
     </row>
     <row r="40">
@@ -1532,17 +1532,17 @@
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>Londres (EGLC)</t>
+          <t>Helsinque (EFHK)</t>
         </is>
       </c>
       <c r="C40" t="n">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="D40" s="2" t="n">
-        <v>0.96875</v>
+        <v>1</v>
       </c>
       <c r="E40" s="3" t="n">
-        <v>0.06505197524359005</v>
+        <v>0.02202204037444169</v>
       </c>
     </row>
     <row r="41">
@@ -1553,17 +1553,17 @@
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>Amsterdã (EHAM)</t>
+          <t>Londres (EGLC)</t>
         </is>
       </c>
       <c r="C41" t="n">
-        <v>54</v>
+        <v>32</v>
       </c>
       <c r="D41" s="2" t="n">
-        <v>0.9814814814814815</v>
+        <v>0.96875</v>
       </c>
       <c r="E41" s="3" t="n">
-        <v>0.05499900040126621</v>
+        <v>0.06505197524359005</v>
       </c>
     </row>
     <row r="42">
@@ -1574,17 +1574,17 @@
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>Varsóvia (EPWA)</t>
+          <t>Amsterdã (EHAM)</t>
         </is>
       </c>
       <c r="C42" t="n">
-        <v>15</v>
+        <v>60</v>
       </c>
       <c r="D42" s="2" t="n">
-        <v>0.9333333333333333</v>
+        <v>0.9833333333333333</v>
       </c>
       <c r="E42" s="3" t="n">
-        <v>0.1573199025875285</v>
+        <v>0.1124566210129819</v>
       </c>
     </row>
     <row r="43">
@@ -1595,17 +1595,17 @@
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>Cidade do Cabo (FACT)</t>
+          <t>Varsóvia (EPWA)</t>
         </is>
       </c>
       <c r="C43" t="n">
-        <v>23</v>
+        <v>15</v>
       </c>
       <c r="D43" s="2" t="n">
-        <v>1</v>
+        <v>0.9333333333333333</v>
       </c>
       <c r="E43" s="3" t="n">
-        <v>0.02646317118320567</v>
+        <v>0.1573199025875285</v>
       </c>
     </row>
     <row r="44">
@@ -1616,17 +1616,17 @@
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>Atlanta (KATL)</t>
+          <t>Cidade do Cabo (FACT)</t>
         </is>
       </c>
       <c r="C44" t="n">
-        <v>16</v>
+        <v>27</v>
       </c>
       <c r="D44" s="2" t="n">
-        <v>0.9375</v>
+        <v>1</v>
       </c>
       <c r="E44" s="3" t="n">
-        <v>0.003500706411286052</v>
+        <v>0.03390174677547726</v>
       </c>
     </row>
     <row r="45">
@@ -1637,17 +1637,17 @@
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>Denver (KBKF)</t>
+          <t>Atlanta (KATL)</t>
         </is>
       </c>
       <c r="C45" t="n">
-        <v>5</v>
+        <v>16</v>
       </c>
       <c r="D45" s="2" t="n">
-        <v>1</v>
+        <v>0.9375</v>
       </c>
       <c r="E45" s="3" t="n">
-        <v>0.08135918956658879</v>
+        <v>0.003500706411286052</v>
       </c>
     </row>
     <row r="46">
@@ -1658,17 +1658,17 @@
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>Dallas (KDAL)</t>
+          <t>Denver (KBKF)</t>
         </is>
       </c>
       <c r="C46" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="D46" s="2" t="n">
         <v>1</v>
       </c>
       <c r="E46" s="3" t="n">
-        <v>0.01731065767370086</v>
+        <v>0.08135918956658879</v>
       </c>
     </row>
     <row r="47">
@@ -1679,17 +1679,17 @@
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>Houston (KHOU)</t>
+          <t>Dallas (KDAL)</t>
         </is>
       </c>
       <c r="C47" t="n">
-        <v>10</v>
+        <v>6</v>
       </c>
       <c r="D47" s="2" t="n">
-        <v>0.6</v>
+        <v>1</v>
       </c>
       <c r="E47" s="3" t="n">
-        <v>-0.05112262463304137</v>
+        <v>0.01731065767370086</v>
       </c>
     </row>
     <row r="48">
@@ -1700,17 +1700,17 @@
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>Los Angeles (KLAX)</t>
+          <t>Houston (KHOU)</t>
         </is>
       </c>
       <c r="C48" t="n">
-        <v>14</v>
+        <v>10</v>
       </c>
       <c r="D48" s="2" t="n">
-        <v>0.8571428571428571</v>
+        <v>0.6</v>
       </c>
       <c r="E48" s="3" t="n">
-        <v>0.01528237604625361</v>
+        <v>-0.05112262463304137</v>
       </c>
     </row>
     <row r="49">
@@ -1721,17 +1721,17 @@
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>Nova York (KLGA)</t>
+          <t>Los Angeles (KLAX)</t>
         </is>
       </c>
       <c r="C49" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="D49" s="2" t="n">
-        <v>0.9375</v>
+        <v>0.8823529411764706</v>
       </c>
       <c r="E49" s="3" t="n">
-        <v>0.09285061569441484</v>
+        <v>0.1905798694257619</v>
       </c>
     </row>
     <row r="50">
@@ -1742,17 +1742,17 @@
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>Miami (KMIA)</t>
+          <t>Nova York (KLGA)</t>
         </is>
       </c>
       <c r="C50" t="n">
-        <v>29</v>
+        <v>16</v>
       </c>
       <c r="D50" s="2" t="n">
-        <v>0.9655172413793104</v>
+        <v>0.9375</v>
       </c>
       <c r="E50" s="3" t="n">
-        <v>0.1437867028586853</v>
+        <v>0.09285061569441484</v>
       </c>
     </row>
     <row r="51">
@@ -1763,17 +1763,17 @@
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>Chicago (KORD)</t>
+          <t>Miami (KMIA)</t>
         </is>
       </c>
       <c r="C51" t="n">
-        <v>21</v>
+        <v>29</v>
       </c>
       <c r="D51" s="2" t="n">
-        <v>1</v>
+        <v>0.9655172413793104</v>
       </c>
       <c r="E51" s="3" t="n">
-        <v>0.04168440738044763</v>
+        <v>0.1437867028586853</v>
       </c>
     </row>
     <row r="52">
@@ -1784,17 +1784,17 @@
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>Seattle (KSEA)</t>
+          <t>Chicago (KORD)</t>
         </is>
       </c>
       <c r="C52" t="n">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="D52" s="2" t="n">
-        <v>0.9545454545454546</v>
+        <v>1</v>
       </c>
       <c r="E52" s="3" t="n">
-        <v>-0.02457179188325269</v>
+        <v>0.04168440738044763</v>
       </c>
     </row>
     <row r="53">
@@ -1805,17 +1805,17 @@
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>Madri (LEMD)</t>
+          <t>Seattle (KSEA)</t>
         </is>
       </c>
       <c r="C53" t="n">
-        <v>4</v>
+        <v>22</v>
       </c>
       <c r="D53" s="2" t="n">
-        <v>1</v>
+        <v>0.9545454545454546</v>
       </c>
       <c r="E53" s="3" t="n">
-        <v>0.005385531300417991</v>
+        <v>-0.02457179188325269</v>
       </c>
     </row>
     <row r="54">
@@ -1826,17 +1826,17 @@
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>Milão (LIMC)</t>
+          <t>Madri (LEMD)</t>
         </is>
       </c>
       <c r="C54" t="n">
-        <v>19</v>
+        <v>4</v>
       </c>
       <c r="D54" s="2" t="n">
         <v>1</v>
       </c>
       <c r="E54" s="3" t="n">
-        <v>0.03465308375945613</v>
+        <v>0.005385531300417991</v>
       </c>
     </row>
     <row r="55">
@@ -1847,17 +1847,17 @@
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>Tel Aviv (LLBG)</t>
+          <t>Milão (LIMC)</t>
         </is>
       </c>
       <c r="C55" t="n">
-        <v>4</v>
+        <v>20</v>
       </c>
       <c r="D55" s="2" t="n">
         <v>1</v>
       </c>
       <c r="E55" s="3" t="n">
-        <v>0.005115058255058735</v>
+        <v>0.04893879804517041</v>
       </c>
     </row>
     <row r="56">
@@ -1868,17 +1868,17 @@
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>Ancara (LTAC)</t>
+          <t>Tel Aviv (LLBG)</t>
         </is>
       </c>
       <c r="C56" t="n">
-        <v>9</v>
+        <v>4</v>
       </c>
       <c r="D56" s="2" t="n">
         <v>1</v>
       </c>
       <c r="E56" s="3" t="n">
-        <v>0.01770727377980937</v>
+        <v>0.005115058255058735</v>
       </c>
     </row>
     <row r="57">
@@ -1889,17 +1889,17 @@
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>Istambul (LTFM)</t>
+          <t>Ancara (LTAC)</t>
         </is>
       </c>
       <c r="C57" t="n">
-        <v>61</v>
+        <v>9</v>
       </c>
       <c r="D57" s="2" t="n">
         <v>1</v>
       </c>
       <c r="E57" s="3" t="n">
-        <v>0.2820296780107753</v>
+        <v>0.01770727377980937</v>
       </c>
     </row>
     <row r="58">
@@ -1910,17 +1910,17 @@
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>Cidade do México (MMMX)</t>
+          <t>Istambul (LTFM)</t>
         </is>
       </c>
       <c r="C58" t="n">
-        <v>17</v>
+        <v>62</v>
       </c>
       <c r="D58" s="2" t="n">
-        <v>0.9411764705882353</v>
+        <v>1</v>
       </c>
       <c r="E58" s="3" t="n">
-        <v>0.02246255388826923</v>
+        <v>0.2832955007955854</v>
       </c>
     </row>
     <row r="59">
@@ -1931,17 +1931,17 @@
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>Wellington (NZWN)</t>
+          <t>Cidade do México (MMMX)</t>
         </is>
       </c>
       <c r="C59" t="n">
-        <v>43</v>
+        <v>20</v>
       </c>
       <c r="D59" s="2" t="n">
-        <v>0.9534883720930233</v>
+        <v>0.95</v>
       </c>
       <c r="E59" s="3" t="n">
-        <v>0.4156127746967782</v>
+        <v>0.03704785368229767</v>
       </c>
     </row>
     <row r="60">
@@ -1952,17 +1952,17 @@
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>Taipé (RCSS)</t>
+          <t>Wellington (NZWN)</t>
         </is>
       </c>
       <c r="C60" t="n">
-        <v>24</v>
+        <v>44</v>
       </c>
       <c r="D60" s="2" t="n">
-        <v>0.9166666666666666</v>
+        <v>0.9545454545454546</v>
       </c>
       <c r="E60" s="3" t="n">
-        <v>0.2310896158327151</v>
+        <v>0.4179193354051783</v>
       </c>
     </row>
     <row r="61">
@@ -1973,17 +1973,17 @@
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>Tóquio (RJTT)</t>
+          <t>Taipé (RCSS)</t>
         </is>
       </c>
       <c r="C61" t="n">
-        <v>40</v>
+        <v>26</v>
       </c>
       <c r="D61" s="2" t="n">
-        <v>1</v>
+        <v>0.9230769230769231</v>
       </c>
       <c r="E61" s="3" t="n">
-        <v>0.218397791157902</v>
+        <v>0.2717562073057582</v>
       </c>
     </row>
     <row r="62">
@@ -1994,17 +1994,17 @@
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>Seul (RKSI)</t>
+          <t>Tóquio (RJTT)</t>
         </is>
       </c>
       <c r="C62" t="n">
-        <v>20</v>
+        <v>43</v>
       </c>
       <c r="D62" s="2" t="n">
-        <v>0.95</v>
+        <v>1</v>
       </c>
       <c r="E62" s="3" t="n">
-        <v>0.2631693719170212</v>
+        <v>0.3332871271739986</v>
       </c>
     </row>
     <row r="63">
@@ -2015,17 +2015,17 @@
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>Manila (RPLL)</t>
+          <t>Seul (RKSI)</t>
         </is>
       </c>
       <c r="C63" t="n">
-        <v>43</v>
+        <v>21</v>
       </c>
       <c r="D63" s="2" t="n">
-        <v>1</v>
+        <v>0.9523809523809523</v>
       </c>
       <c r="E63" s="3" t="n">
-        <v>0.2052968984655665</v>
+        <v>0.27245898940336</v>
       </c>
     </row>
     <row r="64">
@@ -2036,17 +2036,17 @@
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>Buenos Aires (SAEZ)</t>
+          <t>Manila (RPLL)</t>
         </is>
       </c>
       <c r="C64" t="n">
-        <v>36</v>
+        <v>43</v>
       </c>
       <c r="D64" s="2" t="n">
         <v>1</v>
       </c>
       <c r="E64" s="3" t="n">
-        <v>0.5943425580461936</v>
+        <v>0.2052968984655665</v>
       </c>
     </row>
     <row r="65">
@@ -2057,17 +2057,17 @@
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>Guarulhos (SBGR)</t>
+          <t>Buenos Aires (SAEZ)</t>
         </is>
       </c>
       <c r="C65" t="n">
-        <v>38</v>
+        <v>41</v>
       </c>
       <c r="D65" s="2" t="n">
-        <v>0.9736842105263158</v>
+        <v>0.975609756097561</v>
       </c>
       <c r="E65" s="3" t="n">
-        <v>0.1716760837214112</v>
+        <v>0.7351733272975708</v>
       </c>
     </row>
     <row r="66">
@@ -2078,17 +2078,17 @@
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>Moscou (UUWW)</t>
+          <t>Guarulhos (SBGR)</t>
         </is>
       </c>
       <c r="C66" t="n">
-        <v>34</v>
+        <v>38</v>
       </c>
       <c r="D66" s="2" t="n">
-        <v>0.9411764705882353</v>
+        <v>0.9736842105263158</v>
       </c>
       <c r="E66" s="3" t="n">
-        <v>0.4957568473774073</v>
+        <v>0.1716760837214112</v>
       </c>
     </row>
     <row r="67">
@@ -2099,17 +2099,17 @@
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>Kuala Lumpur (WMKK)</t>
+          <t>Moscou (UUWW)</t>
         </is>
       </c>
       <c r="C67" t="n">
-        <v>6</v>
+        <v>36</v>
       </c>
       <c r="D67" s="2" t="n">
-        <v>1</v>
+        <v>0.9444444444444444</v>
       </c>
       <c r="E67" s="3" t="n">
-        <v>0.02281118910147331</v>
+        <v>0.4982893237163585</v>
       </c>
     </row>
     <row r="68">
@@ -2120,17 +2120,17 @@
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>Singapura (WSSS)</t>
+          <t>Kuala Lumpur (WMKK)</t>
         </is>
       </c>
       <c r="C68" t="n">
-        <v>23</v>
+        <v>8</v>
       </c>
       <c r="D68" s="2" t="n">
-        <v>0.9565217391304348</v>
+        <v>1</v>
       </c>
       <c r="E68" s="3" t="n">
-        <v>0.07827536771677449</v>
+        <v>0.03321304116819632</v>
       </c>
     </row>
     <row r="69">
@@ -2141,17 +2141,17 @@
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>Pequim (ZBAA)</t>
+          <t>Singapura (WSSS)</t>
         </is>
       </c>
       <c r="C69" t="n">
-        <v>15</v>
+        <v>24</v>
       </c>
       <c r="D69" s="2" t="n">
-        <v>1</v>
+        <v>0.9583333333333334</v>
       </c>
       <c r="E69" s="3" t="n">
-        <v>0.09900287745257799</v>
+        <v>0.0788284094462868</v>
       </c>
     </row>
     <row r="70">
@@ -2162,17 +2162,17 @@
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>Guangzhou (ZGGG)</t>
+          <t>Pequim (ZBAA)</t>
         </is>
       </c>
       <c r="C70" t="n">
-        <v>35</v>
+        <v>15</v>
       </c>
       <c r="D70" s="2" t="n">
-        <v>0.8857142857142857</v>
+        <v>1</v>
       </c>
       <c r="E70" s="3" t="n">
-        <v>0.1242287830957168</v>
+        <v>0.09900287745257799</v>
       </c>
     </row>
     <row r="71">
@@ -2183,17 +2183,17 @@
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>Shenzhen (ZGSZ)</t>
+          <t>Guangzhou (ZGGG)</t>
         </is>
       </c>
       <c r="C71" t="n">
-        <v>92</v>
+        <v>36</v>
       </c>
       <c r="D71" s="2" t="n">
-        <v>0.9565217391304348</v>
+        <v>0.8888888888888888</v>
       </c>
       <c r="E71" s="3" t="n">
-        <v>0.499676072759845</v>
+        <v>0.1378651467320804</v>
       </c>
     </row>
     <row r="72">
@@ -2204,17 +2204,17 @@
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>Wuhan (ZHHH)</t>
+          <t>Shenzhen (ZGSZ)</t>
         </is>
       </c>
       <c r="C72" t="n">
-        <v>35</v>
+        <v>94</v>
       </c>
       <c r="D72" s="2" t="n">
-        <v>1</v>
+        <v>0.9468085106382979</v>
       </c>
       <c r="E72" s="3" t="n">
-        <v>0.08680414628249902</v>
+        <v>0.469676072759845</v>
       </c>
     </row>
     <row r="73">
@@ -2225,17 +2225,59 @@
       </c>
       <c r="B73" t="inlineStr">
         <is>
+          <t>Wuhan (ZHHH)</t>
+        </is>
+      </c>
+      <c r="C73" t="n">
+        <v>38</v>
+      </c>
+      <c r="D73" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="E73" s="3" t="n">
+        <v>0.0912822137746932</v>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" t="inlineStr">
+        <is>
+          <t>Combinado</t>
+        </is>
+      </c>
+      <c r="B74" t="inlineStr">
+        <is>
           <t>Xangai (ZSPD)</t>
         </is>
       </c>
-      <c r="C73" t="n">
+      <c r="C74" t="n">
         <v>31</v>
       </c>
-      <c r="D73" s="2" t="n">
+      <c r="D74" s="2" t="n">
         <v>0.967741935483871</v>
       </c>
-      <c r="E73" s="3" t="n">
+      <c r="E74" s="3" t="n">
         <v>0.1904499254936535</v>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" t="inlineStr">
+        <is>
+          <t>Combinado</t>
+        </is>
+      </c>
+      <c r="B75" t="inlineStr">
+        <is>
+          <t>Chengdu (ZUUU)</t>
+        </is>
+      </c>
+      <c r="C75" t="n">
+        <v>5</v>
+      </c>
+      <c r="D75" s="2" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="E75" s="3" t="n">
+        <v>-0.02127270710749547</v>
       </c>
     </row>
   </sheetData>
@@ -2287,13 +2329,13 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>1004</v>
+        <v>1024</v>
       </c>
       <c r="C2" s="2" t="n">
-        <v>0.8794999999999999</v>
+        <v>0.8818</v>
       </c>
       <c r="D2" s="2" t="n">
-        <v>0.9907</v>
+        <v>0.9903</v>
       </c>
     </row>
     <row r="3">
@@ -2303,13 +2345,13 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>931</v>
+        <v>953</v>
       </c>
       <c r="C3" s="2" t="n">
-        <v>0.8464</v>
+        <v>0.8499</v>
       </c>
       <c r="D3" s="2" t="n">
-        <v>0.9974</v>
+        <v>0.997</v>
       </c>
     </row>
     <row r="4">
@@ -2319,13 +2361,13 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>895</v>
+        <v>918</v>
       </c>
       <c r="C4" s="2" t="n">
-        <v>0.8715000000000001</v>
+        <v>0.8736</v>
       </c>
       <c r="D4" s="2" t="n">
-        <v>0.9933999999999999</v>
+        <v>0.993</v>
       </c>
     </row>
     <row r="5">
@@ -2335,13 +2377,13 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>1017</v>
+        <v>1038</v>
       </c>
       <c r="C5" s="2" t="n">
-        <v>0.8751</v>
+        <v>0.8776</v>
       </c>
       <c r="D5" s="2" t="n">
-        <v>0.9939</v>
+        <v>0.9937</v>
       </c>
     </row>
     <row r="6">
@@ -2351,13 +2393,13 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>1050</v>
+        <v>1076</v>
       </c>
       <c r="C6" s="2" t="n">
-        <v>0.881</v>
+        <v>0.8838</v>
       </c>
       <c r="D6" s="2" t="n">
-        <v>0.9943</v>
+        <v>0.994</v>
       </c>
     </row>
     <row r="7">
@@ -2367,13 +2409,13 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>1041</v>
+        <v>1065</v>
       </c>
       <c r="C7" s="2" t="n">
-        <v>0.8742</v>
+        <v>0.877</v>
       </c>
       <c r="D7" s="2" t="n">
-        <v>0.996</v>
+        <v>0.9957</v>
       </c>
     </row>
     <row r="8">
@@ -2383,13 +2425,13 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>875</v>
+        <v>900</v>
       </c>
       <c r="C8" s="2" t="n">
-        <v>0.8823</v>
+        <v>0.8856000000000001</v>
       </c>
       <c r="D8" s="2" t="n">
-        <v>0.9913999999999999</v>
+        <v>0.9905</v>
       </c>
     </row>
     <row r="9">
@@ -2399,13 +2441,13 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>1047</v>
+        <v>1070</v>
       </c>
       <c r="C9" s="2" t="n">
-        <v>0.852</v>
+        <v>0.8532999999999999</v>
       </c>
       <c r="D9" s="2" t="n">
-        <v>0.9965000000000001</v>
+        <v>0.9961</v>
       </c>
     </row>
     <row r="10">
@@ -2415,13 +2457,13 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>1040</v>
+        <v>1063</v>
       </c>
       <c r="C10" s="2" t="n">
-        <v>0.8683</v>
+        <v>0.8711</v>
       </c>
       <c r="D10" s="2" t="n">
-        <v>0.9971</v>
+        <v>0.9967</v>
       </c>
     </row>
     <row r="11">
@@ -2431,13 +2473,13 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>1004</v>
+        <v>1026</v>
       </c>
       <c r="C11" s="2" t="n">
-        <v>0.8825</v>
+        <v>0.885</v>
       </c>
       <c r="D11" s="2" t="n">
-        <v>0.9947</v>
+        <v>0.9944</v>
       </c>
     </row>
     <row r="12">
@@ -2447,13 +2489,13 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>993</v>
+        <v>1016</v>
       </c>
       <c r="C12" s="2" t="n">
-        <v>0.8802</v>
+        <v>0.8829</v>
       </c>
       <c r="D12" s="2" t="n">
-        <v>0.9944</v>
+        <v>0.9942</v>
       </c>
     </row>
     <row r="13">
@@ -2463,13 +2505,13 @@
         </is>
       </c>
       <c r="B13" t="n">
-        <v>1015</v>
+        <v>1042</v>
       </c>
       <c r="C13" s="2" t="n">
-        <v>0.8966</v>
+        <v>0.8983</v>
       </c>
       <c r="D13" s="2" t="n">
-        <v>0.9847</v>
+        <v>0.9841</v>
       </c>
     </row>
     <row r="14">
@@ -2479,13 +2521,13 @@
         </is>
       </c>
       <c r="B14" t="n">
-        <v>1009</v>
+        <v>1030</v>
       </c>
       <c r="C14" s="2" t="n">
-        <v>0.8811</v>
+        <v>0.8835</v>
       </c>
       <c r="D14" s="2" t="n">
-        <v>0.9942</v>
+        <v>0.994</v>
       </c>
     </row>
     <row r="15">
@@ -2495,13 +2537,13 @@
         </is>
       </c>
       <c r="B15" t="n">
-        <v>1017</v>
+        <v>1039</v>
       </c>
       <c r="C15" s="2" t="n">
-        <v>0.8653</v>
+        <v>0.8672</v>
       </c>
       <c r="D15" s="2" t="n">
-        <v>0.9933</v>
+        <v>0.9932</v>
       </c>
     </row>
     <row r="16">
@@ -2511,13 +2553,13 @@
         </is>
       </c>
       <c r="B16" t="n">
-        <v>1046</v>
+        <v>1069</v>
       </c>
       <c r="C16" s="2" t="n">
-        <v>0.8901</v>
+        <v>0.8924</v>
       </c>
       <c r="D16" s="2" t="n">
-        <v>0.9958</v>
+        <v>0.9955000000000001</v>
       </c>
     </row>
     <row r="17">
@@ -2527,13 +2569,13 @@
         </is>
       </c>
       <c r="B17" t="n">
-        <v>1016</v>
+        <v>1037</v>
       </c>
       <c r="C17" s="2" t="n">
-        <v>0.875</v>
+        <v>0.8774999999999999</v>
       </c>
       <c r="D17" s="2" t="n">
-        <v>0.9956</v>
+        <v>0.9952</v>
       </c>
     </row>
     <row r="18">
@@ -2543,13 +2585,13 @@
         </is>
       </c>
       <c r="B18" t="n">
-        <v>1071</v>
+        <v>1096</v>
       </c>
       <c r="C18" s="2" t="n">
-        <v>0.8571</v>
+        <v>0.8604000000000001</v>
       </c>
       <c r="D18" s="2" t="n">
-        <v>0.9968</v>
+        <v>0.9966</v>
       </c>
     </row>
     <row r="19">
@@ -2559,13 +2601,13 @@
         </is>
       </c>
       <c r="B19" t="n">
-        <v>1031</v>
+        <v>1052</v>
       </c>
       <c r="C19" s="2" t="n">
-        <v>0.8661</v>
+        <v>0.8688</v>
       </c>
       <c r="D19" s="2" t="n">
-        <v>0.996</v>
+        <v>0.9957</v>
       </c>
     </row>
     <row r="20">
@@ -2575,13 +2617,13 @@
         </is>
       </c>
       <c r="B20" t="n">
-        <v>928</v>
+        <v>949</v>
       </c>
       <c r="C20" s="2" t="n">
-        <v>0.8481</v>
+        <v>0.8514</v>
       </c>
       <c r="D20" s="2" t="n">
-        <v>0.9975000000000001</v>
+        <v>0.9969</v>
       </c>
     </row>
     <row r="21">
@@ -2591,13 +2633,13 @@
         </is>
       </c>
       <c r="B21" t="n">
-        <v>917</v>
+        <v>942</v>
       </c>
       <c r="C21" s="2" t="n">
-        <v>0.8484</v>
+        <v>0.8524</v>
       </c>
       <c r="D21" s="2" t="n">
-        <v>0.9944</v>
+        <v>0.9943</v>
       </c>
     </row>
     <row r="22">
@@ -2607,13 +2649,13 @@
         </is>
       </c>
       <c r="B22" t="n">
-        <v>1059</v>
+        <v>1083</v>
       </c>
       <c r="C22" s="2" t="n">
-        <v>0.8527</v>
+        <v>0.856</v>
       </c>
       <c r="D22" s="2" t="n">
-        <v>0.996</v>
+        <v>0.9956</v>
       </c>
     </row>
     <row r="23">
@@ -2623,13 +2665,13 @@
         </is>
       </c>
       <c r="B23" t="n">
-        <v>997</v>
+        <v>1019</v>
       </c>
       <c r="C23" s="2" t="n">
-        <v>0.9056999999999999</v>
+        <v>0.9078000000000001</v>
       </c>
       <c r="D23" s="2" t="n">
-        <v>0.9899</v>
+        <v>0.9897</v>
       </c>
     </row>
     <row r="24">
@@ -2639,13 +2681,13 @@
         </is>
       </c>
       <c r="B24" t="n">
-        <v>951</v>
+        <v>978</v>
       </c>
       <c r="C24" s="2" t="n">
-        <v>0.8791</v>
+        <v>0.8804</v>
       </c>
       <c r="D24" s="2" t="n">
-        <v>0.99</v>
+        <v>0.9892</v>
       </c>
     </row>
     <row r="25">
@@ -2655,13 +2697,13 @@
         </is>
       </c>
       <c r="B25" t="n">
-        <v>1009</v>
+        <v>1038</v>
       </c>
       <c r="C25" s="2" t="n">
-        <v>0.9326</v>
+        <v>0.9335</v>
       </c>
       <c r="D25" s="2" t="n">
-        <v>0.9932</v>
+        <v>0.9931</v>
       </c>
     </row>
     <row r="26">
@@ -2671,13 +2713,13 @@
         </is>
       </c>
       <c r="B26" t="n">
-        <v>860</v>
+        <v>878</v>
       </c>
       <c r="C26" s="2" t="n">
-        <v>0.8907</v>
+        <v>0.8929</v>
       </c>
       <c r="D26" s="2" t="n">
-        <v>0.9921</v>
+        <v>0.9916</v>
       </c>
     </row>
     <row r="27">
@@ -2687,13 +2729,13 @@
         </is>
       </c>
       <c r="B27" t="n">
-        <v>986</v>
+        <v>1009</v>
       </c>
       <c r="C27" s="2" t="n">
-        <v>0.9147999999999999</v>
+        <v>0.9157999999999999</v>
       </c>
       <c r="D27" s="2" t="n">
-        <v>0.9859</v>
+        <v>0.9857</v>
       </c>
     </row>
     <row r="28">
@@ -2703,13 +2745,13 @@
         </is>
       </c>
       <c r="B28" t="n">
-        <v>987</v>
+        <v>1009</v>
       </c>
       <c r="C28" s="2" t="n">
-        <v>0.9078000000000001</v>
+        <v>0.9098000000000001</v>
       </c>
       <c r="D28" s="2" t="n">
-        <v>0.9866</v>
+        <v>0.9864000000000001</v>
       </c>
     </row>
     <row r="29">
@@ -2719,13 +2761,13 @@
         </is>
       </c>
       <c r="B29" t="n">
-        <v>859</v>
+        <v>881</v>
       </c>
       <c r="C29" s="2" t="n">
-        <v>0.8964</v>
+        <v>0.899</v>
       </c>
       <c r="D29" s="2" t="n">
-        <v>0.9935</v>
+        <v>0.9931</v>
       </c>
     </row>
     <row r="30">
@@ -2735,13 +2777,13 @@
         </is>
       </c>
       <c r="B30" t="n">
-        <v>982</v>
+        <v>1008</v>
       </c>
       <c r="C30" s="2" t="n">
-        <v>0.8829</v>
+        <v>0.8849</v>
       </c>
       <c r="D30" s="2" t="n">
-        <v>0.9917</v>
+        <v>0.9913999999999999</v>
       </c>
     </row>
     <row r="31">
@@ -2751,13 +2793,13 @@
         </is>
       </c>
       <c r="B31" t="n">
-        <v>1024</v>
+        <v>1045</v>
       </c>
       <c r="C31" s="2" t="n">
-        <v>0.877</v>
+        <v>0.8794</v>
       </c>
       <c r="D31" s="2" t="n">
-        <v>0.9928</v>
+        <v>0.9927</v>
       </c>
     </row>
     <row r="32">
@@ -2767,13 +2809,13 @@
         </is>
       </c>
       <c r="B32" t="n">
-        <v>1006</v>
+        <v>1030</v>
       </c>
       <c r="C32" s="2" t="n">
-        <v>0.8817</v>
+        <v>0.8845</v>
       </c>
       <c r="D32" s="2" t="n">
-        <v>0.9898</v>
+        <v>0.9895</v>
       </c>
     </row>
     <row r="33">
@@ -2783,13 +2825,13 @@
         </is>
       </c>
       <c r="B33" t="n">
-        <v>814</v>
+        <v>836</v>
       </c>
       <c r="C33" s="2" t="n">
-        <v>0.8968</v>
+        <v>0.8995</v>
       </c>
       <c r="D33" s="2" t="n">
-        <v>0.9889</v>
+        <v>0.9885</v>
       </c>
     </row>
     <row r="34">
@@ -2799,13 +2841,13 @@
         </is>
       </c>
       <c r="B34" t="n">
-        <v>964</v>
+        <v>986</v>
       </c>
       <c r="C34" s="2" t="n">
-        <v>0.9222</v>
+        <v>0.9239000000000001</v>
       </c>
       <c r="D34" s="2" t="n">
-        <v>0.9909</v>
+        <v>0.9908</v>
       </c>
     </row>
     <row r="35">
@@ -2815,13 +2857,13 @@
         </is>
       </c>
       <c r="B35" t="n">
-        <v>1038</v>
+        <v>1059</v>
       </c>
       <c r="C35" s="2" t="n">
-        <v>0.8671</v>
+        <v>0.8697</v>
       </c>
       <c r="D35" s="2" t="n">
-        <v>0.995</v>
+        <v>0.9944</v>
       </c>
     </row>
     <row r="36">
@@ -2831,13 +2873,13 @@
         </is>
       </c>
       <c r="B36" t="n">
-        <v>820</v>
+        <v>844</v>
       </c>
       <c r="C36" s="2" t="n">
-        <v>0.8976</v>
+        <v>0.8993</v>
       </c>
       <c r="D36" s="2" t="n">
-        <v>0.9909</v>
+        <v>0.9903999999999999</v>
       </c>
     </row>
     <row r="37">
@@ -2847,13 +2889,13 @@
         </is>
       </c>
       <c r="B37" t="n">
-        <v>894</v>
+        <v>918</v>
       </c>
       <c r="C37" s="2" t="n">
-        <v>0.9116</v>
+        <v>0.9118000000000001</v>
       </c>
       <c r="D37" s="2" t="n">
-        <v>0.9926</v>
+        <v>0.9925</v>
       </c>
     </row>
     <row r="38">
@@ -2863,13 +2905,13 @@
         </is>
       </c>
       <c r="B38" t="n">
-        <v>868</v>
+        <v>892</v>
       </c>
       <c r="C38" s="2" t="n">
-        <v>0.8871</v>
+        <v>0.8901</v>
       </c>
       <c r="D38" s="2" t="n">
-        <v>0.9913</v>
+        <v>0.9911</v>
       </c>
     </row>
     <row r="39">
@@ -2879,13 +2921,13 @@
         </is>
       </c>
       <c r="B39" t="n">
-        <v>1047</v>
+        <v>1073</v>
       </c>
       <c r="C39" s="2" t="n">
-        <v>0.8911</v>
+        <v>0.8928</v>
       </c>
       <c r="D39" s="2" t="n">
-        <v>0.9896</v>
+        <v>0.989</v>
       </c>
     </row>
     <row r="40">
@@ -2895,13 +2937,13 @@
         </is>
       </c>
       <c r="B40" t="n">
-        <v>854</v>
+        <v>879</v>
       </c>
       <c r="C40" s="2" t="n">
-        <v>0.8712</v>
+        <v>0.8737</v>
       </c>
       <c r="D40" s="2" t="n">
-        <v>0.9926</v>
+        <v>0.9922</v>
       </c>
     </row>
   </sheetData>
@@ -2965,19 +3007,19 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>0.135</v>
+        <v>0.1331</v>
       </c>
       <c r="C2" t="n">
-        <v>0.135</v>
+        <v>0.1331</v>
       </c>
       <c r="D2" t="n">
-        <v>0.0049</v>
+        <v>0.0047</v>
       </c>
       <c r="E2" t="n">
-        <v>1.0403</v>
+        <v>1.0394</v>
       </c>
       <c r="F2" t="n">
-        <v>0.0742</v>
+        <v>0.07439999999999999</v>
       </c>
     </row>
     <row r="3">
@@ -2987,19 +3029,19 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>0.13</v>
+        <v>0.1287</v>
       </c>
       <c r="C3" t="n">
-        <v>0.13</v>
+        <v>0.1287</v>
       </c>
       <c r="D3" t="n">
-        <v>-0.008500000000000001</v>
+        <v>-0.008999999999999999</v>
       </c>
       <c r="E3" t="n">
-        <v>1.0613</v>
+        <v>1.054</v>
       </c>
       <c r="F3" t="n">
-        <v>0.0815</v>
+        <v>0.08160000000000001</v>
       </c>
     </row>
     <row r="4">
@@ -3009,19 +3051,19 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>0.0509</v>
+        <v>0.0505</v>
       </c>
       <c r="C4" t="n">
         <v>0.0447</v>
       </c>
       <c r="D4" t="n">
-        <v>0.0858</v>
+        <v>0.0871</v>
       </c>
       <c r="E4" t="n">
-        <v>1.0179</v>
+        <v>1.0143</v>
       </c>
       <c r="F4" t="n">
-        <v>0.0629</v>
+        <v>0.06320000000000001</v>
       </c>
     </row>
   </sheetData>
@@ -3050,7 +3092,7 @@
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>2026-07-28T09:48:16+00:00</t>
+          <t>2026-07-31T09:10:36+00:00</t>
         </is>
       </c>
     </row>
@@ -3061,7 +3103,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>3881</v>
+        <v>3998</v>
       </c>
     </row>
     <row r="3">
@@ -3071,7 +3113,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>100</v>
+        <v>103</v>
       </c>
     </row>
     <row r="4">
@@ -3101,7 +3143,7 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>186</v>
+        <v>192</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Arquiva dados, recalibra e atualiza docs (2026-08-01)
</commit_message>
<xml_diff>
--- a/backtest_results/resultados_backtest.xlsx
+++ b/backtest_results/resultados_backtest.xlsx
@@ -516,19 +516,19 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>343</v>
+        <v>353</v>
       </c>
       <c r="C2" s="2" t="n">
-        <v>0.8950437317784257</v>
+        <v>0.8980169971671388</v>
       </c>
       <c r="D2" s="3" t="n">
-        <v>4.560707689951263</v>
+        <v>5.088504951980059</v>
       </c>
       <c r="E2" s="4" t="n">
-        <v>28.02788094283614</v>
+        <v>37.43740614675578</v>
       </c>
       <c r="F2" s="2" t="n">
-        <v>1.640147752218049</v>
+        <v>1.843401560300045</v>
       </c>
       <c r="G2" s="2" t="n">
         <v>0.2170352923628444</v>
@@ -537,7 +537,7 @@
         <v>68</v>
       </c>
       <c r="I2" s="3" t="n">
-        <v>0.8323381924198251</v>
+        <v>0.8298597733711047</v>
       </c>
     </row>
     <row r="3">
@@ -547,28 +547,28 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>1736</v>
+        <v>1758</v>
       </c>
       <c r="C3" s="2" t="n">
-        <v>0.993663594470046</v>
+        <v>0.9931740614334471</v>
       </c>
       <c r="D3" s="3" t="n">
-        <v>1.948048719175096</v>
+        <v>1.916383921866174</v>
       </c>
       <c r="E3" s="4" t="n">
-        <v>2.837148066055549</v>
+        <v>2.789977384684703</v>
       </c>
       <c r="F3" s="2" t="n">
-        <v>0.3549004252321757</v>
+        <v>0.3444314353380216</v>
       </c>
       <c r="G3" s="2" t="n">
         <v>0.08704657533117932</v>
       </c>
       <c r="H3" t="n">
-        <v>34</v>
+        <v>38</v>
       </c>
       <c r="I3" s="3" t="n">
-        <v>0.9857531682027649</v>
+        <v>0.9857326507394768</v>
       </c>
     </row>
     <row r="4">
@@ -578,28 +578,28 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>1259</v>
+        <v>1276</v>
       </c>
       <c r="C4" s="2" t="n">
-        <v>0.9944400317712471</v>
+        <v>0.9945141065830722</v>
       </c>
       <c r="D4" s="3" t="n">
-        <v>1.367908183446105</v>
+        <v>1.344881026706539</v>
       </c>
       <c r="E4" s="4" t="n">
-        <v>2.365867722085081</v>
+        <v>2.329887982588146</v>
       </c>
       <c r="F4" s="2" t="n">
-        <v>0.2850773230877728</v>
+        <v>0.2763272191022512</v>
       </c>
       <c r="G4" s="2" t="n">
         <v>0.08016721391959114</v>
       </c>
       <c r="H4" t="n">
-        <v>20</v>
+        <v>23</v>
       </c>
       <c r="I4" s="3" t="n">
-        <v>0.9866898332009532</v>
+        <v>0.9866508620689655</v>
       </c>
     </row>
     <row r="5">
@@ -609,28 +609,28 @@
         </is>
       </c>
       <c r="B5" s="5" t="n">
-        <v>664</v>
+        <v>673</v>
       </c>
       <c r="C5" s="6" t="n">
-        <v>0.9984939759036144</v>
+        <v>0.9985141158989599</v>
       </c>
       <c r="D5" s="7" t="n">
-        <v>0.765749080790208</v>
+        <v>0.7636952403539042</v>
       </c>
       <c r="E5" s="8" t="n">
-        <v>1.81177862053934</v>
+        <v>1.806991839536587</v>
       </c>
       <c r="F5" s="6" t="n">
-        <v>0.1889846603581167</v>
+        <v>0.186101836239573</v>
       </c>
       <c r="G5" s="6" t="n">
         <v>0.02619857308701179</v>
       </c>
       <c r="H5" s="5" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="I5" s="7" t="n">
-        <v>0.9874239457831325</v>
+        <v>0.9873952451708767</v>
       </c>
     </row>
     <row r="6">
@@ -640,34 +640,34 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>1007</v>
+        <v>1026</v>
       </c>
       <c r="C6" s="2" t="n">
-        <v>0.9632571996027806</v>
+        <v>0.9639376218323586</v>
       </c>
       <c r="D6" s="3" t="n">
-        <v>5.326456770741472</v>
+        <v>5.852200192333963</v>
       </c>
       <c r="E6" s="4" t="n">
-        <v>34.11269547699197</v>
+        <v>43.37465145701749</v>
       </c>
       <c r="F6" s="2" t="n">
-        <v>1.795634550883839</v>
+        <v>1.966740871931507</v>
       </c>
       <c r="G6" s="2" t="n">
         <v>0.1983925675638193</v>
       </c>
       <c r="H6" t="n">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="I6" s="3" t="n">
-        <v>0.9345993048659385</v>
+        <v>0.9331944444444444</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Atualizado em 2026-07-31T09:10:36+00:00 · arquivo de 3998 dias-cidade (~103 dias corridos) · 39 cidades</t>
+          <t>Atualizado em 2026-08-01T09:14:36+00:00 · arquivo de 4037 dias-cidade (~104 dias corridos) · 39 cidades</t>
         </is>
       </c>
     </row>
@@ -969,13 +969,13 @@
         </is>
       </c>
       <c r="C13" t="n">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="D13" s="2" t="n">
-        <v>0.7142857142857143</v>
+        <v>0.7777777777777778</v>
       </c>
       <c r="E13" s="3" t="n">
-        <v>0.1799384187411469</v>
+        <v>0.2432536475736171</v>
       </c>
     </row>
     <row r="14">
@@ -1158,13 +1158,13 @@
         </is>
       </c>
       <c r="C22" t="n">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="D22" s="2" t="n">
-        <v>0.8666666666666667</v>
+        <v>0.875</v>
       </c>
       <c r="E22" s="3" t="n">
-        <v>0.395586087922119</v>
+        <v>0.4027098158278501</v>
       </c>
     </row>
     <row r="23">
@@ -1185,7 +1185,7 @@
         <v>0.9130434782608695</v>
       </c>
       <c r="E23" s="3" t="n">
-        <v>0.2694376024035244</v>
+        <v>0.2662726698561493</v>
       </c>
     </row>
     <row r="24">
@@ -1242,13 +1242,13 @@
         </is>
       </c>
       <c r="C26" t="n">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="D26" s="2" t="n">
         <v>1</v>
       </c>
       <c r="E26" s="3" t="n">
-        <v>0.2056511408541294</v>
+        <v>0.2874693226723112</v>
       </c>
     </row>
     <row r="27">
@@ -1263,13 +1263,13 @@
         </is>
       </c>
       <c r="C27" t="n">
-        <v>20</v>
+        <v>25</v>
       </c>
       <c r="D27" s="2" t="n">
-        <v>0.95</v>
+        <v>0.96</v>
       </c>
       <c r="E27" s="3" t="n">
-        <v>0.7046621818573011</v>
+        <v>1.065024042610816</v>
       </c>
     </row>
     <row r="28">
@@ -1410,13 +1410,13 @@
         </is>
       </c>
       <c r="C34" t="n">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="D34" s="2" t="n">
-        <v>0.8888888888888888</v>
+        <v>0.8913043478260869</v>
       </c>
       <c r="E34" s="3" t="n">
-        <v>0.4067327818601304</v>
+        <v>0.4250759771264026</v>
       </c>
     </row>
     <row r="35">
@@ -1536,13 +1536,13 @@
         </is>
       </c>
       <c r="C40" t="n">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="D40" s="2" t="n">
         <v>1</v>
       </c>
       <c r="E40" s="3" t="n">
-        <v>0.02202204037444169</v>
+        <v>0.02421928104894347</v>
       </c>
     </row>
     <row r="41">
@@ -1620,13 +1620,13 @@
         </is>
       </c>
       <c r="C44" t="n">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="D44" s="2" t="n">
         <v>1</v>
       </c>
       <c r="E44" s="3" t="n">
-        <v>0.03390174677547726</v>
+        <v>0.03800463129073291</v>
       </c>
     </row>
     <row r="45">
@@ -1725,13 +1725,13 @@
         </is>
       </c>
       <c r="C49" t="n">
-        <v>17</v>
+        <v>19</v>
       </c>
       <c r="D49" s="2" t="n">
-        <v>0.8823529411764706</v>
+        <v>0.8947368421052632</v>
       </c>
       <c r="E49" s="3" t="n">
-        <v>0.1905798694257619</v>
+        <v>0.2538950982582321</v>
       </c>
     </row>
     <row r="50">
@@ -1914,13 +1914,13 @@
         </is>
       </c>
       <c r="C58" t="n">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="D58" s="2" t="n">
         <v>1</v>
       </c>
       <c r="E58" s="3" t="n">
-        <v>0.2832955007955854</v>
+        <v>0.2856247950480825</v>
       </c>
     </row>
     <row r="59">
@@ -1956,13 +1956,13 @@
         </is>
       </c>
       <c r="C60" t="n">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="D60" s="2" t="n">
-        <v>0.9545454545454546</v>
+        <v>0.9555555555555556</v>
       </c>
       <c r="E60" s="3" t="n">
-        <v>0.4179193354051783</v>
+        <v>0.4250430633109095</v>
       </c>
     </row>
     <row r="61">
@@ -1983,7 +1983,7 @@
         <v>0.9230769230769231</v>
       </c>
       <c r="E61" s="3" t="n">
-        <v>0.2717562073057582</v>
+        <v>0.2685912747583831</v>
       </c>
     </row>
     <row r="62">
@@ -2040,13 +2040,13 @@
         </is>
       </c>
       <c r="C64" t="n">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="D64" s="2" t="n">
         <v>1</v>
       </c>
       <c r="E64" s="3" t="n">
-        <v>0.2052968984655665</v>
+        <v>0.2871150802837484</v>
       </c>
     </row>
     <row r="65">
@@ -2061,13 +2061,13 @@
         </is>
       </c>
       <c r="C65" t="n">
-        <v>41</v>
+        <v>48</v>
       </c>
       <c r="D65" s="2" t="n">
-        <v>0.975609756097561</v>
+        <v>0.9791666666666666</v>
       </c>
       <c r="E65" s="3" t="n">
-        <v>0.7351733272975708</v>
+        <v>1.081545289061186</v>
       </c>
     </row>
     <row r="66">
@@ -2103,13 +2103,13 @@
         </is>
       </c>
       <c r="C67" t="n">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="D67" s="2" t="n">
-        <v>0.9444444444444444</v>
+        <v>0.9459459459459459</v>
       </c>
       <c r="E67" s="3" t="n">
-        <v>0.4982893237163585</v>
+        <v>0.5003301400428891</v>
       </c>
     </row>
     <row r="68">
@@ -2208,13 +2208,13 @@
         </is>
       </c>
       <c r="C72" t="n">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="D72" s="2" t="n">
-        <v>0.9468085106382979</v>
+        <v>0.9473684210526315</v>
       </c>
       <c r="E72" s="3" t="n">
-        <v>0.469676072759845</v>
+        <v>0.4880192680261172</v>
       </c>
     </row>
     <row r="73">
@@ -2229,13 +2229,13 @@
         </is>
       </c>
       <c r="C73" t="n">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="D73" s="2" t="n">
         <v>1</v>
       </c>
       <c r="E73" s="3" t="n">
-        <v>0.0912822137746932</v>
+        <v>0.0925480365595033</v>
       </c>
     </row>
     <row r="74">
@@ -2329,13 +2329,13 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>1024</v>
+        <v>1031</v>
       </c>
       <c r="C2" s="2" t="n">
-        <v>0.8818</v>
+        <v>0.8826000000000001</v>
       </c>
       <c r="D2" s="2" t="n">
-        <v>0.9903</v>
+        <v>0.9902</v>
       </c>
     </row>
     <row r="3">
@@ -2345,10 +2345,10 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>953</v>
+        <v>960</v>
       </c>
       <c r="C3" s="2" t="n">
-        <v>0.8499</v>
+        <v>0.851</v>
       </c>
       <c r="D3" s="2" t="n">
         <v>0.997</v>
@@ -2361,13 +2361,13 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>918</v>
+        <v>928</v>
       </c>
       <c r="C4" s="2" t="n">
-        <v>0.8736</v>
+        <v>0.875</v>
       </c>
       <c r="D4" s="2" t="n">
-        <v>0.993</v>
+        <v>0.9928</v>
       </c>
     </row>
     <row r="5">
@@ -2377,13 +2377,13 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>1038</v>
+        <v>1045</v>
       </c>
       <c r="C5" s="2" t="n">
-        <v>0.8776</v>
+        <v>0.8784999999999999</v>
       </c>
       <c r="D5" s="2" t="n">
-        <v>0.9937</v>
+        <v>0.9936</v>
       </c>
     </row>
     <row r="6">
@@ -2393,13 +2393,13 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>1076</v>
+        <v>1083</v>
       </c>
       <c r="C6" s="2" t="n">
-        <v>0.8838</v>
+        <v>0.8846000000000001</v>
       </c>
       <c r="D6" s="2" t="n">
-        <v>0.994</v>
+        <v>0.9939</v>
       </c>
     </row>
     <row r="7">
@@ -2409,13 +2409,13 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>1065</v>
+        <v>1073</v>
       </c>
       <c r="C7" s="2" t="n">
-        <v>0.877</v>
+        <v>0.8779</v>
       </c>
       <c r="D7" s="2" t="n">
-        <v>0.9957</v>
+        <v>0.9956</v>
       </c>
     </row>
     <row r="8">
@@ -2425,13 +2425,13 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>900</v>
+        <v>908</v>
       </c>
       <c r="C8" s="2" t="n">
-        <v>0.8856000000000001</v>
+        <v>0.8866000000000001</v>
       </c>
       <c r="D8" s="2" t="n">
-        <v>0.9905</v>
+        <v>0.99</v>
       </c>
     </row>
     <row r="9">
@@ -2441,13 +2441,13 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>1070</v>
+        <v>1078</v>
       </c>
       <c r="C9" s="2" t="n">
-        <v>0.8532999999999999</v>
+        <v>0.8544</v>
       </c>
       <c r="D9" s="2" t="n">
-        <v>0.9961</v>
+        <v>0.996</v>
       </c>
     </row>
     <row r="10">
@@ -2473,13 +2473,13 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>1026</v>
+        <v>1034</v>
       </c>
       <c r="C11" s="2" t="n">
-        <v>0.885</v>
+        <v>0.8859</v>
       </c>
       <c r="D11" s="2" t="n">
-        <v>0.9944</v>
+        <v>0.9943</v>
       </c>
     </row>
     <row r="12">
@@ -2489,10 +2489,10 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>1016</v>
+        <v>1023</v>
       </c>
       <c r="C12" s="2" t="n">
-        <v>0.8829</v>
+        <v>0.8837</v>
       </c>
       <c r="D12" s="2" t="n">
         <v>0.9942</v>
@@ -2505,13 +2505,13 @@
         </is>
       </c>
       <c r="B13" t="n">
-        <v>1042</v>
+        <v>1052</v>
       </c>
       <c r="C13" s="2" t="n">
-        <v>0.8983</v>
+        <v>0.8992</v>
       </c>
       <c r="D13" s="2" t="n">
-        <v>0.9841</v>
+        <v>0.9838</v>
       </c>
     </row>
     <row r="14">
@@ -2521,13 +2521,13 @@
         </is>
       </c>
       <c r="B14" t="n">
-        <v>1030</v>
+        <v>1036</v>
       </c>
       <c r="C14" s="2" t="n">
-        <v>0.8835</v>
+        <v>0.8842</v>
       </c>
       <c r="D14" s="2" t="n">
-        <v>0.994</v>
+        <v>0.9939</v>
       </c>
     </row>
     <row r="15">
@@ -2537,10 +2537,10 @@
         </is>
       </c>
       <c r="B15" t="n">
-        <v>1039</v>
+        <v>1046</v>
       </c>
       <c r="C15" s="2" t="n">
-        <v>0.8672</v>
+        <v>0.8681</v>
       </c>
       <c r="D15" s="2" t="n">
         <v>0.9932</v>
@@ -2553,13 +2553,13 @@
         </is>
       </c>
       <c r="B16" t="n">
-        <v>1069</v>
+        <v>1077</v>
       </c>
       <c r="C16" s="2" t="n">
-        <v>0.8924</v>
+        <v>0.8932</v>
       </c>
       <c r="D16" s="2" t="n">
-        <v>0.9955000000000001</v>
+        <v>0.9954</v>
       </c>
     </row>
     <row r="17">
@@ -2569,10 +2569,10 @@
         </is>
       </c>
       <c r="B17" t="n">
-        <v>1037</v>
+        <v>1043</v>
       </c>
       <c r="C17" s="2" t="n">
-        <v>0.8774999999999999</v>
+        <v>0.8782</v>
       </c>
       <c r="D17" s="2" t="n">
         <v>0.9952</v>
@@ -2585,10 +2585,10 @@
         </is>
       </c>
       <c r="B18" t="n">
-        <v>1096</v>
+        <v>1104</v>
       </c>
       <c r="C18" s="2" t="n">
-        <v>0.8604000000000001</v>
+        <v>0.8614000000000001</v>
       </c>
       <c r="D18" s="2" t="n">
         <v>0.9966</v>
@@ -2601,13 +2601,13 @@
         </is>
       </c>
       <c r="B19" t="n">
-        <v>1052</v>
+        <v>1059</v>
       </c>
       <c r="C19" s="2" t="n">
-        <v>0.8688</v>
+        <v>0.8697</v>
       </c>
       <c r="D19" s="2" t="n">
-        <v>0.9957</v>
+        <v>0.9956</v>
       </c>
     </row>
     <row r="20">
@@ -2617,13 +2617,13 @@
         </is>
       </c>
       <c r="B20" t="n">
-        <v>949</v>
+        <v>955</v>
       </c>
       <c r="C20" s="2" t="n">
-        <v>0.8514</v>
+        <v>0.8524</v>
       </c>
       <c r="D20" s="2" t="n">
-        <v>0.9969</v>
+        <v>0.9968</v>
       </c>
     </row>
     <row r="21">
@@ -2633,10 +2633,10 @@
         </is>
       </c>
       <c r="B21" t="n">
-        <v>942</v>
+        <v>950</v>
       </c>
       <c r="C21" s="2" t="n">
-        <v>0.8524</v>
+        <v>0.8537</v>
       </c>
       <c r="D21" s="2" t="n">
         <v>0.9943</v>
@@ -2649,13 +2649,13 @@
         </is>
       </c>
       <c r="B22" t="n">
-        <v>1083</v>
+        <v>1091</v>
       </c>
       <c r="C22" s="2" t="n">
-        <v>0.856</v>
+        <v>0.857</v>
       </c>
       <c r="D22" s="2" t="n">
-        <v>0.9956</v>
+        <v>0.9954</v>
       </c>
     </row>
     <row r="23">
@@ -2665,13 +2665,13 @@
         </is>
       </c>
       <c r="B23" t="n">
-        <v>1019</v>
+        <v>1028</v>
       </c>
       <c r="C23" s="2" t="n">
-        <v>0.9078000000000001</v>
+        <v>0.9086</v>
       </c>
       <c r="D23" s="2" t="n">
-        <v>0.9897</v>
+        <v>0.9896</v>
       </c>
     </row>
     <row r="24">
@@ -2681,13 +2681,13 @@
         </is>
       </c>
       <c r="B24" t="n">
-        <v>978</v>
+        <v>985</v>
       </c>
       <c r="C24" s="2" t="n">
-        <v>0.8804</v>
+        <v>0.8812</v>
       </c>
       <c r="D24" s="2" t="n">
-        <v>0.9892</v>
+        <v>0.989</v>
       </c>
     </row>
     <row r="25">
@@ -2697,13 +2697,13 @@
         </is>
       </c>
       <c r="B25" t="n">
-        <v>1038</v>
+        <v>1049</v>
       </c>
       <c r="C25" s="2" t="n">
-        <v>0.9335</v>
+        <v>0.9323</v>
       </c>
       <c r="D25" s="2" t="n">
-        <v>0.9931</v>
+        <v>0.993</v>
       </c>
     </row>
     <row r="26">
@@ -2713,13 +2713,13 @@
         </is>
       </c>
       <c r="B26" t="n">
-        <v>878</v>
+        <v>885</v>
       </c>
       <c r="C26" s="2" t="n">
-        <v>0.8929</v>
+        <v>0.8938</v>
       </c>
       <c r="D26" s="2" t="n">
-        <v>0.9916</v>
+        <v>0.9912</v>
       </c>
     </row>
     <row r="27">
@@ -2729,13 +2729,13 @@
         </is>
       </c>
       <c r="B27" t="n">
-        <v>1009</v>
+        <v>1013</v>
       </c>
       <c r="C27" s="2" t="n">
-        <v>0.9157999999999999</v>
+        <v>0.9161</v>
       </c>
       <c r="D27" s="2" t="n">
-        <v>0.9857</v>
+        <v>0.9856</v>
       </c>
     </row>
     <row r="28">
@@ -2745,13 +2745,13 @@
         </is>
       </c>
       <c r="B28" t="n">
-        <v>1009</v>
+        <v>1018</v>
       </c>
       <c r="C28" s="2" t="n">
-        <v>0.9098000000000001</v>
+        <v>0.9106</v>
       </c>
       <c r="D28" s="2" t="n">
-        <v>0.9864000000000001</v>
+        <v>0.9863</v>
       </c>
     </row>
     <row r="29">
@@ -2761,13 +2761,13 @@
         </is>
       </c>
       <c r="B29" t="n">
-        <v>881</v>
+        <v>891</v>
       </c>
       <c r="C29" s="2" t="n">
-        <v>0.899</v>
+        <v>0.9001</v>
       </c>
       <c r="D29" s="2" t="n">
-        <v>0.9931</v>
+        <v>0.993</v>
       </c>
     </row>
     <row r="30">
@@ -2777,10 +2777,10 @@
         </is>
       </c>
       <c r="B30" t="n">
-        <v>1008</v>
+        <v>1019</v>
       </c>
       <c r="C30" s="2" t="n">
-        <v>0.8849</v>
+        <v>0.8852</v>
       </c>
       <c r="D30" s="2" t="n">
         <v>0.9913999999999999</v>
@@ -2793,13 +2793,13 @@
         </is>
       </c>
       <c r="B31" t="n">
-        <v>1045</v>
+        <v>1052</v>
       </c>
       <c r="C31" s="2" t="n">
-        <v>0.8794</v>
+        <v>0.8802</v>
       </c>
       <c r="D31" s="2" t="n">
-        <v>0.9927</v>
+        <v>0.9926</v>
       </c>
     </row>
     <row r="32">
@@ -2809,10 +2809,10 @@
         </is>
       </c>
       <c r="B32" t="n">
-        <v>1030</v>
+        <v>1037</v>
       </c>
       <c r="C32" s="2" t="n">
-        <v>0.8845</v>
+        <v>0.8852</v>
       </c>
       <c r="D32" s="2" t="n">
         <v>0.9895</v>
@@ -2825,13 +2825,13 @@
         </is>
       </c>
       <c r="B33" t="n">
-        <v>836</v>
+        <v>842</v>
       </c>
       <c r="C33" s="2" t="n">
-        <v>0.8995</v>
+        <v>0.9002</v>
       </c>
       <c r="D33" s="2" t="n">
-        <v>0.9885</v>
+        <v>0.9883999999999999</v>
       </c>
     </row>
     <row r="34">
@@ -2841,13 +2841,13 @@
         </is>
       </c>
       <c r="B34" t="n">
-        <v>986</v>
+        <v>994</v>
       </c>
       <c r="C34" s="2" t="n">
-        <v>0.9239000000000001</v>
+        <v>0.9245</v>
       </c>
       <c r="D34" s="2" t="n">
-        <v>0.9908</v>
+        <v>0.9907</v>
       </c>
     </row>
     <row r="35">
@@ -2857,13 +2857,13 @@
         </is>
       </c>
       <c r="B35" t="n">
-        <v>1059</v>
+        <v>1065</v>
       </c>
       <c r="C35" s="2" t="n">
-        <v>0.8697</v>
+        <v>0.8704</v>
       </c>
       <c r="D35" s="2" t="n">
-        <v>0.9944</v>
+        <v>0.9943</v>
       </c>
     </row>
     <row r="36">
@@ -2873,13 +2873,13 @@
         </is>
       </c>
       <c r="B36" t="n">
-        <v>844</v>
+        <v>850</v>
       </c>
       <c r="C36" s="2" t="n">
-        <v>0.8993</v>
+        <v>0.9</v>
       </c>
       <c r="D36" s="2" t="n">
-        <v>0.9903999999999999</v>
+        <v>0.9902</v>
       </c>
     </row>
     <row r="37">
@@ -2889,13 +2889,13 @@
         </is>
       </c>
       <c r="B37" t="n">
-        <v>918</v>
+        <v>925</v>
       </c>
       <c r="C37" s="2" t="n">
-        <v>0.9118000000000001</v>
+        <v>0.9124</v>
       </c>
       <c r="D37" s="2" t="n">
-        <v>0.9925</v>
+        <v>0.9923999999999999</v>
       </c>
     </row>
     <row r="38">
@@ -2905,13 +2905,13 @@
         </is>
       </c>
       <c r="B38" t="n">
-        <v>892</v>
+        <v>900</v>
       </c>
       <c r="C38" s="2" t="n">
-        <v>0.8901</v>
+        <v>0.8911</v>
       </c>
       <c r="D38" s="2" t="n">
-        <v>0.9911</v>
+        <v>0.9909</v>
       </c>
     </row>
     <row r="39">
@@ -2921,13 +2921,13 @@
         </is>
       </c>
       <c r="B39" t="n">
-        <v>1073</v>
+        <v>1080</v>
       </c>
       <c r="C39" s="2" t="n">
-        <v>0.8928</v>
+        <v>0.8935</v>
       </c>
       <c r="D39" s="2" t="n">
-        <v>0.989</v>
+        <v>0.9889</v>
       </c>
     </row>
     <row r="40">
@@ -2937,13 +2937,13 @@
         </is>
       </c>
       <c r="B40" t="n">
-        <v>879</v>
+        <v>886</v>
       </c>
       <c r="C40" s="2" t="n">
-        <v>0.8737</v>
+        <v>0.8747</v>
       </c>
       <c r="D40" s="2" t="n">
-        <v>0.9922</v>
+        <v>0.9919</v>
       </c>
     </row>
   </sheetData>
@@ -3007,16 +3007,16 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>0.1331</v>
+        <v>0.1326</v>
       </c>
       <c r="C2" t="n">
-        <v>0.1331</v>
+        <v>0.1326</v>
       </c>
       <c r="D2" t="n">
-        <v>0.0047</v>
+        <v>0.0045</v>
       </c>
       <c r="E2" t="n">
-        <v>1.0394</v>
+        <v>1.0366</v>
       </c>
       <c r="F2" t="n">
         <v>0.07439999999999999</v>
@@ -3029,16 +3029,16 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>0.1287</v>
+        <v>0.1283</v>
       </c>
       <c r="C3" t="n">
-        <v>0.1287</v>
+        <v>0.1283</v>
       </c>
       <c r="D3" t="n">
-        <v>-0.008999999999999999</v>
+        <v>-0.009299999999999999</v>
       </c>
       <c r="E3" t="n">
-        <v>1.054</v>
+        <v>1.0512</v>
       </c>
       <c r="F3" t="n">
         <v>0.08160000000000001</v>
@@ -3051,19 +3051,19 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>0.0505</v>
+        <v>0.0504</v>
       </c>
       <c r="C4" t="n">
         <v>0.0447</v>
       </c>
       <c r="D4" t="n">
-        <v>0.0871</v>
+        <v>0.08890000000000001</v>
       </c>
       <c r="E4" t="n">
-        <v>1.0143</v>
+        <v>1.0069</v>
       </c>
       <c r="F4" t="n">
-        <v>0.06320000000000001</v>
+        <v>0.0633</v>
       </c>
     </row>
   </sheetData>
@@ -3092,7 +3092,7 @@
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>2026-07-31T09:10:36+00:00</t>
+          <t>2026-08-01T09:14:36+00:00</t>
         </is>
       </c>
     </row>
@@ -3103,7 +3103,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>3998</v>
+        <v>4037</v>
       </c>
     </row>
     <row r="3">
@@ -3113,7 +3113,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>103</v>
+        <v>104</v>
       </c>
     </row>
     <row r="4">

</xml_diff>

<commit_message>
Arquiva dados, recalibra e atualiza docs (2026-08-04)
</commit_message>
<xml_diff>
--- a/backtest_results/resultados_backtest.xlsx
+++ b/backtest_results/resultados_backtest.xlsx
@@ -516,28 +516,28 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>353</v>
+        <v>376</v>
       </c>
       <c r="C2" s="2" t="n">
-        <v>0.8980169971671388</v>
+        <v>0.898936170212766</v>
       </c>
       <c r="D2" s="3" t="n">
-        <v>5.088504951980059</v>
+        <v>5.563470606153434</v>
       </c>
       <c r="E2" s="4" t="n">
-        <v>37.43740614675578</v>
+        <v>47.9117099757488</v>
       </c>
       <c r="F2" s="2" t="n">
-        <v>1.843401560300045</v>
+        <v>1.959047048321784</v>
       </c>
       <c r="G2" s="2" t="n">
         <v>0.2170352923628444</v>
       </c>
       <c r="H2" t="n">
-        <v>68</v>
+        <v>73</v>
       </c>
       <c r="I2" s="3" t="n">
-        <v>0.8298597733711047</v>
+        <v>0.8259135638297872</v>
       </c>
     </row>
     <row r="3">
@@ -547,19 +547,19 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>1758</v>
+        <v>1808</v>
       </c>
       <c r="C3" s="2" t="n">
-        <v>0.9931740614334471</v>
+        <v>0.9933628318584071</v>
       </c>
       <c r="D3" s="3" t="n">
-        <v>1.916383921866174</v>
+        <v>1.98840872976479</v>
       </c>
       <c r="E3" s="4" t="n">
-        <v>2.789977384684703</v>
+        <v>2.896483442803385</v>
       </c>
       <c r="F3" s="2" t="n">
-        <v>0.3444314353380216</v>
+        <v>0.3474000407567095</v>
       </c>
       <c r="G3" s="2" t="n">
         <v>0.08704657533117932</v>
@@ -568,7 +568,7 @@
         <v>38</v>
       </c>
       <c r="I3" s="3" t="n">
-        <v>0.9857326507394768</v>
+        <v>0.9857358960176992</v>
       </c>
     </row>
     <row r="4">
@@ -578,19 +578,19 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>1276</v>
+        <v>1311</v>
       </c>
       <c r="C4" s="2" t="n">
-        <v>0.9945141065830722</v>
+        <v>0.9946605644546148</v>
       </c>
       <c r="D4" s="3" t="n">
-        <v>1.344881026706539</v>
+        <v>1.393234076639585</v>
       </c>
       <c r="E4" s="4" t="n">
-        <v>2.329887982588146</v>
+        <v>2.40759455771909</v>
       </c>
       <c r="F4" s="2" t="n">
-        <v>0.2763272191022512</v>
+        <v>0.2793400235795169</v>
       </c>
       <c r="G4" s="2" t="n">
         <v>0.08016721391959114</v>
@@ -599,7 +599,7 @@
         <v>23</v>
       </c>
       <c r="I4" s="3" t="n">
-        <v>0.9866508620689655</v>
+        <v>0.9866449275362319</v>
       </c>
     </row>
     <row r="5">
@@ -609,19 +609,19 @@
         </is>
       </c>
       <c r="B5" s="5" t="n">
-        <v>673</v>
+        <v>694</v>
       </c>
       <c r="C5" s="6" t="n">
-        <v>0.9985141158989599</v>
+        <v>0.9985590778097982</v>
       </c>
       <c r="D5" s="7" t="n">
-        <v>0.7636952403539042</v>
+        <v>0.7954774270623911</v>
       </c>
       <c r="E5" s="8" t="n">
-        <v>1.806991839536587</v>
+        <v>1.85134776044089</v>
       </c>
       <c r="F5" s="6" t="n">
-        <v>0.186101836239573</v>
+        <v>0.1884930240102944</v>
       </c>
       <c r="G5" s="6" t="n">
         <v>0.02619857308701179</v>
@@ -630,7 +630,7 @@
         <v>6</v>
       </c>
       <c r="I5" s="7" t="n">
-        <v>0.9873952451708767</v>
+        <v>0.987327809798271</v>
       </c>
     </row>
     <row r="6">
@@ -640,34 +640,34 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>1026</v>
+        <v>1070</v>
       </c>
       <c r="C6" s="2" t="n">
-        <v>0.9639376218323586</v>
+        <v>0.9635514018691589</v>
       </c>
       <c r="D6" s="3" t="n">
-        <v>5.852200192333963</v>
+        <v>6.358948033215825</v>
       </c>
       <c r="E6" s="4" t="n">
-        <v>43.37465145701749</v>
+        <v>55.09814680743132</v>
       </c>
       <c r="F6" s="2" t="n">
-        <v>1.966740871931507</v>
+        <v>2.077295842225132</v>
       </c>
       <c r="G6" s="2" t="n">
         <v>0.1983925675638193</v>
       </c>
       <c r="H6" t="n">
-        <v>74</v>
+        <v>79</v>
       </c>
       <c r="I6" s="3" t="n">
-        <v>0.9331944444444444</v>
+        <v>0.9306065420560747</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Atualizado em 2026-08-01T09:14:36+00:00 · arquivo de 4037 dias-cidade (~104 dias corridos) · 39 cidades</t>
+          <t>Atualizado em 2026-08-04T09:15:09+00:00 · arquivo de 4154 dias-cidade (~107 dias corridos) · 39 cidades</t>
         </is>
       </c>
     </row>
@@ -738,13 +738,13 @@
         </is>
       </c>
       <c r="C2" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D2" s="2" t="n">
-        <v>0.6666666666666666</v>
+        <v>0</v>
       </c>
       <c r="E2" s="3" t="n">
-        <v>0.00623474540887469</v>
+        <v>-0.015</v>
       </c>
     </row>
     <row r="3">
@@ -885,13 +885,13 @@
         </is>
       </c>
       <c r="C9" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D9" s="2" t="n">
-        <v>0.5</v>
+        <v>0.6666666666666666</v>
       </c>
       <c r="E9" s="3" t="n">
-        <v>-0.008617021276595745</v>
+        <v>0.09546461137646549</v>
       </c>
     </row>
     <row r="10">
@@ -969,13 +969,13 @@
         </is>
       </c>
       <c r="C13" t="n">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="D13" s="2" t="n">
-        <v>0.7777777777777778</v>
+        <v>0.8181818181818182</v>
       </c>
       <c r="E13" s="3" t="n">
-        <v>0.2432536475736171</v>
+        <v>0.30053294504329</v>
       </c>
     </row>
     <row r="14">
@@ -990,13 +990,13 @@
         </is>
       </c>
       <c r="C14" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="D14" s="2" t="n">
-        <v>0.75</v>
+        <v>0.8</v>
       </c>
       <c r="E14" s="3" t="n">
-        <v>0.0767850392492342</v>
+        <v>0.100241829372691</v>
       </c>
     </row>
     <row r="15">
@@ -1032,13 +1032,13 @@
         </is>
       </c>
       <c r="C16" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="D16" s="2" t="n">
         <v>1</v>
       </c>
       <c r="E16" s="3" t="n">
-        <v>0.02063570816437714</v>
+        <v>0.00563570816437714</v>
       </c>
     </row>
     <row r="17">
@@ -1116,13 +1116,13 @@
         </is>
       </c>
       <c r="C20" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="D20" s="2" t="n">
-        <v>1</v>
+        <v>0.875</v>
       </c>
       <c r="E20" s="3" t="n">
-        <v>0.2123882871456879</v>
+        <v>0.197388287145688</v>
       </c>
     </row>
     <row r="21">
@@ -1158,13 +1158,13 @@
         </is>
       </c>
       <c r="C22" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="D22" s="2" t="n">
-        <v>0.875</v>
+        <v>0.8235294117647058</v>
       </c>
       <c r="E22" s="3" t="n">
-        <v>0.4027098158278501</v>
+        <v>0.3877098158278501</v>
       </c>
     </row>
     <row r="23">
@@ -1179,13 +1179,13 @@
         </is>
       </c>
       <c r="C23" t="n">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="D23" s="2" t="n">
-        <v>0.9130434782608695</v>
+        <v>0.9166666666666666</v>
       </c>
       <c r="E23" s="3" t="n">
-        <v>0.2662726698561493</v>
+        <v>0.2726556485795536</v>
       </c>
     </row>
     <row r="24">
@@ -1242,13 +1242,13 @@
         </is>
       </c>
       <c r="C26" t="n">
-        <v>18</v>
+        <v>23</v>
       </c>
       <c r="D26" s="2" t="n">
         <v>1</v>
       </c>
       <c r="E26" s="3" t="n">
-        <v>0.2874693226723112</v>
+        <v>0.4416585625916054</v>
       </c>
     </row>
     <row r="27">
@@ -1263,13 +1263,13 @@
         </is>
       </c>
       <c r="C27" t="n">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="D27" s="2" t="n">
-        <v>0.96</v>
+        <v>0.9615384615384616</v>
       </c>
       <c r="E27" s="3" t="n">
-        <v>1.065024042610816</v>
+        <v>1.128958468840324</v>
       </c>
     </row>
     <row r="28">
@@ -1284,13 +1284,13 @@
         </is>
       </c>
       <c r="C28" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="D28" s="2" t="n">
-        <v>0.8333333333333334</v>
+        <v>0.8571428571428571</v>
       </c>
       <c r="E28" s="3" t="n">
-        <v>0.1298913520808539</v>
+        <v>0.1687802409697428</v>
       </c>
     </row>
     <row r="29">
@@ -1389,13 +1389,13 @@
         </is>
       </c>
       <c r="C33" t="n">
-        <v>22</v>
+        <v>25</v>
       </c>
       <c r="D33" s="2" t="n">
-        <v>0.8181818181818182</v>
+        <v>0.84</v>
       </c>
       <c r="E33" s="3" t="n">
-        <v>0.1201624281584527</v>
+        <v>0.1619206114997599</v>
       </c>
     </row>
     <row r="34">
@@ -1410,13 +1410,13 @@
         </is>
       </c>
       <c r="C34" t="n">
-        <v>46</v>
+        <v>50</v>
       </c>
       <c r="D34" s="2" t="n">
-        <v>0.8913043478260869</v>
+        <v>0.9</v>
       </c>
       <c r="E34" s="3" t="n">
-        <v>0.4250759771264026</v>
+        <v>0.4507150748707635</v>
       </c>
     </row>
     <row r="35">
@@ -1431,13 +1431,13 @@
         </is>
       </c>
       <c r="C35" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="D35" s="2" t="n">
         <v>1</v>
       </c>
       <c r="E35" s="3" t="n">
-        <v>0.05065203240622935</v>
+        <v>0.05760390406398334</v>
       </c>
     </row>
     <row r="36">
@@ -1473,13 +1473,13 @@
         </is>
       </c>
       <c r="C37" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="D37" s="2" t="n">
-        <v>0.6666666666666666</v>
+        <v>0.8</v>
       </c>
       <c r="E37" s="3" t="n">
-        <v>-0.02417989417989416</v>
+        <v>-0.005541901348352921</v>
       </c>
     </row>
     <row r="38">
@@ -1494,13 +1494,13 @@
         </is>
       </c>
       <c r="C38" t="n">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="D38" s="2" t="n">
-        <v>0.9411764705882353</v>
+        <v>0.9333333333333333</v>
       </c>
       <c r="E38" s="3" t="n">
-        <v>0.02895708859174546</v>
+        <v>0.007722343182870766</v>
       </c>
     </row>
     <row r="39">
@@ -1536,13 +1536,13 @@
         </is>
       </c>
       <c r="C40" t="n">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="D40" s="2" t="n">
         <v>1</v>
       </c>
       <c r="E40" s="3" t="n">
-        <v>0.02421928104894347</v>
+        <v>0.02712646812134217</v>
       </c>
     </row>
     <row r="41">
@@ -1620,13 +1620,13 @@
         </is>
       </c>
       <c r="C44" t="n">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="D44" s="2" t="n">
         <v>1</v>
       </c>
       <c r="E44" s="3" t="n">
-        <v>0.03800463129073291</v>
+        <v>0.04067403580818672</v>
       </c>
     </row>
     <row r="45">
@@ -1641,13 +1641,13 @@
         </is>
       </c>
       <c r="C45" t="n">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="D45" s="2" t="n">
-        <v>0.9375</v>
+        <v>0.9444444444444444</v>
       </c>
       <c r="E45" s="3" t="n">
-        <v>0.003500706411286052</v>
+        <v>0.1093635095478079</v>
       </c>
     </row>
     <row r="46">
@@ -1704,13 +1704,13 @@
         </is>
       </c>
       <c r="C48" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="D48" s="2" t="n">
-        <v>0.6</v>
+        <v>0.6363636363636364</v>
       </c>
       <c r="E48" s="3" t="n">
-        <v>-0.05112262463304137</v>
+        <v>-0.0485585220689388</v>
       </c>
     </row>
     <row r="49">
@@ -1725,13 +1725,13 @@
         </is>
       </c>
       <c r="C49" t="n">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="D49" s="2" t="n">
-        <v>0.8947368421052632</v>
+        <v>0.9047619047619048</v>
       </c>
       <c r="E49" s="3" t="n">
-        <v>0.2538950982582321</v>
+        <v>0.3111743957279052</v>
       </c>
     </row>
     <row r="50">
@@ -1746,13 +1746,13 @@
         </is>
       </c>
       <c r="C50" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="D50" s="2" t="n">
-        <v>0.9375</v>
+        <v>0.9411764705882353</v>
       </c>
       <c r="E50" s="3" t="n">
-        <v>0.09285061569441484</v>
+        <v>0.1163074058178716</v>
       </c>
     </row>
     <row r="51">
@@ -1788,13 +1788,13 @@
         </is>
       </c>
       <c r="C52" t="n">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="D52" s="2" t="n">
         <v>1</v>
       </c>
       <c r="E52" s="3" t="n">
-        <v>0.04168440738044763</v>
+        <v>0.02872522370697825</v>
       </c>
     </row>
     <row r="53">
@@ -1809,13 +1809,13 @@
         </is>
       </c>
       <c r="C53" t="n">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="D53" s="2" t="n">
-        <v>0.9545454545454546</v>
+        <v>0.9565217391304348</v>
       </c>
       <c r="E53" s="3" t="n">
-        <v>-0.02457179188325269</v>
+        <v>-0.02356169087315167</v>
       </c>
     </row>
     <row r="54">
@@ -1899,7 +1899,7 @@
         <v>1</v>
       </c>
       <c r="E57" s="3" t="n">
-        <v>0.01770727377980937</v>
+        <v>0.01971833461439963</v>
       </c>
     </row>
     <row r="58">
@@ -1914,13 +1914,13 @@
         </is>
       </c>
       <c r="C58" t="n">
-        <v>64</v>
+        <v>70</v>
       </c>
       <c r="D58" s="2" t="n">
-        <v>1</v>
+        <v>0.9857142857142858</v>
       </c>
       <c r="E58" s="3" t="n">
-        <v>0.2856247950480825</v>
+        <v>0.2753348375732511</v>
       </c>
     </row>
     <row r="59">
@@ -1956,13 +1956,13 @@
         </is>
       </c>
       <c r="C60" t="n">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="D60" s="2" t="n">
-        <v>0.9555555555555556</v>
+        <v>0.9347826086956522</v>
       </c>
       <c r="E60" s="3" t="n">
-        <v>0.4250430633109095</v>
+        <v>0.4101974315460432</v>
       </c>
     </row>
     <row r="61">
@@ -1977,13 +1977,13 @@
         </is>
       </c>
       <c r="C61" t="n">
-        <v>26</v>
+        <v>29</v>
       </c>
       <c r="D61" s="2" t="n">
-        <v>0.9230769230769231</v>
+        <v>0.9310344827586207</v>
       </c>
       <c r="E61" s="3" t="n">
-        <v>0.2685912747583831</v>
+        <v>0.2782472797296235</v>
       </c>
     </row>
     <row r="62">
@@ -1998,13 +1998,13 @@
         </is>
       </c>
       <c r="C62" t="n">
-        <v>43</v>
+        <v>45</v>
       </c>
       <c r="D62" s="2" t="n">
         <v>1</v>
       </c>
       <c r="E62" s="3" t="n">
-        <v>0.3332871271739986</v>
+        <v>0.334545001546555</v>
       </c>
     </row>
     <row r="63">
@@ -2019,13 +2019,13 @@
         </is>
       </c>
       <c r="C63" t="n">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="D63" s="2" t="n">
-        <v>0.9523809523809523</v>
+        <v>0.9545454545454546</v>
       </c>
       <c r="E63" s="3" t="n">
-        <v>0.27245898940336</v>
+        <v>0.2745518939464943</v>
       </c>
     </row>
     <row r="64">
@@ -2040,13 +2040,13 @@
         </is>
       </c>
       <c r="C64" t="n">
-        <v>44</v>
+        <v>50</v>
       </c>
       <c r="D64" s="2" t="n">
         <v>1</v>
       </c>
       <c r="E64" s="3" t="n">
-        <v>0.2871150802837484</v>
+        <v>0.4419079419334249</v>
       </c>
     </row>
     <row r="65">
@@ -2061,13 +2061,13 @@
         </is>
       </c>
       <c r="C65" t="n">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="D65" s="2" t="n">
-        <v>0.9791666666666666</v>
+        <v>0.9795918367346939</v>
       </c>
       <c r="E65" s="3" t="n">
-        <v>1.081545289061186</v>
+        <v>1.145479715290694</v>
       </c>
     </row>
     <row r="66">
@@ -2082,13 +2082,13 @@
         </is>
       </c>
       <c r="C66" t="n">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="D66" s="2" t="n">
-        <v>0.9736842105263158</v>
+        <v>0.9743589743589743</v>
       </c>
       <c r="E66" s="3" t="n">
-        <v>0.1716760837214112</v>
+        <v>0.2105649726103001</v>
       </c>
     </row>
     <row r="67">
@@ -2187,13 +2187,13 @@
         </is>
       </c>
       <c r="C71" t="n">
-        <v>36</v>
+        <v>40</v>
       </c>
       <c r="D71" s="2" t="n">
-        <v>0.8888888888888888</v>
+        <v>0.9</v>
       </c>
       <c r="E71" s="3" t="n">
-        <v>0.1378651467320804</v>
+        <v>0.1827161135785423</v>
       </c>
     </row>
     <row r="72">
@@ -2208,13 +2208,13 @@
         </is>
       </c>
       <c r="C72" t="n">
-        <v>95</v>
+        <v>100</v>
       </c>
       <c r="D72" s="2" t="n">
-        <v>0.9473684210526315</v>
+        <v>0.95</v>
       </c>
       <c r="E72" s="3" t="n">
-        <v>0.4880192680261172</v>
+        <v>0.5146684667805791</v>
       </c>
     </row>
     <row r="73">
@@ -2229,13 +2229,13 @@
         </is>
       </c>
       <c r="C73" t="n">
-        <v>39</v>
+        <v>41</v>
       </c>
       <c r="D73" s="2" t="n">
         <v>1</v>
       </c>
       <c r="E73" s="3" t="n">
-        <v>0.0925480365595033</v>
+        <v>0.1001035299476396</v>
       </c>
     </row>
     <row r="74">
@@ -2271,13 +2271,13 @@
         </is>
       </c>
       <c r="C75" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="D75" s="2" t="n">
-        <v>0.8</v>
+        <v>0.8571428571428571</v>
       </c>
       <c r="E75" s="3" t="n">
-        <v>-0.02127270710749547</v>
+        <v>-0.002634714275954223</v>
       </c>
     </row>
   </sheetData>
@@ -2329,13 +2329,13 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>1031</v>
+        <v>1053</v>
       </c>
       <c r="C2" s="2" t="n">
-        <v>0.8826000000000001</v>
+        <v>0.8832</v>
       </c>
       <c r="D2" s="2" t="n">
-        <v>0.9902</v>
+        <v>0.9899</v>
       </c>
     </row>
     <row r="3">
@@ -2345,13 +2345,13 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>960</v>
+        <v>981</v>
       </c>
       <c r="C3" s="2" t="n">
-        <v>0.851</v>
+        <v>0.8542</v>
       </c>
       <c r="D3" s="2" t="n">
-        <v>0.997</v>
+        <v>0.9966</v>
       </c>
     </row>
     <row r="4">
@@ -2361,13 +2361,13 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>928</v>
+        <v>958</v>
       </c>
       <c r="C4" s="2" t="n">
-        <v>0.875</v>
+        <v>0.8789</v>
       </c>
       <c r="D4" s="2" t="n">
-        <v>0.9928</v>
+        <v>0.992</v>
       </c>
     </row>
     <row r="5">
@@ -2377,13 +2377,13 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>1045</v>
+        <v>1066</v>
       </c>
       <c r="C5" s="2" t="n">
-        <v>0.8784999999999999</v>
+        <v>0.8809</v>
       </c>
       <c r="D5" s="2" t="n">
-        <v>0.9936</v>
+        <v>0.9935</v>
       </c>
     </row>
     <row r="6">
@@ -2393,13 +2393,13 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>1083</v>
+        <v>1111</v>
       </c>
       <c r="C6" s="2" t="n">
-        <v>0.8846000000000001</v>
+        <v>0.8875</v>
       </c>
       <c r="D6" s="2" t="n">
-        <v>0.9939</v>
+        <v>0.9932</v>
       </c>
     </row>
     <row r="7">
@@ -2409,13 +2409,13 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>1073</v>
+        <v>1098</v>
       </c>
       <c r="C7" s="2" t="n">
-        <v>0.8779</v>
+        <v>0.8807</v>
       </c>
       <c r="D7" s="2" t="n">
-        <v>0.9956</v>
+        <v>0.9949</v>
       </c>
     </row>
     <row r="8">
@@ -2425,13 +2425,13 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>908</v>
+        <v>932</v>
       </c>
       <c r="C8" s="2" t="n">
-        <v>0.8866000000000001</v>
+        <v>0.8873</v>
       </c>
       <c r="D8" s="2" t="n">
-        <v>0.99</v>
+        <v>0.9891</v>
       </c>
     </row>
     <row r="9">
@@ -2441,13 +2441,13 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>1078</v>
+        <v>1101</v>
       </c>
       <c r="C9" s="2" t="n">
-        <v>0.8544</v>
+        <v>0.8574000000000001</v>
       </c>
       <c r="D9" s="2" t="n">
-        <v>0.996</v>
+        <v>0.9955000000000001</v>
       </c>
     </row>
     <row r="10">
@@ -2457,13 +2457,13 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>1063</v>
+        <v>1087</v>
       </c>
       <c r="C10" s="2" t="n">
-        <v>0.8711</v>
+        <v>0.874</v>
       </c>
       <c r="D10" s="2" t="n">
-        <v>0.9967</v>
+        <v>0.9965000000000001</v>
       </c>
     </row>
     <row r="11">
@@ -2473,13 +2473,13 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>1034</v>
+        <v>1055</v>
       </c>
       <c r="C11" s="2" t="n">
-        <v>0.8859</v>
+        <v>0.8882</v>
       </c>
       <c r="D11" s="2" t="n">
-        <v>0.9943</v>
+        <v>0.9942</v>
       </c>
     </row>
     <row r="12">
@@ -2489,13 +2489,13 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>1023</v>
+        <v>1048</v>
       </c>
       <c r="C12" s="2" t="n">
-        <v>0.8837</v>
+        <v>0.8855</v>
       </c>
       <c r="D12" s="2" t="n">
-        <v>0.9942</v>
+        <v>0.994</v>
       </c>
     </row>
     <row r="13">
@@ -2505,13 +2505,13 @@
         </is>
       </c>
       <c r="B13" t="n">
-        <v>1052</v>
+        <v>1079</v>
       </c>
       <c r="C13" s="2" t="n">
-        <v>0.8992</v>
+        <v>0.8999</v>
       </c>
       <c r="D13" s="2" t="n">
-        <v>0.9838</v>
+        <v>0.9833</v>
       </c>
     </row>
     <row r="14">
@@ -2521,13 +2521,13 @@
         </is>
       </c>
       <c r="B14" t="n">
-        <v>1036</v>
+        <v>1059</v>
       </c>
       <c r="C14" s="2" t="n">
-        <v>0.8842</v>
+        <v>0.8867</v>
       </c>
       <c r="D14" s="2" t="n">
-        <v>0.9939</v>
+        <v>0.9935</v>
       </c>
     </row>
     <row r="15">
@@ -2537,13 +2537,13 @@
         </is>
       </c>
       <c r="B15" t="n">
-        <v>1046</v>
+        <v>1069</v>
       </c>
       <c r="C15" s="2" t="n">
-        <v>0.8681</v>
+        <v>0.87</v>
       </c>
       <c r="D15" s="2" t="n">
-        <v>0.9932</v>
+        <v>0.9929</v>
       </c>
     </row>
     <row r="16">
@@ -2553,13 +2553,13 @@
         </is>
       </c>
       <c r="B16" t="n">
-        <v>1077</v>
+        <v>1104</v>
       </c>
       <c r="C16" s="2" t="n">
-        <v>0.8932</v>
+        <v>0.8958</v>
       </c>
       <c r="D16" s="2" t="n">
-        <v>0.9954</v>
+        <v>0.9952</v>
       </c>
     </row>
     <row r="17">
@@ -2569,13 +2569,13 @@
         </is>
       </c>
       <c r="B17" t="n">
-        <v>1043</v>
+        <v>1067</v>
       </c>
       <c r="C17" s="2" t="n">
-        <v>0.8782</v>
+        <v>0.881</v>
       </c>
       <c r="D17" s="2" t="n">
-        <v>0.9952</v>
+        <v>0.9948</v>
       </c>
     </row>
     <row r="18">
@@ -2585,13 +2585,13 @@
         </is>
       </c>
       <c r="B18" t="n">
-        <v>1104</v>
+        <v>1130</v>
       </c>
       <c r="C18" s="2" t="n">
-        <v>0.8614000000000001</v>
+        <v>0.8646</v>
       </c>
       <c r="D18" s="2" t="n">
-        <v>0.9966</v>
+        <v>0.9964</v>
       </c>
     </row>
     <row r="19">
@@ -2601,13 +2601,13 @@
         </is>
       </c>
       <c r="B19" t="n">
-        <v>1059</v>
+        <v>1080</v>
       </c>
       <c r="C19" s="2" t="n">
-        <v>0.8697</v>
+        <v>0.8722</v>
       </c>
       <c r="D19" s="2" t="n">
-        <v>0.9956</v>
+        <v>0.9953</v>
       </c>
     </row>
     <row r="20">
@@ -2617,13 +2617,13 @@
         </is>
       </c>
       <c r="B20" t="n">
-        <v>955</v>
+        <v>975</v>
       </c>
       <c r="C20" s="2" t="n">
-        <v>0.8524</v>
+        <v>0.8554</v>
       </c>
       <c r="D20" s="2" t="n">
-        <v>0.9968</v>
+        <v>0.9962</v>
       </c>
     </row>
     <row r="21">
@@ -2633,13 +2633,13 @@
         </is>
       </c>
       <c r="B21" t="n">
-        <v>950</v>
+        <v>975</v>
       </c>
       <c r="C21" s="2" t="n">
-        <v>0.8537</v>
+        <v>0.8554</v>
       </c>
       <c r="D21" s="2" t="n">
-        <v>0.9943</v>
+        <v>0.9942</v>
       </c>
     </row>
     <row r="22">
@@ -2649,13 +2649,13 @@
         </is>
       </c>
       <c r="B22" t="n">
-        <v>1091</v>
+        <v>1116</v>
       </c>
       <c r="C22" s="2" t="n">
-        <v>0.857</v>
+        <v>0.8602</v>
       </c>
       <c r="D22" s="2" t="n">
-        <v>0.9954</v>
+        <v>0.9949</v>
       </c>
     </row>
     <row r="23">
@@ -2665,13 +2665,13 @@
         </is>
       </c>
       <c r="B23" t="n">
-        <v>1028</v>
+        <v>1063</v>
       </c>
       <c r="C23" s="2" t="n">
-        <v>0.9086</v>
+        <v>0.9087</v>
       </c>
       <c r="D23" s="2" t="n">
-        <v>0.9896</v>
+        <v>0.9883999999999999</v>
       </c>
     </row>
     <row r="24">
@@ -2681,13 +2681,13 @@
         </is>
       </c>
       <c r="B24" t="n">
-        <v>985</v>
+        <v>1004</v>
       </c>
       <c r="C24" s="2" t="n">
-        <v>0.8812</v>
+        <v>0.8835</v>
       </c>
       <c r="D24" s="2" t="n">
-        <v>0.989</v>
+        <v>0.9885</v>
       </c>
     </row>
     <row r="25">
@@ -2697,13 +2697,13 @@
         </is>
       </c>
       <c r="B25" t="n">
-        <v>1049</v>
+        <v>1084</v>
       </c>
       <c r="C25" s="2" t="n">
-        <v>0.9323</v>
+        <v>0.9327</v>
       </c>
       <c r="D25" s="2" t="n">
-        <v>0.993</v>
+        <v>0.9923999999999999</v>
       </c>
     </row>
     <row r="26">
@@ -2713,13 +2713,13 @@
         </is>
       </c>
       <c r="B26" t="n">
-        <v>885</v>
+        <v>908</v>
       </c>
       <c r="C26" s="2" t="n">
-        <v>0.8938</v>
+        <v>0.8965</v>
       </c>
       <c r="D26" s="2" t="n">
-        <v>0.9912</v>
+        <v>0.9903</v>
       </c>
     </row>
     <row r="27">
@@ -2729,13 +2729,13 @@
         </is>
       </c>
       <c r="B27" t="n">
-        <v>1013</v>
+        <v>1034</v>
       </c>
       <c r="C27" s="2" t="n">
-        <v>0.9161</v>
+        <v>0.9167999999999999</v>
       </c>
       <c r="D27" s="2" t="n">
-        <v>0.9856</v>
+        <v>0.9851</v>
       </c>
     </row>
     <row r="28">
@@ -2745,13 +2745,13 @@
         </is>
       </c>
       <c r="B28" t="n">
-        <v>1018</v>
+        <v>1019</v>
       </c>
       <c r="C28" s="2" t="n">
-        <v>0.9106</v>
+        <v>0.9107</v>
       </c>
       <c r="D28" s="2" t="n">
-        <v>0.9863</v>
+        <v>0.9862</v>
       </c>
     </row>
     <row r="29">
@@ -2761,13 +2761,13 @@
         </is>
       </c>
       <c r="B29" t="n">
-        <v>891</v>
+        <v>919</v>
       </c>
       <c r="C29" s="2" t="n">
-        <v>0.9001</v>
+        <v>0.9032</v>
       </c>
       <c r="D29" s="2" t="n">
-        <v>0.993</v>
+        <v>0.9927</v>
       </c>
     </row>
     <row r="30">
@@ -2777,13 +2777,13 @@
         </is>
       </c>
       <c r="B30" t="n">
-        <v>1019</v>
+        <v>1049</v>
       </c>
       <c r="C30" s="2" t="n">
-        <v>0.8852</v>
+        <v>0.8885</v>
       </c>
       <c r="D30" s="2" t="n">
-        <v>0.9913999999999999</v>
+        <v>0.9909</v>
       </c>
     </row>
     <row r="31">
@@ -2793,13 +2793,13 @@
         </is>
       </c>
       <c r="B31" t="n">
-        <v>1052</v>
+        <v>1084</v>
       </c>
       <c r="C31" s="2" t="n">
-        <v>0.8802</v>
+        <v>0.8828</v>
       </c>
       <c r="D31" s="2" t="n">
-        <v>0.9926</v>
+        <v>0.9916</v>
       </c>
     </row>
     <row r="32">
@@ -2809,13 +2809,13 @@
         </is>
       </c>
       <c r="B32" t="n">
-        <v>1037</v>
+        <v>1063</v>
       </c>
       <c r="C32" s="2" t="n">
-        <v>0.8852</v>
+        <v>0.8871</v>
       </c>
       <c r="D32" s="2" t="n">
-        <v>0.9895</v>
+        <v>0.9892</v>
       </c>
     </row>
     <row r="33">
@@ -2825,13 +2825,13 @@
         </is>
       </c>
       <c r="B33" t="n">
-        <v>842</v>
+        <v>860</v>
       </c>
       <c r="C33" s="2" t="n">
-        <v>0.9002</v>
+        <v>0.9023</v>
       </c>
       <c r="D33" s="2" t="n">
-        <v>0.9883999999999999</v>
+        <v>0.988</v>
       </c>
     </row>
     <row r="34">
@@ -2841,13 +2841,13 @@
         </is>
       </c>
       <c r="B34" t="n">
-        <v>994</v>
+        <v>1018</v>
       </c>
       <c r="C34" s="2" t="n">
-        <v>0.9245</v>
+        <v>0.9263</v>
       </c>
       <c r="D34" s="2" t="n">
-        <v>0.9907</v>
+        <v>0.9905</v>
       </c>
     </row>
     <row r="35">
@@ -2857,13 +2857,13 @@
         </is>
       </c>
       <c r="B35" t="n">
-        <v>1065</v>
+        <v>1085</v>
       </c>
       <c r="C35" s="2" t="n">
-        <v>0.8704</v>
+        <v>0.8728</v>
       </c>
       <c r="D35" s="2" t="n">
-        <v>0.9943</v>
+        <v>0.9937</v>
       </c>
     </row>
     <row r="36">
@@ -2873,13 +2873,13 @@
         </is>
       </c>
       <c r="B36" t="n">
-        <v>850</v>
+        <v>875</v>
       </c>
       <c r="C36" s="2" t="n">
-        <v>0.9</v>
+        <v>0.9029</v>
       </c>
       <c r="D36" s="2" t="n">
-        <v>0.9902</v>
+        <v>0.9897</v>
       </c>
     </row>
     <row r="37">
@@ -2889,13 +2889,13 @@
         </is>
       </c>
       <c r="B37" t="n">
-        <v>925</v>
+        <v>956</v>
       </c>
       <c r="C37" s="2" t="n">
-        <v>0.9124</v>
+        <v>0.9079</v>
       </c>
       <c r="D37" s="2" t="n">
-        <v>0.9923999999999999</v>
+        <v>0.9919</v>
       </c>
     </row>
     <row r="38">
@@ -2905,13 +2905,13 @@
         </is>
       </c>
       <c r="B38" t="n">
-        <v>900</v>
+        <v>927</v>
       </c>
       <c r="C38" s="2" t="n">
-        <v>0.8911</v>
+        <v>0.8943</v>
       </c>
       <c r="D38" s="2" t="n">
-        <v>0.9909</v>
+        <v>0.9903999999999999</v>
       </c>
     </row>
     <row r="39">
@@ -2921,13 +2921,13 @@
         </is>
       </c>
       <c r="B39" t="n">
-        <v>1080</v>
+        <v>1100</v>
       </c>
       <c r="C39" s="2" t="n">
-        <v>0.8935</v>
+        <v>0.8955</v>
       </c>
       <c r="D39" s="2" t="n">
-        <v>0.9889</v>
+        <v>0.9882</v>
       </c>
     </row>
     <row r="40">
@@ -2937,13 +2937,13 @@
         </is>
       </c>
       <c r="B40" t="n">
-        <v>886</v>
+        <v>910</v>
       </c>
       <c r="C40" s="2" t="n">
-        <v>0.8747</v>
+        <v>0.8769</v>
       </c>
       <c r="D40" s="2" t="n">
-        <v>0.9919</v>
+        <v>0.9918</v>
       </c>
     </row>
   </sheetData>
@@ -3007,19 +3007,19 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>0.1326</v>
+        <v>0.1307</v>
       </c>
       <c r="C2" t="n">
-        <v>0.1326</v>
+        <v>0.1307</v>
       </c>
       <c r="D2" t="n">
-        <v>0.0045</v>
+        <v>0.0044</v>
       </c>
       <c r="E2" t="n">
-        <v>1.0366</v>
+        <v>1.0393</v>
       </c>
       <c r="F2" t="n">
-        <v>0.07439999999999999</v>
+        <v>0.0746</v>
       </c>
     </row>
     <row r="3">
@@ -3029,16 +3029,16 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>0.1283</v>
+        <v>0.1266</v>
       </c>
       <c r="C3" t="n">
-        <v>0.1283</v>
+        <v>0.1266</v>
       </c>
       <c r="D3" t="n">
-        <v>-0.009299999999999999</v>
+        <v>-0.008200000000000001</v>
       </c>
       <c r="E3" t="n">
-        <v>1.0512</v>
+        <v>1.0573</v>
       </c>
       <c r="F3" t="n">
         <v>0.08160000000000001</v>
@@ -3051,19 +3051,19 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>0.0504</v>
+        <v>0.0501</v>
       </c>
       <c r="C4" t="n">
         <v>0.0447</v>
       </c>
       <c r="D4" t="n">
-        <v>0.08890000000000001</v>
+        <v>0.0901</v>
       </c>
       <c r="E4" t="n">
-        <v>1.0069</v>
+        <v>1.013</v>
       </c>
       <c r="F4" t="n">
-        <v>0.0633</v>
+        <v>0.06320000000000001</v>
       </c>
     </row>
   </sheetData>
@@ -3092,7 +3092,7 @@
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>2026-08-01T09:14:36+00:00</t>
+          <t>2026-08-04T09:15:09+00:00</t>
         </is>
       </c>
     </row>
@@ -3103,7 +3103,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>4037</v>
+        <v>4154</v>
       </c>
     </row>
     <row r="3">
@@ -3113,7 +3113,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>104</v>
+        <v>107</v>
       </c>
     </row>
     <row r="4">
@@ -3143,7 +3143,7 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>192</v>
+        <v>198</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Arquiva dados, recalibra e atualiza docs (2026-08-07)
</commit_message>
<xml_diff>
--- a/backtest_results/resultados_backtest.xlsx
+++ b/backtest_results/resultados_backtest.xlsx
@@ -516,28 +516,28 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>376</v>
+        <v>821</v>
       </c>
       <c r="C2" s="2" t="n">
-        <v>0.898936170212766</v>
+        <v>0.8343483556638246</v>
       </c>
       <c r="D2" s="3" t="n">
-        <v>5.563470606153434</v>
+        <v>8.623489648769622</v>
       </c>
       <c r="E2" s="4" t="n">
-        <v>47.9117099757488</v>
+        <v>203.998157814339</v>
       </c>
       <c r="F2" s="2" t="n">
-        <v>1.959047048321784</v>
+        <v>3.264794083041586</v>
       </c>
       <c r="G2" s="2" t="n">
-        <v>0.2170352923628444</v>
+        <v>0.3062760852327849</v>
       </c>
       <c r="H2" t="n">
-        <v>73</v>
+        <v>282</v>
       </c>
       <c r="I2" s="3" t="n">
-        <v>0.8259135638297872</v>
+        <v>0.7868830694275274</v>
       </c>
     </row>
     <row r="3">
@@ -547,19 +547,19 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>1808</v>
+        <v>1842</v>
       </c>
       <c r="C3" s="2" t="n">
-        <v>0.9933628318584071</v>
+        <v>0.993485342019544</v>
       </c>
       <c r="D3" s="3" t="n">
-        <v>1.98840872976479</v>
+        <v>2.039545780096339</v>
       </c>
       <c r="E3" s="4" t="n">
-        <v>2.896483442803385</v>
+        <v>2.972702866171187</v>
       </c>
       <c r="F3" s="2" t="n">
-        <v>0.3474000407567095</v>
+        <v>0.3459884050303508</v>
       </c>
       <c r="G3" s="2" t="n">
         <v>0.08704657533117932</v>
@@ -568,7 +568,7 @@
         <v>38</v>
       </c>
       <c r="I3" s="3" t="n">
-        <v>0.9857358960176992</v>
+        <v>0.9857266558089034</v>
       </c>
     </row>
     <row r="4">
@@ -578,19 +578,19 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>1311</v>
+        <v>1334</v>
       </c>
       <c r="C4" s="2" t="n">
-        <v>0.9946605644546148</v>
+        <v>0.9947526236881559</v>
       </c>
       <c r="D4" s="3" t="n">
-        <v>1.393234076639585</v>
+        <v>1.427600857501266</v>
       </c>
       <c r="E4" s="4" t="n">
-        <v>2.40759455771909</v>
+        <v>2.454745913306565</v>
       </c>
       <c r="F4" s="2" t="n">
-        <v>0.2793400235795169</v>
+        <v>0.2775132745381776</v>
       </c>
       <c r="G4" s="2" t="n">
         <v>0.08016721391959114</v>
@@ -599,7 +599,7 @@
         <v>23</v>
       </c>
       <c r="I4" s="3" t="n">
-        <v>0.9866449275362319</v>
+        <v>0.9866221889055472</v>
       </c>
     </row>
     <row r="5">
@@ -609,19 +609,19 @@
         </is>
       </c>
       <c r="B5" s="5" t="n">
-        <v>694</v>
+        <v>708</v>
       </c>
       <c r="C5" s="6" t="n">
-        <v>0.9985590778097982</v>
+        <v>0.998587570621469</v>
       </c>
       <c r="D5" s="7" t="n">
-        <v>0.7954774270623911</v>
+        <v>0.8151447231923521</v>
       </c>
       <c r="E5" s="8" t="n">
-        <v>1.85134776044089</v>
+        <v>1.880308522123886</v>
       </c>
       <c r="F5" s="6" t="n">
-        <v>0.1884930240102944</v>
+        <v>0.1879270139333116</v>
       </c>
       <c r="G5" s="6" t="n">
         <v>0.02619857308701179</v>
@@ -630,7 +630,7 @@
         <v>6</v>
       </c>
       <c r="I5" s="7" t="n">
-        <v>0.987327809798271</v>
+        <v>0.987305790960452</v>
       </c>
     </row>
     <row r="6">
@@ -640,34 +640,34 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>1070</v>
+        <v>1529</v>
       </c>
       <c r="C6" s="2" t="n">
-        <v>0.9635514018691589</v>
+        <v>0.9103989535644212</v>
       </c>
       <c r="D6" s="3" t="n">
-        <v>6.358948033215825</v>
+        <v>9.438634371961975</v>
       </c>
       <c r="E6" s="4" t="n">
-        <v>55.09814680743132</v>
+        <v>211.2632753252152</v>
       </c>
       <c r="F6" s="2" t="n">
-        <v>2.077295842225132</v>
+        <v>3.30569151737011</v>
       </c>
       <c r="G6" s="2" t="n">
-        <v>0.1983925675638193</v>
+        <v>0.2892693823308587</v>
       </c>
       <c r="H6" t="n">
-        <v>79</v>
+        <v>288</v>
       </c>
       <c r="I6" s="3" t="n">
-        <v>0.9306065420560747</v>
+        <v>0.8796883584041857</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Atualizado em 2026-08-04T09:15:09+00:00 · arquivo de 4154 dias-cidade (~107 dias corridos) · 39 cidades</t>
+          <t>Atualizado em 2026-08-07T09:13:57+00:00 · arquivo de 4271 dias-cidade (~110 dias corridos) · 39 cidades</t>
         </is>
       </c>
     </row>
@@ -689,7 +689,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E75"/>
+  <dimension ref="A1:E76"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -738,13 +738,13 @@
         </is>
       </c>
       <c r="C2" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="D2" s="2" t="n">
-        <v>0</v>
+        <v>0.6</v>
       </c>
       <c r="E2" s="3" t="n">
-        <v>-0.015</v>
+        <v>-0.075</v>
       </c>
     </row>
     <row r="3">
@@ -759,13 +759,13 @@
         </is>
       </c>
       <c r="C3" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="D3" s="2" t="n">
         <v>1</v>
       </c>
       <c r="E3" s="3" t="n">
-        <v>0.02250133372388761</v>
+        <v>0.02871345493600883</v>
       </c>
     </row>
     <row r="4">
@@ -780,13 +780,13 @@
         </is>
       </c>
       <c r="C4" t="n">
-        <v>4</v>
+        <v>12</v>
       </c>
       <c r="D4" s="2" t="n">
         <v>1</v>
       </c>
       <c r="E4" s="3" t="n">
-        <v>-0.01807874151893931</v>
+        <v>0.06441588010448063</v>
       </c>
     </row>
     <row r="5">
@@ -801,13 +801,13 @@
         </is>
       </c>
       <c r="C5" t="n">
-        <v>8</v>
+        <v>11</v>
       </c>
       <c r="D5" s="2" t="n">
-        <v>0.875</v>
+        <v>0.9090909090909091</v>
       </c>
       <c r="E5" s="3" t="n">
-        <v>0.03322151580128275</v>
+        <v>0.09590495395641901</v>
       </c>
     </row>
     <row r="6">
@@ -822,13 +822,13 @@
         </is>
       </c>
       <c r="C6" t="n">
-        <v>16</v>
+        <v>24</v>
       </c>
       <c r="D6" s="2" t="n">
-        <v>0.9375</v>
+        <v>0.9166666666666666</v>
       </c>
       <c r="E6" s="3" t="n">
-        <v>0.0708055546408668</v>
+        <v>0.1189455334703077</v>
       </c>
     </row>
     <row r="7">
@@ -864,13 +864,13 @@
         </is>
       </c>
       <c r="C8" t="n">
-        <v>8</v>
+        <v>22</v>
       </c>
       <c r="D8" s="2" t="n">
-        <v>1</v>
+        <v>0.7727272727272727</v>
       </c>
       <c r="E8" s="3" t="n">
-        <v>0.007052021389959679</v>
+        <v>0.04730632556038945</v>
       </c>
     </row>
     <row r="9">
@@ -885,13 +885,13 @@
         </is>
       </c>
       <c r="C9" t="n">
-        <v>3</v>
+        <v>9</v>
       </c>
       <c r="D9" s="2" t="n">
-        <v>0.6666666666666666</v>
+        <v>0.8888888888888888</v>
       </c>
       <c r="E9" s="3" t="n">
-        <v>0.09546461137646549</v>
+        <v>0.1222862539916138</v>
       </c>
     </row>
     <row r="10">
@@ -927,13 +927,13 @@
         </is>
       </c>
       <c r="C11" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="D11" s="2" t="n">
-        <v>1</v>
+        <v>0.75</v>
       </c>
       <c r="E11" s="3" t="n">
-        <v>0.01248377447937243</v>
+        <v>0.003303880299478271</v>
       </c>
     </row>
     <row r="12">
@@ -948,13 +948,13 @@
         </is>
       </c>
       <c r="C12" t="n">
-        <v>4</v>
+        <v>11</v>
       </c>
       <c r="D12" s="2" t="n">
-        <v>0</v>
+        <v>0.4545454545454545</v>
       </c>
       <c r="E12" s="3" t="n">
-        <v>-0.06</v>
+        <v>-0.003623464044489731</v>
       </c>
     </row>
     <row r="13">
@@ -969,13 +969,13 @@
         </is>
       </c>
       <c r="C13" t="n">
-        <v>11</v>
+        <v>89</v>
       </c>
       <c r="D13" s="2" t="n">
-        <v>0.8181818181818182</v>
+        <v>0.651685393258427</v>
       </c>
       <c r="E13" s="3" t="n">
-        <v>0.30053294504329</v>
+        <v>0.4118047128216701</v>
       </c>
     </row>
     <row r="14">
@@ -990,13 +990,13 @@
         </is>
       </c>
       <c r="C14" t="n">
-        <v>5</v>
+        <v>9</v>
       </c>
       <c r="D14" s="2" t="n">
-        <v>0.8</v>
+        <v>0.8888888888888888</v>
       </c>
       <c r="E14" s="3" t="n">
-        <v>0.100241829372691</v>
+        <v>0.257403181763825</v>
       </c>
     </row>
     <row r="15">
@@ -1011,13 +1011,13 @@
         </is>
       </c>
       <c r="C15" t="n">
-        <v>9</v>
+        <v>12</v>
       </c>
       <c r="D15" s="2" t="n">
-        <v>0.8888888888888888</v>
+        <v>0.8333333333333334</v>
       </c>
       <c r="E15" s="3" t="n">
-        <v>0.1206121803170523</v>
+        <v>0.1291037681685989</v>
       </c>
     </row>
     <row r="16">
@@ -1032,13 +1032,13 @@
         </is>
       </c>
       <c r="C16" t="n">
-        <v>6</v>
+        <v>12</v>
       </c>
       <c r="D16" s="2" t="n">
-        <v>1</v>
+        <v>0.9166666666666666</v>
       </c>
       <c r="E16" s="3" t="n">
-        <v>0.00563570816437714</v>
+        <v>0.1541296779626947</v>
       </c>
     </row>
     <row r="17">
@@ -1053,13 +1053,13 @@
         </is>
       </c>
       <c r="C17" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="D17" s="2" t="n">
-        <v>0.8333333333333334</v>
+        <v>0.8571428571428571</v>
       </c>
       <c r="E17" s="3" t="n">
-        <v>-0.04666569575854426</v>
+        <v>-0.02618376804770087</v>
       </c>
     </row>
     <row r="18">
@@ -1091,17 +1091,17 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>Ancara (LTAC)</t>
+          <t>Tel Aviv (LLBG)</t>
         </is>
       </c>
       <c r="C19" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="D19" s="2" t="n">
-        <v>1</v>
+        <v>0.3333333333333333</v>
       </c>
       <c r="E19" s="3" t="n">
-        <v>0.007584722969338365</v>
+        <v>-0.005776397515527935</v>
       </c>
     </row>
     <row r="20">
@@ -1112,17 +1112,17 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>Istambul (LTFM)</t>
+          <t>Ancara (LTAC)</t>
         </is>
       </c>
       <c r="C20" t="n">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="D20" s="2" t="n">
-        <v>0.875</v>
+        <v>1</v>
       </c>
       <c r="E20" s="3" t="n">
-        <v>0.197388287145688</v>
+        <v>0.1314966176671566</v>
       </c>
     </row>
     <row r="21">
@@ -1133,17 +1133,17 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>Cidade do México (MMMX)</t>
+          <t>Istambul (LTFM)</t>
         </is>
       </c>
       <c r="C21" t="n">
-        <v>6</v>
+        <v>23</v>
       </c>
       <c r="D21" s="2" t="n">
-        <v>0.8333333333333334</v>
+        <v>0.6956521739130435</v>
       </c>
       <c r="E21" s="3" t="n">
-        <v>0.02092739537784452</v>
+        <v>0.1468422756171502</v>
       </c>
     </row>
     <row r="22">
@@ -1154,17 +1154,17 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>Wellington (NZWN)</t>
+          <t>Cidade do México (MMMX)</t>
         </is>
       </c>
       <c r="C22" t="n">
-        <v>17</v>
+        <v>9</v>
       </c>
       <c r="D22" s="2" t="n">
-        <v>0.8235294117647058</v>
+        <v>0.7777777777777778</v>
       </c>
       <c r="E22" s="3" t="n">
-        <v>0.3877098158278501</v>
+        <v>0.01592739537784452</v>
       </c>
     </row>
     <row r="23">
@@ -1175,17 +1175,17 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>Taipé (RCSS)</t>
+          <t>Wellington (NZWN)</t>
         </is>
       </c>
       <c r="C23" t="n">
-        <v>24</v>
+        <v>47</v>
       </c>
       <c r="D23" s="2" t="n">
-        <v>0.9166666666666666</v>
+        <v>0.7446808510638298</v>
       </c>
       <c r="E23" s="3" t="n">
-        <v>0.2726556485795536</v>
+        <v>0.7074910393505702</v>
       </c>
     </row>
     <row r="24">
@@ -1196,17 +1196,17 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>Tóquio (RJTT)</t>
+          <t>Taipé (RCSS)</t>
         </is>
       </c>
       <c r="C24" t="n">
-        <v>16</v>
+        <v>44</v>
       </c>
       <c r="D24" s="2" t="n">
-        <v>1</v>
+        <v>0.8636363636363636</v>
       </c>
       <c r="E24" s="3" t="n">
-        <v>0.2986899248517935</v>
+        <v>0.4620145470468817</v>
       </c>
     </row>
     <row r="25">
@@ -1217,17 +1217,17 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>Seul (RKSI)</t>
+          <t>Tóquio (RJTT)</t>
         </is>
       </c>
       <c r="C25" t="n">
-        <v>14</v>
+        <v>39</v>
       </c>
       <c r="D25" s="2" t="n">
-        <v>0.9285714285714286</v>
+        <v>0.8461538461538461</v>
       </c>
       <c r="E25" s="3" t="n">
-        <v>0.2659331078030273</v>
+        <v>0.4723217210911316</v>
       </c>
     </row>
     <row r="26">
@@ -1238,17 +1238,17 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>Manila (RPLL)</t>
+          <t>Seul (RKSI)</t>
         </is>
       </c>
       <c r="C26" t="n">
-        <v>23</v>
+        <v>31</v>
       </c>
       <c r="D26" s="2" t="n">
-        <v>1</v>
+        <v>0.9032258064516129</v>
       </c>
       <c r="E26" s="3" t="n">
-        <v>0.4416585625916054</v>
+        <v>0.3159542020951454</v>
       </c>
     </row>
     <row r="27">
@@ -1259,17 +1259,17 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>Buenos Aires (SAEZ)</t>
+          <t>Manila (RPLL)</t>
         </is>
       </c>
       <c r="C27" t="n">
-        <v>26</v>
+        <v>33</v>
       </c>
       <c r="D27" s="2" t="n">
-        <v>0.9615384615384616</v>
+        <v>1</v>
       </c>
       <c r="E27" s="3" t="n">
-        <v>1.128958468840324</v>
+        <v>0.5535944075318887</v>
       </c>
     </row>
     <row r="28">
@@ -1280,17 +1280,17 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>Guarulhos (SBGR)</t>
+          <t>Buenos Aires (SAEZ)</t>
         </is>
       </c>
       <c r="C28" t="n">
-        <v>7</v>
+        <v>43</v>
       </c>
       <c r="D28" s="2" t="n">
-        <v>0.8571428571428571</v>
+        <v>0.8604651162790697</v>
       </c>
       <c r="E28" s="3" t="n">
-        <v>0.1687802409697428</v>
+        <v>1.230616299890604</v>
       </c>
     </row>
     <row r="29">
@@ -1301,7 +1301,7 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>Moscou (UUWW)</t>
+          <t>Guarulhos (SBGR)</t>
         </is>
       </c>
       <c r="C29" t="n">
@@ -1311,7 +1311,7 @@
         <v>0.8571428571428571</v>
       </c>
       <c r="E29" s="3" t="n">
-        <v>0.4721726782662505</v>
+        <v>0.1757981420865279</v>
       </c>
     </row>
     <row r="30">
@@ -1322,17 +1322,17 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>Kuala Lumpur (WMKK)</t>
+          <t>Moscou (UUWW)</t>
         </is>
       </c>
       <c r="C30" t="n">
-        <v>4</v>
+        <v>33</v>
       </c>
       <c r="D30" s="2" t="n">
-        <v>1</v>
+        <v>0.8484848484848485</v>
       </c>
       <c r="E30" s="3" t="n">
-        <v>0.02901832960234521</v>
+        <v>0.6566306201959523</v>
       </c>
     </row>
     <row r="31">
@@ -1343,17 +1343,17 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>Singapura (WSSS)</t>
+          <t>Kuala Lumpur (WMKK)</t>
         </is>
       </c>
       <c r="C31" t="n">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="D31" s="2" t="n">
-        <v>0.9</v>
+        <v>1</v>
       </c>
       <c r="E31" s="3" t="n">
-        <v>0.06741812387731545</v>
+        <v>0.05069786628188186</v>
       </c>
     </row>
     <row r="32">
@@ -1364,17 +1364,17 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>Pequim (ZBAA)</t>
+          <t>Singapura (WSSS)</t>
         </is>
       </c>
       <c r="C32" t="n">
-        <v>7</v>
+        <v>21</v>
       </c>
       <c r="D32" s="2" t="n">
-        <v>1</v>
+        <v>0.9523809523809523</v>
       </c>
       <c r="E32" s="3" t="n">
-        <v>0.09010581559877134</v>
+        <v>0.2046081351060535</v>
       </c>
     </row>
     <row r="33">
@@ -1385,17 +1385,17 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>Guangzhou (ZGGG)</t>
+          <t>Pequim (ZBAA)</t>
         </is>
       </c>
       <c r="C33" t="n">
-        <v>25</v>
+        <v>12</v>
       </c>
       <c r="D33" s="2" t="n">
-        <v>0.84</v>
+        <v>1</v>
       </c>
       <c r="E33" s="3" t="n">
-        <v>0.1619206114997599</v>
+        <v>0.1793830553055883</v>
       </c>
     </row>
     <row r="34">
@@ -1406,17 +1406,17 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>Shenzhen (ZGSZ)</t>
+          <t>Guangzhou (ZGGG)</t>
         </is>
       </c>
       <c r="C34" t="n">
-        <v>50</v>
+        <v>48</v>
       </c>
       <c r="D34" s="2" t="n">
-        <v>0.9</v>
+        <v>0.875</v>
       </c>
       <c r="E34" s="3" t="n">
-        <v>0.4507150748707635</v>
+        <v>0.159388807587754</v>
       </c>
     </row>
     <row r="35">
@@ -1427,17 +1427,17 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>Wuhan (ZHHH)</t>
+          <t>Shenzhen (ZGSZ)</t>
         </is>
       </c>
       <c r="C35" t="n">
-        <v>9</v>
+        <v>100</v>
       </c>
       <c r="D35" s="2" t="n">
-        <v>1</v>
+        <v>0.87</v>
       </c>
       <c r="E35" s="3" t="n">
-        <v>0.05760390406398334</v>
+        <v>0.9809992761363049</v>
       </c>
     </row>
     <row r="36">
@@ -1448,17 +1448,17 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>Xangai (ZSPD)</t>
+          <t>Wuhan (ZHHH)</t>
         </is>
       </c>
       <c r="C36" t="n">
-        <v>12</v>
+        <v>30</v>
       </c>
       <c r="D36" s="2" t="n">
-        <v>0.9166666666666666</v>
+        <v>0.9</v>
       </c>
       <c r="E36" s="3" t="n">
-        <v>0.1685559848260972</v>
+        <v>0.3638157717166314</v>
       </c>
     </row>
     <row r="37">
@@ -1469,38 +1469,38 @@
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>Chengdu (ZUUU)</t>
+          <t>Xangai (ZSPD)</t>
         </is>
       </c>
       <c r="C37" t="n">
-        <v>5</v>
+        <v>29</v>
       </c>
       <c r="D37" s="2" t="n">
-        <v>0.8</v>
+        <v>0.7931034482758621</v>
       </c>
       <c r="E37" s="3" t="n">
-        <v>-0.005541901348352921</v>
+        <v>0.2463086036971679</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>Combinado</t>
+          <t>Edge</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>Toronto (CYYZ)</t>
+          <t>Chengdu (ZUUU)</t>
         </is>
       </c>
       <c r="C38" t="n">
-        <v>15</v>
+        <v>5</v>
       </c>
       <c r="D38" s="2" t="n">
-        <v>0.9333333333333333</v>
+        <v>0.8</v>
       </c>
       <c r="E38" s="3" t="n">
-        <v>0.007722343182870766</v>
+        <v>-0.005541901348352921</v>
       </c>
     </row>
     <row r="39">
@@ -1511,17 +1511,17 @@
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>Munique (EDDM)</t>
+          <t>Toronto (CYYZ)</t>
         </is>
       </c>
       <c r="C39" t="n">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="D39" s="2" t="n">
-        <v>0.9523809523809523</v>
+        <v>0.8947368421052632</v>
       </c>
       <c r="E39" s="3" t="n">
-        <v>0.02897737559373625</v>
+        <v>-0.05227765681712923</v>
       </c>
     </row>
     <row r="40">
@@ -1532,17 +1532,17 @@
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>Helsinque (EFHK)</t>
+          <t>Munique (EDDM)</t>
         </is>
       </c>
       <c r="C40" t="n">
-        <v>34</v>
+        <v>23</v>
       </c>
       <c r="D40" s="2" t="n">
-        <v>1</v>
+        <v>0.9565217391304348</v>
       </c>
       <c r="E40" s="3" t="n">
-        <v>0.02712646812134217</v>
+        <v>0.03518949680585746</v>
       </c>
     </row>
     <row r="41">
@@ -1553,17 +1553,17 @@
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>Londres (EGLC)</t>
+          <t>Helsinque (EFHK)</t>
         </is>
       </c>
       <c r="C41" t="n">
-        <v>32</v>
+        <v>42</v>
       </c>
       <c r="D41" s="2" t="n">
-        <v>0.96875</v>
+        <v>1</v>
       </c>
       <c r="E41" s="3" t="n">
-        <v>0.06505197524359005</v>
+        <v>0.1096210897447621</v>
       </c>
     </row>
     <row r="42">
@@ -1574,17 +1574,17 @@
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>Amsterdã (EHAM)</t>
+          <t>Londres (EGLC)</t>
         </is>
       </c>
       <c r="C42" t="n">
-        <v>60</v>
+        <v>35</v>
       </c>
       <c r="D42" s="2" t="n">
-        <v>0.9833333333333333</v>
+        <v>0.9714285714285714</v>
       </c>
       <c r="E42" s="3" t="n">
-        <v>0.1124566210129819</v>
+        <v>0.1277354133987263</v>
       </c>
     </row>
     <row r="43">
@@ -1595,17 +1595,17 @@
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>Varsóvia (EPWA)</t>
+          <t>Amsterdã (EHAM)</t>
         </is>
       </c>
       <c r="C43" t="n">
-        <v>15</v>
+        <v>72</v>
       </c>
       <c r="D43" s="2" t="n">
-        <v>0.9333333333333333</v>
+        <v>0.9722222222222222</v>
       </c>
       <c r="E43" s="3" t="n">
-        <v>0.1573199025875285</v>
+        <v>0.1657834498465466</v>
       </c>
     </row>
     <row r="44">
@@ -1616,17 +1616,17 @@
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>Cidade do Cabo (FACT)</t>
+          <t>Varsóvia (EPWA)</t>
         </is>
       </c>
       <c r="C44" t="n">
-        <v>30</v>
+        <v>15</v>
       </c>
       <c r="D44" s="2" t="n">
-        <v>1</v>
+        <v>0.9333333333333333</v>
       </c>
       <c r="E44" s="3" t="n">
-        <v>0.04067403580818672</v>
+        <v>0.1573199025875285</v>
       </c>
     </row>
     <row r="45">
@@ -1637,17 +1637,17 @@
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>Atlanta (KATL)</t>
+          <t>Cidade do Cabo (FACT)</t>
         </is>
       </c>
       <c r="C45" t="n">
-        <v>18</v>
+        <v>46</v>
       </c>
       <c r="D45" s="2" t="n">
-        <v>0.9444444444444444</v>
+        <v>0.8913043478260869</v>
       </c>
       <c r="E45" s="3" t="n">
-        <v>0.1093635095478079</v>
+        <v>0.08501528518231299</v>
       </c>
     </row>
     <row r="46">
@@ -1658,17 +1658,17 @@
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>Denver (KBKF)</t>
+          <t>Atlanta (KATL)</t>
         </is>
       </c>
       <c r="C46" t="n">
-        <v>5</v>
+        <v>24</v>
       </c>
       <c r="D46" s="2" t="n">
-        <v>1</v>
+        <v>0.9583333333333334</v>
       </c>
       <c r="E46" s="3" t="n">
-        <v>0.08135918956658879</v>
+        <v>0.1361851521629562</v>
       </c>
     </row>
     <row r="47">
@@ -1679,17 +1679,17 @@
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>Dallas (KDAL)</t>
+          <t>Denver (KBKF)</t>
         </is>
       </c>
       <c r="C47" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="D47" s="2" t="n">
         <v>1</v>
       </c>
       <c r="E47" s="3" t="n">
-        <v>0.01731065767370086</v>
+        <v>0.08135918956658879</v>
       </c>
     </row>
     <row r="48">
@@ -1700,17 +1700,17 @@
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>Houston (KHOU)</t>
+          <t>Dallas (KDAL)</t>
         </is>
       </c>
       <c r="C48" t="n">
-        <v>11</v>
+        <v>8</v>
       </c>
       <c r="D48" s="2" t="n">
-        <v>0.6363636363636364</v>
+        <v>0.875</v>
       </c>
       <c r="E48" s="3" t="n">
-        <v>-0.0485585220689388</v>
+        <v>0.008130763493806696</v>
       </c>
     </row>
     <row r="49">
@@ -1721,17 +1721,17 @@
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>Los Angeles (KLAX)</t>
+          <t>Houston (KHOU)</t>
         </is>
       </c>
       <c r="C49" t="n">
-        <v>21</v>
+        <v>18</v>
       </c>
       <c r="D49" s="2" t="n">
-        <v>0.9047619047619048</v>
+        <v>0.6666666666666666</v>
       </c>
       <c r="E49" s="3" t="n">
-        <v>0.3111743957279052</v>
+        <v>0.007818013886571476</v>
       </c>
     </row>
     <row r="50">
@@ -1742,17 +1742,17 @@
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>Nova York (KLGA)</t>
+          <t>Los Angeles (KLAX)</t>
         </is>
       </c>
       <c r="C50" t="n">
-        <v>17</v>
+        <v>99</v>
       </c>
       <c r="D50" s="2" t="n">
-        <v>0.9411764705882353</v>
+        <v>0.6868686868686869</v>
       </c>
       <c r="E50" s="3" t="n">
-        <v>0.1163074058178716</v>
+        <v>0.4224461635062853</v>
       </c>
     </row>
     <row r="51">
@@ -1763,17 +1763,17 @@
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>Miami (KMIA)</t>
+          <t>Nova York (KLGA)</t>
         </is>
       </c>
       <c r="C51" t="n">
-        <v>29</v>
+        <v>21</v>
       </c>
       <c r="D51" s="2" t="n">
-        <v>0.9655172413793104</v>
+        <v>0.9523809523809523</v>
       </c>
       <c r="E51" s="3" t="n">
-        <v>0.1437867028586853</v>
+        <v>0.2734687582090057</v>
       </c>
     </row>
     <row r="52">
@@ -1784,17 +1784,17 @@
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>Chicago (KORD)</t>
+          <t>Miami (KMIA)</t>
         </is>
       </c>
       <c r="C52" t="n">
-        <v>23</v>
+        <v>32</v>
       </c>
       <c r="D52" s="2" t="n">
-        <v>1</v>
+        <v>0.9375</v>
       </c>
       <c r="E52" s="3" t="n">
-        <v>0.02872522370697825</v>
+        <v>0.152278290710232</v>
       </c>
     </row>
     <row r="53">
@@ -1805,17 +1805,17 @@
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>Seattle (KSEA)</t>
+          <t>Chicago (KORD)</t>
         </is>
       </c>
       <c r="C53" t="n">
-        <v>23</v>
+        <v>29</v>
       </c>
       <c r="D53" s="2" t="n">
-        <v>0.9565217391304348</v>
+        <v>0.9655172413793104</v>
       </c>
       <c r="E53" s="3" t="n">
-        <v>-0.02356169087315167</v>
+        <v>0.1772191935052958</v>
       </c>
     </row>
     <row r="54">
@@ -1826,17 +1826,17 @@
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>Madri (LEMD)</t>
+          <t>Seattle (KSEA)</t>
         </is>
       </c>
       <c r="C54" t="n">
-        <v>4</v>
+        <v>24</v>
       </c>
       <c r="D54" s="2" t="n">
-        <v>1</v>
+        <v>0.9583333333333334</v>
       </c>
       <c r="E54" s="3" t="n">
-        <v>0.005385531300417991</v>
+        <v>-0.003079763162308275</v>
       </c>
     </row>
     <row r="55">
@@ -1847,17 +1847,17 @@
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>Milão (LIMC)</t>
+          <t>Madri (LEMD)</t>
         </is>
       </c>
       <c r="C55" t="n">
-        <v>20</v>
+        <v>4</v>
       </c>
       <c r="D55" s="2" t="n">
         <v>1</v>
       </c>
       <c r="E55" s="3" t="n">
-        <v>0.04893879804517041</v>
+        <v>0.005385531300417991</v>
       </c>
     </row>
     <row r="56">
@@ -1868,17 +1868,17 @@
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>Tel Aviv (LLBG)</t>
+          <t>Milão (LIMC)</t>
         </is>
       </c>
       <c r="C56" t="n">
-        <v>4</v>
+        <v>20</v>
       </c>
       <c r="D56" s="2" t="n">
         <v>1</v>
       </c>
       <c r="E56" s="3" t="n">
-        <v>0.005115058255058735</v>
+        <v>0.04893879804517041</v>
       </c>
     </row>
     <row r="57">
@@ -1889,17 +1889,17 @@
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>Ancara (LTAC)</t>
+          <t>Tel Aviv (LLBG)</t>
         </is>
       </c>
       <c r="C57" t="n">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="D57" s="2" t="n">
-        <v>1</v>
+        <v>0.7142857142857143</v>
       </c>
       <c r="E57" s="3" t="n">
-        <v>0.01971833461439963</v>
+        <v>-0.0006613392604692</v>
       </c>
     </row>
     <row r="58">
@@ -1910,17 +1910,17 @@
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>Istambul (LTFM)</t>
+          <t>Ancara (LTAC)</t>
         </is>
       </c>
       <c r="C58" t="n">
-        <v>70</v>
+        <v>13</v>
       </c>
       <c r="D58" s="2" t="n">
-        <v>0.9857142857142858</v>
+        <v>1</v>
       </c>
       <c r="E58" s="3" t="n">
-        <v>0.2753348375732511</v>
+        <v>0.1436302293122179</v>
       </c>
     </row>
     <row r="59">
@@ -1931,17 +1931,17 @@
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>Cidade do México (MMMX)</t>
+          <t>Istambul (LTFM)</t>
         </is>
       </c>
       <c r="C59" t="n">
-        <v>20</v>
+        <v>87</v>
       </c>
       <c r="D59" s="2" t="n">
-        <v>0.95</v>
+        <v>0.9195402298850575</v>
       </c>
       <c r="E59" s="3" t="n">
-        <v>0.03704785368229767</v>
+        <v>0.2258949095037379</v>
       </c>
     </row>
     <row r="60">
@@ -1952,17 +1952,17 @@
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>Wellington (NZWN)</t>
+          <t>Cidade do México (MMMX)</t>
         </is>
       </c>
       <c r="C60" t="n">
-        <v>46</v>
+        <v>23</v>
       </c>
       <c r="D60" s="2" t="n">
-        <v>0.9347826086956522</v>
+        <v>0.9130434782608695</v>
       </c>
       <c r="E60" s="3" t="n">
-        <v>0.4101974315460432</v>
+        <v>0.03204785368229767</v>
       </c>
     </row>
     <row r="61">
@@ -1973,17 +1973,17 @@
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>Taipé (RCSS)</t>
+          <t>Wellington (NZWN)</t>
         </is>
       </c>
       <c r="C61" t="n">
-        <v>29</v>
+        <v>76</v>
       </c>
       <c r="D61" s="2" t="n">
-        <v>0.9310344827586207</v>
+        <v>0.8421052631578947</v>
       </c>
       <c r="E61" s="3" t="n">
-        <v>0.2782472797296235</v>
+        <v>0.7299786550687631</v>
       </c>
     </row>
     <row r="62">
@@ -1994,17 +1994,17 @@
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>Tóquio (RJTT)</t>
+          <t>Taipé (RCSS)</t>
         </is>
       </c>
       <c r="C62" t="n">
-        <v>45</v>
+        <v>50</v>
       </c>
       <c r="D62" s="2" t="n">
-        <v>1</v>
+        <v>0.88</v>
       </c>
       <c r="E62" s="3" t="n">
-        <v>0.334545001546555</v>
+        <v>0.4681592199264639</v>
       </c>
     </row>
     <row r="63">
@@ -2015,17 +2015,17 @@
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>Seul (RKSI)</t>
+          <t>Tóquio (RJTT)</t>
         </is>
       </c>
       <c r="C63" t="n">
-        <v>22</v>
+        <v>68</v>
       </c>
       <c r="D63" s="2" t="n">
-        <v>0.9545454545454546</v>
+        <v>0.9117647058823529</v>
       </c>
       <c r="E63" s="3" t="n">
-        <v>0.2745518939464943</v>
+        <v>0.5081767977858931</v>
       </c>
     </row>
     <row r="64">
@@ -2036,17 +2036,17 @@
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>Manila (RPLL)</t>
+          <t>Seul (RKSI)</t>
         </is>
       </c>
       <c r="C64" t="n">
-        <v>50</v>
+        <v>39</v>
       </c>
       <c r="D64" s="2" t="n">
-        <v>1</v>
+        <v>0.9230769230769231</v>
       </c>
       <c r="E64" s="3" t="n">
-        <v>0.4419079419334249</v>
+        <v>0.3245729882386124</v>
       </c>
     </row>
     <row r="65">
@@ -2057,17 +2057,17 @@
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>Buenos Aires (SAEZ)</t>
+          <t>Manila (RPLL)</t>
         </is>
       </c>
       <c r="C65" t="n">
-        <v>49</v>
+        <v>60</v>
       </c>
       <c r="D65" s="2" t="n">
-        <v>0.9795918367346939</v>
+        <v>1</v>
       </c>
       <c r="E65" s="3" t="n">
-        <v>1.145479715290694</v>
+        <v>0.5538437868737083</v>
       </c>
     </row>
     <row r="66">
@@ -2078,17 +2078,17 @@
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>Guarulhos (SBGR)</t>
+          <t>Buenos Aires (SAEZ)</t>
         </is>
       </c>
       <c r="C66" t="n">
-        <v>39</v>
+        <v>66</v>
       </c>
       <c r="D66" s="2" t="n">
-        <v>0.9743589743589743</v>
+        <v>0.9090909090909091</v>
       </c>
       <c r="E66" s="3" t="n">
-        <v>0.2105649726103001</v>
+        <v>1.247137546340974</v>
       </c>
     </row>
     <row r="67">
@@ -2099,17 +2099,17 @@
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>Moscou (UUWW)</t>
+          <t>Guarulhos (SBGR)</t>
         </is>
       </c>
       <c r="C67" t="n">
-        <v>37</v>
+        <v>46</v>
       </c>
       <c r="D67" s="2" t="n">
-        <v>0.9459459459459459</v>
+        <v>0.9565217391304348</v>
       </c>
       <c r="E67" s="3" t="n">
-        <v>0.5003301400428891</v>
+        <v>0.2175828737270852</v>
       </c>
     </row>
     <row r="68">
@@ -2120,17 +2120,17 @@
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>Kuala Lumpur (WMKK)</t>
+          <t>Moscou (UUWW)</t>
         </is>
       </c>
       <c r="C68" t="n">
-        <v>8</v>
+        <v>57</v>
       </c>
       <c r="D68" s="2" t="n">
-        <v>1</v>
+        <v>0.9122807017543859</v>
       </c>
       <c r="E68" s="3" t="n">
-        <v>0.03321304116819632</v>
+        <v>0.6869331279378615</v>
       </c>
     </row>
     <row r="69">
@@ -2141,17 +2141,17 @@
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>Singapura (WSSS)</t>
+          <t>Kuala Lumpur (WMKK)</t>
         </is>
       </c>
       <c r="C69" t="n">
-        <v>24</v>
+        <v>12</v>
       </c>
       <c r="D69" s="2" t="n">
-        <v>0.9583333333333334</v>
+        <v>1</v>
       </c>
       <c r="E69" s="3" t="n">
-        <v>0.0788284094462868</v>
+        <v>0.05489257784773297</v>
       </c>
     </row>
     <row r="70">
@@ -2162,17 +2162,17 @@
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>Pequim (ZBAA)</t>
+          <t>Singapura (WSSS)</t>
         </is>
       </c>
       <c r="C70" t="n">
-        <v>15</v>
+        <v>35</v>
       </c>
       <c r="D70" s="2" t="n">
-        <v>1</v>
+        <v>0.9714285714285714</v>
       </c>
       <c r="E70" s="3" t="n">
-        <v>0.09900287745257799</v>
+        <v>0.2160184206750249</v>
       </c>
     </row>
     <row r="71">
@@ -2183,17 +2183,17 @@
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>Guangzhou (ZGGG)</t>
+          <t>Pequim (ZBAA)</t>
         </is>
       </c>
       <c r="C71" t="n">
-        <v>40</v>
+        <v>21</v>
       </c>
       <c r="D71" s="2" t="n">
-        <v>0.9</v>
+        <v>1</v>
       </c>
       <c r="E71" s="3" t="n">
-        <v>0.1827161135785423</v>
+        <v>0.189545939944205</v>
       </c>
     </row>
     <row r="72">
@@ -2204,17 +2204,17 @@
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>Shenzhen (ZGSZ)</t>
+          <t>Guangzhou (ZGGG)</t>
         </is>
       </c>
       <c r="C72" t="n">
-        <v>100</v>
+        <v>64</v>
       </c>
       <c r="D72" s="2" t="n">
-        <v>0.95</v>
+        <v>0.90625</v>
       </c>
       <c r="E72" s="3" t="n">
-        <v>0.5146684667805791</v>
+        <v>0.1818619914153925</v>
       </c>
     </row>
     <row r="73">
@@ -2225,17 +2225,17 @@
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>Wuhan (ZHHH)</t>
+          <t>Shenzhen (ZGSZ)</t>
         </is>
       </c>
       <c r="C73" t="n">
-        <v>41</v>
+        <v>152</v>
       </c>
       <c r="D73" s="2" t="n">
-        <v>1</v>
+        <v>0.9144736842105263</v>
       </c>
       <c r="E73" s="3" t="n">
-        <v>0.1001035299476396</v>
+        <v>1.048598493280787</v>
       </c>
     </row>
     <row r="74">
@@ -2246,17 +2246,17 @@
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>Xangai (ZSPD)</t>
+          <t>Wuhan (ZHHH)</t>
         </is>
       </c>
       <c r="C74" t="n">
-        <v>31</v>
+        <v>62</v>
       </c>
       <c r="D74" s="2" t="n">
-        <v>0.967741935483871</v>
+        <v>0.9516129032258065</v>
       </c>
       <c r="E74" s="3" t="n">
-        <v>0.1904499254936535</v>
+        <v>0.4063153976002876</v>
       </c>
     </row>
     <row r="75">
@@ -2267,16 +2267,37 @@
       </c>
       <c r="B75" t="inlineStr">
         <is>
+          <t>Xangai (ZSPD)</t>
+        </is>
+      </c>
+      <c r="C75" t="n">
+        <v>48</v>
+      </c>
+      <c r="D75" s="2" t="n">
+        <v>0.875</v>
+      </c>
+      <c r="E75" s="3" t="n">
+        <v>0.2682025443647241</v>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" t="inlineStr">
+        <is>
+          <t>Combinado</t>
+        </is>
+      </c>
+      <c r="B76" t="inlineStr">
+        <is>
           <t>Chengdu (ZUUU)</t>
         </is>
       </c>
-      <c r="C75" t="n">
+      <c r="C76" t="n">
         <v>7</v>
       </c>
-      <c r="D75" s="2" t="n">
+      <c r="D76" s="2" t="n">
         <v>0.8571428571428571</v>
       </c>
-      <c r="E75" s="3" t="n">
+      <c r="E76" s="3" t="n">
         <v>-0.002634714275954223</v>
       </c>
     </row>
@@ -2329,13 +2350,13 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>1053</v>
+        <v>895</v>
       </c>
       <c r="C2" s="2" t="n">
-        <v>0.8832</v>
+        <v>0.8816000000000001</v>
       </c>
       <c r="D2" s="2" t="n">
-        <v>0.9899</v>
+        <v>0.9916</v>
       </c>
     </row>
     <row r="3">
@@ -2345,13 +2366,13 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>981</v>
+        <v>952</v>
       </c>
       <c r="C3" s="2" t="n">
-        <v>0.8542</v>
+        <v>0.8519</v>
       </c>
       <c r="D3" s="2" t="n">
-        <v>0.9966</v>
+        <v>0.9969</v>
       </c>
     </row>
     <row r="4">
@@ -2361,13 +2382,13 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>958</v>
+        <v>895</v>
       </c>
       <c r="C4" s="2" t="n">
-        <v>0.8789</v>
+        <v>0.8793</v>
       </c>
       <c r="D4" s="2" t="n">
-        <v>0.992</v>
+        <v>0.9931</v>
       </c>
     </row>
     <row r="5">
@@ -2377,13 +2398,13 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>1066</v>
+        <v>982</v>
       </c>
       <c r="C5" s="2" t="n">
-        <v>0.8809</v>
+        <v>0.8768</v>
       </c>
       <c r="D5" s="2" t="n">
-        <v>0.9935</v>
+        <v>0.9939</v>
       </c>
     </row>
     <row r="6">
@@ -2393,13 +2414,13 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>1111</v>
+        <v>1068</v>
       </c>
       <c r="C6" s="2" t="n">
-        <v>0.8875</v>
+        <v>0.8904</v>
       </c>
       <c r="D6" s="2" t="n">
-        <v>0.9932</v>
+        <v>0.9928</v>
       </c>
     </row>
     <row r="7">
@@ -2409,13 +2430,13 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>1098</v>
+        <v>1022</v>
       </c>
       <c r="C7" s="2" t="n">
-        <v>0.8807</v>
+        <v>0.8757</v>
       </c>
       <c r="D7" s="2" t="n">
-        <v>0.9949</v>
+        <v>0.9958</v>
       </c>
     </row>
     <row r="8">
@@ -2425,13 +2446,13 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>932</v>
+        <v>844</v>
       </c>
       <c r="C8" s="2" t="n">
-        <v>0.8873</v>
+        <v>0.8885999999999999</v>
       </c>
       <c r="D8" s="2" t="n">
-        <v>0.9891</v>
+        <v>0.9895</v>
       </c>
     </row>
     <row r="9">
@@ -2441,13 +2462,13 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>1101</v>
+        <v>1046</v>
       </c>
       <c r="C9" s="2" t="n">
-        <v>0.8574000000000001</v>
+        <v>0.8604000000000001</v>
       </c>
       <c r="D9" s="2" t="n">
-        <v>0.9955000000000001</v>
+        <v>0.9958</v>
       </c>
     </row>
     <row r="10">
@@ -2457,13 +2478,13 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>1087</v>
+        <v>1040</v>
       </c>
       <c r="C10" s="2" t="n">
-        <v>0.874</v>
+        <v>0.8712</v>
       </c>
       <c r="D10" s="2" t="n">
-        <v>0.9965000000000001</v>
+        <v>0.9971</v>
       </c>
     </row>
     <row r="11">
@@ -2473,13 +2494,13 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>1055</v>
+        <v>971</v>
       </c>
       <c r="C11" s="2" t="n">
-        <v>0.8882</v>
+        <v>0.895</v>
       </c>
       <c r="D11" s="2" t="n">
-        <v>0.9942</v>
+        <v>0.9947</v>
       </c>
     </row>
     <row r="12">
@@ -2489,13 +2510,13 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>1048</v>
+        <v>990</v>
       </c>
       <c r="C12" s="2" t="n">
-        <v>0.8855</v>
+        <v>0.8838</v>
       </c>
       <c r="D12" s="2" t="n">
-        <v>0.994</v>
+        <v>0.9928</v>
       </c>
     </row>
     <row r="13">
@@ -2505,13 +2526,13 @@
         </is>
       </c>
       <c r="B13" t="n">
-        <v>1079</v>
+        <v>941</v>
       </c>
       <c r="C13" s="2" t="n">
-        <v>0.8999</v>
+        <v>0.9182</v>
       </c>
       <c r="D13" s="2" t="n">
-        <v>0.9833</v>
+        <v>0.9801</v>
       </c>
     </row>
     <row r="14">
@@ -2521,13 +2542,13 @@
         </is>
       </c>
       <c r="B14" t="n">
-        <v>1059</v>
+        <v>969</v>
       </c>
       <c r="C14" s="2" t="n">
-        <v>0.8867</v>
+        <v>0.8895999999999999</v>
       </c>
       <c r="D14" s="2" t="n">
-        <v>0.9935</v>
+        <v>0.9926</v>
       </c>
     </row>
     <row r="15">
@@ -2537,13 +2558,13 @@
         </is>
       </c>
       <c r="B15" t="n">
-        <v>1069</v>
+        <v>1014</v>
       </c>
       <c r="C15" s="2" t="n">
-        <v>0.87</v>
+        <v>0.8826000000000001</v>
       </c>
       <c r="D15" s="2" t="n">
-        <v>0.9929</v>
+        <v>0.9937</v>
       </c>
     </row>
     <row r="16">
@@ -2553,13 +2574,13 @@
         </is>
       </c>
       <c r="B16" t="n">
-        <v>1104</v>
+        <v>1061</v>
       </c>
       <c r="C16" s="2" t="n">
-        <v>0.8958</v>
+        <v>0.8935</v>
       </c>
       <c r="D16" s="2" t="n">
-        <v>0.9952</v>
+        <v>0.9946</v>
       </c>
     </row>
     <row r="17">
@@ -2569,13 +2590,13 @@
         </is>
       </c>
       <c r="B17" t="n">
-        <v>1067</v>
+        <v>1003</v>
       </c>
       <c r="C17" s="2" t="n">
-        <v>0.881</v>
+        <v>0.8774</v>
       </c>
       <c r="D17" s="2" t="n">
-        <v>0.9948</v>
+        <v>0.9945000000000001</v>
       </c>
     </row>
     <row r="18">
@@ -2585,13 +2606,13 @@
         </is>
       </c>
       <c r="B18" t="n">
-        <v>1130</v>
+        <v>1094</v>
       </c>
       <c r="C18" s="2" t="n">
-        <v>0.8646</v>
+        <v>0.8656</v>
       </c>
       <c r="D18" s="2" t="n">
-        <v>0.9964</v>
+        <v>0.9962</v>
       </c>
     </row>
     <row r="19">
@@ -2601,13 +2622,13 @@
         </is>
       </c>
       <c r="B19" t="n">
-        <v>1080</v>
+        <v>996</v>
       </c>
       <c r="C19" s="2" t="n">
-        <v>0.8722</v>
+        <v>0.8655</v>
       </c>
       <c r="D19" s="2" t="n">
-        <v>0.9953</v>
+        <v>0.9959</v>
       </c>
     </row>
     <row r="20">
@@ -2617,13 +2638,13 @@
         </is>
       </c>
       <c r="B20" t="n">
-        <v>975</v>
+        <v>931</v>
       </c>
       <c r="C20" s="2" t="n">
-        <v>0.8554</v>
+        <v>0.8507</v>
       </c>
       <c r="D20" s="2" t="n">
-        <v>0.9962</v>
+        <v>0.997</v>
       </c>
     </row>
     <row r="21">
@@ -2633,13 +2654,13 @@
         </is>
       </c>
       <c r="B21" t="n">
-        <v>975</v>
+        <v>918</v>
       </c>
       <c r="C21" s="2" t="n">
-        <v>0.8554</v>
+        <v>0.8529</v>
       </c>
       <c r="D21" s="2" t="n">
-        <v>0.9942</v>
+        <v>0.9947</v>
       </c>
     </row>
     <row r="22">
@@ -2649,13 +2670,13 @@
         </is>
       </c>
       <c r="B22" t="n">
-        <v>1116</v>
+        <v>1051</v>
       </c>
       <c r="C22" s="2" t="n">
-        <v>0.8602</v>
+        <v>0.8554</v>
       </c>
       <c r="D22" s="2" t="n">
-        <v>0.9949</v>
+        <v>0.9959</v>
       </c>
     </row>
     <row r="23">
@@ -2665,13 +2686,13 @@
         </is>
       </c>
       <c r="B23" t="n">
-        <v>1063</v>
+        <v>985</v>
       </c>
       <c r="C23" s="2" t="n">
-        <v>0.9087</v>
+        <v>0.9107</v>
       </c>
       <c r="D23" s="2" t="n">
-        <v>0.9883999999999999</v>
+        <v>0.9887</v>
       </c>
     </row>
     <row r="24">
@@ -2681,13 +2702,13 @@
         </is>
       </c>
       <c r="B24" t="n">
-        <v>1004</v>
+        <v>870</v>
       </c>
       <c r="C24" s="2" t="n">
-        <v>0.8835</v>
+        <v>0.8724</v>
       </c>
       <c r="D24" s="2" t="n">
-        <v>0.9885</v>
+        <v>0.991</v>
       </c>
     </row>
     <row r="25">
@@ -2697,13 +2718,13 @@
         </is>
       </c>
       <c r="B25" t="n">
-        <v>1084</v>
+        <v>1056</v>
       </c>
       <c r="C25" s="2" t="n">
-        <v>0.9327</v>
+        <v>0.9413</v>
       </c>
       <c r="D25" s="2" t="n">
-        <v>0.9923999999999999</v>
+        <v>0.9923</v>
       </c>
     </row>
     <row r="26">
@@ -2713,13 +2734,13 @@
         </is>
       </c>
       <c r="B26" t="n">
-        <v>908</v>
+        <v>851</v>
       </c>
       <c r="C26" s="2" t="n">
-        <v>0.8965</v>
+        <v>0.8919</v>
       </c>
       <c r="D26" s="2" t="n">
-        <v>0.9903</v>
+        <v>0.986</v>
       </c>
     </row>
     <row r="27">
@@ -2729,13 +2750,13 @@
         </is>
       </c>
       <c r="B27" t="n">
-        <v>1034</v>
+        <v>920</v>
       </c>
       <c r="C27" s="2" t="n">
-        <v>0.9167999999999999</v>
+        <v>0.9174</v>
       </c>
       <c r="D27" s="2" t="n">
-        <v>0.9851</v>
+        <v>0.9867</v>
       </c>
     </row>
     <row r="28">
@@ -2745,13 +2766,13 @@
         </is>
       </c>
       <c r="B28" t="n">
-        <v>1019</v>
+        <v>876</v>
       </c>
       <c r="C28" s="2" t="n">
-        <v>0.9107</v>
+        <v>0.9041</v>
       </c>
       <c r="D28" s="2" t="n">
-        <v>0.9862</v>
+        <v>0.9855</v>
       </c>
     </row>
     <row r="29">
@@ -2761,13 +2782,13 @@
         </is>
       </c>
       <c r="B29" t="n">
-        <v>919</v>
+        <v>877</v>
       </c>
       <c r="C29" s="2" t="n">
-        <v>0.9032</v>
+        <v>0.9065</v>
       </c>
       <c r="D29" s="2" t="n">
-        <v>0.9927</v>
+        <v>0.992</v>
       </c>
     </row>
     <row r="30">
@@ -2777,13 +2798,13 @@
         </is>
       </c>
       <c r="B30" t="n">
-        <v>1049</v>
+        <v>963</v>
       </c>
       <c r="C30" s="2" t="n">
-        <v>0.8885</v>
+        <v>0.8879</v>
       </c>
       <c r="D30" s="2" t="n">
-        <v>0.9909</v>
+        <v>0.9912</v>
       </c>
     </row>
     <row r="31">
@@ -2793,13 +2814,13 @@
         </is>
       </c>
       <c r="B31" t="n">
-        <v>1084</v>
+        <v>1011</v>
       </c>
       <c r="C31" s="2" t="n">
-        <v>0.8828</v>
+        <v>0.8773</v>
       </c>
       <c r="D31" s="2" t="n">
-        <v>0.9916</v>
+        <v>0.9921</v>
       </c>
     </row>
     <row r="32">
@@ -2809,13 +2830,13 @@
         </is>
       </c>
       <c r="B32" t="n">
-        <v>1063</v>
+        <v>936</v>
       </c>
       <c r="C32" s="2" t="n">
-        <v>0.8871</v>
+        <v>0.89</v>
       </c>
       <c r="D32" s="2" t="n">
-        <v>0.9892</v>
+        <v>0.9883</v>
       </c>
     </row>
     <row r="33">
@@ -2825,13 +2846,13 @@
         </is>
       </c>
       <c r="B33" t="n">
-        <v>860</v>
+        <v>733</v>
       </c>
       <c r="C33" s="2" t="n">
-        <v>0.9023</v>
+        <v>0.8922</v>
       </c>
       <c r="D33" s="2" t="n">
-        <v>0.988</v>
+        <v>0.9912</v>
       </c>
     </row>
     <row r="34">
@@ -2841,13 +2862,13 @@
         </is>
       </c>
       <c r="B34" t="n">
-        <v>1018</v>
+        <v>943</v>
       </c>
       <c r="C34" s="2" t="n">
-        <v>0.9263</v>
+        <v>0.9236</v>
       </c>
       <c r="D34" s="2" t="n">
-        <v>0.9905</v>
+        <v>0.9903</v>
       </c>
     </row>
     <row r="35">
@@ -2857,13 +2878,13 @@
         </is>
       </c>
       <c r="B35" t="n">
-        <v>1085</v>
+        <v>998</v>
       </c>
       <c r="C35" s="2" t="n">
-        <v>0.8728</v>
+        <v>0.8717</v>
       </c>
       <c r="D35" s="2" t="n">
-        <v>0.9937</v>
+        <v>0.9943</v>
       </c>
     </row>
     <row r="36">
@@ -2873,13 +2894,13 @@
         </is>
       </c>
       <c r="B36" t="n">
-        <v>875</v>
+        <v>793</v>
       </c>
       <c r="C36" s="2" t="n">
-        <v>0.9029</v>
+        <v>0.9142</v>
       </c>
       <c r="D36" s="2" t="n">
-        <v>0.9897</v>
+        <v>0.9861</v>
       </c>
     </row>
     <row r="37">
@@ -2889,13 +2910,13 @@
         </is>
       </c>
       <c r="B37" t="n">
-        <v>956</v>
+        <v>934</v>
       </c>
       <c r="C37" s="2" t="n">
-        <v>0.9079</v>
+        <v>0.9111</v>
       </c>
       <c r="D37" s="2" t="n">
-        <v>0.9919</v>
+        <v>0.9905</v>
       </c>
     </row>
     <row r="38">
@@ -2905,13 +2926,13 @@
         </is>
       </c>
       <c r="B38" t="n">
-        <v>927</v>
+        <v>836</v>
       </c>
       <c r="C38" s="2" t="n">
-        <v>0.8943</v>
+        <v>0.89</v>
       </c>
       <c r="D38" s="2" t="n">
-        <v>0.9903999999999999</v>
+        <v>0.9927</v>
       </c>
     </row>
     <row r="39">
@@ -2921,13 +2942,13 @@
         </is>
       </c>
       <c r="B39" t="n">
-        <v>1100</v>
+        <v>1020</v>
       </c>
       <c r="C39" s="2" t="n">
-        <v>0.8955</v>
+        <v>0.9098000000000001</v>
       </c>
       <c r="D39" s="2" t="n">
-        <v>0.9882</v>
+        <v>0.9887</v>
       </c>
     </row>
     <row r="40">
@@ -2937,13 +2958,13 @@
         </is>
       </c>
       <c r="B40" t="n">
-        <v>910</v>
+        <v>807</v>
       </c>
       <c r="C40" s="2" t="n">
-        <v>0.8769</v>
+        <v>0.8823</v>
       </c>
       <c r="D40" s="2" t="n">
-        <v>0.9918</v>
+        <v>0.9915</v>
       </c>
     </row>
   </sheetData>
@@ -3007,16 +3028,16 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>0.1307</v>
+        <v>0.129</v>
       </c>
       <c r="C2" t="n">
-        <v>0.1307</v>
+        <v>0.1191</v>
       </c>
       <c r="D2" t="n">
-        <v>0.0044</v>
+        <v>-0.0014</v>
       </c>
       <c r="E2" t="n">
-        <v>1.0393</v>
+        <v>1.0442</v>
       </c>
       <c r="F2" t="n">
         <v>0.0746</v>
@@ -3029,16 +3050,16 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>0.1266</v>
+        <v>0.1256</v>
       </c>
       <c r="C3" t="n">
-        <v>0.1266</v>
+        <v>0.1256</v>
       </c>
       <c r="D3" t="n">
-        <v>-0.008200000000000001</v>
+        <v>-0.0075</v>
       </c>
       <c r="E3" t="n">
-        <v>1.0573</v>
+        <v>1.0607</v>
       </c>
       <c r="F3" t="n">
         <v>0.08160000000000001</v>
@@ -3051,19 +3072,19 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>0.0501</v>
+        <v>0.0499</v>
       </c>
       <c r="C4" t="n">
-        <v>0.0447</v>
+        <v>0.0446</v>
       </c>
       <c r="D4" t="n">
-        <v>0.0901</v>
+        <v>0.09130000000000001</v>
       </c>
       <c r="E4" t="n">
-        <v>1.013</v>
+        <v>1.0138</v>
       </c>
       <c r="F4" t="n">
-        <v>0.06320000000000001</v>
+        <v>0.0631</v>
       </c>
     </row>
   </sheetData>
@@ -3092,7 +3113,7 @@
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>2026-08-04T09:15:09+00:00</t>
+          <t>2026-08-07T09:13:57+00:00</t>
         </is>
       </c>
     </row>
@@ -3103,7 +3124,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>4154</v>
+        <v>4271</v>
       </c>
     </row>
     <row r="3">
@@ -3113,7 +3134,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>107</v>
+        <v>110</v>
       </c>
     </row>
     <row r="4">
@@ -3143,7 +3164,7 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>198</v>
+        <v>206</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Arquiva dados, recalibra e atualiza docs (2026-08-10)
</commit_message>
<xml_diff>
--- a/backtest_results/resultados_backtest.xlsx
+++ b/backtest_results/resultados_backtest.xlsx
@@ -516,28 +516,28 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>821</v>
+        <v>450</v>
       </c>
       <c r="C2" s="2" t="n">
-        <v>0.8343483556638246</v>
+        <v>0.8733333333333333</v>
       </c>
       <c r="D2" s="3" t="n">
-        <v>8.623489648769622</v>
+        <v>6.744648574982978</v>
       </c>
       <c r="E2" s="4" t="n">
-        <v>203.998157814339</v>
+        <v>135.9557172833742</v>
       </c>
       <c r="F2" s="2" t="n">
-        <v>3.264794083041586</v>
+        <v>2.684586107663417</v>
       </c>
       <c r="G2" s="2" t="n">
-        <v>0.3062760852327849</v>
+        <v>0.317247950343665</v>
       </c>
       <c r="H2" t="n">
-        <v>282</v>
+        <v>104</v>
       </c>
       <c r="I2" s="3" t="n">
-        <v>0.7868830694275274</v>
+        <v>0.8069733333333333</v>
       </c>
     </row>
     <row r="3">
@@ -547,28 +547,28 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>1842</v>
+        <v>1880</v>
       </c>
       <c r="C3" s="2" t="n">
-        <v>0.993485342019544</v>
+        <v>0.9930851063829788</v>
       </c>
       <c r="D3" s="3" t="n">
-        <v>2.039545780096339</v>
+        <v>2.048300104592252</v>
       </c>
       <c r="E3" s="4" t="n">
-        <v>2.972702866171187</v>
+        <v>2.977331809451109</v>
       </c>
       <c r="F3" s="2" t="n">
-        <v>0.3459884050303508</v>
+        <v>0.3359642656289785</v>
       </c>
       <c r="G3" s="2" t="n">
-        <v>0.08704657533117932</v>
+        <v>0.08704657533117899</v>
       </c>
       <c r="H3" t="n">
-        <v>38</v>
+        <v>41</v>
       </c>
       <c r="I3" s="3" t="n">
-        <v>0.9857266558089034</v>
+        <v>0.9857095744680852</v>
       </c>
     </row>
     <row r="4">
@@ -578,28 +578,28 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>1334</v>
+        <v>1361</v>
       </c>
       <c r="C4" s="2" t="n">
-        <v>0.9947526236881559</v>
+        <v>0.9948567229977957</v>
       </c>
       <c r="D4" s="3" t="n">
-        <v>1.427600857501266</v>
+        <v>1.451175947349657</v>
       </c>
       <c r="E4" s="4" t="n">
-        <v>2.454745913306565</v>
+        <v>2.48951910355694</v>
       </c>
       <c r="F4" s="2" t="n">
-        <v>0.2775132745381776</v>
+        <v>0.2739823091529194</v>
       </c>
       <c r="G4" s="2" t="n">
         <v>0.08016721391959114</v>
       </c>
       <c r="H4" t="n">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="I4" s="3" t="n">
-        <v>0.9866221889055472</v>
+        <v>0.9865907421013961</v>
       </c>
     </row>
     <row r="5">
@@ -609,19 +609,19 @@
         </is>
       </c>
       <c r="B5" s="5" t="n">
-        <v>708</v>
+        <v>726</v>
       </c>
       <c r="C5" s="6" t="n">
-        <v>0.998587570621469</v>
+        <v>0.9986225895316805</v>
       </c>
       <c r="D5" s="7" t="n">
-        <v>0.8151447231923521</v>
+        <v>0.8410733032525365</v>
       </c>
       <c r="E5" s="8" t="n">
-        <v>1.880308522123886</v>
+        <v>1.922289010908064</v>
       </c>
       <c r="F5" s="6" t="n">
-        <v>0.1879270139333116</v>
+        <v>0.1894606875452871</v>
       </c>
       <c r="G5" s="6" t="n">
         <v>0.02619857308701179</v>
@@ -630,7 +630,7 @@
         <v>6</v>
       </c>
       <c r="I5" s="7" t="n">
-        <v>0.987305790960452</v>
+        <v>0.9872699724517907</v>
       </c>
     </row>
     <row r="6">
@@ -640,34 +640,34 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>1529</v>
+        <v>1176</v>
       </c>
       <c r="C6" s="2" t="n">
-        <v>0.9103989535644212</v>
+        <v>0.9506802721088435</v>
       </c>
       <c r="D6" s="3" t="n">
-        <v>9.438634371961975</v>
+        <v>7.585721878235514</v>
       </c>
       <c r="E6" s="4" t="n">
-        <v>211.2632753252152</v>
+        <v>139.5288597750242</v>
       </c>
       <c r="F6" s="2" t="n">
-        <v>3.30569151737011</v>
+        <v>2.710050618573619</v>
       </c>
       <c r="G6" s="2" t="n">
-        <v>0.2892693823308587</v>
+        <v>0.3007452058777901</v>
       </c>
       <c r="H6" t="n">
-        <v>288</v>
+        <v>110</v>
       </c>
       <c r="I6" s="3" t="n">
-        <v>0.8796883584041857</v>
+        <v>0.9182789115646258</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Atualizado em 2026-08-07T09:13:57+00:00 · arquivo de 4271 dias-cidade (~110 dias corridos) · 39 cidades</t>
+          <t>Atualizado em 2026-08-10T09:12:06+00:00 · arquivo de 4388 dias-cidade (~113 dias corridos) · 39 cidades</t>
         </is>
       </c>
     </row>
@@ -738,13 +738,13 @@
         </is>
       </c>
       <c r="C2" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="D2" s="2" t="n">
-        <v>0.6</v>
+        <v>0.5</v>
       </c>
       <c r="E2" s="3" t="n">
-        <v>-0.075</v>
+        <v>-0.03</v>
       </c>
     </row>
     <row r="3">
@@ -759,13 +759,13 @@
         </is>
       </c>
       <c r="C3" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="D3" s="2" t="n">
         <v>1</v>
       </c>
       <c r="E3" s="3" t="n">
-        <v>0.02871345493600883</v>
+        <v>0.02250133372388761</v>
       </c>
     </row>
     <row r="4">
@@ -780,13 +780,13 @@
         </is>
       </c>
       <c r="C4" t="n">
-        <v>12</v>
+        <v>6</v>
       </c>
       <c r="D4" s="2" t="n">
-        <v>1</v>
+        <v>0.8333333333333334</v>
       </c>
       <c r="E4" s="3" t="n">
-        <v>0.06441588010448063</v>
+        <v>0.07431891929977413</v>
       </c>
     </row>
     <row r="5">
@@ -801,13 +801,13 @@
         </is>
       </c>
       <c r="C5" t="n">
-        <v>11</v>
+        <v>8</v>
       </c>
       <c r="D5" s="2" t="n">
-        <v>0.9090909090909091</v>
+        <v>0.75</v>
       </c>
       <c r="E5" s="3" t="n">
-        <v>0.09590495395641901</v>
+        <v>-0.06526472273082738</v>
       </c>
     </row>
     <row r="6">
@@ -822,13 +822,13 @@
         </is>
       </c>
       <c r="C6" t="n">
-        <v>24</v>
+        <v>11</v>
       </c>
       <c r="D6" s="2" t="n">
-        <v>0.9166666666666666</v>
+        <v>0.9090909090909091</v>
       </c>
       <c r="E6" s="3" t="n">
-        <v>0.1189455334703077</v>
+        <v>-0.01281695079576209</v>
       </c>
     </row>
     <row r="7">
@@ -849,7 +849,7 @@
         <v>0.8</v>
       </c>
       <c r="E7" s="3" t="n">
-        <v>0.1431748022405707</v>
+        <v>0.1406418288239204</v>
       </c>
     </row>
     <row r="8">
@@ -864,13 +864,13 @@
         </is>
       </c>
       <c r="C8" t="n">
-        <v>22</v>
+        <v>9</v>
       </c>
       <c r="D8" s="2" t="n">
-        <v>0.7727272727272727</v>
+        <v>0.6666666666666666</v>
       </c>
       <c r="E8" s="3" t="n">
-        <v>0.04730632556038945</v>
+        <v>-0.01506240674211111</v>
       </c>
     </row>
     <row r="9">
@@ -885,13 +885,13 @@
         </is>
       </c>
       <c r="C9" t="n">
-        <v>9</v>
+        <v>3</v>
       </c>
       <c r="D9" s="2" t="n">
-        <v>0.8888888888888888</v>
+        <v>0.6666666666666666</v>
       </c>
       <c r="E9" s="3" t="n">
-        <v>0.1222862539916138</v>
+        <v>0.1294782168186424</v>
       </c>
     </row>
     <row r="10">
@@ -927,13 +927,13 @@
         </is>
       </c>
       <c r="C11" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="D11" s="2" t="n">
-        <v>0.75</v>
+        <v>1</v>
       </c>
       <c r="E11" s="3" t="n">
-        <v>0.003303880299478271</v>
+        <v>0.00610079575596818</v>
       </c>
     </row>
     <row r="12">
@@ -948,13 +948,13 @@
         </is>
       </c>
       <c r="C12" t="n">
-        <v>11</v>
+        <v>6</v>
       </c>
       <c r="D12" s="2" t="n">
-        <v>0.4545454545454545</v>
+        <v>0.3333333333333333</v>
       </c>
       <c r="E12" s="3" t="n">
-        <v>-0.003623464044489731</v>
+        <v>-0.03415492957746477</v>
       </c>
     </row>
     <row r="13">
@@ -969,13 +969,13 @@
         </is>
       </c>
       <c r="C13" t="n">
-        <v>89</v>
+        <v>21</v>
       </c>
       <c r="D13" s="2" t="n">
-        <v>0.651685393258427</v>
+        <v>0.8571428571428571</v>
       </c>
       <c r="E13" s="3" t="n">
-        <v>0.4118047128216701</v>
+        <v>0.4579984840521444</v>
       </c>
     </row>
     <row r="14">
@@ -990,13 +990,13 @@
         </is>
       </c>
       <c r="C14" t="n">
-        <v>9</v>
+        <v>3</v>
       </c>
       <c r="D14" s="2" t="n">
-        <v>0.8888888888888888</v>
+        <v>0.6666666666666666</v>
       </c>
       <c r="E14" s="3" t="n">
-        <v>0.257403181763825</v>
+        <v>0.05099887572722163</v>
       </c>
     </row>
     <row r="15">
@@ -1011,13 +1011,13 @@
         </is>
       </c>
       <c r="C15" t="n">
-        <v>12</v>
+        <v>8</v>
       </c>
       <c r="D15" s="2" t="n">
-        <v>0.8333333333333334</v>
+        <v>0.75</v>
       </c>
       <c r="E15" s="3" t="n">
-        <v>0.1291037681685989</v>
+        <v>0.04707558652443192</v>
       </c>
     </row>
     <row r="16">
@@ -1032,13 +1032,13 @@
         </is>
       </c>
       <c r="C16" t="n">
-        <v>12</v>
+        <v>4</v>
       </c>
       <c r="D16" s="2" t="n">
-        <v>0.9166666666666666</v>
+        <v>1</v>
       </c>
       <c r="E16" s="3" t="n">
-        <v>0.1541296779626947</v>
+        <v>0.02573492529537737</v>
       </c>
     </row>
     <row r="17">
@@ -1053,13 +1053,13 @@
         </is>
       </c>
       <c r="C17" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="D17" s="2" t="n">
-        <v>0.8571428571428571</v>
+        <v>0.8333333333333334</v>
       </c>
       <c r="E17" s="3" t="n">
-        <v>-0.02618376804770087</v>
+        <v>-0.04666569575854426</v>
       </c>
     </row>
     <row r="18">
@@ -1074,13 +1074,13 @@
         </is>
       </c>
       <c r="C18" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="D18" s="2" t="n">
         <v>1</v>
       </c>
       <c r="E18" s="3" t="n">
-        <v>0.02847840283119394</v>
+        <v>0.01419268854547966</v>
       </c>
     </row>
     <row r="19">
@@ -1095,13 +1095,13 @@
         </is>
       </c>
       <c r="C19" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D19" s="2" t="n">
-        <v>0.3333333333333333</v>
+        <v>0</v>
       </c>
       <c r="E19" s="3" t="n">
-        <v>-0.005776397515527935</v>
+        <v>-0.015</v>
       </c>
     </row>
     <row r="20">
@@ -1116,13 +1116,13 @@
         </is>
       </c>
       <c r="C20" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="D20" s="2" t="n">
         <v>1</v>
       </c>
       <c r="E20" s="3" t="n">
-        <v>0.1314966176671566</v>
+        <v>0.02592791823561056</v>
       </c>
     </row>
     <row r="21">
@@ -1137,13 +1137,13 @@
         </is>
       </c>
       <c r="C21" t="n">
-        <v>23</v>
+        <v>10</v>
       </c>
       <c r="D21" s="2" t="n">
-        <v>0.6956521739130435</v>
+        <v>0.5</v>
       </c>
       <c r="E21" s="3" t="n">
-        <v>0.1468422756171502</v>
+        <v>-0.04853875397650686</v>
       </c>
     </row>
     <row r="22">
@@ -1158,13 +1158,13 @@
         </is>
       </c>
       <c r="C22" t="n">
-        <v>9</v>
+        <v>4</v>
       </c>
       <c r="D22" s="2" t="n">
-        <v>0.7777777777777778</v>
+        <v>0.75</v>
       </c>
       <c r="E22" s="3" t="n">
-        <v>0.01592739537784452</v>
+        <v>-0.01709668829975063</v>
       </c>
     </row>
     <row r="23">
@@ -1179,13 +1179,13 @@
         </is>
       </c>
       <c r="C23" t="n">
-        <v>47</v>
+        <v>24</v>
       </c>
       <c r="D23" s="2" t="n">
-        <v>0.7446808510638298</v>
+        <v>0.8333333333333334</v>
       </c>
       <c r="E23" s="3" t="n">
-        <v>0.7074910393505702</v>
+        <v>0.4972467102262322</v>
       </c>
     </row>
     <row r="24">
@@ -1200,13 +1200,13 @@
         </is>
       </c>
       <c r="C24" t="n">
-        <v>44</v>
+        <v>23</v>
       </c>
       <c r="D24" s="2" t="n">
-        <v>0.8636363636363636</v>
+        <v>0.9565217391304348</v>
       </c>
       <c r="E24" s="3" t="n">
-        <v>0.4620145470468817</v>
+        <v>0.2869825159383541</v>
       </c>
     </row>
     <row r="25">
@@ -1221,13 +1221,13 @@
         </is>
       </c>
       <c r="C25" t="n">
-        <v>39</v>
+        <v>24</v>
       </c>
       <c r="D25" s="2" t="n">
-        <v>0.8461538461538461</v>
+        <v>0.8333333333333334</v>
       </c>
       <c r="E25" s="3" t="n">
-        <v>0.4723217210911316</v>
+        <v>0.2363717485679154</v>
       </c>
     </row>
     <row r="26">
@@ -1242,13 +1242,13 @@
         </is>
       </c>
       <c r="C26" t="n">
-        <v>31</v>
+        <v>18</v>
       </c>
       <c r="D26" s="2" t="n">
-        <v>0.9032258064516129</v>
+        <v>0.9444444444444444</v>
       </c>
       <c r="E26" s="3" t="n">
-        <v>0.3159542020951454</v>
+        <v>0.1981192944401984</v>
       </c>
     </row>
     <row r="27">
@@ -1263,13 +1263,13 @@
         </is>
       </c>
       <c r="C27" t="n">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="D27" s="2" t="n">
         <v>1</v>
       </c>
       <c r="E27" s="3" t="n">
-        <v>0.5535944075318887</v>
+        <v>0.8221975485570969</v>
       </c>
     </row>
     <row r="28">
@@ -1284,13 +1284,13 @@
         </is>
       </c>
       <c r="C28" t="n">
-        <v>43</v>
+        <v>32</v>
       </c>
       <c r="D28" s="2" t="n">
-        <v>0.8604651162790697</v>
+        <v>0.90625</v>
       </c>
       <c r="E28" s="3" t="n">
-        <v>1.230616299890604</v>
+        <v>1.281152704143795</v>
       </c>
     </row>
     <row r="29">
@@ -1305,13 +1305,13 @@
         </is>
       </c>
       <c r="C29" t="n">
-        <v>14</v>
+        <v>10</v>
       </c>
       <c r="D29" s="2" t="n">
-        <v>0.8571428571428571</v>
+        <v>0.9</v>
       </c>
       <c r="E29" s="3" t="n">
-        <v>0.1757981420865279</v>
+        <v>0.1572290064307805</v>
       </c>
     </row>
     <row r="30">
@@ -1326,13 +1326,13 @@
         </is>
       </c>
       <c r="C30" t="n">
-        <v>33</v>
+        <v>17</v>
       </c>
       <c r="D30" s="2" t="n">
-        <v>0.8484848484848485</v>
+        <v>1</v>
       </c>
       <c r="E30" s="3" t="n">
-        <v>0.6566306201959523</v>
+        <v>0.3588116893818861</v>
       </c>
     </row>
     <row r="31">
@@ -1347,13 +1347,13 @@
         </is>
       </c>
       <c r="C31" t="n">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="D31" s="2" t="n">
         <v>1</v>
       </c>
       <c r="E31" s="3" t="n">
-        <v>0.05069786628188186</v>
+        <v>0.07820345241955598</v>
       </c>
     </row>
     <row r="32">
@@ -1368,13 +1368,13 @@
         </is>
       </c>
       <c r="C32" t="n">
-        <v>21</v>
+        <v>15</v>
       </c>
       <c r="D32" s="2" t="n">
-        <v>0.9523809523809523</v>
+        <v>0.9333333333333333</v>
       </c>
       <c r="E32" s="3" t="n">
-        <v>0.2046081351060535</v>
+        <v>0.1205477225213461</v>
       </c>
     </row>
     <row r="33">
@@ -1389,13 +1389,13 @@
         </is>
       </c>
       <c r="C33" t="n">
-        <v>12</v>
+        <v>8</v>
       </c>
       <c r="D33" s="2" t="n">
         <v>1</v>
       </c>
       <c r="E33" s="3" t="n">
-        <v>0.1793830553055883</v>
+        <v>0.09340663731887164</v>
       </c>
     </row>
     <row r="34">
@@ -1410,13 +1410,13 @@
         </is>
       </c>
       <c r="C34" t="n">
-        <v>48</v>
+        <v>16</v>
       </c>
       <c r="D34" s="2" t="n">
         <v>0.875</v>
       </c>
       <c r="E34" s="3" t="n">
-        <v>0.159388807587754</v>
+        <v>0.428628714046834</v>
       </c>
     </row>
     <row r="35">
@@ -1431,13 +1431,13 @@
         </is>
       </c>
       <c r="C35" t="n">
-        <v>100</v>
+        <v>74</v>
       </c>
       <c r="D35" s="2" t="n">
-        <v>0.87</v>
+        <v>0.8783783783783784</v>
       </c>
       <c r="E35" s="3" t="n">
-        <v>0.9809992761363049</v>
+        <v>0.8611178896791831</v>
       </c>
     </row>
     <row r="36">
@@ -1452,13 +1452,13 @@
         </is>
       </c>
       <c r="C36" t="n">
-        <v>30</v>
+        <v>17</v>
       </c>
       <c r="D36" s="2" t="n">
-        <v>0.9</v>
+        <v>0.8823529411764706</v>
       </c>
       <c r="E36" s="3" t="n">
-        <v>0.3638157717166314</v>
+        <v>0.3696888882744743</v>
       </c>
     </row>
     <row r="37">
@@ -1473,13 +1473,13 @@
         </is>
       </c>
       <c r="C37" t="n">
-        <v>29</v>
+        <v>12</v>
       </c>
       <c r="D37" s="2" t="n">
-        <v>0.7931034482758621</v>
+        <v>0.9166666666666666</v>
       </c>
       <c r="E37" s="3" t="n">
-        <v>0.2463086036971679</v>
+        <v>0.1393609616271082</v>
       </c>
     </row>
     <row r="38">
@@ -1494,13 +1494,13 @@
         </is>
       </c>
       <c r="C38" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="D38" s="2" t="n">
-        <v>0.8</v>
+        <v>1</v>
       </c>
       <c r="E38" s="3" t="n">
-        <v>-0.005541901348352921</v>
+        <v>0.02445809865164708</v>
       </c>
     </row>
     <row r="39">
@@ -1515,13 +1515,13 @@
         </is>
       </c>
       <c r="C39" t="n">
-        <v>19</v>
+        <v>16</v>
       </c>
       <c r="D39" s="2" t="n">
-        <v>0.8947368421052632</v>
+        <v>0.9375</v>
       </c>
       <c r="E39" s="3" t="n">
-        <v>-0.05227765681712923</v>
+        <v>-0.007277656817129237</v>
       </c>
     </row>
     <row r="40">
@@ -1536,13 +1536,13 @@
         </is>
       </c>
       <c r="C40" t="n">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="D40" s="2" t="n">
-        <v>0.9565217391304348</v>
+        <v>0.9523809523809523</v>
       </c>
       <c r="E40" s="3" t="n">
-        <v>0.03518949680585746</v>
+        <v>0.02897737559373625</v>
       </c>
     </row>
     <row r="41">
@@ -1557,13 +1557,13 @@
         </is>
       </c>
       <c r="C41" t="n">
-        <v>42</v>
+        <v>36</v>
       </c>
       <c r="D41" s="2" t="n">
-        <v>1</v>
+        <v>0.9722222222222222</v>
       </c>
       <c r="E41" s="3" t="n">
-        <v>0.1096210897447621</v>
+        <v>0.1195241289400556</v>
       </c>
     </row>
     <row r="42">
@@ -1578,13 +1578,13 @@
         </is>
       </c>
       <c r="C42" t="n">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="D42" s="2" t="n">
-        <v>0.9714285714285714</v>
+        <v>0.9393939393939394</v>
       </c>
       <c r="E42" s="3" t="n">
-        <v>0.1277354133987263</v>
+        <v>-0.03288122155900778</v>
       </c>
     </row>
     <row r="43">
@@ -1599,13 +1599,13 @@
         </is>
       </c>
       <c r="C43" t="n">
-        <v>72</v>
+        <v>59</v>
       </c>
       <c r="D43" s="2" t="n">
-        <v>0.9722222222222222</v>
+        <v>0.9830508474576272</v>
       </c>
       <c r="E43" s="3" t="n">
-        <v>0.1657834498465466</v>
+        <v>0.03402096558047677</v>
       </c>
     </row>
     <row r="44">
@@ -1626,7 +1626,7 @@
         <v>0.9333333333333333</v>
       </c>
       <c r="E44" s="3" t="n">
-        <v>0.1573199025875285</v>
+        <v>0.1547869291708782</v>
       </c>
     </row>
     <row r="45">
@@ -1641,13 +1641,13 @@
         </is>
       </c>
       <c r="C45" t="n">
-        <v>46</v>
+        <v>33</v>
       </c>
       <c r="D45" s="2" t="n">
-        <v>0.8913043478260869</v>
+        <v>0.9090909090909091</v>
       </c>
       <c r="E45" s="3" t="n">
-        <v>0.08501528518231299</v>
+        <v>0.02264655287981242</v>
       </c>
     </row>
     <row r="46">
@@ -1662,13 +1662,13 @@
         </is>
       </c>
       <c r="C46" t="n">
-        <v>24</v>
+        <v>19</v>
       </c>
       <c r="D46" s="2" t="n">
-        <v>0.9583333333333334</v>
+        <v>0.9473684210526315</v>
       </c>
       <c r="E46" s="3" t="n">
-        <v>0.1361851521629562</v>
+        <v>0.1464698984951394</v>
       </c>
     </row>
     <row r="47">
@@ -1704,13 +1704,13 @@
         </is>
       </c>
       <c r="C48" t="n">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="D48" s="2" t="n">
-        <v>0.875</v>
+        <v>1</v>
       </c>
       <c r="E48" s="3" t="n">
-        <v>0.008130763493806696</v>
+        <v>0.0109276789502966</v>
       </c>
     </row>
     <row r="49">
@@ -1725,13 +1725,13 @@
         </is>
       </c>
       <c r="C49" t="n">
-        <v>18</v>
+        <v>13</v>
       </c>
       <c r="D49" s="2" t="n">
-        <v>0.6666666666666666</v>
+        <v>0.6923076923076923</v>
       </c>
       <c r="E49" s="3" t="n">
-        <v>0.007818013886571476</v>
+        <v>-0.02271345164640357</v>
       </c>
     </row>
     <row r="50">
@@ -1746,13 +1746,13 @@
         </is>
       </c>
       <c r="C50" t="n">
-        <v>99</v>
+        <v>31</v>
       </c>
       <c r="D50" s="2" t="n">
-        <v>0.6868686868686869</v>
+        <v>0.9032258064516129</v>
       </c>
       <c r="E50" s="3" t="n">
-        <v>0.4224461635062853</v>
+        <v>0.4686399347367595</v>
       </c>
     </row>
     <row r="51">
@@ -1767,13 +1767,13 @@
         </is>
       </c>
       <c r="C51" t="n">
-        <v>21</v>
+        <v>15</v>
       </c>
       <c r="D51" s="2" t="n">
-        <v>0.9523809523809523</v>
+        <v>0.9333333333333333</v>
       </c>
       <c r="E51" s="3" t="n">
-        <v>0.2734687582090057</v>
+        <v>0.06706445217240228</v>
       </c>
     </row>
     <row r="52">
@@ -1788,13 +1788,13 @@
         </is>
       </c>
       <c r="C52" t="n">
-        <v>32</v>
+        <v>28</v>
       </c>
       <c r="D52" s="2" t="n">
-        <v>0.9375</v>
+        <v>0.9285714285714286</v>
       </c>
       <c r="E52" s="3" t="n">
-        <v>0.152278290710232</v>
+        <v>0.07025010906606494</v>
       </c>
     </row>
     <row r="53">
@@ -1809,13 +1809,13 @@
         </is>
       </c>
       <c r="C53" t="n">
-        <v>29</v>
+        <v>21</v>
       </c>
       <c r="D53" s="2" t="n">
-        <v>0.9655172413793104</v>
+        <v>1</v>
       </c>
       <c r="E53" s="3" t="n">
-        <v>0.1772191935052958</v>
+        <v>0.04882444083797849</v>
       </c>
     </row>
     <row r="54">
@@ -1830,13 +1830,13 @@
         </is>
       </c>
       <c r="C54" t="n">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="D54" s="2" t="n">
-        <v>0.9583333333333334</v>
+        <v>0.9565217391304348</v>
       </c>
       <c r="E54" s="3" t="n">
-        <v>-0.003079763162308275</v>
+        <v>-0.02356169087315167</v>
       </c>
     </row>
     <row r="55">
@@ -1872,13 +1872,13 @@
         </is>
       </c>
       <c r="C56" t="n">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="D56" s="2" t="n">
         <v>1</v>
       </c>
       <c r="E56" s="3" t="n">
-        <v>0.04893879804517041</v>
+        <v>0.03465308375945613</v>
       </c>
     </row>
     <row r="57">
@@ -1893,13 +1893,13 @@
         </is>
       </c>
       <c r="C57" t="n">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="D57" s="2" t="n">
-        <v>0.7142857142857143</v>
+        <v>0.8</v>
       </c>
       <c r="E57" s="3" t="n">
-        <v>-0.0006613392604692</v>
+        <v>-0.009884941744941264</v>
       </c>
     </row>
     <row r="58">
@@ -1914,13 +1914,13 @@
         </is>
       </c>
       <c r="C58" t="n">
-        <v>13</v>
+        <v>10</v>
       </c>
       <c r="D58" s="2" t="n">
         <v>1</v>
       </c>
       <c r="E58" s="3" t="n">
-        <v>0.1436302293122179</v>
+        <v>0.03806152988067182</v>
       </c>
     </row>
     <row r="59">
@@ -1935,13 +1935,13 @@
         </is>
       </c>
       <c r="C59" t="n">
-        <v>87</v>
+        <v>75</v>
       </c>
       <c r="D59" s="2" t="n">
-        <v>0.9195402298850575</v>
+        <v>0.9333333333333333</v>
       </c>
       <c r="E59" s="3" t="n">
-        <v>0.2258949095037379</v>
+        <v>0.03307798247418333</v>
       </c>
     </row>
     <row r="60">
@@ -1956,13 +1956,13 @@
         </is>
       </c>
       <c r="C60" t="n">
-        <v>23</v>
+        <v>18</v>
       </c>
       <c r="D60" s="2" t="n">
-        <v>0.9130434782608695</v>
+        <v>0.9444444444444444</v>
       </c>
       <c r="E60" s="3" t="n">
-        <v>0.03204785368229767</v>
+        <v>-0.0009762299952974871</v>
       </c>
     </row>
     <row r="61">
@@ -1977,13 +1977,13 @@
         </is>
       </c>
       <c r="C61" t="n">
-        <v>76</v>
+        <v>54</v>
       </c>
       <c r="D61" s="2" t="n">
-        <v>0.8421052631578947</v>
+        <v>0.9259259259259259</v>
       </c>
       <c r="E61" s="3" t="n">
-        <v>0.7299786550687631</v>
+        <v>0.5212571685840192</v>
       </c>
     </row>
     <row r="62">
@@ -1998,13 +1998,13 @@
         </is>
       </c>
       <c r="C62" t="n">
-        <v>50</v>
+        <v>33</v>
       </c>
       <c r="D62" s="2" t="n">
-        <v>0.88</v>
+        <v>0.9696969696969697</v>
       </c>
       <c r="E62" s="3" t="n">
-        <v>0.4681592199264639</v>
+        <v>0.2995551262996995</v>
       </c>
     </row>
     <row r="63">
@@ -2019,13 +2019,13 @@
         </is>
       </c>
       <c r="C63" t="n">
-        <v>68</v>
+        <v>53</v>
       </c>
       <c r="D63" s="2" t="n">
-        <v>0.9117647058823529</v>
+        <v>0.9245283018867925</v>
       </c>
       <c r="E63" s="3" t="n">
-        <v>0.5081767977858931</v>
+        <v>0.2722268252626769</v>
       </c>
     </row>
     <row r="64">
@@ -2040,13 +2040,13 @@
         </is>
       </c>
       <c r="C64" t="n">
-        <v>39</v>
+        <v>26</v>
       </c>
       <c r="D64" s="2" t="n">
-        <v>0.9230769230769231</v>
+        <v>0.9615384615384616</v>
       </c>
       <c r="E64" s="3" t="n">
-        <v>0.3245729882386124</v>
+        <v>0.2067380805836653</v>
       </c>
     </row>
     <row r="65">
@@ -2061,13 +2061,13 @@
         </is>
       </c>
       <c r="C65" t="n">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="D65" s="2" t="n">
         <v>1</v>
       </c>
       <c r="E65" s="3" t="n">
-        <v>0.5538437868737083</v>
+        <v>0.8242657924132389</v>
       </c>
     </row>
     <row r="66">
@@ -2082,13 +2082,13 @@
         </is>
       </c>
       <c r="C66" t="n">
-        <v>66</v>
+        <v>55</v>
       </c>
       <c r="D66" s="2" t="n">
-        <v>0.9090909090909091</v>
+        <v>0.9454545454545454</v>
       </c>
       <c r="E66" s="3" t="n">
-        <v>1.247137546340974</v>
+        <v>1.297673950594165</v>
       </c>
     </row>
     <row r="67">
@@ -2103,13 +2103,13 @@
         </is>
       </c>
       <c r="C67" t="n">
-        <v>46</v>
+        <v>42</v>
       </c>
       <c r="D67" s="2" t="n">
-        <v>0.9565217391304348</v>
+        <v>0.9761904761904762</v>
       </c>
       <c r="E67" s="3" t="n">
-        <v>0.2175828737270852</v>
+        <v>0.1990137380713378</v>
       </c>
     </row>
     <row r="68">
@@ -2124,13 +2124,13 @@
         </is>
       </c>
       <c r="C68" t="n">
-        <v>57</v>
+        <v>41</v>
       </c>
       <c r="D68" s="2" t="n">
-        <v>0.9122807017543859</v>
+        <v>1</v>
       </c>
       <c r="E68" s="3" t="n">
-        <v>0.6869331279378615</v>
+        <v>0.3891141971237955</v>
       </c>
     </row>
     <row r="69">
@@ -2145,13 +2145,13 @@
         </is>
       </c>
       <c r="C69" t="n">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="D69" s="2" t="n">
         <v>1</v>
       </c>
       <c r="E69" s="3" t="n">
-        <v>0.05489257784773297</v>
+        <v>0.083921006625001</v>
       </c>
     </row>
     <row r="70">
@@ -2166,13 +2166,13 @@
         </is>
       </c>
       <c r="C70" t="n">
-        <v>35</v>
+        <v>30</v>
       </c>
       <c r="D70" s="2" t="n">
-        <v>0.9714285714285714</v>
+        <v>0.9666666666666667</v>
       </c>
       <c r="E70" s="3" t="n">
-        <v>0.2160184206750249</v>
+        <v>0.133019150081222</v>
       </c>
     </row>
     <row r="71">
@@ -2187,13 +2187,13 @@
         </is>
       </c>
       <c r="C71" t="n">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="D71" s="2" t="n">
         <v>1</v>
       </c>
       <c r="E71" s="3" t="n">
-        <v>0.189545939944205</v>
+        <v>0.105030430626852</v>
       </c>
     </row>
     <row r="72">
@@ -2208,13 +2208,13 @@
         </is>
       </c>
       <c r="C72" t="n">
-        <v>64</v>
+        <v>35</v>
       </c>
       <c r="D72" s="2" t="n">
-        <v>0.90625</v>
+        <v>0.9428571428571428</v>
       </c>
       <c r="E72" s="3" t="n">
-        <v>0.1818619914153925</v>
+        <v>0.4558937776199615</v>
       </c>
     </row>
     <row r="73">
@@ -2229,13 +2229,13 @@
         </is>
       </c>
       <c r="C73" t="n">
-        <v>152</v>
+        <v>126</v>
       </c>
       <c r="D73" s="2" t="n">
-        <v>0.9144736842105263</v>
+        <v>0.9285714285714286</v>
       </c>
       <c r="E73" s="3" t="n">
-        <v>1.048598493280787</v>
+        <v>0.9287171068236656</v>
       </c>
     </row>
     <row r="74">
@@ -2250,13 +2250,13 @@
         </is>
       </c>
       <c r="C74" t="n">
-        <v>62</v>
+        <v>50</v>
       </c>
       <c r="D74" s="2" t="n">
-        <v>0.9516129032258065</v>
+        <v>0.96</v>
       </c>
       <c r="E74" s="3" t="n">
-        <v>0.4063153976002876</v>
+        <v>0.4133007487385147</v>
       </c>
     </row>
     <row r="75">
@@ -2271,13 +2271,13 @@
         </is>
       </c>
       <c r="C75" t="n">
-        <v>48</v>
+        <v>31</v>
       </c>
       <c r="D75" s="2" t="n">
-        <v>0.875</v>
+        <v>0.967741935483871</v>
       </c>
       <c r="E75" s="3" t="n">
-        <v>0.2682025443647241</v>
+        <v>0.1612549022946645</v>
       </c>
     </row>
     <row r="76">
@@ -2292,13 +2292,13 @@
         </is>
       </c>
       <c r="C76" t="n">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="D76" s="2" t="n">
-        <v>0.8571428571428571</v>
+        <v>1</v>
       </c>
       <c r="E76" s="3" t="n">
-        <v>-0.002634714275954223</v>
+        <v>0.02736528572404578</v>
       </c>
     </row>
   </sheetData>
@@ -2350,13 +2350,13 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>895</v>
+        <v>891</v>
       </c>
       <c r="C2" s="2" t="n">
-        <v>0.8816000000000001</v>
+        <v>0.8833</v>
       </c>
       <c r="D2" s="2" t="n">
-        <v>0.9916</v>
+        <v>0.9923999999999999</v>
       </c>
     </row>
     <row r="3">
@@ -2366,10 +2366,10 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>952</v>
+        <v>962</v>
       </c>
       <c r="C3" s="2" t="n">
-        <v>0.8519</v>
+        <v>0.8534</v>
       </c>
       <c r="D3" s="2" t="n">
         <v>0.9969</v>
@@ -2382,13 +2382,13 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>895</v>
+        <v>901</v>
       </c>
       <c r="C4" s="2" t="n">
-        <v>0.8793</v>
+        <v>0.8801</v>
       </c>
       <c r="D4" s="2" t="n">
-        <v>0.9931</v>
+        <v>0.9933999999999999</v>
       </c>
     </row>
     <row r="5">
@@ -2398,13 +2398,13 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>982</v>
+        <v>991</v>
       </c>
       <c r="C5" s="2" t="n">
-        <v>0.8768</v>
+        <v>0.8789</v>
       </c>
       <c r="D5" s="2" t="n">
-        <v>0.9939</v>
+        <v>0.994</v>
       </c>
     </row>
     <row r="6">
@@ -2414,13 +2414,13 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>1068</v>
+        <v>1075</v>
       </c>
       <c r="C6" s="2" t="n">
-        <v>0.8904</v>
+        <v>0.8884</v>
       </c>
       <c r="D6" s="2" t="n">
-        <v>0.9928</v>
+        <v>0.9929</v>
       </c>
     </row>
     <row r="7">
@@ -2430,13 +2430,13 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>1022</v>
+        <v>1039</v>
       </c>
       <c r="C7" s="2" t="n">
-        <v>0.8757</v>
+        <v>0.8778</v>
       </c>
       <c r="D7" s="2" t="n">
-        <v>0.9958</v>
+        <v>0.9957</v>
       </c>
     </row>
     <row r="8">
@@ -2446,13 +2446,13 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>844</v>
+        <v>837</v>
       </c>
       <c r="C8" s="2" t="n">
-        <v>0.8885999999999999</v>
+        <v>0.8913</v>
       </c>
       <c r="D8" s="2" t="n">
-        <v>0.9895</v>
+        <v>0.9917</v>
       </c>
     </row>
     <row r="9">
@@ -2462,13 +2462,13 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>1046</v>
+        <v>1057</v>
       </c>
       <c r="C9" s="2" t="n">
-        <v>0.8604000000000001</v>
+        <v>0.8628</v>
       </c>
       <c r="D9" s="2" t="n">
-        <v>0.9958</v>
+        <v>0.9955000000000001</v>
       </c>
     </row>
     <row r="10">
@@ -2478,13 +2478,13 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>1040</v>
+        <v>1060</v>
       </c>
       <c r="C10" s="2" t="n">
-        <v>0.8712</v>
+        <v>0.8736</v>
       </c>
       <c r="D10" s="2" t="n">
-        <v>0.9971</v>
+        <v>0.9969</v>
       </c>
     </row>
     <row r="11">
@@ -2494,13 +2494,13 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>971</v>
+        <v>980</v>
       </c>
       <c r="C11" s="2" t="n">
-        <v>0.895</v>
+        <v>0.898</v>
       </c>
       <c r="D11" s="2" t="n">
-        <v>0.9947</v>
+        <v>0.9946</v>
       </c>
     </row>
     <row r="12">
@@ -2510,13 +2510,13 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>990</v>
+        <v>997</v>
       </c>
       <c r="C12" s="2" t="n">
-        <v>0.8838</v>
+        <v>0.8917</v>
       </c>
       <c r="D12" s="2" t="n">
-        <v>0.9928</v>
+        <v>0.9936</v>
       </c>
     </row>
     <row r="13">
@@ -2526,13 +2526,13 @@
         </is>
       </c>
       <c r="B13" t="n">
-        <v>941</v>
+        <v>915</v>
       </c>
       <c r="C13" s="2" t="n">
-        <v>0.9182</v>
+        <v>0.9486</v>
       </c>
       <c r="D13" s="2" t="n">
-        <v>0.9801</v>
+        <v>0.9843</v>
       </c>
     </row>
     <row r="14">
@@ -2542,13 +2542,13 @@
         </is>
       </c>
       <c r="B14" t="n">
-        <v>969</v>
+        <v>978</v>
       </c>
       <c r="C14" s="2" t="n">
-        <v>0.8895999999999999</v>
+        <v>0.8885</v>
       </c>
       <c r="D14" s="2" t="n">
-        <v>0.9926</v>
+        <v>0.9928</v>
       </c>
     </row>
     <row r="15">
@@ -2558,13 +2558,13 @@
         </is>
       </c>
       <c r="B15" t="n">
-        <v>1014</v>
+        <v>1025</v>
       </c>
       <c r="C15" s="2" t="n">
-        <v>0.8826000000000001</v>
+        <v>0.8849</v>
       </c>
       <c r="D15" s="2" t="n">
-        <v>0.9937</v>
+        <v>0.9942</v>
       </c>
     </row>
     <row r="16">
@@ -2574,13 +2574,13 @@
         </is>
       </c>
       <c r="B16" t="n">
-        <v>1061</v>
+        <v>1072</v>
       </c>
       <c r="C16" s="2" t="n">
-        <v>0.8935</v>
+        <v>0.8965</v>
       </c>
       <c r="D16" s="2" t="n">
-        <v>0.9946</v>
+        <v>0.9948</v>
       </c>
     </row>
     <row r="17">
@@ -2590,10 +2590,10 @@
         </is>
       </c>
       <c r="B17" t="n">
-        <v>1003</v>
+        <v>1013</v>
       </c>
       <c r="C17" s="2" t="n">
-        <v>0.8774</v>
+        <v>0.8806</v>
       </c>
       <c r="D17" s="2" t="n">
         <v>0.9945000000000001</v>
@@ -2606,13 +2606,13 @@
         </is>
       </c>
       <c r="B18" t="n">
-        <v>1094</v>
+        <v>1113</v>
       </c>
       <c r="C18" s="2" t="n">
-        <v>0.8656</v>
+        <v>0.8688</v>
       </c>
       <c r="D18" s="2" t="n">
-        <v>0.9962</v>
+        <v>0.9963</v>
       </c>
     </row>
     <row r="19">
@@ -2622,13 +2622,13 @@
         </is>
       </c>
       <c r="B19" t="n">
-        <v>996</v>
+        <v>1010</v>
       </c>
       <c r="C19" s="2" t="n">
-        <v>0.8655</v>
+        <v>0.8673</v>
       </c>
       <c r="D19" s="2" t="n">
-        <v>0.9959</v>
+        <v>0.9956</v>
       </c>
     </row>
     <row r="20">
@@ -2638,10 +2638,10 @@
         </is>
       </c>
       <c r="B20" t="n">
-        <v>931</v>
+        <v>936</v>
       </c>
       <c r="C20" s="2" t="n">
-        <v>0.8507</v>
+        <v>0.8515</v>
       </c>
       <c r="D20" s="2" t="n">
         <v>0.997</v>
@@ -2654,13 +2654,13 @@
         </is>
       </c>
       <c r="B21" t="n">
-        <v>918</v>
+        <v>932</v>
       </c>
       <c r="C21" s="2" t="n">
-        <v>0.8529</v>
+        <v>0.8562</v>
       </c>
       <c r="D21" s="2" t="n">
-        <v>0.9947</v>
+        <v>0.9951</v>
       </c>
     </row>
     <row r="22">
@@ -2670,13 +2670,13 @@
         </is>
       </c>
       <c r="B22" t="n">
-        <v>1051</v>
+        <v>1059</v>
       </c>
       <c r="C22" s="2" t="n">
-        <v>0.8554</v>
+        <v>0.8565</v>
       </c>
       <c r="D22" s="2" t="n">
-        <v>0.9959</v>
+        <v>0.9957</v>
       </c>
     </row>
     <row r="23">
@@ -2686,13 +2686,13 @@
         </is>
       </c>
       <c r="B23" t="n">
-        <v>985</v>
+        <v>1008</v>
       </c>
       <c r="C23" s="2" t="n">
-        <v>0.9107</v>
+        <v>0.9137</v>
       </c>
       <c r="D23" s="2" t="n">
-        <v>0.9887</v>
+        <v>0.9901</v>
       </c>
     </row>
     <row r="24">
@@ -2702,13 +2702,13 @@
         </is>
       </c>
       <c r="B24" t="n">
-        <v>870</v>
+        <v>865</v>
       </c>
       <c r="C24" s="2" t="n">
-        <v>0.8724</v>
+        <v>0.8717</v>
       </c>
       <c r="D24" s="2" t="n">
-        <v>0.991</v>
+        <v>0.9915</v>
       </c>
     </row>
     <row r="25">
@@ -2718,13 +2718,13 @@
         </is>
       </c>
       <c r="B25" t="n">
-        <v>1056</v>
+        <v>1065</v>
       </c>
       <c r="C25" s="2" t="n">
-        <v>0.9413</v>
+        <v>0.9502</v>
       </c>
       <c r="D25" s="2" t="n">
-        <v>0.9923</v>
+        <v>0.9927</v>
       </c>
     </row>
     <row r="26">
@@ -2734,13 +2734,13 @@
         </is>
       </c>
       <c r="B26" t="n">
-        <v>851</v>
+        <v>862</v>
       </c>
       <c r="C26" s="2" t="n">
-        <v>0.8919</v>
+        <v>0.8991</v>
       </c>
       <c r="D26" s="2" t="n">
-        <v>0.986</v>
+        <v>0.9889</v>
       </c>
     </row>
     <row r="27">
@@ -2750,13 +2750,13 @@
         </is>
       </c>
       <c r="B27" t="n">
-        <v>920</v>
+        <v>926</v>
       </c>
       <c r="C27" s="2" t="n">
-        <v>0.9174</v>
+        <v>0.9298</v>
       </c>
       <c r="D27" s="2" t="n">
-        <v>0.9867</v>
+        <v>0.9896</v>
       </c>
     </row>
     <row r="28">
@@ -2766,13 +2766,13 @@
         </is>
       </c>
       <c r="B28" t="n">
-        <v>876</v>
+        <v>862</v>
       </c>
       <c r="C28" s="2" t="n">
-        <v>0.9041</v>
+        <v>0.9049</v>
       </c>
       <c r="D28" s="2" t="n">
-        <v>0.9855</v>
+        <v>0.9893999999999999</v>
       </c>
     </row>
     <row r="29">
@@ -2782,13 +2782,13 @@
         </is>
       </c>
       <c r="B29" t="n">
-        <v>877</v>
+        <v>896</v>
       </c>
       <c r="C29" s="2" t="n">
-        <v>0.9065</v>
+        <v>0.9085</v>
       </c>
       <c r="D29" s="2" t="n">
-        <v>0.992</v>
+        <v>0.9927</v>
       </c>
     </row>
     <row r="30">
@@ -2798,13 +2798,13 @@
         </is>
       </c>
       <c r="B30" t="n">
-        <v>963</v>
+        <v>962</v>
       </c>
       <c r="C30" s="2" t="n">
-        <v>0.8879</v>
+        <v>0.8898</v>
       </c>
       <c r="D30" s="2" t="n">
-        <v>0.9912</v>
+        <v>0.9915</v>
       </c>
     </row>
     <row r="31">
@@ -2814,13 +2814,13 @@
         </is>
       </c>
       <c r="B31" t="n">
-        <v>1011</v>
+        <v>1018</v>
       </c>
       <c r="C31" s="2" t="n">
-        <v>0.8773</v>
+        <v>0.8802</v>
       </c>
       <c r="D31" s="2" t="n">
-        <v>0.9921</v>
+        <v>0.9926</v>
       </c>
     </row>
     <row r="32">
@@ -2830,13 +2830,13 @@
         </is>
       </c>
       <c r="B32" t="n">
-        <v>936</v>
+        <v>939</v>
       </c>
       <c r="C32" s="2" t="n">
-        <v>0.89</v>
+        <v>0.8967000000000001</v>
       </c>
       <c r="D32" s="2" t="n">
-        <v>0.9883</v>
+        <v>0.989</v>
       </c>
     </row>
     <row r="33">
@@ -2846,13 +2846,13 @@
         </is>
       </c>
       <c r="B33" t="n">
-        <v>733</v>
+        <v>731</v>
       </c>
       <c r="C33" s="2" t="n">
-        <v>0.8922</v>
+        <v>0.8933</v>
       </c>
       <c r="D33" s="2" t="n">
-        <v>0.9912</v>
+        <v>0.992</v>
       </c>
     </row>
     <row r="34">
@@ -2862,13 +2862,13 @@
         </is>
       </c>
       <c r="B34" t="n">
-        <v>943</v>
+        <v>956</v>
       </c>
       <c r="C34" s="2" t="n">
-        <v>0.9236</v>
+        <v>0.9257</v>
       </c>
       <c r="D34" s="2" t="n">
-        <v>0.9903</v>
+        <v>0.9913999999999999</v>
       </c>
     </row>
     <row r="35">
@@ -2878,13 +2878,13 @@
         </is>
       </c>
       <c r="B35" t="n">
-        <v>998</v>
+        <v>1007</v>
       </c>
       <c r="C35" s="2" t="n">
-        <v>0.8717</v>
+        <v>0.8729</v>
       </c>
       <c r="D35" s="2" t="n">
-        <v>0.9943</v>
+        <v>0.994</v>
       </c>
     </row>
     <row r="36">
@@ -2894,13 +2894,13 @@
         </is>
       </c>
       <c r="B36" t="n">
-        <v>793</v>
+        <v>798</v>
       </c>
       <c r="C36" s="2" t="n">
-        <v>0.9142</v>
+        <v>0.9173</v>
       </c>
       <c r="D36" s="2" t="n">
-        <v>0.9861</v>
+        <v>0.988</v>
       </c>
     </row>
     <row r="37">
@@ -2910,13 +2910,13 @@
         </is>
       </c>
       <c r="B37" t="n">
-        <v>934</v>
+        <v>936</v>
       </c>
       <c r="C37" s="2" t="n">
-        <v>0.9111</v>
+        <v>0.9071</v>
       </c>
       <c r="D37" s="2" t="n">
-        <v>0.9905</v>
+        <v>0.9913999999999999</v>
       </c>
     </row>
     <row r="38">
@@ -2926,13 +2926,13 @@
         </is>
       </c>
       <c r="B38" t="n">
-        <v>836</v>
+        <v>840</v>
       </c>
       <c r="C38" s="2" t="n">
-        <v>0.89</v>
+        <v>0.8929</v>
       </c>
       <c r="D38" s="2" t="n">
-        <v>0.9927</v>
+        <v>0.9937</v>
       </c>
     </row>
     <row r="39">
@@ -2942,13 +2942,13 @@
         </is>
       </c>
       <c r="B39" t="n">
-        <v>1020</v>
+        <v>1032</v>
       </c>
       <c r="C39" s="2" t="n">
-        <v>0.9098000000000001</v>
+        <v>0.9186</v>
       </c>
       <c r="D39" s="2" t="n">
-        <v>0.9887</v>
+        <v>0.9909</v>
       </c>
     </row>
     <row r="40">
@@ -2958,13 +2958,13 @@
         </is>
       </c>
       <c r="B40" t="n">
-        <v>807</v>
+        <v>806</v>
       </c>
       <c r="C40" s="2" t="n">
-        <v>0.8823</v>
+        <v>0.8821</v>
       </c>
       <c r="D40" s="2" t="n">
-        <v>0.9915</v>
+        <v>0.9918</v>
       </c>
     </row>
   </sheetData>
@@ -3028,16 +3028,16 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>0.129</v>
+        <v>0.1273</v>
       </c>
       <c r="C2" t="n">
-        <v>0.1191</v>
+        <v>0.1184</v>
       </c>
       <c r="D2" t="n">
-        <v>-0.0014</v>
+        <v>-0.0011</v>
       </c>
       <c r="E2" t="n">
-        <v>1.0442</v>
+        <v>1.0493</v>
       </c>
       <c r="F2" t="n">
         <v>0.0746</v>
@@ -3050,19 +3050,19 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>0.1256</v>
+        <v>0.1246</v>
       </c>
       <c r="C3" t="n">
-        <v>0.1256</v>
+        <v>0.1127</v>
       </c>
       <c r="D3" t="n">
-        <v>-0.0075</v>
+        <v>-0.0089</v>
       </c>
       <c r="E3" t="n">
-        <v>1.0607</v>
+        <v>1.059</v>
       </c>
       <c r="F3" t="n">
-        <v>0.08160000000000001</v>
+        <v>0.0818</v>
       </c>
     </row>
     <row r="4">
@@ -3072,19 +3072,19 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>0.0499</v>
+        <v>0.0494</v>
       </c>
       <c r="C4" t="n">
-        <v>0.0446</v>
+        <v>0.0444</v>
       </c>
       <c r="D4" t="n">
-        <v>0.09130000000000001</v>
+        <v>0.0927</v>
       </c>
       <c r="E4" t="n">
-        <v>1.0138</v>
+        <v>1.0142</v>
       </c>
       <c r="F4" t="n">
-        <v>0.0631</v>
+        <v>0.063</v>
       </c>
     </row>
   </sheetData>
@@ -3113,7 +3113,7 @@
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>2026-08-07T09:13:57+00:00</t>
+          <t>2026-08-10T09:12:06+00:00</t>
         </is>
       </c>
     </row>
@@ -3124,7 +3124,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>4271</v>
+        <v>4388</v>
       </c>
     </row>
     <row r="3">
@@ -3134,7 +3134,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>110</v>
+        <v>113</v>
       </c>
     </row>
     <row r="4">
@@ -3164,7 +3164,7 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>206</v>
+        <v>210</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Exclui Shenzhen e recalcula o backtest
</commit_message>
<xml_diff>
--- a/backtest_results/resultados_backtest.xlsx
+++ b/backtest_results/resultados_backtest.xlsx
@@ -516,28 +516,28 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>450</v>
+        <v>390</v>
       </c>
       <c r="C2" s="2" t="n">
-        <v>0.8733333333333333</v>
+        <v>0.8743589743589744</v>
       </c>
       <c r="D2" s="3" t="n">
-        <v>6.744648574982978</v>
+        <v>6.055273071034335</v>
       </c>
       <c r="E2" s="4" t="n">
-        <v>135.9557172833742</v>
+        <v>94.20530983932451</v>
       </c>
       <c r="F2" s="2" t="n">
-        <v>2.684586107663417</v>
+        <v>2.342649263472548</v>
       </c>
       <c r="G2" s="2" t="n">
         <v>0.317247950343665</v>
       </c>
       <c r="H2" t="n">
-        <v>104</v>
+        <v>85</v>
       </c>
       <c r="I2" s="3" t="n">
-        <v>0.8069733333333333</v>
+        <v>0.8029948717948718</v>
       </c>
     </row>
     <row r="3">
@@ -547,28 +547,28 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>1880</v>
+        <v>1761</v>
       </c>
       <c r="C3" s="2" t="n">
-        <v>0.9930851063829788</v>
+        <v>0.9926178307779671</v>
       </c>
       <c r="D3" s="3" t="n">
-        <v>2.048300104592252</v>
+        <v>1.929343391232834</v>
       </c>
       <c r="E3" s="4" t="n">
-        <v>2.977331809451109</v>
+        <v>2.860342411305598</v>
       </c>
       <c r="F3" s="2" t="n">
-        <v>0.3359642656289785</v>
+        <v>0.3218218517432809</v>
       </c>
       <c r="G3" s="2" t="n">
-        <v>0.08704657533117899</v>
+        <v>0.07901949101919936</v>
       </c>
       <c r="H3" t="n">
-        <v>41</v>
+        <v>38</v>
       </c>
       <c r="I3" s="3" t="n">
-        <v>0.9857095744680852</v>
+        <v>0.9856785917092561</v>
       </c>
     </row>
     <row r="4">
@@ -578,28 +578,28 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>1361</v>
+        <v>1283</v>
       </c>
       <c r="C4" s="2" t="n">
-        <v>0.9948567229977957</v>
+        <v>0.9945440374123149</v>
       </c>
       <c r="D4" s="3" t="n">
-        <v>1.451175947349657</v>
+        <v>1.385736794077846</v>
       </c>
       <c r="E4" s="4" t="n">
-        <v>2.48951910355694</v>
+        <v>2.407740757845219</v>
       </c>
       <c r="F4" s="2" t="n">
-        <v>0.2739823091529194</v>
+        <v>0.2627352849259024</v>
       </c>
       <c r="G4" s="2" t="n">
-        <v>0.08016721391959114</v>
+        <v>0.07313459803799172</v>
       </c>
       <c r="H4" t="n">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="I4" s="3" t="n">
-        <v>0.9865907421013961</v>
+        <v>0.9865315666406859</v>
       </c>
     </row>
     <row r="5">
@@ -609,19 +609,19 @@
         </is>
       </c>
       <c r="B5" s="5" t="n">
-        <v>726</v>
+        <v>681</v>
       </c>
       <c r="C5" s="6" t="n">
-        <v>0.9986225895316805</v>
+        <v>0.9985315712187959</v>
       </c>
       <c r="D5" s="7" t="n">
-        <v>0.8410733032525365</v>
+        <v>0.7859325595763096</v>
       </c>
       <c r="E5" s="8" t="n">
-        <v>1.922289010908064</v>
+        <v>1.854295813834358</v>
       </c>
       <c r="F5" s="6" t="n">
-        <v>0.1894606875452871</v>
+        <v>0.1781428972849284</v>
       </c>
       <c r="G5" s="6" t="n">
         <v>0.02619857308701179</v>
@@ -630,7 +630,7 @@
         <v>6</v>
       </c>
       <c r="I5" s="7" t="n">
-        <v>0.9872699724517907</v>
+        <v>0.9872254038179149</v>
       </c>
     </row>
     <row r="6">
@@ -640,34 +640,34 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>1176</v>
+        <v>1071</v>
       </c>
       <c r="C6" s="2" t="n">
-        <v>0.9506802721088435</v>
+        <v>0.9533146591970122</v>
       </c>
       <c r="D6" s="3" t="n">
-        <v>7.585721878235514</v>
+        <v>6.841205630610644</v>
       </c>
       <c r="E6" s="4" t="n">
-        <v>139.5288597750242</v>
+        <v>101.5157720795613</v>
       </c>
       <c r="F6" s="2" t="n">
-        <v>2.710050618573619</v>
+        <v>2.409635975505925</v>
       </c>
       <c r="G6" s="2" t="n">
         <v>0.3007452058777901</v>
       </c>
       <c r="H6" t="n">
-        <v>110</v>
+        <v>91</v>
       </c>
       <c r="I6" s="3" t="n">
-        <v>0.9182789115646258</v>
+        <v>0.920138655462185</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Atualizado em 2026-08-10T09:12:06+00:00 · arquivo de 4388 dias-cidade (~113 dias corridos) · 39 cidades</t>
+          <t>Atualizado em 2026-08-11T09:39:37+00:00 · arquivo de 4286 dias-cidade (~113 dias corridos) · 38 cidades</t>
         </is>
       </c>
     </row>
@@ -689,7 +689,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E76"/>
+  <dimension ref="A1:E74"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -738,13 +738,13 @@
         </is>
       </c>
       <c r="C2" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="D2" s="2" t="n">
-        <v>0.5</v>
+        <v>0.75</v>
       </c>
       <c r="E2" s="3" t="n">
-        <v>-0.03</v>
+        <v>-0.00876525459112531</v>
       </c>
     </row>
     <row r="3">
@@ -822,13 +822,13 @@
         </is>
       </c>
       <c r="C6" t="n">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="D6" s="2" t="n">
-        <v>0.9090909090909091</v>
+        <v>0.9285714285714286</v>
       </c>
       <c r="E6" s="3" t="n">
-        <v>-0.01281695079576209</v>
+        <v>0.05183875767161625</v>
       </c>
     </row>
     <row r="7">
@@ -885,13 +885,13 @@
         </is>
       </c>
       <c r="C9" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D9" s="2" t="n">
-        <v>0.6666666666666666</v>
+        <v>0.75</v>
       </c>
       <c r="E9" s="3" t="n">
-        <v>0.1294782168186424</v>
+        <v>0.1693383566787822</v>
       </c>
     </row>
     <row r="10">
@@ -975,7 +975,7 @@
         <v>0.8571428571428571</v>
       </c>
       <c r="E13" s="3" t="n">
-        <v>0.4579984840521444</v>
+        <v>0.4626455303825978</v>
       </c>
     </row>
     <row r="14">
@@ -1137,13 +1137,13 @@
         </is>
       </c>
       <c r="C21" t="n">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="D21" s="2" t="n">
         <v>0.5</v>
       </c>
       <c r="E21" s="3" t="n">
-        <v>-0.04853875397650686</v>
+        <v>-0.02840361884137172</v>
       </c>
     </row>
     <row r="22">
@@ -1179,13 +1179,13 @@
         </is>
       </c>
       <c r="C23" t="n">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="D23" s="2" t="n">
-        <v>0.8333333333333334</v>
+        <v>0.84</v>
       </c>
       <c r="E23" s="3" t="n">
-        <v>0.4972467102262322</v>
+        <v>0.4822467102262322</v>
       </c>
     </row>
     <row r="24">
@@ -1221,13 +1221,13 @@
         </is>
       </c>
       <c r="C25" t="n">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="D25" s="2" t="n">
-        <v>0.8333333333333334</v>
+        <v>0.84</v>
       </c>
       <c r="E25" s="3" t="n">
-        <v>0.2363717485679154</v>
+        <v>0.2493660988504013</v>
       </c>
     </row>
     <row r="26">
@@ -1263,13 +1263,13 @@
         </is>
       </c>
       <c r="C27" t="n">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="D27" s="2" t="n">
         <v>1</v>
       </c>
       <c r="E27" s="3" t="n">
-        <v>0.8221975485570969</v>
+        <v>1.022497848857397</v>
       </c>
     </row>
     <row r="28">
@@ -1290,7 +1290,7 @@
         <v>0.90625</v>
       </c>
       <c r="E28" s="3" t="n">
-        <v>1.281152704143795</v>
+        <v>1.043572058982505</v>
       </c>
     </row>
     <row r="29">
@@ -1311,7 +1311,7 @@
         <v>0.9</v>
       </c>
       <c r="E29" s="3" t="n">
-        <v>0.1572290064307805</v>
+        <v>0.1591315939498064</v>
       </c>
     </row>
     <row r="30">
@@ -1410,13 +1410,13 @@
         </is>
       </c>
       <c r="C34" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="D34" s="2" t="n">
-        <v>0.875</v>
+        <v>0.8823529411764706</v>
       </c>
       <c r="E34" s="3" t="n">
-        <v>0.428628714046834</v>
+        <v>0.4393706852539215</v>
       </c>
     </row>
     <row r="35">
@@ -1427,17 +1427,17 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>Shenzhen (ZGSZ)</t>
+          <t>Wuhan (ZHHH)</t>
         </is>
       </c>
       <c r="C35" t="n">
-        <v>74</v>
+        <v>19</v>
       </c>
       <c r="D35" s="2" t="n">
-        <v>0.8783783783783784</v>
+        <v>0.8947368421052632</v>
       </c>
       <c r="E35" s="3" t="n">
-        <v>0.8611178896791831</v>
+        <v>0.4175399346554238</v>
       </c>
     </row>
     <row r="36">
@@ -1448,17 +1448,17 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>Wuhan (ZHHH)</t>
+          <t>Xangai (ZSPD)</t>
         </is>
       </c>
       <c r="C36" t="n">
-        <v>17</v>
+        <v>12</v>
       </c>
       <c r="D36" s="2" t="n">
-        <v>0.8823529411764706</v>
+        <v>0.9166666666666666</v>
       </c>
       <c r="E36" s="3" t="n">
-        <v>0.3696888882744743</v>
+        <v>0.1393609616271082</v>
       </c>
     </row>
     <row r="37">
@@ -1469,38 +1469,38 @@
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>Xangai (ZSPD)</t>
+          <t>Chengdu (ZUUU)</t>
         </is>
       </c>
       <c r="C37" t="n">
-        <v>12</v>
+        <v>3</v>
       </c>
       <c r="D37" s="2" t="n">
-        <v>0.9166666666666666</v>
+        <v>1</v>
       </c>
       <c r="E37" s="3" t="n">
-        <v>0.1393609616271082</v>
+        <v>0.02445809865164708</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>Edge</t>
+          <t>Combinado</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>Chengdu (ZUUU)</t>
+          <t>Toronto (CYYZ)</t>
         </is>
       </c>
       <c r="C38" t="n">
-        <v>3</v>
+        <v>18</v>
       </c>
       <c r="D38" s="2" t="n">
-        <v>1</v>
+        <v>0.9444444444444444</v>
       </c>
       <c r="E38" s="3" t="n">
-        <v>0.02445809865164708</v>
+        <v>0.01395708859174546</v>
       </c>
     </row>
     <row r="39">
@@ -1511,17 +1511,17 @@
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>Toronto (CYYZ)</t>
+          <t>Munique (EDDM)</t>
         </is>
       </c>
       <c r="C39" t="n">
-        <v>16</v>
+        <v>21</v>
       </c>
       <c r="D39" s="2" t="n">
-        <v>0.9375</v>
+        <v>0.9523809523809523</v>
       </c>
       <c r="E39" s="3" t="n">
-        <v>-0.007277656817129237</v>
+        <v>0.02897737559373625</v>
       </c>
     </row>
     <row r="40">
@@ -1532,17 +1532,17 @@
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>Munique (EDDM)</t>
+          <t>Helsinque (EFHK)</t>
         </is>
       </c>
       <c r="C40" t="n">
-        <v>21</v>
+        <v>36</v>
       </c>
       <c r="D40" s="2" t="n">
-        <v>0.9523809523809523</v>
+        <v>0.9722222222222222</v>
       </c>
       <c r="E40" s="3" t="n">
-        <v>0.02897737559373625</v>
+        <v>0.1195241289400556</v>
       </c>
     </row>
     <row r="41">
@@ -1553,17 +1553,17 @@
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>Helsinque (EFHK)</t>
+          <t>Londres (EGLC)</t>
         </is>
       </c>
       <c r="C41" t="n">
-        <v>36</v>
+        <v>33</v>
       </c>
       <c r="D41" s="2" t="n">
-        <v>0.9722222222222222</v>
+        <v>0.9393939393939394</v>
       </c>
       <c r="E41" s="3" t="n">
-        <v>0.1195241289400556</v>
+        <v>-0.03288122155900778</v>
       </c>
     </row>
     <row r="42">
@@ -1574,17 +1574,17 @@
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>Londres (EGLC)</t>
+          <t>Amsterdã (EHAM)</t>
         </is>
       </c>
       <c r="C42" t="n">
-        <v>33</v>
+        <v>62</v>
       </c>
       <c r="D42" s="2" t="n">
-        <v>0.9393939393939394</v>
+        <v>0.9838709677419355</v>
       </c>
       <c r="E42" s="3" t="n">
-        <v>-0.03288122155900778</v>
+        <v>0.09960525579400151</v>
       </c>
     </row>
     <row r="43">
@@ -1595,17 +1595,17 @@
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>Amsterdã (EHAM)</t>
+          <t>Varsóvia (EPWA)</t>
         </is>
       </c>
       <c r="C43" t="n">
-        <v>59</v>
+        <v>15</v>
       </c>
       <c r="D43" s="2" t="n">
-        <v>0.9830508474576272</v>
+        <v>0.9333333333333333</v>
       </c>
       <c r="E43" s="3" t="n">
-        <v>0.03402096558047677</v>
+        <v>0.1547869291708782</v>
       </c>
     </row>
     <row r="44">
@@ -1616,17 +1616,17 @@
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>Varsóvia (EPWA)</t>
+          <t>Cidade do Cabo (FACT)</t>
         </is>
       </c>
       <c r="C44" t="n">
-        <v>15</v>
+        <v>35</v>
       </c>
       <c r="D44" s="2" t="n">
-        <v>0.9333333333333333</v>
+        <v>0.9142857142857143</v>
       </c>
       <c r="E44" s="3" t="n">
-        <v>0.1547869291708782</v>
+        <v>0.02446541739413485</v>
       </c>
     </row>
     <row r="45">
@@ -1637,17 +1637,17 @@
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>Cidade do Cabo (FACT)</t>
+          <t>Atlanta (KATL)</t>
         </is>
       </c>
       <c r="C45" t="n">
-        <v>33</v>
+        <v>20</v>
       </c>
       <c r="D45" s="2" t="n">
-        <v>0.9090909090909091</v>
+        <v>0.95</v>
       </c>
       <c r="E45" s="3" t="n">
-        <v>0.02264655287981242</v>
+        <v>0.1863300383552792</v>
       </c>
     </row>
     <row r="46">
@@ -1658,17 +1658,17 @@
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>Atlanta (KATL)</t>
+          <t>Denver (KBKF)</t>
         </is>
       </c>
       <c r="C46" t="n">
-        <v>19</v>
+        <v>5</v>
       </c>
       <c r="D46" s="2" t="n">
-        <v>0.9473684210526315</v>
+        <v>1</v>
       </c>
       <c r="E46" s="3" t="n">
-        <v>0.1464698984951394</v>
+        <v>0.08135918956658879</v>
       </c>
     </row>
     <row r="47">
@@ -1679,7 +1679,7 @@
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>Denver (KBKF)</t>
+          <t>Dallas (KDAL)</t>
         </is>
       </c>
       <c r="C47" t="n">
@@ -1689,7 +1689,7 @@
         <v>1</v>
       </c>
       <c r="E47" s="3" t="n">
-        <v>0.08135918956658879</v>
+        <v>0.0109276789502966</v>
       </c>
     </row>
     <row r="48">
@@ -1700,17 +1700,17 @@
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>Dallas (KDAL)</t>
+          <t>Houston (KHOU)</t>
         </is>
       </c>
       <c r="C48" t="n">
-        <v>5</v>
+        <v>13</v>
       </c>
       <c r="D48" s="2" t="n">
-        <v>1</v>
+        <v>0.6923076923076923</v>
       </c>
       <c r="E48" s="3" t="n">
-        <v>0.0109276789502966</v>
+        <v>-0.02271345164640357</v>
       </c>
     </row>
     <row r="49">
@@ -1721,17 +1721,17 @@
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>Houston (KHOU)</t>
+          <t>Los Angeles (KLAX)</t>
         </is>
       </c>
       <c r="C49" t="n">
-        <v>13</v>
+        <v>31</v>
       </c>
       <c r="D49" s="2" t="n">
-        <v>0.6923076923076923</v>
+        <v>0.9032258064516129</v>
       </c>
       <c r="E49" s="3" t="n">
-        <v>-0.02271345164640357</v>
+        <v>0.473286981067213</v>
       </c>
     </row>
     <row r="50">
@@ -1742,17 +1742,17 @@
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>Los Angeles (KLAX)</t>
+          <t>Nova York (KLGA)</t>
         </is>
       </c>
       <c r="C50" t="n">
-        <v>31</v>
+        <v>15</v>
       </c>
       <c r="D50" s="2" t="n">
-        <v>0.9032258064516129</v>
+        <v>0.9333333333333333</v>
       </c>
       <c r="E50" s="3" t="n">
-        <v>0.4686399347367595</v>
+        <v>0.06706445217240228</v>
       </c>
     </row>
     <row r="51">
@@ -1763,17 +1763,17 @@
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>Nova York (KLGA)</t>
+          <t>Miami (KMIA)</t>
         </is>
       </c>
       <c r="C51" t="n">
-        <v>15</v>
+        <v>28</v>
       </c>
       <c r="D51" s="2" t="n">
-        <v>0.9333333333333333</v>
+        <v>0.9285714285714286</v>
       </c>
       <c r="E51" s="3" t="n">
-        <v>0.06706445217240228</v>
+        <v>0.07025010906606494</v>
       </c>
     </row>
     <row r="52">
@@ -1784,17 +1784,17 @@
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>Miami (KMIA)</t>
+          <t>Chicago (KORD)</t>
         </is>
       </c>
       <c r="C52" t="n">
-        <v>28</v>
+        <v>21</v>
       </c>
       <c r="D52" s="2" t="n">
-        <v>0.9285714285714286</v>
+        <v>1</v>
       </c>
       <c r="E52" s="3" t="n">
-        <v>0.07025010906606494</v>
+        <v>0.04882444083797849</v>
       </c>
     </row>
     <row r="53">
@@ -1805,17 +1805,17 @@
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>Chicago (KORD)</t>
+          <t>Seattle (KSEA)</t>
         </is>
       </c>
       <c r="C53" t="n">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="D53" s="2" t="n">
-        <v>1</v>
+        <v>0.9565217391304348</v>
       </c>
       <c r="E53" s="3" t="n">
-        <v>0.04882444083797849</v>
+        <v>-0.02356169087315167</v>
       </c>
     </row>
     <row r="54">
@@ -1826,17 +1826,17 @@
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>Seattle (KSEA)</t>
+          <t>Madri (LEMD)</t>
         </is>
       </c>
       <c r="C54" t="n">
-        <v>23</v>
+        <v>4</v>
       </c>
       <c r="D54" s="2" t="n">
-        <v>0.9565217391304348</v>
+        <v>1</v>
       </c>
       <c r="E54" s="3" t="n">
-        <v>-0.02356169087315167</v>
+        <v>0.005385531300417991</v>
       </c>
     </row>
     <row r="55">
@@ -1847,17 +1847,17 @@
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>Madri (LEMD)</t>
+          <t>Milão (LIMC)</t>
         </is>
       </c>
       <c r="C55" t="n">
-        <v>4</v>
+        <v>19</v>
       </c>
       <c r="D55" s="2" t="n">
         <v>1</v>
       </c>
       <c r="E55" s="3" t="n">
-        <v>0.005385531300417991</v>
+        <v>0.03465308375945613</v>
       </c>
     </row>
     <row r="56">
@@ -1868,17 +1868,17 @@
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>Milão (LIMC)</t>
+          <t>Tel Aviv (LLBG)</t>
         </is>
       </c>
       <c r="C56" t="n">
-        <v>19</v>
+        <v>5</v>
       </c>
       <c r="D56" s="2" t="n">
-        <v>1</v>
+        <v>0.8</v>
       </c>
       <c r="E56" s="3" t="n">
-        <v>0.03465308375945613</v>
+        <v>-0.009884941744941264</v>
       </c>
     </row>
     <row r="57">
@@ -1889,17 +1889,17 @@
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>Tel Aviv (LLBG)</t>
+          <t>Ancara (LTAC)</t>
         </is>
       </c>
       <c r="C57" t="n">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="D57" s="2" t="n">
-        <v>0.8</v>
+        <v>1</v>
       </c>
       <c r="E57" s="3" t="n">
-        <v>-0.009884941744941264</v>
+        <v>0.03806152988067182</v>
       </c>
     </row>
     <row r="58">
@@ -1910,17 +1910,17 @@
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>Ancara (LTAC)</t>
+          <t>Istambul (LTFM)</t>
         </is>
       </c>
       <c r="C58" t="n">
-        <v>10</v>
+        <v>77</v>
       </c>
       <c r="D58" s="2" t="n">
-        <v>1</v>
+        <v>0.9220779220779221</v>
       </c>
       <c r="E58" s="3" t="n">
-        <v>0.03806152988067182</v>
+        <v>0.05522417844390874</v>
       </c>
     </row>
     <row r="59">
@@ -1931,17 +1931,17 @@
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>Istambul (LTFM)</t>
+          <t>Cidade do México (MMMX)</t>
         </is>
       </c>
       <c r="C59" t="n">
-        <v>75</v>
+        <v>18</v>
       </c>
       <c r="D59" s="2" t="n">
-        <v>0.9333333333333333</v>
+        <v>0.9444444444444444</v>
       </c>
       <c r="E59" s="3" t="n">
-        <v>0.03307798247418333</v>
+        <v>-0.0009762299952974871</v>
       </c>
     </row>
     <row r="60">
@@ -1952,17 +1952,17 @@
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>Cidade do México (MMMX)</t>
+          <t>Wellington (NZWN)</t>
         </is>
       </c>
       <c r="C60" t="n">
-        <v>18</v>
+        <v>55</v>
       </c>
       <c r="D60" s="2" t="n">
-        <v>0.9444444444444444</v>
+        <v>0.9272727272727272</v>
       </c>
       <c r="E60" s="3" t="n">
-        <v>-0.0009762299952974871</v>
+        <v>0.5062571685840191</v>
       </c>
     </row>
     <row r="61">
@@ -1973,17 +1973,17 @@
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>Wellington (NZWN)</t>
+          <t>Taipé (RCSS)</t>
         </is>
       </c>
       <c r="C61" t="n">
-        <v>54</v>
+        <v>33</v>
       </c>
       <c r="D61" s="2" t="n">
-        <v>0.9259259259259259</v>
+        <v>0.9696969696969697</v>
       </c>
       <c r="E61" s="3" t="n">
-        <v>0.5212571685840192</v>
+        <v>0.2995551262996995</v>
       </c>
     </row>
     <row r="62">
@@ -1994,17 +1994,17 @@
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>Taipé (RCSS)</t>
+          <t>Tóquio (RJTT)</t>
         </is>
       </c>
       <c r="C62" t="n">
-        <v>33</v>
+        <v>54</v>
       </c>
       <c r="D62" s="2" t="n">
-        <v>0.9696969696969697</v>
+        <v>0.9259259259259259</v>
       </c>
       <c r="E62" s="3" t="n">
-        <v>0.2995551262996995</v>
+        <v>0.2852211755451628</v>
       </c>
     </row>
     <row r="63">
@@ -2015,17 +2015,17 @@
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>Tóquio (RJTT)</t>
+          <t>Seul (RKSI)</t>
         </is>
       </c>
       <c r="C63" t="n">
-        <v>53</v>
+        <v>26</v>
       </c>
       <c r="D63" s="2" t="n">
-        <v>0.9245283018867925</v>
+        <v>0.9615384615384616</v>
       </c>
       <c r="E63" s="3" t="n">
-        <v>0.2722268252626769</v>
+        <v>0.2067380805836653</v>
       </c>
     </row>
     <row r="64">
@@ -2036,17 +2036,17 @@
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>Seul (RKSI)</t>
+          <t>Manila (RPLL)</t>
         </is>
       </c>
       <c r="C64" t="n">
-        <v>26</v>
+        <v>63</v>
       </c>
       <c r="D64" s="2" t="n">
-        <v>0.9615384615384616</v>
+        <v>1</v>
       </c>
       <c r="E64" s="3" t="n">
-        <v>0.2067380805836653</v>
+        <v>1.025169714443921</v>
       </c>
     </row>
     <row r="65">
@@ -2057,17 +2057,17 @@
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>Manila (RPLL)</t>
+          <t>Buenos Aires (SAEZ)</t>
         </is>
       </c>
       <c r="C65" t="n">
-        <v>61</v>
+        <v>55</v>
       </c>
       <c r="D65" s="2" t="n">
-        <v>1</v>
+        <v>0.9454545454545454</v>
       </c>
       <c r="E65" s="3" t="n">
-        <v>0.8242657924132389</v>
+        <v>1.060093305432875</v>
       </c>
     </row>
     <row r="66">
@@ -2078,17 +2078,17 @@
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>Buenos Aires (SAEZ)</t>
+          <t>Guarulhos (SBGR)</t>
         </is>
       </c>
       <c r="C66" t="n">
-        <v>55</v>
+        <v>42</v>
       </c>
       <c r="D66" s="2" t="n">
-        <v>0.9454545454545454</v>
+        <v>0.9761904761904762</v>
       </c>
       <c r="E66" s="3" t="n">
-        <v>1.297673950594165</v>
+        <v>0.2009163255903637</v>
       </c>
     </row>
     <row r="67">
@@ -2099,17 +2099,17 @@
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>Guarulhos (SBGR)</t>
+          <t>Moscou (UUWW)</t>
         </is>
       </c>
       <c r="C67" t="n">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="D67" s="2" t="n">
-        <v>0.9761904761904762</v>
+        <v>1</v>
       </c>
       <c r="E67" s="3" t="n">
-        <v>0.1990137380713378</v>
+        <v>0.3891141971237955</v>
       </c>
     </row>
     <row r="68">
@@ -2120,17 +2120,17 @@
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>Moscou (UUWW)</t>
+          <t>Kuala Lumpur (WMKK)</t>
         </is>
       </c>
       <c r="C68" t="n">
-        <v>41</v>
+        <v>11</v>
       </c>
       <c r="D68" s="2" t="n">
         <v>1</v>
       </c>
       <c r="E68" s="3" t="n">
-        <v>0.3891141971237955</v>
+        <v>0.083921006625001</v>
       </c>
     </row>
     <row r="69">
@@ -2141,17 +2141,17 @@
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>Kuala Lumpur (WMKK)</t>
+          <t>Singapura (WSSS)</t>
         </is>
       </c>
       <c r="C69" t="n">
-        <v>11</v>
+        <v>30</v>
       </c>
       <c r="D69" s="2" t="n">
-        <v>1</v>
+        <v>0.9666666666666667</v>
       </c>
       <c r="E69" s="3" t="n">
-        <v>0.083921006625001</v>
+        <v>0.133019150081222</v>
       </c>
     </row>
     <row r="70">
@@ -2162,17 +2162,17 @@
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>Singapura (WSSS)</t>
+          <t>Pequim (ZBAA)</t>
         </is>
       </c>
       <c r="C70" t="n">
-        <v>30</v>
+        <v>19</v>
       </c>
       <c r="D70" s="2" t="n">
-        <v>0.9666666666666667</v>
+        <v>1</v>
       </c>
       <c r="E70" s="3" t="n">
-        <v>0.133019150081222</v>
+        <v>0.105030430626852</v>
       </c>
     </row>
     <row r="71">
@@ -2183,17 +2183,17 @@
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>Pequim (ZBAA)</t>
+          <t>Guangzhou (ZGGG)</t>
         </is>
       </c>
       <c r="C71" t="n">
-        <v>19</v>
+        <v>39</v>
       </c>
       <c r="D71" s="2" t="n">
-        <v>1</v>
+        <v>0.9487179487179487</v>
       </c>
       <c r="E71" s="3" t="n">
-        <v>0.105030430626852</v>
+        <v>0.473128471739481</v>
       </c>
     </row>
     <row r="72">
@@ -2204,17 +2204,17 @@
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>Guangzhou (ZGGG)</t>
+          <t>Wuhan (ZHHH)</t>
         </is>
       </c>
       <c r="C72" t="n">
-        <v>35</v>
+        <v>52</v>
       </c>
       <c r="D72" s="2" t="n">
-        <v>0.9428571428571428</v>
+        <v>0.9615384615384616</v>
       </c>
       <c r="E72" s="3" t="n">
-        <v>0.4558937776199615</v>
+        <v>0.4611517951194642</v>
       </c>
     </row>
     <row r="73">
@@ -2225,17 +2225,17 @@
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>Shenzhen (ZGSZ)</t>
+          <t>Xangai (ZSPD)</t>
         </is>
       </c>
       <c r="C73" t="n">
-        <v>126</v>
+        <v>31</v>
       </c>
       <c r="D73" s="2" t="n">
-        <v>0.9285714285714286</v>
+        <v>0.967741935483871</v>
       </c>
       <c r="E73" s="3" t="n">
-        <v>0.9287171068236656</v>
+        <v>0.1612549022946645</v>
       </c>
     </row>
     <row r="74">
@@ -2246,59 +2246,17 @@
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>Wuhan (ZHHH)</t>
+          <t>Chengdu (ZUUU)</t>
         </is>
       </c>
       <c r="C74" t="n">
-        <v>50</v>
+        <v>6</v>
       </c>
       <c r="D74" s="2" t="n">
-        <v>0.96</v>
+        <v>1</v>
       </c>
       <c r="E74" s="3" t="n">
-        <v>0.4133007487385147</v>
-      </c>
-    </row>
-    <row r="75">
-      <c r="A75" t="inlineStr">
-        <is>
-          <t>Combinado</t>
-        </is>
-      </c>
-      <c r="B75" t="inlineStr">
-        <is>
-          <t>Xangai (ZSPD)</t>
-        </is>
-      </c>
-      <c r="C75" t="n">
-        <v>31</v>
-      </c>
-      <c r="D75" s="2" t="n">
-        <v>0.967741935483871</v>
-      </c>
-      <c r="E75" s="3" t="n">
-        <v>0.1612549022946645</v>
-      </c>
-    </row>
-    <row r="76">
-      <c r="A76" t="inlineStr">
-        <is>
-          <t>Combinado</t>
-        </is>
-      </c>
-      <c r="B76" t="inlineStr">
-        <is>
-          <t>Chengdu (ZUUU)</t>
-        </is>
-      </c>
-      <c r="C76" t="n">
-        <v>5</v>
-      </c>
-      <c r="D76" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="E76" s="3" t="n">
-        <v>0.02736528572404578</v>
+        <v>0.02796890745442807</v>
       </c>
     </row>
   </sheetData>
@@ -2312,7 +2270,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D40"/>
+  <dimension ref="A1:D39"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
@@ -2353,10 +2311,10 @@
         <v>891</v>
       </c>
       <c r="C2" s="2" t="n">
-        <v>0.8833</v>
+        <v>0.8844</v>
       </c>
       <c r="D2" s="2" t="n">
-        <v>0.9923999999999999</v>
+        <v>0.9925</v>
       </c>
     </row>
     <row r="3">
@@ -2382,13 +2340,13 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>901</v>
+        <v>897</v>
       </c>
       <c r="C4" s="2" t="n">
-        <v>0.8801</v>
+        <v>0.8807</v>
       </c>
       <c r="D4" s="2" t="n">
-        <v>0.9933999999999999</v>
+        <v>0.9938</v>
       </c>
     </row>
     <row r="5">
@@ -2401,10 +2359,10 @@
         <v>991</v>
       </c>
       <c r="C5" s="2" t="n">
-        <v>0.8789</v>
+        <v>0.8799</v>
       </c>
       <c r="D5" s="2" t="n">
-        <v>0.994</v>
+        <v>0.9942</v>
       </c>
     </row>
     <row r="6">
@@ -2414,13 +2372,13 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>1075</v>
+        <v>1065</v>
       </c>
       <c r="C6" s="2" t="n">
-        <v>0.8884</v>
+        <v>0.8901</v>
       </c>
       <c r="D6" s="2" t="n">
-        <v>0.9929</v>
+        <v>0.9941</v>
       </c>
     </row>
     <row r="7">
@@ -2430,13 +2388,13 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>1039</v>
+        <v>1038</v>
       </c>
       <c r="C7" s="2" t="n">
-        <v>0.8778</v>
+        <v>0.8776</v>
       </c>
       <c r="D7" s="2" t="n">
-        <v>0.9957</v>
+        <v>0.9959</v>
       </c>
     </row>
     <row r="8">
@@ -2449,10 +2407,10 @@
         <v>837</v>
       </c>
       <c r="C8" s="2" t="n">
-        <v>0.8913</v>
+        <v>0.8925</v>
       </c>
       <c r="D8" s="2" t="n">
-        <v>0.9917</v>
+        <v>0.9918</v>
       </c>
     </row>
     <row r="9">
@@ -2484,7 +2442,7 @@
         <v>0.8736</v>
       </c>
       <c r="D10" s="2" t="n">
-        <v>0.9969</v>
+        <v>0.997</v>
       </c>
     </row>
     <row r="11">
@@ -2510,13 +2468,13 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>997</v>
+        <v>998</v>
       </c>
       <c r="C12" s="2" t="n">
-        <v>0.8917</v>
+        <v>0.8918</v>
       </c>
       <c r="D12" s="2" t="n">
-        <v>0.9936</v>
+        <v>0.9935</v>
       </c>
     </row>
     <row r="13">
@@ -2526,13 +2484,13 @@
         </is>
       </c>
       <c r="B13" t="n">
-        <v>915</v>
+        <v>916</v>
       </c>
       <c r="C13" s="2" t="n">
-        <v>0.9486</v>
+        <v>0.9487</v>
       </c>
       <c r="D13" s="2" t="n">
-        <v>0.9843</v>
+        <v>0.9844000000000001</v>
       </c>
     </row>
     <row r="14">
@@ -2542,10 +2500,10 @@
         </is>
       </c>
       <c r="B14" t="n">
-        <v>978</v>
+        <v>979</v>
       </c>
       <c r="C14" s="2" t="n">
-        <v>0.8885</v>
+        <v>0.8897</v>
       </c>
       <c r="D14" s="2" t="n">
         <v>0.9928</v>
@@ -2580,7 +2538,7 @@
         <v>0.8965</v>
       </c>
       <c r="D16" s="2" t="n">
-        <v>0.9948</v>
+        <v>0.9949</v>
       </c>
     </row>
     <row r="17">
@@ -2670,13 +2628,13 @@
         </is>
       </c>
       <c r="B22" t="n">
-        <v>1059</v>
+        <v>1058</v>
       </c>
       <c r="C22" s="2" t="n">
-        <v>0.8565</v>
+        <v>0.8573</v>
       </c>
       <c r="D22" s="2" t="n">
-        <v>0.9957</v>
+        <v>0.9959</v>
       </c>
     </row>
     <row r="23">
@@ -2686,13 +2644,13 @@
         </is>
       </c>
       <c r="B23" t="n">
-        <v>1008</v>
+        <v>999</v>
       </c>
       <c r="C23" s="2" t="n">
-        <v>0.9137</v>
+        <v>0.9149</v>
       </c>
       <c r="D23" s="2" t="n">
-        <v>0.9901</v>
+        <v>0.9911</v>
       </c>
     </row>
     <row r="24">
@@ -2702,13 +2660,13 @@
         </is>
       </c>
       <c r="B24" t="n">
-        <v>865</v>
+        <v>864</v>
       </c>
       <c r="C24" s="2" t="n">
-        <v>0.8717</v>
+        <v>0.8715000000000001</v>
       </c>
       <c r="D24" s="2" t="n">
-        <v>0.9915</v>
+        <v>0.9916</v>
       </c>
     </row>
     <row r="25">
@@ -2718,13 +2676,13 @@
         </is>
       </c>
       <c r="B25" t="n">
-        <v>1065</v>
+        <v>1048</v>
       </c>
       <c r="C25" s="2" t="n">
-        <v>0.9502</v>
+        <v>0.9504</v>
       </c>
       <c r="D25" s="2" t="n">
-        <v>0.9927</v>
+        <v>0.9942</v>
       </c>
     </row>
     <row r="26">
@@ -2734,13 +2692,13 @@
         </is>
       </c>
       <c r="B26" t="n">
-        <v>862</v>
+        <v>859</v>
       </c>
       <c r="C26" s="2" t="n">
-        <v>0.8991</v>
+        <v>0.8987000000000001</v>
       </c>
       <c r="D26" s="2" t="n">
-        <v>0.9889</v>
+        <v>0.9893999999999999</v>
       </c>
     </row>
     <row r="27">
@@ -2750,13 +2708,13 @@
         </is>
       </c>
       <c r="B27" t="n">
-        <v>926</v>
+        <v>922</v>
       </c>
       <c r="C27" s="2" t="n">
-        <v>0.9298</v>
+        <v>0.9295</v>
       </c>
       <c r="D27" s="2" t="n">
-        <v>0.9896</v>
+        <v>0.99</v>
       </c>
     </row>
     <row r="28">
@@ -2766,10 +2724,10 @@
         </is>
       </c>
       <c r="B28" t="n">
-        <v>862</v>
+        <v>861</v>
       </c>
       <c r="C28" s="2" t="n">
-        <v>0.9049</v>
+        <v>0.9048</v>
       </c>
       <c r="D28" s="2" t="n">
         <v>0.9893999999999999</v>
@@ -2782,13 +2740,13 @@
         </is>
       </c>
       <c r="B29" t="n">
-        <v>896</v>
+        <v>894</v>
       </c>
       <c r="C29" s="2" t="n">
-        <v>0.9085</v>
+        <v>0.9094</v>
       </c>
       <c r="D29" s="2" t="n">
-        <v>0.9927</v>
+        <v>0.9931</v>
       </c>
     </row>
     <row r="30">
@@ -2798,13 +2756,13 @@
         </is>
       </c>
       <c r="B30" t="n">
-        <v>962</v>
+        <v>956</v>
       </c>
       <c r="C30" s="2" t="n">
-        <v>0.8898</v>
+        <v>0.8902</v>
       </c>
       <c r="D30" s="2" t="n">
-        <v>0.9915</v>
+        <v>0.9922</v>
       </c>
     </row>
     <row r="31">
@@ -2814,13 +2772,13 @@
         </is>
       </c>
       <c r="B31" t="n">
-        <v>1018</v>
+        <v>1009</v>
       </c>
       <c r="C31" s="2" t="n">
-        <v>0.8802</v>
+        <v>0.8811</v>
       </c>
       <c r="D31" s="2" t="n">
-        <v>0.9926</v>
+        <v>0.9935</v>
       </c>
     </row>
     <row r="32">
@@ -2830,13 +2788,13 @@
         </is>
       </c>
       <c r="B32" t="n">
-        <v>939</v>
+        <v>936</v>
       </c>
       <c r="C32" s="2" t="n">
-        <v>0.8967000000000001</v>
+        <v>0.8974</v>
       </c>
       <c r="D32" s="2" t="n">
-        <v>0.989</v>
+        <v>0.9893</v>
       </c>
     </row>
     <row r="33">
@@ -2852,7 +2810,7 @@
         <v>0.8933</v>
       </c>
       <c r="D33" s="2" t="n">
-        <v>0.992</v>
+        <v>0.9921</v>
       </c>
     </row>
     <row r="34">
@@ -2862,13 +2820,13 @@
         </is>
       </c>
       <c r="B34" t="n">
-        <v>956</v>
+        <v>952</v>
       </c>
       <c r="C34" s="2" t="n">
-        <v>0.9257</v>
+        <v>0.9254</v>
       </c>
       <c r="D34" s="2" t="n">
-        <v>0.9913999999999999</v>
+        <v>0.9918</v>
       </c>
     </row>
     <row r="35">
@@ -2878,13 +2836,13 @@
         </is>
       </c>
       <c r="B35" t="n">
-        <v>1007</v>
+        <v>1006</v>
       </c>
       <c r="C35" s="2" t="n">
-        <v>0.8729</v>
+        <v>0.8728</v>
       </c>
       <c r="D35" s="2" t="n">
-        <v>0.994</v>
+        <v>0.9941</v>
       </c>
     </row>
     <row r="36">
@@ -2894,76 +2852,60 @@
         </is>
       </c>
       <c r="B36" t="n">
-        <v>798</v>
+        <v>796</v>
       </c>
       <c r="C36" s="2" t="n">
-        <v>0.9173</v>
+        <v>0.9171</v>
       </c>
       <c r="D36" s="2" t="n">
-        <v>0.988</v>
+        <v>0.9883</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>Shenzhen (ZGSZ)</t>
+          <t>Wuhan (ZHHH)</t>
         </is>
       </c>
       <c r="B37" t="n">
-        <v>936</v>
+        <v>839</v>
       </c>
       <c r="C37" s="2" t="n">
-        <v>0.9071</v>
+        <v>0.8927</v>
       </c>
       <c r="D37" s="2" t="n">
-        <v>0.9913999999999999</v>
+        <v>0.9938</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>Wuhan (ZHHH)</t>
+          <t>Xangai (ZSPD)</t>
         </is>
       </c>
       <c r="B38" t="n">
-        <v>840</v>
+        <v>1022</v>
       </c>
       <c r="C38" s="2" t="n">
-        <v>0.8929</v>
+        <v>0.9177999999999999</v>
       </c>
       <c r="D38" s="2" t="n">
-        <v>0.9937</v>
+        <v>0.9917</v>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>Xangai (ZSPD)</t>
+          <t>Chengdu (ZUUU)</t>
         </is>
       </c>
       <c r="B39" t="n">
-        <v>1032</v>
+        <v>806</v>
       </c>
       <c r="C39" s="2" t="n">
-        <v>0.9186</v>
+        <v>0.8821</v>
       </c>
       <c r="D39" s="2" t="n">
-        <v>0.9909</v>
-      </c>
-    </row>
-    <row r="40">
-      <c r="A40" t="inlineStr">
-        <is>
-          <t>Chengdu (ZUUU)</t>
-        </is>
-      </c>
-      <c r="B40" t="n">
-        <v>806</v>
-      </c>
-      <c r="C40" s="2" t="n">
-        <v>0.8821</v>
-      </c>
-      <c r="D40" s="2" t="n">
         <v>0.9918</v>
       </c>
     </row>
@@ -3028,19 +2970,19 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>0.1273</v>
+        <v>0.1277</v>
       </c>
       <c r="C2" t="n">
-        <v>0.1184</v>
+        <v>0.119</v>
       </c>
       <c r="D2" t="n">
-        <v>-0.0011</v>
+        <v>0.0002</v>
       </c>
       <c r="E2" t="n">
-        <v>1.0493</v>
+        <v>1.0569</v>
       </c>
       <c r="F2" t="n">
-        <v>0.0746</v>
+        <v>0.074</v>
       </c>
     </row>
     <row r="3">
@@ -3050,19 +2992,19 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>0.1246</v>
+        <v>0.1248</v>
       </c>
       <c r="C3" t="n">
-        <v>0.1127</v>
+        <v>0.1129</v>
       </c>
       <c r="D3" t="n">
-        <v>-0.0089</v>
+        <v>-0.005</v>
       </c>
       <c r="E3" t="n">
-        <v>1.059</v>
+        <v>1.0706</v>
       </c>
       <c r="F3" t="n">
-        <v>0.0818</v>
+        <v>0.0805</v>
       </c>
     </row>
     <row r="4">
@@ -3072,19 +3014,19 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>0.0494</v>
+        <v>0.044</v>
       </c>
       <c r="C4" t="n">
-        <v>0.0444</v>
+        <v>0.0395</v>
       </c>
       <c r="D4" t="n">
-        <v>0.0927</v>
+        <v>0.1188</v>
       </c>
       <c r="E4" t="n">
-        <v>1.0142</v>
+        <v>0.9935</v>
       </c>
       <c r="F4" t="n">
-        <v>0.063</v>
+        <v>0.0622</v>
       </c>
     </row>
   </sheetData>
@@ -3113,7 +3055,7 @@
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>2026-08-10T09:12:06+00:00</t>
+          <t>2026-08-11T09:39:37+00:00</t>
         </is>
       </c>
     </row>
@@ -3124,7 +3066,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>4388</v>
+        <v>4286</v>
       </c>
     </row>
     <row r="3">
@@ -3144,7 +3086,7 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>39</v>
+        <v>38</v>
       </c>
     </row>
     <row r="5">
@@ -3164,7 +3106,7 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>210</v>
+        <v>54</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Arquiva dados, recalibra e atualiza docs (2026-08-13)
</commit_message>
<xml_diff>
--- a/backtest_results/resultados_backtest.xlsx
+++ b/backtest_results/resultados_backtest.xlsx
@@ -516,28 +516,28 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>390</v>
+        <v>393</v>
       </c>
       <c r="C2" s="2" t="n">
-        <v>0.8743589743589744</v>
+        <v>0.8829516539440203</v>
       </c>
       <c r="D2" s="3" t="n">
-        <v>6.055273071034335</v>
+        <v>6.170987216982523</v>
       </c>
       <c r="E2" s="4" t="n">
-        <v>94.20530983932451</v>
+        <v>108.5707361553694</v>
       </c>
       <c r="F2" s="2" t="n">
-        <v>2.342649263472548</v>
+        <v>2.361069119863112</v>
       </c>
       <c r="G2" s="2" t="n">
-        <v>0.317247950343665</v>
+        <v>0.3059017866796615</v>
       </c>
       <c r="H2" t="n">
-        <v>85</v>
+        <v>80</v>
       </c>
       <c r="I2" s="3" t="n">
-        <v>0.8029948717948718</v>
+        <v>0.8081094147582697</v>
       </c>
     </row>
     <row r="3">
@@ -547,19 +547,19 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>1761</v>
+        <v>1809</v>
       </c>
       <c r="C3" s="2" t="n">
-        <v>0.9926178307779671</v>
+        <v>0.9928137092316197</v>
       </c>
       <c r="D3" s="3" t="n">
-        <v>1.929343391232834</v>
+        <v>1.999446258407061</v>
       </c>
       <c r="E3" s="4" t="n">
-        <v>2.860342411305598</v>
+        <v>2.982231980851253</v>
       </c>
       <c r="F3" s="2" t="n">
-        <v>0.3218218517432809</v>
+        <v>0.3265579606000797</v>
       </c>
       <c r="G3" s="2" t="n">
         <v>0.07901949101919936</v>
@@ -568,7 +568,7 @@
         <v>38</v>
       </c>
       <c r="I3" s="3" t="n">
-        <v>0.9856785917092561</v>
+        <v>0.9856779988944168</v>
       </c>
     </row>
     <row r="4">
@@ -578,19 +578,19 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>1283</v>
+        <v>1318</v>
       </c>
       <c r="C4" s="2" t="n">
-        <v>0.9945440374123149</v>
+        <v>0.9946889226100152</v>
       </c>
       <c r="D4" s="3" t="n">
-        <v>1.385736794077846</v>
+        <v>1.436865517384735</v>
       </c>
       <c r="E4" s="4" t="n">
-        <v>2.407740757845219</v>
+        <v>2.500419900830992</v>
       </c>
       <c r="F4" s="2" t="n">
-        <v>0.2627352849259024</v>
+        <v>0.2674603518109306</v>
       </c>
       <c r="G4" s="2" t="n">
         <v>0.07313459803799172</v>
@@ -599,7 +599,7 @@
         <v>22</v>
       </c>
       <c r="I4" s="3" t="n">
-        <v>0.9865315666406859</v>
+        <v>0.9865083459787557</v>
       </c>
     </row>
     <row r="5">
@@ -609,19 +609,19 @@
         </is>
       </c>
       <c r="B5" s="5" t="n">
-        <v>681</v>
+        <v>696</v>
       </c>
       <c r="C5" s="6" t="n">
-        <v>0.9985315712187959</v>
+        <v>0.9985632183908046</v>
       </c>
       <c r="D5" s="7" t="n">
-        <v>0.7859325595763096</v>
+        <v>0.8035315105952537</v>
       </c>
       <c r="E5" s="8" t="n">
-        <v>1.854295813834358</v>
+        <v>1.883070576824799</v>
       </c>
       <c r="F5" s="6" t="n">
-        <v>0.1781428972849284</v>
+        <v>0.1778397014998288</v>
       </c>
       <c r="G5" s="6" t="n">
         <v>0.02619857308701179</v>
@@ -630,7 +630,7 @@
         <v>6</v>
       </c>
       <c r="I5" s="7" t="n">
-        <v>0.9872254038179149</v>
+        <v>0.9872514367816093</v>
       </c>
     </row>
     <row r="6">
@@ -640,34 +640,34 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>1071</v>
+        <v>1089</v>
       </c>
       <c r="C6" s="2" t="n">
-        <v>0.9533146591970122</v>
+        <v>0.9568411386593205</v>
       </c>
       <c r="D6" s="3" t="n">
-        <v>6.841205630610644</v>
+        <v>6.974518727577776</v>
       </c>
       <c r="E6" s="4" t="n">
-        <v>101.5157720795613</v>
+        <v>117.6336736923698</v>
       </c>
       <c r="F6" s="2" t="n">
-        <v>2.409635975505925</v>
+        <v>2.43148674708239</v>
       </c>
       <c r="G6" s="2" t="n">
-        <v>0.3007452058777901</v>
+        <v>0.2893750111453259</v>
       </c>
       <c r="H6" t="n">
-        <v>91</v>
+        <v>86</v>
       </c>
       <c r="I6" s="3" t="n">
-        <v>0.920138655462185</v>
+        <v>0.9226023875114785</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Atualizado em 2026-08-11T09:39:37+00:00 · arquivo de 4286 dias-cidade (~113 dias corridos) · 38 cidades</t>
+          <t>Atualizado em 2026-08-13T09:14:08+00:00 · arquivo de 4400 dias-cidade (~116 dias corridos) · 38 cidades</t>
         </is>
       </c>
     </row>
@@ -738,13 +738,13 @@
         </is>
       </c>
       <c r="C2" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D2" s="2" t="n">
-        <v>0.75</v>
+        <v>0.6666666666666666</v>
       </c>
       <c r="E2" s="3" t="n">
-        <v>-0.00876525459112531</v>
+        <v>0.00623474540887469</v>
       </c>
     </row>
     <row r="3">
@@ -780,13 +780,13 @@
         </is>
       </c>
       <c r="C4" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="D4" s="2" t="n">
-        <v>0.8333333333333334</v>
+        <v>1</v>
       </c>
       <c r="E4" s="3" t="n">
-        <v>0.07431891929977413</v>
+        <v>0.07235985497228876</v>
       </c>
     </row>
     <row r="5">
@@ -801,13 +801,13 @@
         </is>
       </c>
       <c r="C5" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="D5" s="2" t="n">
-        <v>0.75</v>
+        <v>0.8571428571428571</v>
       </c>
       <c r="E5" s="3" t="n">
-        <v>-0.06526472273082738</v>
+        <v>-0.05026472273082738</v>
       </c>
     </row>
     <row r="6">
@@ -849,7 +849,7 @@
         <v>0.8</v>
       </c>
       <c r="E7" s="3" t="n">
-        <v>0.1406418288239204</v>
+        <v>0.1400478635114946</v>
       </c>
     </row>
     <row r="8">
@@ -864,13 +864,13 @@
         </is>
       </c>
       <c r="C8" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="D8" s="2" t="n">
-        <v>0.6666666666666666</v>
+        <v>0.75</v>
       </c>
       <c r="E8" s="3" t="n">
-        <v>-0.01506240674211111</v>
+        <v>-6.24067421111079e-05</v>
       </c>
     </row>
     <row r="9">
@@ -951,10 +951,10 @@
         <v>6</v>
       </c>
       <c r="D12" s="2" t="n">
-        <v>0.3333333333333333</v>
+        <v>0.5</v>
       </c>
       <c r="E12" s="3" t="n">
-        <v>-0.03415492957746477</v>
+        <v>-0.02348484848484846</v>
       </c>
     </row>
     <row r="13">
@@ -969,13 +969,13 @@
         </is>
       </c>
       <c r="C13" t="n">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="D13" s="2" t="n">
-        <v>0.8571428571428571</v>
+        <v>0.8421052631578947</v>
       </c>
       <c r="E13" s="3" t="n">
-        <v>0.4626455303825978</v>
+        <v>0.3374431186685581</v>
       </c>
     </row>
     <row r="14">
@@ -1182,10 +1182,10 @@
         <v>25</v>
       </c>
       <c r="D23" s="2" t="n">
-        <v>0.84</v>
+        <v>0.88</v>
       </c>
       <c r="E23" s="3" t="n">
-        <v>0.4822467102262322</v>
+        <v>0.5037997203487682</v>
       </c>
     </row>
     <row r="24">
@@ -1206,7 +1206,7 @@
         <v>0.9565217391304348</v>
       </c>
       <c r="E24" s="3" t="n">
-        <v>0.2869825159383541</v>
+        <v>0.2916596476873091</v>
       </c>
     </row>
     <row r="25">
@@ -1221,13 +1221,13 @@
         </is>
       </c>
       <c r="C25" t="n">
-        <v>25</v>
+        <v>29</v>
       </c>
       <c r="D25" s="2" t="n">
-        <v>0.84</v>
+        <v>0.8275862068965517</v>
       </c>
       <c r="E25" s="3" t="n">
-        <v>0.2493660988504013</v>
+        <v>0.2933607142431768</v>
       </c>
     </row>
     <row r="26">
@@ -1245,10 +1245,10 @@
         <v>18</v>
       </c>
       <c r="D26" s="2" t="n">
-        <v>0.9444444444444444</v>
+        <v>0.8888888888888888</v>
       </c>
       <c r="E26" s="3" t="n">
-        <v>0.1981192944401984</v>
+        <v>0.1451882599574397</v>
       </c>
     </row>
     <row r="27">
@@ -1263,13 +1263,13 @@
         </is>
       </c>
       <c r="C27" t="n">
-        <v>33</v>
+        <v>38</v>
       </c>
       <c r="D27" s="2" t="n">
         <v>1</v>
       </c>
       <c r="E27" s="3" t="n">
-        <v>1.022497848857397</v>
+        <v>1.132460979000862</v>
       </c>
     </row>
     <row r="28">
@@ -1284,13 +1284,13 @@
         </is>
       </c>
       <c r="C28" t="n">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="D28" s="2" t="n">
-        <v>0.90625</v>
+        <v>0.9090909090909091</v>
       </c>
       <c r="E28" s="3" t="n">
-        <v>1.043572058982505</v>
+        <v>1.069571862761213</v>
       </c>
     </row>
     <row r="29">
@@ -1305,13 +1305,13 @@
         </is>
       </c>
       <c r="C29" t="n">
-        <v>10</v>
+        <v>7</v>
       </c>
       <c r="D29" s="2" t="n">
-        <v>0.9</v>
+        <v>1</v>
       </c>
       <c r="E29" s="3" t="n">
-        <v>0.1591315939498064</v>
+        <v>0.1502427050609175</v>
       </c>
     </row>
     <row r="30">
@@ -1326,13 +1326,13 @@
         </is>
       </c>
       <c r="C30" t="n">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="D30" s="2" t="n">
         <v>1</v>
       </c>
       <c r="E30" s="3" t="n">
-        <v>0.3588116893818861</v>
+        <v>0.4097165460561873</v>
       </c>
     </row>
     <row r="31">
@@ -1473,13 +1473,13 @@
         </is>
       </c>
       <c r="C37" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="D37" s="2" t="n">
-        <v>1</v>
+        <v>0.8</v>
       </c>
       <c r="E37" s="3" t="n">
-        <v>0.02445809865164708</v>
+        <v>0.0169849803720772</v>
       </c>
     </row>
     <row r="38">
@@ -1494,13 +1494,13 @@
         </is>
       </c>
       <c r="C38" t="n">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="D38" s="2" t="n">
-        <v>0.9444444444444444</v>
+        <v>0.9411764705882353</v>
       </c>
       <c r="E38" s="3" t="n">
-        <v>0.01395708859174546</v>
+        <v>0.02895708859174546</v>
       </c>
     </row>
     <row r="39">
@@ -1536,13 +1536,13 @@
         </is>
       </c>
       <c r="C40" t="n">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="D40" s="2" t="n">
-        <v>0.9722222222222222</v>
+        <v>1</v>
       </c>
       <c r="E40" s="3" t="n">
-        <v>0.1195241289400556</v>
+        <v>0.1175650646125702</v>
       </c>
     </row>
     <row r="41">
@@ -1557,13 +1557,13 @@
         </is>
       </c>
       <c r="C41" t="n">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="D41" s="2" t="n">
-        <v>0.9393939393939394</v>
+        <v>0.96875</v>
       </c>
       <c r="E41" s="3" t="n">
-        <v>-0.03288122155900778</v>
+        <v>-0.01788122155900777</v>
       </c>
     </row>
     <row r="42">
@@ -1605,7 +1605,7 @@
         <v>0.9333333333333333</v>
       </c>
       <c r="E43" s="3" t="n">
-        <v>0.1547869291708782</v>
+        <v>0.1541929638584525</v>
       </c>
     </row>
     <row r="44">
@@ -1620,13 +1620,13 @@
         </is>
       </c>
       <c r="C44" t="n">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="D44" s="2" t="n">
-        <v>0.9142857142857143</v>
+        <v>0.9411764705882353</v>
       </c>
       <c r="E44" s="3" t="n">
-        <v>0.02446541739413485</v>
+        <v>0.03946541739413485</v>
       </c>
     </row>
     <row r="45">
@@ -1704,13 +1704,13 @@
         </is>
       </c>
       <c r="C48" t="n">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="D48" s="2" t="n">
-        <v>0.6923076923076923</v>
+        <v>0.8</v>
       </c>
       <c r="E48" s="3" t="n">
-        <v>-0.02271345164640357</v>
+        <v>-0.007956425350090768</v>
       </c>
     </row>
     <row r="49">
@@ -1725,13 +1725,13 @@
         </is>
       </c>
       <c r="C49" t="n">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="D49" s="2" t="n">
-        <v>0.9032258064516129</v>
+        <v>0.9</v>
       </c>
       <c r="E49" s="3" t="n">
-        <v>0.473286981067213</v>
+        <v>0.3486376110826856</v>
       </c>
     </row>
     <row r="50">
@@ -1935,13 +1935,13 @@
         </is>
       </c>
       <c r="C59" t="n">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="D59" s="2" t="n">
-        <v>0.9444444444444444</v>
+        <v>0.9473684210526315</v>
       </c>
       <c r="E59" s="3" t="n">
-        <v>-0.0009762299952974871</v>
+        <v>3.387101480352948e-05</v>
       </c>
     </row>
     <row r="60">
@@ -1959,10 +1959,10 @@
         <v>55</v>
       </c>
       <c r="D60" s="2" t="n">
-        <v>0.9272727272727272</v>
+        <v>0.9454545454545454</v>
       </c>
       <c r="E60" s="3" t="n">
-        <v>0.5062571685840191</v>
+        <v>0.527810178706555</v>
       </c>
     </row>
     <row r="61">
@@ -1983,7 +1983,7 @@
         <v>0.9696969696969697</v>
       </c>
       <c r="E61" s="3" t="n">
-        <v>0.2995551262996995</v>
+        <v>0.3042322580486544</v>
       </c>
     </row>
     <row r="62">
@@ -1998,13 +1998,13 @@
         </is>
       </c>
       <c r="C62" t="n">
-        <v>54</v>
+        <v>59</v>
       </c>
       <c r="D62" s="2" t="n">
-        <v>0.9259259259259259</v>
+        <v>0.9152542372881356</v>
       </c>
       <c r="E62" s="3" t="n">
-        <v>0.2852211755451628</v>
+        <v>0.3298194126683207</v>
       </c>
     </row>
     <row r="63">
@@ -2022,10 +2022,10 @@
         <v>26</v>
       </c>
       <c r="D63" s="2" t="n">
-        <v>0.9615384615384616</v>
+        <v>0.9230769230769231</v>
       </c>
       <c r="E63" s="3" t="n">
-        <v>0.2067380805836653</v>
+        <v>0.1538070461009067</v>
       </c>
     </row>
     <row r="64">
@@ -2040,13 +2040,13 @@
         </is>
       </c>
       <c r="C64" t="n">
-        <v>63</v>
+        <v>68</v>
       </c>
       <c r="D64" s="2" t="n">
         <v>1</v>
       </c>
       <c r="E64" s="3" t="n">
-        <v>1.025169714443921</v>
+        <v>1.135132844587386</v>
       </c>
     </row>
     <row r="65">
@@ -2061,13 +2061,13 @@
         </is>
       </c>
       <c r="C65" t="n">
-        <v>55</v>
+        <v>58</v>
       </c>
       <c r="D65" s="2" t="n">
-        <v>0.9454545454545454</v>
+        <v>0.9482758620689655</v>
       </c>
       <c r="E65" s="3" t="n">
-        <v>1.060093305432875</v>
+        <v>1.088215444802068</v>
       </c>
     </row>
     <row r="66">
@@ -2082,13 +2082,13 @@
         </is>
       </c>
       <c r="C66" t="n">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="D66" s="2" t="n">
-        <v>0.9761904761904762</v>
+        <v>1</v>
       </c>
       <c r="E66" s="3" t="n">
-        <v>0.2009163255903637</v>
+        <v>0.1942552138828612</v>
       </c>
     </row>
     <row r="67">
@@ -2103,13 +2103,13 @@
         </is>
       </c>
       <c r="C67" t="n">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="D67" s="2" t="n">
         <v>1</v>
       </c>
       <c r="E67" s="3" t="n">
-        <v>0.3891141971237955</v>
+        <v>0.4400190537980967</v>
       </c>
     </row>
     <row r="68">
@@ -2187,13 +2187,13 @@
         </is>
       </c>
       <c r="C71" t="n">
-        <v>39</v>
+        <v>42</v>
       </c>
       <c r="D71" s="2" t="n">
-        <v>0.9487179487179487</v>
+        <v>0.9523809523809523</v>
       </c>
       <c r="E71" s="3" t="n">
-        <v>0.473128471739481</v>
+        <v>0.4761634770379517</v>
       </c>
     </row>
     <row r="72">
@@ -2229,13 +2229,13 @@
         </is>
       </c>
       <c r="C73" t="n">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="D73" s="2" t="n">
-        <v>0.967741935483871</v>
+        <v>0.9696969696969697</v>
       </c>
       <c r="E73" s="3" t="n">
-        <v>0.1612549022946645</v>
+        <v>0.163537343820718</v>
       </c>
     </row>
     <row r="74">
@@ -2250,13 +2250,13 @@
         </is>
       </c>
       <c r="C74" t="n">
-        <v>6</v>
+        <v>9</v>
       </c>
       <c r="D74" s="2" t="n">
-        <v>1</v>
+        <v>0.8888888888888888</v>
       </c>
       <c r="E74" s="3" t="n">
-        <v>0.02796890745442807</v>
+        <v>0.02217347092371431</v>
       </c>
     </row>
   </sheetData>
@@ -2308,13 +2308,13 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>891</v>
+        <v>918</v>
       </c>
       <c r="C2" s="2" t="n">
-        <v>0.8844</v>
+        <v>0.8856000000000001</v>
       </c>
       <c r="D2" s="2" t="n">
-        <v>0.9925</v>
+        <v>0.9915</v>
       </c>
     </row>
     <row r="3">
@@ -2324,13 +2324,13 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>962</v>
+        <v>978</v>
       </c>
       <c r="C3" s="2" t="n">
-        <v>0.8534</v>
+        <v>0.8558</v>
       </c>
       <c r="D3" s="2" t="n">
-        <v>0.9969</v>
+        <v>0.997</v>
       </c>
     </row>
     <row r="4">
@@ -2340,13 +2340,13 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>897</v>
+        <v>923</v>
       </c>
       <c r="C4" s="2" t="n">
-        <v>0.8807</v>
+        <v>0.8819</v>
       </c>
       <c r="D4" s="2" t="n">
-        <v>0.9938</v>
+        <v>0.9927</v>
       </c>
     </row>
     <row r="5">
@@ -2356,13 +2356,13 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>991</v>
+        <v>1021</v>
       </c>
       <c r="C5" s="2" t="n">
-        <v>0.8799</v>
+        <v>0.8825</v>
       </c>
       <c r="D5" s="2" t="n">
-        <v>0.9942</v>
+        <v>0.9932</v>
       </c>
     </row>
     <row r="6">
@@ -2372,13 +2372,13 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>1065</v>
+        <v>1085</v>
       </c>
       <c r="C6" s="2" t="n">
-        <v>0.8901</v>
+        <v>0.8912</v>
       </c>
       <c r="D6" s="2" t="n">
-        <v>0.9941</v>
+        <v>0.994</v>
       </c>
     </row>
     <row r="7">
@@ -2388,13 +2388,13 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>1038</v>
+        <v>1060</v>
       </c>
       <c r="C7" s="2" t="n">
-        <v>0.8776</v>
+        <v>0.8802</v>
       </c>
       <c r="D7" s="2" t="n">
-        <v>0.9959</v>
+        <v>0.9955000000000001</v>
       </c>
     </row>
     <row r="8">
@@ -2404,13 +2404,13 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>837</v>
+        <v>852</v>
       </c>
       <c r="C8" s="2" t="n">
-        <v>0.8925</v>
+        <v>0.8944</v>
       </c>
       <c r="D8" s="2" t="n">
-        <v>0.9918</v>
+        <v>0.9915</v>
       </c>
     </row>
     <row r="9">
@@ -2420,13 +2420,13 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>1057</v>
+        <v>1076</v>
       </c>
       <c r="C9" s="2" t="n">
-        <v>0.8628</v>
+        <v>0.8652</v>
       </c>
       <c r="D9" s="2" t="n">
-        <v>0.9955000000000001</v>
+        <v>0.9951</v>
       </c>
     </row>
     <row r="10">
@@ -2436,13 +2436,13 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>1060</v>
+        <v>1079</v>
       </c>
       <c r="C10" s="2" t="n">
-        <v>0.8736</v>
+        <v>0.8758</v>
       </c>
       <c r="D10" s="2" t="n">
-        <v>0.997</v>
+        <v>0.9968</v>
       </c>
     </row>
     <row r="11">
@@ -2452,13 +2452,13 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>980</v>
+        <v>1001</v>
       </c>
       <c r="C11" s="2" t="n">
-        <v>0.898</v>
+        <v>0.9001</v>
       </c>
       <c r="D11" s="2" t="n">
-        <v>0.9946</v>
+        <v>0.9943</v>
       </c>
     </row>
     <row r="12">
@@ -2468,13 +2468,13 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>998</v>
+        <v>1025</v>
       </c>
       <c r="C12" s="2" t="n">
-        <v>0.8918</v>
+        <v>0.8946</v>
       </c>
       <c r="D12" s="2" t="n">
-        <v>0.9935</v>
+        <v>0.9932</v>
       </c>
     </row>
     <row r="13">
@@ -2484,13 +2484,13 @@
         </is>
       </c>
       <c r="B13" t="n">
-        <v>916</v>
+        <v>954</v>
       </c>
       <c r="C13" s="2" t="n">
-        <v>0.9487</v>
+        <v>0.9465</v>
       </c>
       <c r="D13" s="2" t="n">
-        <v>0.9844000000000001</v>
+        <v>0.9841</v>
       </c>
     </row>
     <row r="14">
@@ -2500,13 +2500,13 @@
         </is>
       </c>
       <c r="B14" t="n">
-        <v>979</v>
+        <v>997</v>
       </c>
       <c r="C14" s="2" t="n">
-        <v>0.8897</v>
+        <v>0.8917</v>
       </c>
       <c r="D14" s="2" t="n">
-        <v>0.9928</v>
+        <v>0.993</v>
       </c>
     </row>
     <row r="15">
@@ -2516,13 +2516,13 @@
         </is>
       </c>
       <c r="B15" t="n">
-        <v>1025</v>
+        <v>1045</v>
       </c>
       <c r="C15" s="2" t="n">
-        <v>0.8849</v>
+        <v>0.8871</v>
       </c>
       <c r="D15" s="2" t="n">
-        <v>0.9942</v>
+        <v>0.994</v>
       </c>
     </row>
     <row r="16">
@@ -2532,13 +2532,13 @@
         </is>
       </c>
       <c r="B16" t="n">
-        <v>1072</v>
+        <v>1088</v>
       </c>
       <c r="C16" s="2" t="n">
-        <v>0.8965</v>
+        <v>0.898</v>
       </c>
       <c r="D16" s="2" t="n">
-        <v>0.9949</v>
+        <v>0.9951</v>
       </c>
     </row>
     <row r="17">
@@ -2548,13 +2548,13 @@
         </is>
       </c>
       <c r="B17" t="n">
-        <v>1013</v>
+        <v>1035</v>
       </c>
       <c r="C17" s="2" t="n">
-        <v>0.8806</v>
+        <v>0.8821</v>
       </c>
       <c r="D17" s="2" t="n">
-        <v>0.9945000000000001</v>
+        <v>0.9943</v>
       </c>
     </row>
     <row r="18">
@@ -2564,13 +2564,13 @@
         </is>
       </c>
       <c r="B18" t="n">
-        <v>1113</v>
+        <v>1138</v>
       </c>
       <c r="C18" s="2" t="n">
-        <v>0.8688</v>
+        <v>0.8708</v>
       </c>
       <c r="D18" s="2" t="n">
-        <v>0.9963</v>
+        <v>0.9962</v>
       </c>
     </row>
     <row r="19">
@@ -2580,13 +2580,13 @@
         </is>
       </c>
       <c r="B19" t="n">
-        <v>1010</v>
+        <v>1027</v>
       </c>
       <c r="C19" s="2" t="n">
-        <v>0.8673</v>
+        <v>0.8695000000000001</v>
       </c>
       <c r="D19" s="2" t="n">
-        <v>0.9956</v>
+        <v>0.9958</v>
       </c>
     </row>
     <row r="20">
@@ -2596,13 +2596,13 @@
         </is>
       </c>
       <c r="B20" t="n">
-        <v>936</v>
+        <v>951</v>
       </c>
       <c r="C20" s="2" t="n">
-        <v>0.8515</v>
+        <v>0.8538</v>
       </c>
       <c r="D20" s="2" t="n">
-        <v>0.997</v>
+        <v>0.9966</v>
       </c>
     </row>
     <row r="21">
@@ -2612,13 +2612,13 @@
         </is>
       </c>
       <c r="B21" t="n">
-        <v>932</v>
+        <v>955</v>
       </c>
       <c r="C21" s="2" t="n">
-        <v>0.8562</v>
+        <v>0.8597</v>
       </c>
       <c r="D21" s="2" t="n">
-        <v>0.9951</v>
+        <v>0.9954</v>
       </c>
     </row>
     <row r="22">
@@ -2628,13 +2628,13 @@
         </is>
       </c>
       <c r="B22" t="n">
-        <v>1058</v>
+        <v>1080</v>
       </c>
       <c r="C22" s="2" t="n">
-        <v>0.8573</v>
+        <v>0.8602</v>
       </c>
       <c r="D22" s="2" t="n">
-        <v>0.9959</v>
+        <v>0.9954</v>
       </c>
     </row>
     <row r="23">
@@ -2644,13 +2644,13 @@
         </is>
       </c>
       <c r="B23" t="n">
-        <v>999</v>
+        <v>1019</v>
       </c>
       <c r="C23" s="2" t="n">
-        <v>0.9149</v>
+        <v>0.9156</v>
       </c>
       <c r="D23" s="2" t="n">
-        <v>0.9911</v>
+        <v>0.9913999999999999</v>
       </c>
     </row>
     <row r="24">
@@ -2660,13 +2660,13 @@
         </is>
       </c>
       <c r="B24" t="n">
-        <v>864</v>
+        <v>882</v>
       </c>
       <c r="C24" s="2" t="n">
-        <v>0.8715000000000001</v>
+        <v>0.8719</v>
       </c>
       <c r="D24" s="2" t="n">
-        <v>0.9916</v>
+        <v>0.9917</v>
       </c>
     </row>
     <row r="25">
@@ -2676,13 +2676,13 @@
         </is>
       </c>
       <c r="B25" t="n">
-        <v>1048</v>
+        <v>1068</v>
       </c>
       <c r="C25" s="2" t="n">
-        <v>0.9504</v>
+        <v>0.9513</v>
       </c>
       <c r="D25" s="2" t="n">
-        <v>0.9942</v>
+        <v>0.9946</v>
       </c>
     </row>
     <row r="26">
@@ -2692,13 +2692,13 @@
         </is>
       </c>
       <c r="B26" t="n">
-        <v>859</v>
+        <v>877</v>
       </c>
       <c r="C26" s="2" t="n">
-        <v>0.8987000000000001</v>
+        <v>0.8997000000000001</v>
       </c>
       <c r="D26" s="2" t="n">
-        <v>0.9893999999999999</v>
+        <v>0.9897</v>
       </c>
     </row>
     <row r="27">
@@ -2708,13 +2708,13 @@
         </is>
       </c>
       <c r="B27" t="n">
-        <v>922</v>
+        <v>956</v>
       </c>
       <c r="C27" s="2" t="n">
-        <v>0.9295</v>
+        <v>0.9288999999999999</v>
       </c>
       <c r="D27" s="2" t="n">
-        <v>0.99</v>
+        <v>0.9897</v>
       </c>
     </row>
     <row r="28">
@@ -2724,13 +2724,13 @@
         </is>
       </c>
       <c r="B28" t="n">
-        <v>861</v>
+        <v>868</v>
       </c>
       <c r="C28" s="2" t="n">
-        <v>0.9048</v>
+        <v>0.9032</v>
       </c>
       <c r="D28" s="2" t="n">
-        <v>0.9893999999999999</v>
+        <v>0.9895</v>
       </c>
     </row>
     <row r="29">
@@ -2740,13 +2740,13 @@
         </is>
       </c>
       <c r="B29" t="n">
-        <v>894</v>
+        <v>929</v>
       </c>
       <c r="C29" s="2" t="n">
-        <v>0.9094</v>
+        <v>0.9127999999999999</v>
       </c>
       <c r="D29" s="2" t="n">
-        <v>0.9931</v>
+        <v>0.9923999999999999</v>
       </c>
     </row>
     <row r="30">
@@ -2756,13 +2756,13 @@
         </is>
       </c>
       <c r="B30" t="n">
-        <v>956</v>
+        <v>992</v>
       </c>
       <c r="C30" s="2" t="n">
-        <v>0.8902</v>
+        <v>0.8921</v>
       </c>
       <c r="D30" s="2" t="n">
-        <v>0.9922</v>
+        <v>0.991</v>
       </c>
     </row>
     <row r="31">
@@ -2772,13 +2772,13 @@
         </is>
       </c>
       <c r="B31" t="n">
-        <v>1009</v>
+        <v>1039</v>
       </c>
       <c r="C31" s="2" t="n">
-        <v>0.8811</v>
+        <v>0.8826000000000001</v>
       </c>
       <c r="D31" s="2" t="n">
-        <v>0.9935</v>
+        <v>0.9929</v>
       </c>
     </row>
     <row r="32">
@@ -2788,13 +2788,13 @@
         </is>
       </c>
       <c r="B32" t="n">
-        <v>936</v>
+        <v>961</v>
       </c>
       <c r="C32" s="2" t="n">
-        <v>0.8974</v>
+        <v>0.9001</v>
       </c>
       <c r="D32" s="2" t="n">
-        <v>0.9893</v>
+        <v>0.9893999999999999</v>
       </c>
     </row>
     <row r="33">
@@ -2804,13 +2804,13 @@
         </is>
       </c>
       <c r="B33" t="n">
-        <v>731</v>
+        <v>762</v>
       </c>
       <c r="C33" s="2" t="n">
-        <v>0.8933</v>
+        <v>0.8963</v>
       </c>
       <c r="D33" s="2" t="n">
-        <v>0.9921</v>
+        <v>0.9899</v>
       </c>
     </row>
     <row r="34">
@@ -2820,13 +2820,13 @@
         </is>
       </c>
       <c r="B34" t="n">
-        <v>952</v>
+        <v>972</v>
       </c>
       <c r="C34" s="2" t="n">
-        <v>0.9254</v>
+        <v>0.927</v>
       </c>
       <c r="D34" s="2" t="n">
-        <v>0.9918</v>
+        <v>0.9923</v>
       </c>
     </row>
     <row r="35">
@@ -2836,13 +2836,13 @@
         </is>
       </c>
       <c r="B35" t="n">
-        <v>1006</v>
+        <v>1037</v>
       </c>
       <c r="C35" s="2" t="n">
-        <v>0.8728</v>
+        <v>0.8756</v>
       </c>
       <c r="D35" s="2" t="n">
-        <v>0.9941</v>
+        <v>0.9937</v>
       </c>
     </row>
     <row r="36">
@@ -2852,13 +2852,13 @@
         </is>
       </c>
       <c r="B36" t="n">
-        <v>796</v>
+        <v>822</v>
       </c>
       <c r="C36" s="2" t="n">
-        <v>0.9171</v>
+        <v>0.9185</v>
       </c>
       <c r="D36" s="2" t="n">
-        <v>0.9883</v>
+        <v>0.9877</v>
       </c>
     </row>
     <row r="37">
@@ -2868,13 +2868,13 @@
         </is>
       </c>
       <c r="B37" t="n">
-        <v>839</v>
+        <v>860</v>
       </c>
       <c r="C37" s="2" t="n">
-        <v>0.8927</v>
+        <v>0.8953</v>
       </c>
       <c r="D37" s="2" t="n">
-        <v>0.9938</v>
+        <v>0.9937</v>
       </c>
     </row>
     <row r="38">
@@ -2884,13 +2884,13 @@
         </is>
       </c>
       <c r="B38" t="n">
-        <v>1022</v>
+        <v>1053</v>
       </c>
       <c r="C38" s="2" t="n">
-        <v>0.9177999999999999</v>
+        <v>0.9202</v>
       </c>
       <c r="D38" s="2" t="n">
-        <v>0.9917</v>
+        <v>0.9918</v>
       </c>
     </row>
     <row r="39">
@@ -2900,13 +2900,13 @@
         </is>
       </c>
       <c r="B39" t="n">
-        <v>806</v>
+        <v>829</v>
       </c>
       <c r="C39" s="2" t="n">
-        <v>0.8821</v>
+        <v>0.8842</v>
       </c>
       <c r="D39" s="2" t="n">
-        <v>0.9918</v>
+        <v>0.9913999999999999</v>
       </c>
     </row>
   </sheetData>
@@ -2970,19 +2970,19 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>0.1277</v>
+        <v>0.1262</v>
       </c>
       <c r="C2" t="n">
-        <v>0.119</v>
+        <v>0.1184</v>
       </c>
       <c r="D2" t="n">
-        <v>0.0002</v>
+        <v>0.0005999999999999999</v>
       </c>
       <c r="E2" t="n">
-        <v>1.0569</v>
+        <v>1.053</v>
       </c>
       <c r="F2" t="n">
-        <v>0.074</v>
+        <v>0.0741</v>
       </c>
     </row>
     <row r="3">
@@ -2992,19 +2992,19 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>0.1248</v>
+        <v>0.1235</v>
       </c>
       <c r="C3" t="n">
-        <v>0.1129</v>
+        <v>0.1125</v>
       </c>
       <c r="D3" t="n">
-        <v>-0.005</v>
+        <v>-0.0039</v>
       </c>
       <c r="E3" t="n">
-        <v>1.0706</v>
+        <v>1.0497</v>
       </c>
       <c r="F3" t="n">
-        <v>0.0805</v>
+        <v>0.081</v>
       </c>
     </row>
     <row r="4">
@@ -3014,16 +3014,16 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>0.044</v>
+        <v>0.0437</v>
       </c>
       <c r="C4" t="n">
         <v>0.0395</v>
       </c>
       <c r="D4" t="n">
-        <v>0.1188</v>
+        <v>0.1185</v>
       </c>
       <c r="E4" t="n">
-        <v>0.9935</v>
+        <v>0.9966</v>
       </c>
       <c r="F4" t="n">
         <v>0.0622</v>
@@ -3055,7 +3055,7 @@
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>2026-08-11T09:39:37+00:00</t>
+          <t>2026-08-13T09:14:08+00:00</t>
         </is>
       </c>
     </row>
@@ -3066,7 +3066,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>4286</v>
+        <v>4400</v>
       </c>
     </row>
     <row r="3">
@@ -3076,7 +3076,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>113</v>
+        <v>116</v>
       </c>
     </row>
     <row r="4">

</xml_diff>

<commit_message>
Arquiva dados, recalibra e atualiza docs (2026-08-16)
</commit_message>
<xml_diff>
--- a/backtest_results/resultados_backtest.xlsx
+++ b/backtest_results/resultados_backtest.xlsx
@@ -516,28 +516,28 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>393</v>
+        <v>406</v>
       </c>
       <c r="C2" s="2" t="n">
-        <v>0.8829516539440203</v>
+        <v>0.8817733990147784</v>
       </c>
       <c r="D2" s="3" t="n">
-        <v>6.170987216982523</v>
+        <v>6.459970248427571</v>
       </c>
       <c r="E2" s="4" t="n">
-        <v>108.5707361553694</v>
+        <v>138.0515286908054</v>
       </c>
       <c r="F2" s="2" t="n">
-        <v>2.361069119863112</v>
+        <v>2.463428209490314</v>
       </c>
       <c r="G2" s="2" t="n">
         <v>0.3059017866796615</v>
       </c>
       <c r="H2" t="n">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="I2" s="3" t="n">
-        <v>0.8081094147582697</v>
+        <v>0.806076354679803</v>
       </c>
     </row>
     <row r="3">
@@ -547,19 +547,19 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>1809</v>
+        <v>1870</v>
       </c>
       <c r="C3" s="2" t="n">
-        <v>0.9928137092316197</v>
+        <v>0.993048128342246</v>
       </c>
       <c r="D3" s="3" t="n">
-        <v>1.999446258407061</v>
+        <v>2.090463989889831</v>
       </c>
       <c r="E3" s="4" t="n">
-        <v>2.982231980851253</v>
+        <v>3.132793327630674</v>
       </c>
       <c r="F3" s="2" t="n">
-        <v>0.3265579606000797</v>
+        <v>0.333597613678595</v>
       </c>
       <c r="G3" s="2" t="n">
         <v>0.07901949101919936</v>
@@ -568,7 +568,7 @@
         <v>38</v>
       </c>
       <c r="I3" s="3" t="n">
-        <v>0.9856779988944168</v>
+        <v>0.9856676470588235</v>
       </c>
     </row>
     <row r="4">
@@ -578,19 +578,19 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>1318</v>
+        <v>1358</v>
       </c>
       <c r="C4" s="2" t="n">
-        <v>0.9946889226100152</v>
+        <v>0.9948453608247423</v>
       </c>
       <c r="D4" s="3" t="n">
-        <v>1.436865517384735</v>
+        <v>1.490314975974403</v>
       </c>
       <c r="E4" s="4" t="n">
-        <v>2.500419900830992</v>
+        <v>2.588333286910503</v>
       </c>
       <c r="F4" s="2" t="n">
-        <v>0.2674603518109306</v>
+        <v>0.2709332414341799</v>
       </c>
       <c r="G4" s="2" t="n">
         <v>0.07313459803799172</v>
@@ -599,7 +599,7 @@
         <v>22</v>
       </c>
       <c r="I4" s="3" t="n">
-        <v>0.9865083459787557</v>
+        <v>0.986519145802651</v>
       </c>
     </row>
     <row r="5">
@@ -609,19 +609,19 @@
         </is>
       </c>
       <c r="B5" s="5" t="n">
-        <v>696</v>
+        <v>718</v>
       </c>
       <c r="C5" s="6" t="n">
-        <v>0.9985632183908046</v>
+        <v>0.9986072423398329</v>
       </c>
       <c r="D5" s="7" t="n">
-        <v>0.8035315105952537</v>
+        <v>0.8316523566005093</v>
       </c>
       <c r="E5" s="8" t="n">
-        <v>1.883070576824799</v>
+        <v>1.925451863494174</v>
       </c>
       <c r="F5" s="6" t="n">
-        <v>0.1778397014998288</v>
+        <v>0.1795895707681392</v>
       </c>
       <c r="G5" s="6" t="n">
         <v>0.02619857308701179</v>
@@ -630,7 +630,7 @@
         <v>6</v>
       </c>
       <c r="I5" s="7" t="n">
-        <v>0.9872514367816093</v>
+        <v>0.9872569637883009</v>
       </c>
     </row>
     <row r="6">
@@ -640,34 +640,34 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>1089</v>
+        <v>1124</v>
       </c>
       <c r="C6" s="2" t="n">
-        <v>0.9568411386593205</v>
+        <v>0.9564056939501779</v>
       </c>
       <c r="D6" s="3" t="n">
-        <v>6.974518727577776</v>
+        <v>7.29162260502808</v>
       </c>
       <c r="E6" s="4" t="n">
-        <v>117.6336736923698</v>
+        <v>148.4552533035217</v>
       </c>
       <c r="F6" s="2" t="n">
-        <v>2.43148674708239</v>
+        <v>2.527451637528832</v>
       </c>
       <c r="G6" s="2" t="n">
         <v>0.2893750111453259</v>
       </c>
       <c r="H6" t="n">
-        <v>86</v>
+        <v>88</v>
       </c>
       <c r="I6" s="3" t="n">
-        <v>0.9226023875114785</v>
+        <v>0.9218127224199288</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Atualizado em 2026-08-13T09:14:08+00:00 · arquivo de 4400 dias-cidade (~116 dias corridos) · 38 cidades</t>
+          <t>Atualizado em 2026-08-16T09:13:23+00:00 · arquivo de 4514 dias-cidade (~119 dias corridos) · 38 cidades</t>
         </is>
       </c>
     </row>
@@ -822,13 +822,13 @@
         </is>
       </c>
       <c r="C6" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="D6" s="2" t="n">
-        <v>0.9285714285714286</v>
+        <v>0.9333333333333333</v>
       </c>
       <c r="E6" s="3" t="n">
-        <v>0.05183875767161625</v>
+        <v>0.08976979215437488</v>
       </c>
     </row>
     <row r="7">
@@ -906,13 +906,13 @@
         </is>
       </c>
       <c r="C10" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="D10" s="2" t="n">
         <v>1</v>
       </c>
       <c r="E10" s="3" t="n">
-        <v>0.08075556783620651</v>
+        <v>0.1398271598597436</v>
       </c>
     </row>
     <row r="11">
@@ -969,13 +969,13 @@
         </is>
       </c>
       <c r="C13" t="n">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="D13" s="2" t="n">
-        <v>0.8421052631578947</v>
+        <v>0.8095238095238095</v>
       </c>
       <c r="E13" s="3" t="n">
-        <v>0.3374431186685581</v>
+        <v>0.4099163061417456</v>
       </c>
     </row>
     <row r="14">
@@ -1200,13 +1200,13 @@
         </is>
       </c>
       <c r="C24" t="n">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="D24" s="2" t="n">
-        <v>0.9565217391304348</v>
+        <v>0.9583333333333334</v>
       </c>
       <c r="E24" s="3" t="n">
-        <v>0.2916596476873091</v>
+        <v>0.2974797535074149</v>
       </c>
     </row>
     <row r="25">
@@ -1221,13 +1221,13 @@
         </is>
       </c>
       <c r="C25" t="n">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="D25" s="2" t="n">
-        <v>0.8275862068965517</v>
+        <v>0.8333333333333334</v>
       </c>
       <c r="E25" s="3" t="n">
-        <v>0.2933607142431768</v>
+        <v>0.3168175043666336</v>
       </c>
     </row>
     <row r="26">
@@ -1242,13 +1242,13 @@
         </is>
       </c>
       <c r="C26" t="n">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="D26" s="2" t="n">
-        <v>0.8888888888888888</v>
+        <v>0.8421052631578947</v>
       </c>
       <c r="E26" s="3" t="n">
-        <v>0.1451882599574397</v>
+        <v>0.1301882599574397</v>
       </c>
     </row>
     <row r="27">
@@ -1263,13 +1263,13 @@
         </is>
       </c>
       <c r="C27" t="n">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="D27" s="2" t="n">
         <v>1</v>
       </c>
       <c r="E27" s="3" t="n">
-        <v>1.132460979000862</v>
+        <v>1.161062265699533</v>
       </c>
     </row>
     <row r="28">
@@ -1284,13 +1284,13 @@
         </is>
       </c>
       <c r="C28" t="n">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="D28" s="2" t="n">
-        <v>0.9090909090909091</v>
+        <v>0.9117647058823529</v>
       </c>
       <c r="E28" s="3" t="n">
-        <v>1.069571862761213</v>
+        <v>1.080682973872324</v>
       </c>
     </row>
     <row r="29">
@@ -1353,7 +1353,7 @@
         <v>1</v>
       </c>
       <c r="E31" s="3" t="n">
-        <v>0.07820345241955598</v>
+        <v>0.08205930778991248</v>
       </c>
     </row>
     <row r="32">
@@ -1410,13 +1410,13 @@
         </is>
       </c>
       <c r="C34" t="n">
-        <v>17</v>
+        <v>19</v>
       </c>
       <c r="D34" s="2" t="n">
-        <v>0.8823529411764706</v>
+        <v>0.8947368421052632</v>
       </c>
       <c r="E34" s="3" t="n">
-        <v>0.4393706852539215</v>
+        <v>0.4977156372755733</v>
       </c>
     </row>
     <row r="35">
@@ -1437,7 +1437,7 @@
         <v>0.8947368421052632</v>
       </c>
       <c r="E35" s="3" t="n">
-        <v>0.4175399346554238</v>
+        <v>0.420857050975636</v>
       </c>
     </row>
     <row r="36">
@@ -1536,13 +1536,13 @@
         </is>
       </c>
       <c r="C40" t="n">
-        <v>34</v>
+        <v>38</v>
       </c>
       <c r="D40" s="2" t="n">
         <v>1</v>
       </c>
       <c r="E40" s="3" t="n">
-        <v>0.1175650646125702</v>
+        <v>0.1214041311470947</v>
       </c>
     </row>
     <row r="41">
@@ -1578,13 +1578,13 @@
         </is>
       </c>
       <c r="C42" t="n">
-        <v>62</v>
+        <v>65</v>
       </c>
       <c r="D42" s="2" t="n">
-        <v>0.9838709677419355</v>
+        <v>0.9846153846153847</v>
       </c>
       <c r="E42" s="3" t="n">
-        <v>0.09960525579400151</v>
+        <v>0.1394545648489197</v>
       </c>
     </row>
     <row r="43">
@@ -1662,13 +1662,13 @@
         </is>
       </c>
       <c r="C46" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="D46" s="2" t="n">
         <v>1</v>
       </c>
       <c r="E46" s="3" t="n">
-        <v>0.08135918956658879</v>
+        <v>0.1404307815901259</v>
       </c>
     </row>
     <row r="47">
@@ -1725,13 +1725,13 @@
         </is>
       </c>
       <c r="C49" t="n">
-        <v>30</v>
+        <v>32</v>
       </c>
       <c r="D49" s="2" t="n">
-        <v>0.9</v>
+        <v>0.875</v>
       </c>
       <c r="E49" s="3" t="n">
-        <v>0.3486376110826856</v>
+        <v>0.421110798555873</v>
       </c>
     </row>
     <row r="50">
@@ -1788,13 +1788,13 @@
         </is>
       </c>
       <c r="C52" t="n">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="D52" s="2" t="n">
         <v>1</v>
       </c>
       <c r="E52" s="3" t="n">
-        <v>0.04882444083797849</v>
+        <v>0.05090032520708471</v>
       </c>
     </row>
     <row r="53">
@@ -1914,13 +1914,13 @@
         </is>
       </c>
       <c r="C58" t="n">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="D58" s="2" t="n">
-        <v>0.9220779220779221</v>
+        <v>0.9230769230769231</v>
       </c>
       <c r="E58" s="3" t="n">
-        <v>0.05522417844390874</v>
+        <v>0.05789358296136255</v>
       </c>
     </row>
     <row r="59">
@@ -1977,13 +1977,13 @@
         </is>
       </c>
       <c r="C61" t="n">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="D61" s="2" t="n">
-        <v>0.9696969696969697</v>
+        <v>0.9705882352941176</v>
       </c>
       <c r="E61" s="3" t="n">
-        <v>0.3042322580486544</v>
+        <v>0.3100523638687603</v>
       </c>
     </row>
     <row r="62">
@@ -1998,13 +1998,13 @@
         </is>
       </c>
       <c r="C62" t="n">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="D62" s="2" t="n">
-        <v>0.9152542372881356</v>
+        <v>0.9166666666666666</v>
       </c>
       <c r="E62" s="3" t="n">
-        <v>0.3298194126683207</v>
+        <v>0.3532762027917775</v>
       </c>
     </row>
     <row r="63">
@@ -2019,13 +2019,13 @@
         </is>
       </c>
       <c r="C63" t="n">
-        <v>26</v>
+        <v>29</v>
       </c>
       <c r="D63" s="2" t="n">
-        <v>0.9230769230769231</v>
+        <v>0.896551724137931</v>
       </c>
       <c r="E63" s="3" t="n">
-        <v>0.1538070461009067</v>
+        <v>0.1408291032364176</v>
       </c>
     </row>
     <row r="64">
@@ -2040,13 +2040,13 @@
         </is>
       </c>
       <c r="C64" t="n">
-        <v>68</v>
+        <v>70</v>
       </c>
       <c r="D64" s="2" t="n">
         <v>1</v>
       </c>
       <c r="E64" s="3" t="n">
-        <v>1.135132844587386</v>
+        <v>1.163734131286057</v>
       </c>
     </row>
     <row r="65">
@@ -2061,13 +2061,13 @@
         </is>
       </c>
       <c r="C65" t="n">
-        <v>58</v>
+        <v>62</v>
       </c>
       <c r="D65" s="2" t="n">
-        <v>0.9482758620689655</v>
+        <v>0.9516129032258065</v>
       </c>
       <c r="E65" s="3" t="n">
-        <v>1.088215444802068</v>
+        <v>1.107128487947707</v>
       </c>
     </row>
     <row r="66">
@@ -2082,13 +2082,13 @@
         </is>
       </c>
       <c r="C66" t="n">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="D66" s="2" t="n">
         <v>1</v>
       </c>
       <c r="E66" s="3" t="n">
-        <v>0.1942552138828612</v>
+        <v>0.1957780565224551</v>
       </c>
     </row>
     <row r="67">
@@ -2103,13 +2103,13 @@
         </is>
       </c>
       <c r="C67" t="n">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="D67" s="2" t="n">
         <v>1</v>
       </c>
       <c r="E67" s="3" t="n">
-        <v>0.4400190537980967</v>
+        <v>0.4414903881461434</v>
       </c>
     </row>
     <row r="68">
@@ -2124,13 +2124,13 @@
         </is>
       </c>
       <c r="C68" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="D68" s="2" t="n">
         <v>1</v>
       </c>
       <c r="E68" s="3" t="n">
-        <v>0.083921006625001</v>
+        <v>0.08832990372486982</v>
       </c>
     </row>
     <row r="69">
@@ -2166,13 +2166,13 @@
         </is>
       </c>
       <c r="C70" t="n">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="D70" s="2" t="n">
         <v>1</v>
       </c>
       <c r="E70" s="3" t="n">
-        <v>0.105030430626852</v>
+        <v>0.1068629009192208</v>
       </c>
     </row>
     <row r="71">
@@ -2187,13 +2187,13 @@
         </is>
       </c>
       <c r="C71" t="n">
-        <v>42</v>
+        <v>46</v>
       </c>
       <c r="D71" s="2" t="n">
-        <v>0.9523809523809523</v>
+        <v>0.9565217391304348</v>
       </c>
       <c r="E71" s="3" t="n">
-        <v>0.4761634770379517</v>
+        <v>0.5357156725203681</v>
       </c>
     </row>
     <row r="72">
@@ -2208,13 +2208,13 @@
         </is>
       </c>
       <c r="C72" t="n">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="D72" s="2" t="n">
-        <v>0.9615384615384616</v>
+        <v>0.9622641509433962</v>
       </c>
       <c r="E72" s="3" t="n">
-        <v>0.4611517951194642</v>
+        <v>0.4651231640818506</v>
       </c>
     </row>
     <row r="73">
@@ -2229,13 +2229,13 @@
         </is>
       </c>
       <c r="C73" t="n">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="D73" s="2" t="n">
-        <v>0.9696969696969697</v>
+        <v>0.9705882352941176</v>
       </c>
       <c r="E73" s="3" t="n">
-        <v>0.163537343820718</v>
+        <v>0.1640903855502303</v>
       </c>
     </row>
     <row r="74">
@@ -2308,10 +2308,10 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>918</v>
+        <v>924</v>
       </c>
       <c r="C2" s="2" t="n">
-        <v>0.8856000000000001</v>
+        <v>0.8864</v>
       </c>
       <c r="D2" s="2" t="n">
         <v>0.9915</v>
@@ -2324,13 +2324,13 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>978</v>
+        <v>992</v>
       </c>
       <c r="C3" s="2" t="n">
-        <v>0.8558</v>
+        <v>0.8579</v>
       </c>
       <c r="D3" s="2" t="n">
-        <v>0.997</v>
+        <v>0.9968</v>
       </c>
     </row>
     <row r="4">
@@ -2340,13 +2340,13 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>923</v>
+        <v>943</v>
       </c>
       <c r="C4" s="2" t="n">
-        <v>0.8819</v>
+        <v>0.8855</v>
       </c>
       <c r="D4" s="2" t="n">
-        <v>0.9927</v>
+        <v>0.9925</v>
       </c>
     </row>
     <row r="5">
@@ -2356,13 +2356,13 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>1021</v>
+        <v>1036</v>
       </c>
       <c r="C5" s="2" t="n">
-        <v>0.8825</v>
+        <v>0.8842</v>
       </c>
       <c r="D5" s="2" t="n">
-        <v>0.9932</v>
+        <v>0.9931</v>
       </c>
     </row>
     <row r="6">
@@ -2372,13 +2372,13 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>1085</v>
+        <v>1106</v>
       </c>
       <c r="C6" s="2" t="n">
-        <v>0.8912</v>
+        <v>0.8933</v>
       </c>
       <c r="D6" s="2" t="n">
-        <v>0.994</v>
+        <v>0.9936</v>
       </c>
     </row>
     <row r="7">
@@ -2388,13 +2388,13 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>1060</v>
+        <v>1075</v>
       </c>
       <c r="C7" s="2" t="n">
-        <v>0.8802</v>
+        <v>0.8819</v>
       </c>
       <c r="D7" s="2" t="n">
-        <v>0.9955000000000001</v>
+        <v>0.9954</v>
       </c>
     </row>
     <row r="8">
@@ -2404,13 +2404,13 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>852</v>
+        <v>859</v>
       </c>
       <c r="C8" s="2" t="n">
-        <v>0.8944</v>
+        <v>0.8952</v>
       </c>
       <c r="D8" s="2" t="n">
-        <v>0.9915</v>
+        <v>0.9913999999999999</v>
       </c>
     </row>
     <row r="9">
@@ -2420,13 +2420,13 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>1076</v>
+        <v>1085</v>
       </c>
       <c r="C9" s="2" t="n">
-        <v>0.8652</v>
+        <v>0.8663999999999999</v>
       </c>
       <c r="D9" s="2" t="n">
-        <v>0.9951</v>
+        <v>0.995</v>
       </c>
     </row>
     <row r="10">
@@ -2436,13 +2436,13 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>1079</v>
+        <v>1099</v>
       </c>
       <c r="C10" s="2" t="n">
-        <v>0.8758</v>
+        <v>0.8781</v>
       </c>
       <c r="D10" s="2" t="n">
-        <v>0.9968</v>
+        <v>0.9965000000000001</v>
       </c>
     </row>
     <row r="11">
@@ -2452,13 +2452,13 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>1001</v>
+        <v>1012</v>
       </c>
       <c r="C11" s="2" t="n">
-        <v>0.9001</v>
+        <v>0.9012</v>
       </c>
       <c r="D11" s="2" t="n">
-        <v>0.9943</v>
+        <v>0.9944</v>
       </c>
     </row>
     <row r="12">
@@ -2468,13 +2468,13 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>1025</v>
+        <v>1039</v>
       </c>
       <c r="C12" s="2" t="n">
-        <v>0.8946</v>
+        <v>0.8961</v>
       </c>
       <c r="D12" s="2" t="n">
-        <v>0.9932</v>
+        <v>0.9928</v>
       </c>
     </row>
     <row r="13">
@@ -2484,13 +2484,13 @@
         </is>
       </c>
       <c r="B13" t="n">
-        <v>954</v>
+        <v>985</v>
       </c>
       <c r="C13" s="2" t="n">
-        <v>0.9465</v>
+        <v>0.9472</v>
       </c>
       <c r="D13" s="2" t="n">
-        <v>0.9841</v>
+        <v>0.9836</v>
       </c>
     </row>
     <row r="14">
@@ -2500,13 +2500,13 @@
         </is>
       </c>
       <c r="B14" t="n">
-        <v>997</v>
+        <v>1011</v>
       </c>
       <c r="C14" s="2" t="n">
-        <v>0.8917</v>
+        <v>0.8932</v>
       </c>
       <c r="D14" s="2" t="n">
-        <v>0.993</v>
+        <v>0.9927</v>
       </c>
     </row>
     <row r="15">
@@ -2516,13 +2516,13 @@
         </is>
       </c>
       <c r="B15" t="n">
-        <v>1045</v>
+        <v>1066</v>
       </c>
       <c r="C15" s="2" t="n">
-        <v>0.8871</v>
+        <v>0.8893</v>
       </c>
       <c r="D15" s="2" t="n">
-        <v>0.994</v>
+        <v>0.9936</v>
       </c>
     </row>
     <row r="16">
@@ -2532,13 +2532,13 @@
         </is>
       </c>
       <c r="B16" t="n">
-        <v>1088</v>
+        <v>1110</v>
       </c>
       <c r="C16" s="2" t="n">
-        <v>0.898</v>
+        <v>0.9</v>
       </c>
       <c r="D16" s="2" t="n">
-        <v>0.9951</v>
+        <v>0.9947</v>
       </c>
     </row>
     <row r="17">
@@ -2548,10 +2548,10 @@
         </is>
       </c>
       <c r="B17" t="n">
-        <v>1035</v>
+        <v>1048</v>
       </c>
       <c r="C17" s="2" t="n">
-        <v>0.8821</v>
+        <v>0.8826000000000001</v>
       </c>
       <c r="D17" s="2" t="n">
         <v>0.9943</v>
@@ -2564,13 +2564,13 @@
         </is>
       </c>
       <c r="B18" t="n">
-        <v>1138</v>
+        <v>1158</v>
       </c>
       <c r="C18" s="2" t="n">
-        <v>0.8708</v>
+        <v>0.8722</v>
       </c>
       <c r="D18" s="2" t="n">
-        <v>0.9962</v>
+        <v>0.9959</v>
       </c>
     </row>
     <row r="19">
@@ -2580,13 +2580,13 @@
         </is>
       </c>
       <c r="B19" t="n">
-        <v>1027</v>
+        <v>1042</v>
       </c>
       <c r="C19" s="2" t="n">
-        <v>0.8695000000000001</v>
+        <v>0.8714</v>
       </c>
       <c r="D19" s="2" t="n">
-        <v>0.9958</v>
+        <v>0.9957</v>
       </c>
     </row>
     <row r="20">
@@ -2596,13 +2596,13 @@
         </is>
       </c>
       <c r="B20" t="n">
-        <v>951</v>
+        <v>961</v>
       </c>
       <c r="C20" s="2" t="n">
-        <v>0.8538</v>
+        <v>0.8554</v>
       </c>
       <c r="D20" s="2" t="n">
-        <v>0.9966</v>
+        <v>0.9963</v>
       </c>
     </row>
     <row r="21">
@@ -2612,13 +2612,13 @@
         </is>
       </c>
       <c r="B21" t="n">
-        <v>955</v>
+        <v>974</v>
       </c>
       <c r="C21" s="2" t="n">
-        <v>0.8597</v>
+        <v>0.8624000000000001</v>
       </c>
       <c r="D21" s="2" t="n">
-        <v>0.9954</v>
+        <v>0.9951</v>
       </c>
     </row>
     <row r="22">
@@ -2628,13 +2628,13 @@
         </is>
       </c>
       <c r="B22" t="n">
-        <v>1080</v>
+        <v>1093</v>
       </c>
       <c r="C22" s="2" t="n">
-        <v>0.8602</v>
+        <v>0.8618</v>
       </c>
       <c r="D22" s="2" t="n">
-        <v>0.9954</v>
+        <v>0.9953</v>
       </c>
     </row>
     <row r="23">
@@ -2644,13 +2644,13 @@
         </is>
       </c>
       <c r="B23" t="n">
-        <v>1019</v>
+        <v>1044</v>
       </c>
       <c r="C23" s="2" t="n">
-        <v>0.9156</v>
+        <v>0.9176</v>
       </c>
       <c r="D23" s="2" t="n">
-        <v>0.9913999999999999</v>
+        <v>0.9913</v>
       </c>
     </row>
     <row r="24">
@@ -2660,13 +2660,13 @@
         </is>
       </c>
       <c r="B24" t="n">
-        <v>882</v>
+        <v>891</v>
       </c>
       <c r="C24" s="2" t="n">
-        <v>0.8719</v>
+        <v>0.8732</v>
       </c>
       <c r="D24" s="2" t="n">
-        <v>0.9917</v>
+        <v>0.9911</v>
       </c>
     </row>
     <row r="25">
@@ -2676,13 +2676,13 @@
         </is>
       </c>
       <c r="B25" t="n">
-        <v>1068</v>
+        <v>1091</v>
       </c>
       <c r="C25" s="2" t="n">
-        <v>0.9513</v>
+        <v>0.9523</v>
       </c>
       <c r="D25" s="2" t="n">
-        <v>0.9946</v>
+        <v>0.9942</v>
       </c>
     </row>
     <row r="26">
@@ -2692,13 +2692,13 @@
         </is>
       </c>
       <c r="B26" t="n">
-        <v>877</v>
+        <v>895</v>
       </c>
       <c r="C26" s="2" t="n">
-        <v>0.8997000000000001</v>
+        <v>0.9016999999999999</v>
       </c>
       <c r="D26" s="2" t="n">
-        <v>0.9897</v>
+        <v>0.9893</v>
       </c>
     </row>
     <row r="27">
@@ -2708,13 +2708,13 @@
         </is>
       </c>
       <c r="B27" t="n">
-        <v>956</v>
+        <v>977</v>
       </c>
       <c r="C27" s="2" t="n">
-        <v>0.9288999999999999</v>
+        <v>0.9304</v>
       </c>
       <c r="D27" s="2" t="n">
-        <v>0.9897</v>
+        <v>0.9891</v>
       </c>
     </row>
     <row r="28">
@@ -2727,10 +2727,10 @@
         <v>868</v>
       </c>
       <c r="C28" s="2" t="n">
-        <v>0.9032</v>
+        <v>0.9021</v>
       </c>
       <c r="D28" s="2" t="n">
-        <v>0.9895</v>
+        <v>0.9892</v>
       </c>
     </row>
     <row r="29">
@@ -2740,13 +2740,13 @@
         </is>
       </c>
       <c r="B29" t="n">
-        <v>929</v>
+        <v>948</v>
       </c>
       <c r="C29" s="2" t="n">
-        <v>0.9127999999999999</v>
+        <v>0.9146</v>
       </c>
       <c r="D29" s="2" t="n">
-        <v>0.9923999999999999</v>
+        <v>0.9919</v>
       </c>
     </row>
     <row r="30">
@@ -2756,13 +2756,13 @@
         </is>
       </c>
       <c r="B30" t="n">
-        <v>992</v>
+        <v>1012</v>
       </c>
       <c r="C30" s="2" t="n">
-        <v>0.8921</v>
+        <v>0.8953</v>
       </c>
       <c r="D30" s="2" t="n">
-        <v>0.991</v>
+        <v>0.9909</v>
       </c>
     </row>
     <row r="31">
@@ -2772,13 +2772,13 @@
         </is>
       </c>
       <c r="B31" t="n">
-        <v>1039</v>
+        <v>1055</v>
       </c>
       <c r="C31" s="2" t="n">
-        <v>0.8826000000000001</v>
+        <v>0.8844</v>
       </c>
       <c r="D31" s="2" t="n">
-        <v>0.9929</v>
+        <v>0.9927</v>
       </c>
     </row>
     <row r="32">
@@ -2788,13 +2788,13 @@
         </is>
       </c>
       <c r="B32" t="n">
-        <v>961</v>
+        <v>975</v>
       </c>
       <c r="C32" s="2" t="n">
-        <v>0.9001</v>
+        <v>0.9015</v>
       </c>
       <c r="D32" s="2" t="n">
-        <v>0.9893999999999999</v>
+        <v>0.9892</v>
       </c>
     </row>
     <row r="33">
@@ -2804,13 +2804,13 @@
         </is>
       </c>
       <c r="B33" t="n">
-        <v>762</v>
+        <v>772</v>
       </c>
       <c r="C33" s="2" t="n">
-        <v>0.8963</v>
+        <v>0.8977000000000001</v>
       </c>
       <c r="D33" s="2" t="n">
-        <v>0.9899</v>
+        <v>0.9898</v>
       </c>
     </row>
     <row r="34">
@@ -2820,13 +2820,13 @@
         </is>
       </c>
       <c r="B34" t="n">
-        <v>972</v>
+        <v>989</v>
       </c>
       <c r="C34" s="2" t="n">
-        <v>0.927</v>
+        <v>0.9282</v>
       </c>
       <c r="D34" s="2" t="n">
-        <v>0.9923</v>
+        <v>0.9921</v>
       </c>
     </row>
     <row r="35">
@@ -2836,13 +2836,13 @@
         </is>
       </c>
       <c r="B35" t="n">
-        <v>1037</v>
+        <v>1049</v>
       </c>
       <c r="C35" s="2" t="n">
-        <v>0.8756</v>
+        <v>0.877</v>
       </c>
       <c r="D35" s="2" t="n">
-        <v>0.9937</v>
+        <v>0.9933999999999999</v>
       </c>
     </row>
     <row r="36">
@@ -2852,13 +2852,13 @@
         </is>
       </c>
       <c r="B36" t="n">
-        <v>822</v>
+        <v>839</v>
       </c>
       <c r="C36" s="2" t="n">
-        <v>0.9185</v>
+        <v>0.919</v>
       </c>
       <c r="D36" s="2" t="n">
-        <v>0.9877</v>
+        <v>0.9874000000000001</v>
       </c>
     </row>
     <row r="37">
@@ -2868,13 +2868,13 @@
         </is>
       </c>
       <c r="B37" t="n">
-        <v>860</v>
+        <v>869</v>
       </c>
       <c r="C37" s="2" t="n">
-        <v>0.8953</v>
+        <v>0.8964</v>
       </c>
       <c r="D37" s="2" t="n">
-        <v>0.9937</v>
+        <v>0.9935</v>
       </c>
     </row>
     <row r="38">
@@ -2884,13 +2884,13 @@
         </is>
       </c>
       <c r="B38" t="n">
-        <v>1053</v>
+        <v>1076</v>
       </c>
       <c r="C38" s="2" t="n">
-        <v>0.9202</v>
+        <v>0.9219000000000001</v>
       </c>
       <c r="D38" s="2" t="n">
-        <v>0.9918</v>
+        <v>0.9916</v>
       </c>
     </row>
     <row r="39">
@@ -2900,13 +2900,13 @@
         </is>
       </c>
       <c r="B39" t="n">
-        <v>829</v>
+        <v>840</v>
       </c>
       <c r="C39" s="2" t="n">
-        <v>0.8842</v>
+        <v>0.8821</v>
       </c>
       <c r="D39" s="2" t="n">
-        <v>0.9913999999999999</v>
+        <v>0.9905</v>
       </c>
     </row>
   </sheetData>
@@ -2970,19 +2970,19 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>0.1262</v>
+        <v>0.1247</v>
       </c>
       <c r="C2" t="n">
-        <v>0.1184</v>
+        <v>0.1177</v>
       </c>
       <c r="D2" t="n">
-        <v>0.0005999999999999999</v>
+        <v>0.0007</v>
       </c>
       <c r="E2" t="n">
-        <v>1.053</v>
+        <v>1.0436</v>
       </c>
       <c r="F2" t="n">
-        <v>0.0741</v>
+        <v>0.07439999999999999</v>
       </c>
     </row>
     <row r="3">
@@ -2992,19 +2992,19 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>0.1235</v>
+        <v>0.1219</v>
       </c>
       <c r="C3" t="n">
-        <v>0.1125</v>
+        <v>0.1119</v>
       </c>
       <c r="D3" t="n">
-        <v>-0.0039</v>
+        <v>-0.0035</v>
       </c>
       <c r="E3" t="n">
-        <v>1.0497</v>
+        <v>1.0389</v>
       </c>
       <c r="F3" t="n">
-        <v>0.081</v>
+        <v>0.0814</v>
       </c>
     </row>
     <row r="4">
@@ -3014,19 +3014,19 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>0.0437</v>
+        <v>0.0433</v>
       </c>
       <c r="C4" t="n">
-        <v>0.0395</v>
+        <v>0.0393</v>
       </c>
       <c r="D4" t="n">
-        <v>0.1185</v>
+        <v>0.1205</v>
       </c>
       <c r="E4" t="n">
-        <v>0.9966</v>
+        <v>1.0004</v>
       </c>
       <c r="F4" t="n">
-        <v>0.0622</v>
+        <v>0.0621</v>
       </c>
     </row>
   </sheetData>
@@ -3055,7 +3055,7 @@
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>2026-08-13T09:14:08+00:00</t>
+          <t>2026-08-16T09:13:23+00:00</t>
         </is>
       </c>
     </row>
@@ -3066,7 +3066,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>4400</v>
+        <v>4514</v>
       </c>
     </row>
     <row r="3">
@@ -3076,7 +3076,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>116</v>
+        <v>119</v>
       </c>
     </row>
     <row r="4">
@@ -3106,7 +3106,7 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>54</v>
+        <v>56</v>
       </c>
     </row>
   </sheetData>

</xml_diff>